<commit_message>
Seccion Noticias sincronizadas desde excel y rediseño de menu princioal 2x2
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -8,21 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\Resurrection Fest 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46E09D60-C65E-44D7-8A88-9019CFBA16C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7EBB27-212F-493A-BC53-AF45B5616BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
+    <workbookView xWindow="3930" yWindow="2535" windowWidth="21600" windowHeight="12645" activeTab="6" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
   </bookViews>
   <sheets>
     <sheet name="Edición" sheetId="1" r:id="rId1"/>
     <sheet name="Artistas" sheetId="2" r:id="rId2"/>
     <sheet name="Actuaciones" sheetId="3" r:id="rId3"/>
     <sheet name="Firmas" sheetId="4" r:id="rId4"/>
-    <sheet name="Escenarios" sheetId="5" r:id="rId5"/>
+    <sheet name="Hoja1" sheetId="6" r:id="rId5"/>
+    <sheet name="Escenarios" sheetId="5" r:id="rId6"/>
+    <sheet name="Noticias" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="2" hidden="1">Actuaciones!$A$1:$F$94</definedName>
     <definedName name="DatosExternos_1" localSheetId="1" hidden="1">Artistas!$A$1:$F$94</definedName>
-    <definedName name="DatosExternos_1" localSheetId="4" hidden="1">Escenarios!$A$1:$D$5</definedName>
+    <definedName name="DatosExternos_1" localSheetId="5" hidden="1">Escenarios!$A$1:$D$5</definedName>
     <definedName name="DatosExternos_1" localSheetId="3" hidden="1">Firmas!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -66,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="459">
   <si>
     <t>ID</t>
   </si>
@@ -1073,9 +1075,6 @@
     <t>DOWN TO SUFFER</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Down to Suffer es una banda joven cántabra de cinco integrantes (Julen, Dabi, Jesús, Mario y Samu) que nace para renovar el proyecto Burning the Waves. Con tres singles publicados, sacan a primeros de 2026 el que es su primer EP "Eclipse"</t>
   </si>
   <si>
@@ -1413,6 +1412,39 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Imagen</t>
+  </si>
+  <si>
+    <t>Noticia</t>
+  </si>
+  <si>
+    <t>https://scontent.fbio3-1.fna.fbcdn.net/v/t39.99422-6/736343148_1348783289919456_2872457055456058256_n.png?stp=dst-jpg_tt6&amp;cstp=mx1080x1350&amp;ctp=s1080x1350&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=scXNdlGehAYQ7kNvwErRBlD&amp;_nc_oc=AdqWCbGf0CGjMl8jaWEgwLj-3mSoGqf8p_cZ5FA1c0Mo_VvvfBhFNvc0BXj_SnjbC_c&amp;_nc_zt=14&amp;_nc_ht=scontent.fbio3-1.fna&amp;_nc_gid=DU5FkyvKhp9xssnjhwmdXg&amp;_nc_ss=7b2a8&amp;oh=00_AQCvNzvgxpKqAcfB1YIdDXCEaeRGLZ36Wd_DE1-yhrrG4A&amp;oe=6A4D9041</t>
+  </si>
+  <si>
+    <t>Horarios de pulseración y Taquillas</t>
+  </si>
+  <si>
+    <t>Entradilla</t>
+  </si>
+  <si>
+    <t>https://scontent.fbio3-1.fna.fbcdn.net/v/t39.99422-6/736349305_1614637920087864_3569990565911515227_n.png?stp=dst-jpg_tt6&amp;cstp=mx1080x1350&amp;ctp=s1080x1350&amp;_nc_cat=102&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=zPmnLukVoIYQ7kNvwE2GiNK&amp;_nc_oc=AdoXqW6ucmn4rG8zsr9Wbq6NaWOSpcL0cK-ZUpbB5FKWzZ9xSkzADoJhPcVePt1eGgQ&amp;_nc_zt=14&amp;_nc_ht=scontent.fbio3-1.fna&amp;_nc_gid=Xbjgn1d33gh-fK7BeNyAVw&amp;_nc_ss=7b2a8&amp;oh=00_AQC3LrvliBlGOGyQ3fcHAarvOe1Y-g-bUU80Kd6FZQK8Ag&amp;oe=6A4D8B54</t>
+  </si>
+  <si>
+    <t>Localización de Taquillas, Pulseras, Incidencias y Recinto</t>
+  </si>
+  <si>
+    <t>https://scontent.fbio3-2.fna.fbcdn.net/v/t39.99422-6/734826776_1435094478510075_4957313761417329896_n.png?stp=dst-jpg_tt6&amp;cstp=mx1080x1350&amp;ctp=s1080x1350&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=bP-Qc4Spn0oQ7kNvwF_qKQ9&amp;_nc_oc=Adpuq1rQ_9CoTNZSFQ143ZiR_t-sVL3bfulg-8WBN9X30EsBoD1V6EM8ZKyx1ki66sk&amp;_nc_zt=14&amp;_nc_ht=scontent.fbio3-2.fna&amp;_nc_gid=To2SavWz1QfhkKPSahpvWQ&amp;_nc_ss=7b2a8&amp;oh=00_AQAwRMUETRoyn2nWrvqMHqjniQ9AYLKAP1vjZXtEM1eGeA&amp;oe=6A4DA47F</t>
+  </si>
+  <si>
+    <t>Buses hasta/desde el recinto</t>
+  </si>
+  <si>
+    <t>El precio del billete por cada trayecto es de 1,60€, excepto la conexión con Vicedo en la que el importe es de 3,20€ por cada viaje.</t>
+  </si>
+  <si>
+    <t>Fecha_noticia</t>
   </si>
 </sst>
 </file>
@@ -1422,7 +1454,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1430,16 +1462,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1447,30 +1499,109 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="26">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="9"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <border outline="0">
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1533,6 +1664,15 @@
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1667,10 +1807,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}" name="Resu_2026_Escenarios" displayName="Resu_2026_Escenarios" ref="A1:D5" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D5" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{F5497620-A4CF-4BD7-A8E7-28E1CF6E3857}" uniqueName="3" name="Orden" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="23"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}" name="Tabla6" displayName="Tabla6" ref="A1:D4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:D4" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}"/>
+  <tableColumns count="4">
+    <tableColumn id="4" xr3:uid="{A9DF3F42-14AF-4444-B7F6-F1AEF4BD9D15}" name="Fecha_noticia"/>
+    <tableColumn id="1" xr3:uid="{ED6D7AFD-A899-4CB1-8175-CE9A81F451C6}" name="Imagen"/>
+    <tableColumn id="2" xr3:uid="{545525B9-095E-43D5-8AE1-AB4557388772}" name="Entradilla"/>
+    <tableColumn id="3" xr3:uid="{DFE6B929-436E-49E7-B1BF-617E4CF938E4}" name="Noticia"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2001,27 +2154,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B1" t="s">
+        <v>439</v>
+      </c>
+      <c r="C1" t="s">
         <v>440</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>441</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>442</v>
       </c>
-      <c r="E1" t="s">
-        <v>443</v>
-      </c>
       <c r="F1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B2">
         <v>2026</v>
@@ -2033,10 +2186,10 @@
         <v>46207</v>
       </c>
       <c r="E2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -2062,7 +2215,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2442,10 +2595,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B20" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C20" t="s">
         <v>14</v>
@@ -3471,161 +3624,161 @@
         <v>14</v>
       </c>
       <c r="D71" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E71" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F71" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>336</v>
+      </c>
+      <c r="B72" t="s">
         <v>337</v>
-      </c>
-      <c r="B72" t="s">
-        <v>338</v>
       </c>
       <c r="C72" t="s">
         <v>25</v>
       </c>
       <c r="D72" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E72" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F72" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>339</v>
+      </c>
+      <c r="B73" t="s">
         <v>340</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
+        <v>446</v>
+      </c>
+      <c r="D73" t="s">
+        <v>447</v>
+      </c>
+      <c r="E73" t="s">
         <v>341</v>
       </c>
-      <c r="C73" t="s">
+      <c r="F73" t="s">
         <v>447</v>
-      </c>
-      <c r="D73" t="s">
-        <v>448</v>
-      </c>
-      <c r="E73" t="s">
-        <v>342</v>
-      </c>
-      <c r="F73" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>342</v>
+      </c>
+      <c r="B74" t="s">
         <v>343</v>
-      </c>
-      <c r="B74" t="s">
-        <v>344</v>
       </c>
       <c r="C74" t="s">
         <v>14</v>
       </c>
       <c r="D74" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E74" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F74" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>345</v>
+      </c>
+      <c r="B75" t="s">
         <v>346</v>
-      </c>
-      <c r="B75" t="s">
-        <v>347</v>
       </c>
       <c r="C75" t="s">
         <v>14</v>
       </c>
       <c r="D75" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E75" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F75" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>348</v>
+      </c>
+      <c r="B76" t="s">
         <v>349</v>
-      </c>
-      <c r="B76" t="s">
-        <v>350</v>
       </c>
       <c r="C76" t="s">
         <v>14</v>
       </c>
       <c r="D76" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E76" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F76" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>351</v>
+      </c>
+      <c r="B77" t="s">
         <v>352</v>
       </c>
-      <c r="B77" t="s">
-        <v>353</v>
-      </c>
       <c r="C77" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D77" t="s">
         <v>115</v>
       </c>
       <c r="E77" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F77" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>354</v>
+      </c>
+      <c r="B78" t="s">
         <v>355</v>
-      </c>
-      <c r="B78" t="s">
-        <v>356</v>
       </c>
       <c r="C78" t="s">
         <v>73</v>
       </c>
       <c r="D78" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E78" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F78" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>357</v>
+      </c>
+      <c r="B79" t="s">
         <v>358</v>
-      </c>
-      <c r="B79" t="s">
-        <v>359</v>
       </c>
       <c r="C79" t="s">
         <v>73</v>
@@ -3634,78 +3787,78 @@
         <v>9</v>
       </c>
       <c r="E79" t="s">
+        <v>359</v>
+      </c>
+      <c r="F79" t="s">
         <v>360</v>
-      </c>
-      <c r="F79" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>361</v>
+      </c>
+      <c r="B80" t="s">
         <v>362</v>
-      </c>
-      <c r="B80" t="s">
-        <v>363</v>
       </c>
       <c r="C80" t="s">
         <v>73</v>
       </c>
       <c r="D80" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E80" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F80" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>364</v>
+      </c>
+      <c r="B81" t="s">
         <v>365</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>366</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>367</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>368</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>369</v>
-      </c>
-      <c r="F81" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>370</v>
+      </c>
+      <c r="B82" t="s">
         <v>371</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
+        <v>447</v>
+      </c>
+      <c r="D82" t="s">
+        <v>447</v>
+      </c>
+      <c r="E82" t="s">
         <v>372</v>
       </c>
-      <c r="C82" t="s">
-        <v>448</v>
-      </c>
-      <c r="D82" t="s">
-        <v>448</v>
-      </c>
-      <c r="E82" t="s">
-        <v>373</v>
-      </c>
       <c r="F82" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>373</v>
+      </c>
+      <c r="B83" t="s">
         <v>374</v>
-      </c>
-      <c r="B83" t="s">
-        <v>375</v>
       </c>
       <c r="C83" t="s">
         <v>52</v>
@@ -3714,138 +3867,138 @@
         <v>142</v>
       </c>
       <c r="E83" t="s">
+        <v>375</v>
+      </c>
+      <c r="F83" t="s">
         <v>376</v>
-      </c>
-      <c r="F83" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>377</v>
+      </c>
+      <c r="B84" t="s">
         <v>378</v>
-      </c>
-      <c r="B84" t="s">
-        <v>379</v>
       </c>
       <c r="C84" t="s">
         <v>31</v>
       </c>
       <c r="D84" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E84" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F84" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>380</v>
+      </c>
+      <c r="B85" t="s">
         <v>381</v>
       </c>
-      <c r="B85" t="s">
-        <v>382</v>
-      </c>
       <c r="C85" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D85" t="s">
         <v>53</v>
       </c>
       <c r="E85" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F85" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>383</v>
+      </c>
+      <c r="B86" t="s">
         <v>384</v>
-      </c>
-      <c r="B86" t="s">
-        <v>385</v>
       </c>
       <c r="C86" t="s">
         <v>52</v>
       </c>
       <c r="D86" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E86" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F86" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>386</v>
+      </c>
+      <c r="B87" t="s">
         <v>387</v>
-      </c>
-      <c r="B87" t="s">
-        <v>388</v>
       </c>
       <c r="C87" t="s">
         <v>52</v>
       </c>
       <c r="D87" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E87" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F87" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>389</v>
+      </c>
+      <c r="B88" t="s">
         <v>390</v>
-      </c>
-      <c r="B88" t="s">
-        <v>391</v>
       </c>
       <c r="C88" t="s">
         <v>31</v>
       </c>
       <c r="D88" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E88" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F88" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>392</v>
+      </c>
+      <c r="B89" t="s">
         <v>393</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
+        <v>447</v>
+      </c>
+      <c r="D89" t="s">
+        <v>447</v>
+      </c>
+      <c r="E89" t="s">
         <v>394</v>
       </c>
-      <c r="C89" t="s">
-        <v>448</v>
-      </c>
-      <c r="D89" t="s">
-        <v>448</v>
-      </c>
-      <c r="E89" t="s">
-        <v>395</v>
-      </c>
       <c r="F89" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>395</v>
+      </c>
+      <c r="B90" t="s">
         <v>396</v>
-      </c>
-      <c r="B90" t="s">
-        <v>397</v>
       </c>
       <c r="C90" t="s">
         <v>52</v>
@@ -3854,90 +4007,90 @@
         <v>62</v>
       </c>
       <c r="E90" t="s">
+        <v>397</v>
+      </c>
+      <c r="F90" t="s">
         <v>398</v>
-      </c>
-      <c r="F90" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>399</v>
+      </c>
+      <c r="B91" t="s">
         <v>400</v>
-      </c>
-      <c r="B91" t="s">
-        <v>401</v>
       </c>
       <c r="C91" t="s">
         <v>52</v>
       </c>
       <c r="D91" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E91" t="s">
+        <v>401</v>
+      </c>
+      <c r="F91" t="s">
         <v>402</v>
-      </c>
-      <c r="F91" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>403</v>
+      </c>
+      <c r="B92" t="s">
         <v>404</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
+        <v>447</v>
+      </c>
+      <c r="D92" t="s">
+        <v>447</v>
+      </c>
+      <c r="E92" t="s">
         <v>405</v>
       </c>
-      <c r="C92" t="s">
-        <v>448</v>
-      </c>
-      <c r="D92" t="s">
-        <v>448</v>
-      </c>
-      <c r="E92" t="s">
-        <v>406</v>
-      </c>
       <c r="F92" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>406</v>
+      </c>
+      <c r="B93" t="s">
         <v>407</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
+        <v>447</v>
+      </c>
+      <c r="D93" t="s">
+        <v>447</v>
+      </c>
+      <c r="E93" t="s">
         <v>408</v>
       </c>
-      <c r="C93" t="s">
-        <v>448</v>
-      </c>
-      <c r="D93" t="s">
-        <v>448</v>
-      </c>
-      <c r="E93" t="s">
-        <v>409</v>
-      </c>
       <c r="F93" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>409</v>
+      </c>
+      <c r="B94" t="s">
         <v>410</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
+        <v>447</v>
+      </c>
+      <c r="D94" t="s">
+        <v>447</v>
+      </c>
+      <c r="E94" t="s">
         <v>411</v>
       </c>
-      <c r="C94" t="s">
-        <v>448</v>
-      </c>
-      <c r="D94" t="s">
-        <v>448</v>
-      </c>
-      <c r="E94" t="s">
-        <v>412</v>
-      </c>
       <c r="F94" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -3959,22 +4112,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B1" t="s">
         <v>415</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>416</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>419</v>
-      </c>
-      <c r="F1" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -3985,7 +4138,7 @@
         <v>46204</v>
       </c>
       <c r="C2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D2" s="2">
         <v>0.64236111111111116</v>
@@ -3994,7 +4147,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="F2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4005,7 +4158,7 @@
         <v>46204</v>
       </c>
       <c r="C3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D3" s="2">
         <v>0.64236111111111116</v>
@@ -4014,7 +4167,7 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4025,7 +4178,7 @@
         <v>46204</v>
       </c>
       <c r="C4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D4" s="2">
         <v>0.67708333333333337</v>
@@ -4034,7 +4187,7 @@
         <v>0.70486111111111116</v>
       </c>
       <c r="F4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -4045,7 +4198,7 @@
         <v>46204</v>
       </c>
       <c r="C5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D5" s="2">
         <v>0.70486111111111116</v>
@@ -4054,7 +4207,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="F5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -4065,7 +4218,7 @@
         <v>46204</v>
       </c>
       <c r="C6" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D6" s="2">
         <v>0.70486111111111116</v>
@@ -4074,7 +4227,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="F6" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -4085,7 +4238,7 @@
         <v>46204</v>
       </c>
       <c r="C7" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D7" s="2">
         <v>0.73958333333333337</v>
@@ -4094,7 +4247,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -4105,7 +4258,7 @@
         <v>46204</v>
       </c>
       <c r="C8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D8" s="2">
         <v>0.73958333333333337</v>
@@ -4114,7 +4267,7 @@
         <v>0.77430555555555558</v>
       </c>
       <c r="F8" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -4125,7 +4278,7 @@
         <v>46204</v>
       </c>
       <c r="C9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D9" s="2">
         <v>0.77083333333333337</v>
@@ -4134,7 +4287,7 @@
         <v>0.80555555555555558</v>
       </c>
       <c r="F9" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -4145,7 +4298,7 @@
         <v>46204</v>
       </c>
       <c r="C10" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D10" s="2">
         <v>0.77083333333333337</v>
@@ -4154,7 +4307,7 @@
         <v>0.80555555555555558</v>
       </c>
       <c r="F10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -4165,7 +4318,7 @@
         <v>46204</v>
       </c>
       <c r="C11" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D11" s="2">
         <v>0.80555555555555558</v>
@@ -4174,7 +4327,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="F11" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -4185,7 +4338,7 @@
         <v>46204</v>
       </c>
       <c r="C12" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D12" s="2">
         <v>0.80555555555555558</v>
@@ -4194,7 +4347,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="F12" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -4205,7 +4358,7 @@
         <v>46204</v>
       </c>
       <c r="C13" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D13" s="2">
         <v>0.83680555555555558</v>
@@ -4214,7 +4367,7 @@
         <v>0.87847222222222221</v>
       </c>
       <c r="F13" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -4225,7 +4378,7 @@
         <v>46204</v>
       </c>
       <c r="C14" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D14" s="2">
         <v>0.84027777777777779</v>
@@ -4234,7 +4387,7 @@
         <v>0.875</v>
       </c>
       <c r="F14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -4245,7 +4398,7 @@
         <v>46204</v>
       </c>
       <c r="C15" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D15" s="2">
         <v>0.875</v>
@@ -4254,7 +4407,7 @@
         <v>0.90972222222222221</v>
       </c>
       <c r="F15" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -4265,7 +4418,7 @@
         <v>46204</v>
       </c>
       <c r="C16" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D16" s="2">
         <v>0.875</v>
@@ -4274,7 +4427,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="F16" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -4285,7 +4438,7 @@
         <v>46204</v>
       </c>
       <c r="C17" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D17" s="2">
         <v>0.90972222222222221</v>
@@ -4294,7 +4447,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F17" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -4305,7 +4458,7 @@
         <v>46204</v>
       </c>
       <c r="C18" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D18" s="2">
         <v>0.91666666666666663</v>
@@ -4314,7 +4467,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F18" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -4325,7 +4478,7 @@
         <v>46204</v>
       </c>
       <c r="C19" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D19" s="2">
         <v>0.95833333333333337</v>
@@ -4334,18 +4487,18 @@
         <v>0.99652777777777779</v>
       </c>
       <c r="F19" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B20" s="1">
         <v>46204</v>
       </c>
       <c r="C20" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D20" s="2">
         <v>0.95833333333333337</v>
@@ -4354,7 +4507,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -4365,7 +4518,7 @@
         <v>46204</v>
       </c>
       <c r="C21" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D21" s="2">
         <v>0</v>
@@ -4374,7 +4527,7 @@
         <v>7.6388888888888895E-2</v>
       </c>
       <c r="F21" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -4385,7 +4538,7 @@
         <v>46204</v>
       </c>
       <c r="C22" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D22" s="2">
         <v>0</v>
@@ -4394,7 +4547,7 @@
         <v>4.8611111111111112E-2</v>
       </c>
       <c r="F22" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -4405,7 +4558,7 @@
         <v>46204</v>
       </c>
       <c r="C23" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D23" s="2">
         <v>4.8611111111111112E-2</v>
@@ -4414,7 +4567,7 @@
         <v>9.7222222222222224E-2</v>
       </c>
       <c r="F23" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -4425,7 +4578,7 @@
         <v>46204</v>
       </c>
       <c r="C24" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D24" s="2">
         <v>7.6388888888888895E-2</v>
@@ -4434,7 +4587,7 @@
         <v>0.125</v>
       </c>
       <c r="F24" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -4445,7 +4598,7 @@
         <v>46205</v>
       </c>
       <c r="C25" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D25" s="2">
         <v>0.63888888888888884</v>
@@ -4454,7 +4607,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F25" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -4465,7 +4618,7 @@
         <v>46205</v>
       </c>
       <c r="C26" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D26" s="2">
         <v>0.64236111111111116</v>
@@ -4474,7 +4627,7 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F26" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -4485,7 +4638,7 @@
         <v>46205</v>
       </c>
       <c r="C27" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D27" s="2">
         <v>0.65625</v>
@@ -4494,7 +4647,7 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F27" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -4505,7 +4658,7 @@
         <v>46205</v>
       </c>
       <c r="C28" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D28" s="2">
         <v>0.67361111111111116</v>
@@ -4514,7 +4667,7 @@
         <v>0.70138888888888884</v>
       </c>
       <c r="F28" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -4525,7 +4678,7 @@
         <v>46205</v>
       </c>
       <c r="C29" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D29" s="2">
         <v>0.69097222222222221</v>
@@ -4534,7 +4687,7 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F29" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -4545,7 +4698,7 @@
         <v>46205</v>
       </c>
       <c r="C30" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D30" s="2">
         <v>0.70138888888888884</v>
@@ -4554,7 +4707,7 @@
         <v>0.73611111111111116</v>
       </c>
       <c r="F30" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -4565,7 +4718,7 @@
         <v>46205</v>
       </c>
       <c r="C31" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D31" s="2">
         <v>0.72222222222222221</v>
@@ -4574,7 +4727,7 @@
         <v>0.76388888888888884</v>
       </c>
       <c r="F31" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -4585,7 +4738,7 @@
         <v>46205</v>
       </c>
       <c r="C32" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D32" s="2">
         <v>0.73611111111111116</v>
@@ -4594,7 +4747,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F32" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -4605,7 +4758,7 @@
         <v>46205</v>
       </c>
       <c r="C33" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D33" s="2">
         <v>0.76388888888888884</v>
@@ -4614,7 +4767,7 @@
         <v>0.8125</v>
       </c>
       <c r="F33" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -4625,7 +4778,7 @@
         <v>46205</v>
       </c>
       <c r="C34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D34" s="2">
         <v>0.77083333333333337</v>
@@ -4634,7 +4787,7 @@
         <v>0.8125</v>
       </c>
       <c r="F34" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -4645,7 +4798,7 @@
         <v>46205</v>
       </c>
       <c r="C35" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D35" s="2">
         <v>0.8125</v>
@@ -4654,7 +4807,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F35" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -4665,7 +4818,7 @@
         <v>46205</v>
       </c>
       <c r="C36" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D36" s="2">
         <v>0.8125</v>
@@ -4674,7 +4827,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F36" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -4685,7 +4838,7 @@
         <v>46205</v>
       </c>
       <c r="C37" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D37" s="2">
         <v>0.85416666666666663</v>
@@ -4694,7 +4847,7 @@
         <v>0.89583333333333337</v>
       </c>
       <c r="F37" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -4705,7 +4858,7 @@
         <v>46205</v>
       </c>
       <c r="C38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D38" s="2">
         <v>0.86805555555555558</v>
@@ -4714,7 +4867,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F38" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -4725,7 +4878,7 @@
         <v>46205</v>
       </c>
       <c r="C39" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D39" s="2">
         <v>0.89930555555555558</v>
@@ -4734,7 +4887,7 @@
         <v>0.94097222222222221</v>
       </c>
       <c r="F39" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -4745,7 +4898,7 @@
         <v>46205</v>
       </c>
       <c r="C40" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D40" s="2">
         <v>0.94097222222222221</v>
@@ -4754,7 +4907,7 @@
         <v>0.98263888888888884</v>
       </c>
       <c r="F40" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -4765,7 +4918,7 @@
         <v>46205</v>
       </c>
       <c r="C41" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D41" s="2">
         <v>0.96527777777777779</v>
@@ -4774,7 +4927,7 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F41" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -4785,7 +4938,7 @@
         <v>46205</v>
       </c>
       <c r="C42" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D42" s="2">
         <v>0.98958333333333337</v>
@@ -4794,7 +4947,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="F42" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -4805,7 +4958,7 @@
         <v>46205</v>
       </c>
       <c r="C43" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D43" s="2">
         <v>1.3888888888888888E-2</v>
@@ -4814,7 +4967,7 @@
         <v>6.5972222222222224E-2</v>
       </c>
       <c r="F43" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -4825,7 +4978,7 @@
         <v>46205</v>
       </c>
       <c r="C44" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D44" s="2">
         <v>4.1666666666666664E-2</v>
@@ -4834,7 +4987,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F44" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -4845,7 +4998,7 @@
         <v>46205</v>
       </c>
       <c r="C45" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D45" s="2">
         <v>6.5972222222222224E-2</v>
@@ -4854,7 +5007,7 @@
         <v>0.10069444444444445</v>
       </c>
       <c r="F45" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -4865,7 +5018,7 @@
         <v>46205</v>
       </c>
       <c r="C46" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D46" s="2">
         <v>0.10069444444444445</v>
@@ -4874,7 +5027,7 @@
         <v>0.1423611111111111</v>
       </c>
       <c r="F46" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -4885,7 +5038,7 @@
         <v>46206</v>
       </c>
       <c r="C47" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D47" s="2">
         <v>0.62847222222222221</v>
@@ -4894,7 +5047,7 @@
         <v>0.65972222222222221</v>
       </c>
       <c r="F47" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -4905,7 +5058,7 @@
         <v>46206</v>
       </c>
       <c r="C48" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D48" s="2">
         <v>0.62847222222222221</v>
@@ -4914,7 +5067,7 @@
         <v>0.65625</v>
       </c>
       <c r="F48" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -4925,7 +5078,7 @@
         <v>46206</v>
       </c>
       <c r="C49" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D49" s="2">
         <v>0.65972222222222221</v>
@@ -4934,7 +5087,7 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F49" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -4945,7 +5098,7 @@
         <v>46206</v>
       </c>
       <c r="C50" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D50" s="2">
         <v>0.65972222222222221</v>
@@ -4954,7 +5107,7 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F50" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -4965,7 +5118,7 @@
         <v>46206</v>
       </c>
       <c r="C51" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D51" s="2">
         <v>0.69097222222222221</v>
@@ -4974,7 +5127,7 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F51" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -4985,7 +5138,7 @@
         <v>46206</v>
       </c>
       <c r="C52" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D52" s="2">
         <v>0.69097222222222221</v>
@@ -4994,7 +5147,7 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F52" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -5005,7 +5158,7 @@
         <v>46206</v>
       </c>
       <c r="C53" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D53" s="2">
         <v>0.72222222222222221</v>
@@ -5014,7 +5167,7 @@
         <v>0.75694444444444442</v>
       </c>
       <c r="F53" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -5025,7 +5178,7 @@
         <v>46206</v>
       </c>
       <c r="C54" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D54" s="2">
         <v>0.72222222222222221</v>
@@ -5034,7 +5187,7 @@
         <v>0.75694444444444442</v>
       </c>
       <c r="F54" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -5045,7 +5198,7 @@
         <v>46206</v>
       </c>
       <c r="C55" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D55" s="2">
         <v>0.75694444444444442</v>
@@ -5054,7 +5207,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F55" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -5065,7 +5218,7 @@
         <v>46206</v>
       </c>
       <c r="C56" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D56" s="2">
         <v>0.75694444444444442</v>
@@ -5074,7 +5227,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F56" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -5085,7 +5238,7 @@
         <v>46206</v>
       </c>
       <c r="C57" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D57" s="2">
         <v>0.79166666666666663</v>
@@ -5094,7 +5247,7 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="F57" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -5105,7 +5258,7 @@
         <v>46206</v>
       </c>
       <c r="C58" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D58" s="2">
         <v>0.79166666666666663</v>
@@ -5114,7 +5267,7 @@
         <v>0.82638888888888884</v>
       </c>
       <c r="F58" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -5125,7 +5278,7 @@
         <v>46206</v>
       </c>
       <c r="C59" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D59" s="2">
         <v>0.83333333333333337</v>
@@ -5134,7 +5287,7 @@
         <v>0.86805555555555558</v>
       </c>
       <c r="F59" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -5145,7 +5298,7 @@
         <v>46206</v>
       </c>
       <c r="C60" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D60" s="2">
         <v>0.83333333333333337</v>
@@ -5154,7 +5307,7 @@
         <v>0.86805555555555558</v>
       </c>
       <c r="F60" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -5165,7 +5318,7 @@
         <v>46206</v>
       </c>
       <c r="C61" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D61" s="2">
         <v>0.86805555555555558</v>
@@ -5174,7 +5327,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="F61" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -5185,7 +5338,7 @@
         <v>46206</v>
       </c>
       <c r="C62" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D62" s="2">
         <v>0.86805555555555558</v>
@@ -5194,7 +5347,7 @@
         <v>0.90972222222222221</v>
       </c>
       <c r="F62" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -5205,7 +5358,7 @@
         <v>46206</v>
       </c>
       <c r="C63" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D63" s="2">
         <v>0.91666666666666663</v>
@@ -5214,7 +5367,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F63" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -5225,7 +5378,7 @@
         <v>46206</v>
       </c>
       <c r="C64" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D64" s="2">
         <v>0.91666666666666663</v>
@@ -5234,7 +5387,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F64" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -5245,7 +5398,7 @@
         <v>46206</v>
       </c>
       <c r="C65" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D65" s="2">
         <v>0.95833333333333337</v>
@@ -5254,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -5265,7 +5418,7 @@
         <v>46206</v>
       </c>
       <c r="C66" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D66" s="2">
         <v>0.96527777777777779</v>
@@ -5274,7 +5427,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="F66" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -5285,7 +5438,7 @@
         <v>46206</v>
       </c>
       <c r="C67" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D67" s="2">
         <v>2.4305555555555556E-2</v>
@@ -5294,7 +5447,7 @@
         <v>5.9027777777777776E-2</v>
       </c>
       <c r="F67" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -5305,7 +5458,7 @@
         <v>46206</v>
       </c>
       <c r="C68" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D68" s="2">
         <v>2.4305555555555556E-2</v>
@@ -5314,7 +5467,7 @@
         <v>7.2916666666666671E-2</v>
       </c>
       <c r="F68" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -5325,7 +5478,7 @@
         <v>46206</v>
       </c>
       <c r="C69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D69" s="2">
         <v>5.9027777777777776E-2</v>
@@ -5334,7 +5487,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -5345,7 +5498,7 @@
         <v>46206</v>
       </c>
       <c r="C70" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D70" s="2">
         <v>6.9444444444444448E-2</v>
@@ -5354,18 +5507,18 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F70" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B71" s="1">
         <v>46207</v>
       </c>
       <c r="C71" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D71" s="2">
         <v>0.61805555555555558</v>
@@ -5374,7 +5527,7 @@
         <v>0.65277777777777779</v>
       </c>
       <c r="F71" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -5385,7 +5538,7 @@
         <v>46207</v>
       </c>
       <c r="C72" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D72" s="2">
         <v>0.61805555555555558</v>
@@ -5394,18 +5547,18 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F72" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B73" s="1">
         <v>46207</v>
       </c>
       <c r="C73" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D73" s="2">
         <v>0.65277777777777779</v>
@@ -5414,18 +5567,18 @@
         <v>0.68402777777777779</v>
       </c>
       <c r="F73" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B74" s="1">
         <v>46207</v>
       </c>
       <c r="C74" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D74" s="2">
         <v>0.65277777777777779</v>
@@ -5434,18 +5587,18 @@
         <v>0.68402777777777779</v>
       </c>
       <c r="F74" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B75" s="1">
         <v>46207</v>
       </c>
       <c r="C75" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D75" s="2">
         <v>0.68402777777777779</v>
@@ -5454,18 +5607,18 @@
         <v>0.71875</v>
       </c>
       <c r="F75" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B76" s="1">
         <v>46207</v>
       </c>
       <c r="C76" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D76" s="2">
         <v>0.68402777777777779</v>
@@ -5474,18 +5627,18 @@
         <v>0.71875</v>
       </c>
       <c r="F76" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B77" s="1">
         <v>46207</v>
       </c>
       <c r="C77" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D77" s="2">
         <v>0.71875</v>
@@ -5494,18 +5647,18 @@
         <v>0.75347222222222221</v>
       </c>
       <c r="F77" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B78" s="1">
         <v>46207</v>
       </c>
       <c r="C78" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D78" s="2">
         <v>0.71875</v>
@@ -5514,18 +5667,18 @@
         <v>0.75347222222222221</v>
       </c>
       <c r="F78" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B79" s="1">
         <v>46207</v>
       </c>
       <c r="C79" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D79" s="2">
         <v>0.75347222222222221</v>
@@ -5534,18 +5687,18 @@
         <v>0.79513888888888884</v>
       </c>
       <c r="F79" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B80" s="1">
         <v>46207</v>
       </c>
       <c r="C80" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D80" s="2">
         <v>0.76041666666666663</v>
@@ -5554,18 +5707,18 @@
         <v>0.79513888888888884</v>
       </c>
       <c r="F80" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B81" s="1">
         <v>46207</v>
       </c>
       <c r="C81" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D81" s="2">
         <v>0.79513888888888884</v>
@@ -5574,18 +5727,18 @@
         <v>0.82986111111111116</v>
       </c>
       <c r="F81" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B82" s="1">
         <v>46207</v>
       </c>
       <c r="C82" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D82" s="2">
         <v>0.79513888888888884</v>
@@ -5594,18 +5747,18 @@
         <v>0.82986111111111116</v>
       </c>
       <c r="F82" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B83" s="1">
         <v>46207</v>
       </c>
       <c r="C83" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D83" s="2">
         <v>0.82986111111111116</v>
@@ -5614,18 +5767,18 @@
         <v>0.87152777777777779</v>
       </c>
       <c r="F83" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B84" s="1">
         <v>46207</v>
       </c>
       <c r="C84" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D84" s="2">
         <v>0.82986111111111116</v>
@@ -5634,18 +5787,18 @@
         <v>0.87152777777777779</v>
       </c>
       <c r="F84" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B85" s="1">
         <v>46207</v>
       </c>
       <c r="C85" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D85" s="2">
         <v>0.87152777777777779</v>
@@ -5654,18 +5807,18 @@
         <v>0.91319444444444442</v>
       </c>
       <c r="F85" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B86" s="1">
         <v>46207</v>
       </c>
       <c r="C86" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D86" s="2">
         <v>0.87152777777777779</v>
@@ -5674,18 +5827,18 @@
         <v>0.91319444444444442</v>
       </c>
       <c r="F86" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B87" s="1">
         <v>46207</v>
       </c>
       <c r="C87" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D87" s="2">
         <v>0.91319444444444442</v>
@@ -5694,18 +5847,18 @@
         <v>0.96527777777777779</v>
       </c>
       <c r="F87" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B88" s="1">
         <v>46207</v>
       </c>
       <c r="C88" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D88" s="2">
         <v>0.91319444444444442</v>
@@ -5714,18 +5867,18 @@
         <v>0.95486111111111116</v>
       </c>
       <c r="F88" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B89" s="1">
         <v>46207</v>
       </c>
       <c r="C89" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D89" s="2">
         <v>0.96527777777777779</v>
@@ -5734,18 +5887,18 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F89" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B90" s="1">
         <v>46207</v>
       </c>
       <c r="C90" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D90" s="2">
         <v>0.96527777777777779</v>
@@ -5754,18 +5907,18 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F90" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B91" s="1">
         <v>46207</v>
       </c>
       <c r="C91" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D91" s="2">
         <v>2.0833333333333332E-2</v>
@@ -5774,18 +5927,18 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F91" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B92" s="1">
         <v>46207</v>
       </c>
       <c r="C92" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D92" s="2">
         <v>3.4722222222222224E-2</v>
@@ -5794,18 +5947,18 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F92" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B93" s="1">
         <v>46207</v>
       </c>
       <c r="C93" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D93" s="2">
         <v>9.0277777777777776E-2</v>
@@ -5814,18 +5967,18 @@
         <v>0.1423611111111111</v>
       </c>
       <c r="F93" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B94" s="1">
         <v>46207</v>
       </c>
       <c r="C94" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D94" s="2">
         <v>9.0277777777777776E-2</v>
@@ -5834,7 +5987,7 @@
         <v>0.1388888888888889</v>
       </c>
       <c r="F94" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -5857,19 +6010,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B1" t="s">
         <v>415</v>
       </c>
-      <c r="B1" t="s">
-        <v>416</v>
-      </c>
       <c r="C1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D1" t="s">
         <v>418</v>
       </c>
-      <c r="D1" t="s">
-        <v>419</v>
-      </c>
       <c r="E1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -5886,7 +6039,7 @@
         <v>0.82638888888888884</v>
       </c>
       <c r="E2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -5903,7 +6056,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -5920,7 +6073,7 @@
         <v>0.875</v>
       </c>
       <c r="E4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -5937,7 +6090,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="E5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -5954,7 +6107,7 @@
         <v>0.8125</v>
       </c>
       <c r="E6" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -5971,12 +6124,12 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B8" s="1">
         <v>46207</v>
@@ -5988,12 +6141,12 @@
         <v>0.6875</v>
       </c>
       <c r="E8" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B9" s="1">
         <v>46207</v>
@@ -6005,12 +6158,12 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="E9" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B10" s="1">
         <v>46207</v>
@@ -6022,7 +6175,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -6034,6 +6187,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F98B513-13BD-497E-9297-59EEA952D49F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6BE1310-03D4-41E8-8E99-89C5D710B0D7}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6052,66 +6214,141 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1" t="s">
         <v>428</v>
-      </c>
-      <c r="D1" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>437</v>
+        <v>436</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CDB14F4-F5C1-44FB-8AC4-31FDC06E2D66}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="55.28515625" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" customWidth="1"/>
+    <col min="4" max="4" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>448</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>46202</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46203</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B4" t="s">
+        <v>455</v>
+      </c>
+      <c r="C4" t="s">
+        <v>456</v>
+      </c>
+      <c r="D4" t="s">
+        <v>457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Soporte multifestival dinamico parametrizado desde la hoja Edicion del Excel
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -8,23 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\Resurrection Fest 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7EBB27-212F-493A-BC53-AF45B5616BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6C4466A-C584-4A0A-A232-473DD095D060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3930" yWindow="2535" windowWidth="21600" windowHeight="12645" activeTab="6" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
+    <workbookView xWindow="5190" yWindow="3045" windowWidth="21600" windowHeight="12645" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
   </bookViews>
   <sheets>
     <sheet name="Edición" sheetId="1" r:id="rId1"/>
     <sheet name="Artistas" sheetId="2" r:id="rId2"/>
     <sheet name="Actuaciones" sheetId="3" r:id="rId3"/>
     <sheet name="Firmas" sheetId="4" r:id="rId4"/>
-    <sheet name="Hoja1" sheetId="6" r:id="rId5"/>
-    <sheet name="Escenarios" sheetId="5" r:id="rId6"/>
-    <sheet name="Noticias" sheetId="7" r:id="rId7"/>
+    <sheet name="Escenarios" sheetId="5" r:id="rId5"/>
+    <sheet name="Noticias" sheetId="7" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="2" hidden="1">Actuaciones!$A$1:$F$94</definedName>
     <definedName name="DatosExternos_1" localSheetId="1" hidden="1">Artistas!$A$1:$F$94</definedName>
-    <definedName name="DatosExternos_1" localSheetId="5" hidden="1">Escenarios!$A$1:$D$5</definedName>
+    <definedName name="DatosExternos_1" localSheetId="4" hidden="1">Escenarios!$A$1:$D$5</definedName>
     <definedName name="DatosExternos_1" localSheetId="3" hidden="1">Firmas!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -68,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="474">
   <si>
     <t>ID</t>
   </si>
@@ -1381,9 +1380,6 @@
     <t>#e67e22</t>
   </si>
   <si>
-    <t>Festival</t>
-  </si>
-  <si>
     <t>Resurrection Fest</t>
   </si>
   <si>
@@ -1445,6 +1441,54 @@
   </si>
   <si>
     <t>Fecha_noticia</t>
+  </si>
+  <si>
+    <t>Nombre Festival</t>
+  </si>
+  <si>
+    <t>resurrection-fest</t>
+  </si>
+  <si>
+    <t>resurrection-fest-2026</t>
+  </si>
+  <si>
+    <t>Nombre visible</t>
+  </si>
+  <si>
+    <t>Resurrection Fest E.G.</t>
+  </si>
+  <si>
+    <t>Inicio cuenta atrás</t>
+  </si>
+  <si>
+    <t>Hora inicio parrilla</t>
+  </si>
+  <si>
+    <t>Hora fin parrilla</t>
+  </si>
+  <si>
+    <t>Logo</t>
+  </si>
+  <si>
+    <t>logo.svg</t>
+  </si>
+  <si>
+    <t>Cartel</t>
+  </si>
+  <si>
+    <t>cartel.jpg</t>
+  </si>
+  <si>
+    <t>Mapa</t>
+  </si>
+  <si>
+    <t>mapa.jpg</t>
+  </si>
+  <si>
+    <t>Festival ID</t>
+  </si>
+  <si>
+    <t>Edicion ID</t>
   </si>
 </sst>
 </file>
@@ -1454,7 +1498,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1466,6 +1510,12 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1547,61 +1597,45 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="30">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="9"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-      </border>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1666,13 +1700,42 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <border outline="0">
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="9"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1745,30 +1808,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{62006AC5-8661-4769-8EA1-C477E01879E4}" name="Tabla5" displayName="Tabla5" ref="A1:F2" totalsRowShown="0">
-  <autoFilter ref="A1:F2" xr:uid="{62006AC5-8661-4769-8EA1-C477E01879E4}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{15AFF007-6ACF-476C-992B-C418B464D377}" name="Festival"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{62006AC5-8661-4769-8EA1-C477E01879E4}" name="Tabla5" displayName="Tabla5" ref="A1:O2" totalsRowShown="0">
+  <autoFilter ref="A1:O2" xr:uid="{62006AC5-8661-4769-8EA1-C477E01879E4}"/>
+  <tableColumns count="15">
+    <tableColumn id="7" xr3:uid="{4459CFC1-77B1-4D5A-823E-D9A1B93BB199}" name="Festival ID"/>
+    <tableColumn id="8" xr3:uid="{E45D7BC9-7855-48A0-B74F-E245C77DA393}" name="Edicion ID"/>
+    <tableColumn id="1" xr3:uid="{15AFF007-6ACF-476C-992B-C418B464D377}" name="Nombre Festival"/>
+    <tableColumn id="9" xr3:uid="{5EC016F7-E39E-413B-95DF-669EEED6A9AF}" name="Nombre visible"/>
     <tableColumn id="2" xr3:uid="{EB5B3C98-C24C-4EE9-8B98-948B3E8364A7}" name="Año"/>
-    <tableColumn id="3" xr3:uid="{34EE02C0-F635-48F0-8270-9D93DA60F2E2}" name="Fecha inicio" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{38046547-49A7-4BEC-9673-353E2A7A0C72}" name="Fecha fin" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{34EE02C0-F635-48F0-8270-9D93DA60F2E2}" name="Fecha inicio" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{38046547-49A7-4BEC-9673-353E2A7A0C72}" name="Fecha fin" dataDxfId="25"/>
     <tableColumn id="5" xr3:uid="{B0EE68D7-240A-432E-828B-412D863DB860}" name="Localidad"/>
     <tableColumn id="6" xr3:uid="{CAF5BBDD-2799-4D36-8E8C-4828C6BBCC14}" name="Zona horaria"/>
+    <tableColumn id="10" xr3:uid="{EA18A59F-5EAD-45EB-993D-FEBE14308766}" name="Inicio cuenta atrás"/>
+    <tableColumn id="11" xr3:uid="{7E841A91-CA6F-42AC-A6D7-C2DDBEF7FDE9}" name="Hora inicio parrilla"/>
+    <tableColumn id="12" xr3:uid="{679CDA01-6531-4963-95DC-7D385312E7BB}" name="Hora fin parrilla" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{D631FCFB-A23A-4D9C-86E8-0BC2DF22E081}" name="Logo" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{3C554932-14D5-453C-A155-0A57136B8251}" name="Cartel" dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{1F28B6E7-6238-4EAA-87BF-E0E067554DD7}" name="Mapa" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}" name="Resu_2026_Bandas" displayName="Resu_2026_Bandas" ref="A1:F94" tableType="queryTable" totalsRowShown="0" headerRowDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}" name="Resu_2026_Bandas" displayName="Resu_2026_Bandas" ref="A1:F94" tableType="queryTable" totalsRowShown="0" headerRowDxfId="24">
   <autoFilter ref="A1:F94" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{332FF7D4-1975-45FA-8763-D1A083D8FE2F}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{922EB2D7-BDCF-4797-BFF0-8A22CB9C6F39}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{CB14A298-32C9-4122-BD30-3016D41B6015}" uniqueName="3" name="País" queryTableFieldId="3" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{99176C72-F021-473F-B769-6C3E0FCBDE7B}" uniqueName="4" name="Género principal" queryTableFieldId="4" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{56414A58-1DFA-4995-9EFD-80C971999C52}" uniqueName="5" name="Descripción" queryTableFieldId="5" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{C4CC863B-2259-457A-A08B-CB7F95AA821B}" uniqueName="6" name="YouTube" queryTableFieldId="6" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{332FF7D4-1975-45FA-8763-D1A083D8FE2F}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{922EB2D7-BDCF-4797-BFF0-8A22CB9C6F39}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{CB14A298-32C9-4122-BD30-3016D41B6015}" uniqueName="3" name="País" queryTableFieldId="3" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{99176C72-F021-473F-B769-6C3E0FCBDE7B}" uniqueName="4" name="Género principal" queryTableFieldId="4" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{56414A58-1DFA-4995-9EFD-80C971999C52}" uniqueName="5" name="Descripción" queryTableFieldId="5" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{C4CC863B-2259-457A-A08B-CB7F95AA821B}" uniqueName="6" name="YouTube" queryTableFieldId="6" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1778,12 +1850,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2BEC583C-339F-4B73-8C37-E33B77FB98D9}" name="Resu_2026_Horarios" displayName="Resu_2026_Horarios" ref="A1:F94" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F94" xr:uid="{2BEC583C-339F-4B73-8C37-E33B77FB98D9}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{260FA184-5F84-4B0D-B8F2-A1F3A5C706A9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{72ACC8A8-5988-40D3-A47C-4720A05E6BED}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{CAF50085-3E03-439C-A8FE-6EA34C1F0B6C}" uniqueName="3" name="Escenario" queryTableFieldId="3" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{CA173E7C-1376-4FF5-96B1-C85971DA9824}" uniqueName="4" name="Inicio" queryTableFieldId="4" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{875B5625-99D4-4511-9BA8-407A3DDD9913}" uniqueName="5" name="Fin" queryTableFieldId="5" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{894E47A5-100E-431A-B533-57698097335B}" uniqueName="6" name="Estado" queryTableFieldId="6" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{260FA184-5F84-4B0D-B8F2-A1F3A5C706A9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{72ACC8A8-5988-40D3-A47C-4720A05E6BED}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{CAF50085-3E03-439C-A8FE-6EA34C1F0B6C}" uniqueName="3" name="Escenario" queryTableFieldId="3" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{CA173E7C-1376-4FF5-96B1-C85971DA9824}" uniqueName="4" name="Inicio" queryTableFieldId="4" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{875B5625-99D4-4511-9BA8-407A3DDD9913}" uniqueName="5" name="Fin" queryTableFieldId="5" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{894E47A5-100E-431A-B533-57698097335B}" uniqueName="6" name="Estado" queryTableFieldId="6" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1793,11 +1865,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{35F91919-D6D4-4F94-9D8E-919ABF494188}" name="Resu_2026_Firmas" displayName="Resu_2026_Firmas" ref="A1:E10" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E10" xr:uid="{35F91919-D6D4-4F94-9D8E-919ABF494188}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A4CC5F35-5249-43F3-AC88-309620CC12F9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{153952D1-13AC-4C33-A40B-32C07B5BEEE6}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{B03BDDBD-33D4-444F-BAB1-30CED98305E7}" uniqueName="3" name="Inicio" queryTableFieldId="3" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{F0D8F161-D930-4F98-9BDA-95DEFECCCB15}" uniqueName="4" name="Fin" queryTableFieldId="4" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{23CD0C9B-12E2-4544-B3AB-BE082393F99E}" uniqueName="5" name="Ubicación" queryTableFieldId="5" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{A4CC5F35-5249-43F3-AC88-309620CC12F9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{153952D1-13AC-4C33-A40B-32C07B5BEEE6}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{B03BDDBD-33D4-444F-BAB1-30CED98305E7}" uniqueName="3" name="Inicio" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{F0D8F161-D930-4F98-9BDA-95DEFECCCB15}" uniqueName="4" name="Fin" queryTableFieldId="4" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{23CD0C9B-12E2-4544-B3AB-BE082393F99E}" uniqueName="5" name="Ubicación" queryTableFieldId="5" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1807,17 +1879,17 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}" name="Resu_2026_Escenarios" displayName="Resu_2026_Escenarios" ref="A1:D5" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D5" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{F5497620-A4CF-4BD7-A8E7-28E1CF6E3857}" uniqueName="3" name="Orden" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}" name="Tabla6" displayName="Tabla6" ref="A1:D4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}" name="Tabla6" displayName="Tabla6" ref="A1:D4" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
   <autoFilter ref="A1:D4" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}"/>
   <tableColumns count="4">
     <tableColumn id="4" xr3:uid="{A9DF3F42-14AF-4444-B7F6-F1AEF4BD9D15}" name="Fecha_noticia"/>
@@ -2146,53 +2218,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B08E700-C8E3-464D-B8AB-B5A6F11794E6}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="5" width="23" customWidth="1"/>
+    <col min="11" max="11" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1" t="s">
+        <v>461</v>
+      </c>
+      <c r="E1" t="s">
+        <v>438</v>
+      </c>
+      <c r="F1" t="s">
+        <v>439</v>
+      </c>
+      <c r="G1" t="s">
+        <v>440</v>
+      </c>
+      <c r="H1" t="s">
+        <v>441</v>
+      </c>
+      <c r="I1" t="s">
+        <v>443</v>
+      </c>
+      <c r="J1" t="s">
+        <v>463</v>
+      </c>
+      <c r="K1" t="s">
+        <v>464</v>
+      </c>
+      <c r="L1" t="s">
+        <v>465</v>
+      </c>
+      <c r="M1" t="s">
+        <v>466</v>
+      </c>
+      <c r="N1" t="s">
+        <v>468</v>
+      </c>
+      <c r="O1" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C2" t="s">
         <v>437</v>
       </c>
-      <c r="B1" t="s">
-        <v>439</v>
-      </c>
-      <c r="C1" t="s">
-        <v>440</v>
-      </c>
-      <c r="D1" t="s">
-        <v>441</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E2">
+        <v>2026</v>
+      </c>
+      <c r="F2" s="3">
+        <v>46204</v>
+      </c>
+      <c r="G2" s="3">
+        <v>46207</v>
+      </c>
+      <c r="H2" t="s">
         <v>442</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I2" t="s">
         <v>444</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>438</v>
-      </c>
-      <c r="B2">
-        <v>2026</v>
-      </c>
-      <c r="C2" s="3">
+      <c r="J2" s="1">
         <v>46204</v>
       </c>
-      <c r="D2" s="3">
-        <v>46207</v>
-      </c>
-      <c r="E2" t="s">
-        <v>443</v>
-      </c>
-      <c r="F2" t="s">
-        <v>445</v>
+      <c r="K2" s="10">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="L2" s="10">
+        <v>0.14583333333333334</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>467</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>471</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -3624,13 +3754,13 @@
         <v>14</v>
       </c>
       <c r="D71" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E71" t="s">
         <v>335</v>
       </c>
       <c r="F71" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -3644,13 +3774,13 @@
         <v>25</v>
       </c>
       <c r="D72" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E72" t="s">
         <v>338</v>
       </c>
       <c r="F72" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -3661,16 +3791,16 @@
         <v>340</v>
       </c>
       <c r="C73" t="s">
+        <v>445</v>
+      </c>
+      <c r="D73" t="s">
         <v>446</v>
-      </c>
-      <c r="D73" t="s">
-        <v>447</v>
       </c>
       <c r="E73" t="s">
         <v>341</v>
       </c>
       <c r="F73" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -3684,13 +3814,13 @@
         <v>14</v>
       </c>
       <c r="D74" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E74" t="s">
         <v>344</v>
       </c>
       <c r="F74" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -3704,13 +3834,13 @@
         <v>14</v>
       </c>
       <c r="D75" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E75" t="s">
         <v>347</v>
       </c>
       <c r="F75" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -3724,13 +3854,13 @@
         <v>14</v>
       </c>
       <c r="D76" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E76" t="s">
         <v>350</v>
       </c>
       <c r="F76" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3741,7 +3871,7 @@
         <v>352</v>
       </c>
       <c r="C77" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D77" t="s">
         <v>115</v>
@@ -3750,7 +3880,7 @@
         <v>353</v>
       </c>
       <c r="F77" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -3764,13 +3894,13 @@
         <v>73</v>
       </c>
       <c r="D78" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E78" t="s">
         <v>356</v>
       </c>
       <c r="F78" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -3804,13 +3934,13 @@
         <v>73</v>
       </c>
       <c r="D80" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E80" t="s">
         <v>363</v>
       </c>
       <c r="F80" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -3841,16 +3971,16 @@
         <v>371</v>
       </c>
       <c r="C82" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D82" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E82" t="s">
         <v>372</v>
       </c>
       <c r="F82" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -3884,13 +4014,13 @@
         <v>31</v>
       </c>
       <c r="D84" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E84" t="s">
         <v>379</v>
       </c>
       <c r="F84" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -3901,7 +4031,7 @@
         <v>381</v>
       </c>
       <c r="C85" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D85" t="s">
         <v>53</v>
@@ -3910,7 +4040,7 @@
         <v>382</v>
       </c>
       <c r="F85" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -3924,13 +4054,13 @@
         <v>52</v>
       </c>
       <c r="D86" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E86" t="s">
         <v>385</v>
       </c>
       <c r="F86" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3944,13 +4074,13 @@
         <v>52</v>
       </c>
       <c r="D87" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E87" t="s">
         <v>388</v>
       </c>
       <c r="F87" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3964,13 +4094,13 @@
         <v>31</v>
       </c>
       <c r="D88" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E88" t="s">
         <v>391</v>
       </c>
       <c r="F88" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -3981,16 +4111,16 @@
         <v>393</v>
       </c>
       <c r="C89" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D89" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E89" t="s">
         <v>394</v>
       </c>
       <c r="F89" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -4041,16 +4171,16 @@
         <v>404</v>
       </c>
       <c r="C92" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D92" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E92" t="s">
         <v>405</v>
       </c>
       <c r="F92" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -4061,16 +4191,16 @@
         <v>407</v>
       </c>
       <c r="C93" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D93" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E93" t="s">
         <v>408</v>
       </c>
       <c r="F93" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -4081,16 +4211,16 @@
         <v>410</v>
       </c>
       <c r="C94" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D94" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E94" t="s">
         <v>411</v>
       </c>
       <c r="F94" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -6187,15 +6317,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F98B513-13BD-497E-9297-59EEA952D49F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6BE1310-03D4-41E8-8E99-89C5D710B0D7}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6284,7 +6405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CDB14F4-F5C1-44FB-8AC4-31FDC06E2D66}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6297,16 +6418,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>448</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>452</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -6314,13 +6435,13 @@
         <v>46202</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>450</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>451</v>
-      </c>
       <c r="D2" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -6328,13 +6449,13 @@
         <v>46203</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>454</v>
-      </c>
       <c r="D3" s="7" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -6342,13 +6463,13 @@
         <v>46204</v>
       </c>
       <c r="B4" t="s">
+        <v>454</v>
+      </c>
+      <c r="C4" t="s">
         <v>455</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>456</v>
-      </c>
-      <c r="D4" t="s">
-        <v>457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sincronizacion de nombres de imagenes actualizados des excel
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\Resurrection Fest 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6C4466A-C584-4A0A-A232-473DD095D060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98704AD-35FC-4045-8365-AFBCD8403138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5190" yWindow="3045" windowWidth="21600" windowHeight="12645" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
   </bookViews>
   <sheets>
     <sheet name="Edición" sheetId="1" r:id="rId1"/>
@@ -1470,25 +1470,25 @@
     <t>Logo</t>
   </si>
   <si>
-    <t>logo.svg</t>
-  </si>
-  <si>
     <t>Cartel</t>
   </si>
   <si>
-    <t>cartel.jpg</t>
-  </si>
-  <si>
     <t>Mapa</t>
   </si>
   <si>
-    <t>mapa.jpg</t>
-  </si>
-  <si>
     <t>Festival ID</t>
   </si>
   <si>
     <t>Edicion ID</t>
+  </si>
+  <si>
+    <t>cartelresu2026.jpg</t>
+  </si>
+  <si>
+    <t>maparesu2026.jpg</t>
+  </si>
+  <si>
+    <t>logoresu2026.jpg</t>
   </si>
 </sst>
 </file>
@@ -1617,16 +1617,42 @@
   </cellStyles>
   <dxfs count="30">
     <dxf>
-      <numFmt numFmtId="25" formatCode="h:mm"/>
+      <border outline="0">
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="25" formatCode="h:mm"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="25" formatCode="h:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="h:mm"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="9"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1692,50 +1718,24 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="9"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1816,31 +1816,31 @@
     <tableColumn id="1" xr3:uid="{15AFF007-6ACF-476C-992B-C418B464D377}" name="Nombre Festival"/>
     <tableColumn id="9" xr3:uid="{5EC016F7-E39E-413B-95DF-669EEED6A9AF}" name="Nombre visible"/>
     <tableColumn id="2" xr3:uid="{EB5B3C98-C24C-4EE9-8B98-948B3E8364A7}" name="Año"/>
-    <tableColumn id="3" xr3:uid="{34EE02C0-F635-48F0-8270-9D93DA60F2E2}" name="Fecha inicio" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{38046547-49A7-4BEC-9673-353E2A7A0C72}" name="Fecha fin" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{34EE02C0-F635-48F0-8270-9D93DA60F2E2}" name="Fecha inicio" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{38046547-49A7-4BEC-9673-353E2A7A0C72}" name="Fecha fin" dataDxfId="28"/>
     <tableColumn id="5" xr3:uid="{B0EE68D7-240A-432E-828B-412D863DB860}" name="Localidad"/>
     <tableColumn id="6" xr3:uid="{CAF5BBDD-2799-4D36-8E8C-4828C6BBCC14}" name="Zona horaria"/>
     <tableColumn id="10" xr3:uid="{EA18A59F-5EAD-45EB-993D-FEBE14308766}" name="Inicio cuenta atrás"/>
     <tableColumn id="11" xr3:uid="{7E841A91-CA6F-42AC-A6D7-C2DDBEF7FDE9}" name="Hora inicio parrilla"/>
-    <tableColumn id="12" xr3:uid="{679CDA01-6531-4963-95DC-7D385312E7BB}" name="Hora fin parrilla" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{D631FCFB-A23A-4D9C-86E8-0BC2DF22E081}" name="Logo" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{3C554932-14D5-453C-A155-0A57136B8251}" name="Cartel" dataDxfId="1"/>
-    <tableColumn id="15" xr3:uid="{1F28B6E7-6238-4EAA-87BF-E0E067554DD7}" name="Mapa" dataDxfId="0"/>
+    <tableColumn id="12" xr3:uid="{679CDA01-6531-4963-95DC-7D385312E7BB}" name="Hora fin parrilla" dataDxfId="27"/>
+    <tableColumn id="13" xr3:uid="{D631FCFB-A23A-4D9C-86E8-0BC2DF22E081}" name="Logo" dataDxfId="26"/>
+    <tableColumn id="14" xr3:uid="{3C554932-14D5-453C-A155-0A57136B8251}" name="Cartel" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{1F28B6E7-6238-4EAA-87BF-E0E067554DD7}" name="Mapa" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}" name="Resu_2026_Bandas" displayName="Resu_2026_Bandas" ref="A1:F94" tableType="queryTable" totalsRowShown="0" headerRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}" name="Resu_2026_Bandas" displayName="Resu_2026_Bandas" ref="A1:F94" tableType="queryTable" totalsRowShown="0" headerRowDxfId="23">
   <autoFilter ref="A1:F94" xr:uid="{A719971D-B9A1-4CC5-8C2E-97805706D491}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{332FF7D4-1975-45FA-8763-D1A083D8FE2F}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{922EB2D7-BDCF-4797-BFF0-8A22CB9C6F39}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{CB14A298-32C9-4122-BD30-3016D41B6015}" uniqueName="3" name="País" queryTableFieldId="3" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{99176C72-F021-473F-B769-6C3E0FCBDE7B}" uniqueName="4" name="Género principal" queryTableFieldId="4" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{56414A58-1DFA-4995-9EFD-80C971999C52}" uniqueName="5" name="Descripción" queryTableFieldId="5" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{C4CC863B-2259-457A-A08B-CB7F95AA821B}" uniqueName="6" name="YouTube" queryTableFieldId="6" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{332FF7D4-1975-45FA-8763-D1A083D8FE2F}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{922EB2D7-BDCF-4797-BFF0-8A22CB9C6F39}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{CB14A298-32C9-4122-BD30-3016D41B6015}" uniqueName="3" name="País" queryTableFieldId="3" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{99176C72-F021-473F-B769-6C3E0FCBDE7B}" uniqueName="4" name="Género principal" queryTableFieldId="4" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{56414A58-1DFA-4995-9EFD-80C971999C52}" uniqueName="5" name="Descripción" queryTableFieldId="5" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{C4CC863B-2259-457A-A08B-CB7F95AA821B}" uniqueName="6" name="YouTube" queryTableFieldId="6" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1850,12 +1850,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2BEC583C-339F-4B73-8C37-E33B77FB98D9}" name="Resu_2026_Horarios" displayName="Resu_2026_Horarios" ref="A1:F94" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F94" xr:uid="{2BEC583C-339F-4B73-8C37-E33B77FB98D9}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{260FA184-5F84-4B0D-B8F2-A1F3A5C706A9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{72ACC8A8-5988-40D3-A47C-4720A05E6BED}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{CAF50085-3E03-439C-A8FE-6EA34C1F0B6C}" uniqueName="3" name="Escenario" queryTableFieldId="3" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{CA173E7C-1376-4FF5-96B1-C85971DA9824}" uniqueName="4" name="Inicio" queryTableFieldId="4" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{875B5625-99D4-4511-9BA8-407A3DDD9913}" uniqueName="5" name="Fin" queryTableFieldId="5" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{894E47A5-100E-431A-B533-57698097335B}" uniqueName="6" name="Estado" queryTableFieldId="6" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{260FA184-5F84-4B0D-B8F2-A1F3A5C706A9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{72ACC8A8-5988-40D3-A47C-4720A05E6BED}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{CAF50085-3E03-439C-A8FE-6EA34C1F0B6C}" uniqueName="3" name="Escenario" queryTableFieldId="3" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{CA173E7C-1376-4FF5-96B1-C85971DA9824}" uniqueName="4" name="Inicio" queryTableFieldId="4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{875B5625-99D4-4511-9BA8-407A3DDD9913}" uniqueName="5" name="Fin" queryTableFieldId="5" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{894E47A5-100E-431A-B533-57698097335B}" uniqueName="6" name="Estado" queryTableFieldId="6" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1865,11 +1865,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{35F91919-D6D4-4F94-9D8E-919ABF494188}" name="Resu_2026_Firmas" displayName="Resu_2026_Firmas" ref="A1:E10" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E10" xr:uid="{35F91919-D6D4-4F94-9D8E-919ABF494188}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A4CC5F35-5249-43F3-AC88-309620CC12F9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{153952D1-13AC-4C33-A40B-32C07B5BEEE6}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{B03BDDBD-33D4-444F-BAB1-30CED98305E7}" uniqueName="3" name="Inicio" queryTableFieldId="3" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{F0D8F161-D930-4F98-9BDA-95DEFECCCB15}" uniqueName="4" name="Fin" queryTableFieldId="4" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{23CD0C9B-12E2-4544-B3AB-BE082393F99E}" uniqueName="5" name="Ubicación" queryTableFieldId="5" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{A4CC5F35-5249-43F3-AC88-309620CC12F9}" uniqueName="1" name="Artista ID" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{153952D1-13AC-4C33-A40B-32C07B5BEEE6}" uniqueName="2" name="Fecha" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{B03BDDBD-33D4-444F-BAB1-30CED98305E7}" uniqueName="3" name="Inicio" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F0D8F161-D930-4F98-9BDA-95DEFECCCB15}" uniqueName="4" name="Fin" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{23CD0C9B-12E2-4544-B3AB-BE082393F99E}" uniqueName="5" name="Ubicación" queryTableFieldId="5" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1879,17 +1879,17 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}" name="Resu_2026_Escenarios" displayName="Resu_2026_Escenarios" ref="A1:D5" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D5" xr:uid="{0027EA80-5A4C-4A67-ADB8-6F31BD527ABA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{614D9728-7FFB-4B06-8156-8D500F75516B}" uniqueName="1" name="ID" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{E740DF2C-7892-4626-9796-22C8AF4FF580}" uniqueName="2" name="Nombre" queryTableFieldId="2" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{F5497620-A4CF-4BD7-A8E7-28E1CF6E3857}" uniqueName="3" name="Orden" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{B90C1FC5-5741-4BA5-830D-2FB32CB93A79}" uniqueName="4" name="Color" queryTableFieldId="4" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}" name="Tabla6" displayName="Tabla6" ref="A1:D4" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}" name="Tabla6" displayName="Tabla6" ref="A1:D4" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:D4" xr:uid="{D12BEC07-ED97-4613-8F5D-310274F55997}"/>
   <tableColumns count="4">
     <tableColumn id="4" xr3:uid="{A9DF3F42-14AF-4444-B7F6-F1AEF4BD9D15}" name="Fecha_noticia"/>
@@ -2225,14 +2225,15 @@
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
     <col min="3" max="5" width="23" customWidth="1"/>
     <col min="11" max="11" width="21.140625" customWidth="1"/>
+    <col min="13" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="B1" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="C1" t="s">
         <v>458</v>
@@ -2268,10 +2269,10 @@
         <v>466</v>
       </c>
       <c r="N1" t="s">
+        <v>467</v>
+      </c>
+      <c r="O1" t="s">
         <v>468</v>
-      </c>
-      <c r="O1" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -2312,13 +2313,13 @@
         <v>0.14583333333333334</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadir mensaje fin de festival
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\Resurrection Fest 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D536C28-A2F5-4BDE-8C18-6B4C957B0035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E8B58A-E94A-456F-91D9-BE7F1A71A13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{680F1EA4-1A24-48E6-8465-A31DBABEE799}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="493">
   <si>
     <t>ID</t>
   </si>
@@ -747,9 +747,6 @@
     <t>NUKORE</t>
   </si>
   <si>
-    <t>Harcore</t>
-  </si>
-  <si>
     <t>Con una sólida trayectoria que ya supera los 20 años, la banda vitoriana Nukore es un referente de autenticidad y tesón en la escena nacional. Desde su formación, han sabido perfeccionar su mezcla implacable entre nu metal, hardcore, rap y metal alternativo dejando canciones brutales a lo largo de sus seis referencias de estudio 🙌  Si te mola el hardcore noventero y el nu metal y bandas como Rage Against The Machine, Biohazard, Suicidal Tendencies o Stuck Mojo, no te lo pienses y vente a verlos el viernes 3 de julio al Ritual Stage de una 🤘</t>
   </si>
   <si>
@@ -1549,9 +1546,6 @@
   </si>
   <si>
     <t>https://www.youtube.com/watch?v=JVF6e_LSO2k</t>
-  </si>
-  <si>
-    <t>Post Harcore</t>
   </si>
 </sst>
 </file>
@@ -2304,63 +2298,63 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>461</v>
+      </c>
+      <c r="B1" t="s">
         <v>462</v>
       </c>
-      <c r="B1" t="s">
-        <v>463</v>
-      </c>
       <c r="C1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="E1" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1" t="s">
         <v>432</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>433</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>434</v>
       </c>
-      <c r="H1" t="s">
-        <v>435</v>
-      </c>
       <c r="I1" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J1" t="s">
+        <v>455</v>
+      </c>
+      <c r="K1" t="s">
         <v>456</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>457</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>458</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>459</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>460</v>
-      </c>
-      <c r="O1" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B2" t="s">
         <v>452</v>
       </c>
-      <c r="B2" t="s">
-        <v>453</v>
-      </c>
       <c r="C2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E2">
         <v>2026</v>
@@ -2372,10 +2366,10 @@
         <v>46207</v>
       </c>
       <c r="H2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="I2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="J2" s="1">
         <v>46204</v>
@@ -2387,13 +2381,13 @@
         <v>0.14583333333333334</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="N2" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="O2" s="10" t="s">
         <v>464</v>
-      </c>
-      <c r="O2" s="10" t="s">
-        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -2420,7 +2414,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2489,7 +2483,7 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
@@ -2800,10 +2794,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B20" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C20" t="s">
         <v>14</v>
@@ -3009,7 +3003,7 @@
         <v>107</v>
       </c>
       <c r="D30" t="s">
-        <v>494</v>
+        <v>238</v>
       </c>
       <c r="E30" t="s">
         <v>144</v>
@@ -3109,7 +3103,7 @@
         <v>50</v>
       </c>
       <c r="D35" t="s">
-        <v>494</v>
+        <v>238</v>
       </c>
       <c r="E35" t="s">
         <v>169</v>
@@ -3369,41 +3363,41 @@
         <v>14</v>
       </c>
       <c r="D48" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" t="s">
         <v>226</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>227</v>
-      </c>
-      <c r="F48" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>228</v>
+      </c>
+      <c r="B49" t="s">
         <v>229</v>
-      </c>
-      <c r="B49" t="s">
-        <v>230</v>
       </c>
       <c r="C49" t="s">
         <v>14</v>
       </c>
       <c r="D49" t="s">
-        <v>226</v>
+        <v>60</v>
       </c>
       <c r="E49" t="s">
+        <v>230</v>
+      </c>
+      <c r="F49" t="s">
         <v>231</v>
-      </c>
-      <c r="F49" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>232</v>
+      </c>
+      <c r="B50" t="s">
         <v>233</v>
-      </c>
-      <c r="B50" t="s">
-        <v>234</v>
       </c>
       <c r="C50" t="s">
         <v>14</v>
@@ -3412,78 +3406,78 @@
         <v>149</v>
       </c>
       <c r="E50" t="s">
+        <v>234</v>
+      </c>
+      <c r="F50" t="s">
         <v>235</v>
-      </c>
-      <c r="F50" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>236</v>
+      </c>
+      <c r="B51" t="s">
         <v>237</v>
-      </c>
-      <c r="B51" t="s">
-        <v>238</v>
       </c>
       <c r="C51" t="s">
         <v>14</v>
       </c>
       <c r="D51" t="s">
+        <v>238</v>
+      </c>
+      <c r="E51" t="s">
         <v>239</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
         <v>240</v>
-      </c>
-      <c r="F51" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>241</v>
+      </c>
+      <c r="B52" t="s">
         <v>242</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>243</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>244</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>245</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>246</v>
-      </c>
-      <c r="F52" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>247</v>
+      </c>
+      <c r="B53" t="s">
         <v>248</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>249</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>250</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>251</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>252</v>
-      </c>
-      <c r="F53" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>253</v>
+      </c>
+      <c r="B54" t="s">
         <v>254</v>
-      </c>
-      <c r="B54" t="s">
-        <v>255</v>
       </c>
       <c r="C54" t="s">
         <v>14</v>
@@ -3492,78 +3486,78 @@
         <v>81</v>
       </c>
       <c r="E54" t="s">
+        <v>255</v>
+      </c>
+      <c r="F54" t="s">
         <v>256</v>
-      </c>
-      <c r="F54" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>257</v>
+      </c>
+      <c r="B55" t="s">
         <v>258</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
+        <v>243</v>
+      </c>
+      <c r="D55" t="s">
         <v>259</v>
       </c>
-      <c r="C55" t="s">
-        <v>244</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>260</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
         <v>261</v>
-      </c>
-      <c r="F55" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>262</v>
+      </c>
+      <c r="B56" t="s">
         <v>263</v>
-      </c>
-      <c r="B56" t="s">
-        <v>264</v>
       </c>
       <c r="C56" t="s">
         <v>34</v>
       </c>
       <c r="D56" t="s">
+        <v>264</v>
+      </c>
+      <c r="E56" t="s">
         <v>265</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
         <v>266</v>
-      </c>
-      <c r="F56" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>267</v>
+      </c>
+      <c r="B57" t="s">
         <v>268</v>
-      </c>
-      <c r="B57" t="s">
-        <v>269</v>
       </c>
       <c r="C57" t="s">
         <v>107</v>
       </c>
       <c r="D57" t="s">
+        <v>269</v>
+      </c>
+      <c r="E57" t="s">
         <v>270</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>271</v>
-      </c>
-      <c r="F57" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>272</v>
+      </c>
+      <c r="B58" t="s">
         <v>273</v>
-      </c>
-      <c r="B58" t="s">
-        <v>274</v>
       </c>
       <c r="C58" t="s">
         <v>50</v>
@@ -3572,58 +3566,58 @@
         <v>60</v>
       </c>
       <c r="E58" t="s">
+        <v>274</v>
+      </c>
+      <c r="F58" t="s">
         <v>275</v>
-      </c>
-      <c r="F58" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>276</v>
+      </c>
+      <c r="B59" t="s">
         <v>277</v>
-      </c>
-      <c r="B59" t="s">
-        <v>278</v>
       </c>
       <c r="C59" t="s">
         <v>50</v>
       </c>
       <c r="D59" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E59" t="s">
+        <v>278</v>
+      </c>
+      <c r="F59" t="s">
         <v>279</v>
-      </c>
-      <c r="F59" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>280</v>
+      </c>
+      <c r="B60" t="s">
         <v>281</v>
-      </c>
-      <c r="B60" t="s">
-        <v>282</v>
       </c>
       <c r="C60" t="s">
         <v>107</v>
       </c>
       <c r="D60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E60" t="s">
+        <v>282</v>
+      </c>
+      <c r="F60" t="s">
         <v>283</v>
-      </c>
-      <c r="F60" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>284</v>
+      </c>
+      <c r="B61" t="s">
         <v>285</v>
-      </c>
-      <c r="B61" t="s">
-        <v>286</v>
       </c>
       <c r="C61" t="s">
         <v>50</v>
@@ -3632,18 +3626,18 @@
         <v>9</v>
       </c>
       <c r="E61" t="s">
+        <v>286</v>
+      </c>
+      <c r="F61" t="s">
         <v>287</v>
-      </c>
-      <c r="F61" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>288</v>
+      </c>
+      <c r="B62" t="s">
         <v>289</v>
-      </c>
-      <c r="B62" t="s">
-        <v>290</v>
       </c>
       <c r="C62" t="s">
         <v>50</v>
@@ -3652,38 +3646,38 @@
         <v>9</v>
       </c>
       <c r="E62" t="s">
+        <v>290</v>
+      </c>
+      <c r="F62" t="s">
         <v>291</v>
-      </c>
-      <c r="F62" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>292</v>
+      </c>
+      <c r="B63" t="s">
         <v>293</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
+        <v>243</v>
+      </c>
+      <c r="D63" t="s">
+        <v>264</v>
+      </c>
+      <c r="E63" t="s">
         <v>294</v>
       </c>
-      <c r="C63" t="s">
-        <v>244</v>
-      </c>
-      <c r="D63" t="s">
-        <v>265</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>295</v>
-      </c>
-      <c r="F63" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>296</v>
+      </c>
+      <c r="B64" t="s">
         <v>297</v>
-      </c>
-      <c r="B64" t="s">
-        <v>298</v>
       </c>
       <c r="C64" t="s">
         <v>50</v>
@@ -3692,18 +3686,18 @@
         <v>177</v>
       </c>
       <c r="E64" t="s">
+        <v>298</v>
+      </c>
+      <c r="F64" t="s">
         <v>299</v>
-      </c>
-      <c r="F64" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>300</v>
+      </c>
+      <c r="B65" t="s">
         <v>301</v>
-      </c>
-      <c r="B65" t="s">
-        <v>302</v>
       </c>
       <c r="C65" t="s">
         <v>50</v>
@@ -3712,18 +3706,18 @@
         <v>139</v>
       </c>
       <c r="E65" t="s">
+        <v>302</v>
+      </c>
+      <c r="F65" t="s">
         <v>303</v>
-      </c>
-      <c r="F65" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>304</v>
+      </c>
+      <c r="B66" t="s">
         <v>305</v>
-      </c>
-      <c r="B66" t="s">
-        <v>306</v>
       </c>
       <c r="C66" t="s">
         <v>50</v>
@@ -3732,18 +3726,18 @@
         <v>60</v>
       </c>
       <c r="E66" t="s">
+        <v>306</v>
+      </c>
+      <c r="F66" t="s">
         <v>307</v>
-      </c>
-      <c r="F66" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>308</v>
+      </c>
+      <c r="B67" t="s">
         <v>309</v>
-      </c>
-      <c r="B67" t="s">
-        <v>310</v>
       </c>
       <c r="C67" t="s">
         <v>50</v>
@@ -3752,78 +3746,78 @@
         <v>9</v>
       </c>
       <c r="E67" t="s">
+        <v>310</v>
+      </c>
+      <c r="F67" t="s">
         <v>311</v>
-      </c>
-      <c r="F67" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>312</v>
+      </c>
+      <c r="B68" t="s">
         <v>313</v>
-      </c>
-      <c r="B68" t="s">
-        <v>314</v>
       </c>
       <c r="C68" t="s">
         <v>148</v>
       </c>
       <c r="D68" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E68" t="s">
+        <v>314</v>
+      </c>
+      <c r="F68" t="s">
         <v>315</v>
-      </c>
-      <c r="F68" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>316</v>
+      </c>
+      <c r="B69" t="s">
         <v>317</v>
-      </c>
-      <c r="B69" t="s">
-        <v>318</v>
       </c>
       <c r="C69" t="s">
         <v>50</v>
       </c>
       <c r="D69" t="s">
+        <v>318</v>
+      </c>
+      <c r="E69" t="s">
         <v>319</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>320</v>
-      </c>
-      <c r="F69" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>321</v>
+      </c>
+      <c r="B70" t="s">
         <v>322</v>
-      </c>
-      <c r="B70" t="s">
-        <v>323</v>
       </c>
       <c r="C70" t="s">
         <v>50</v>
       </c>
       <c r="D70" t="s">
+        <v>323</v>
+      </c>
+      <c r="E70" t="s">
         <v>324</v>
       </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>325</v>
-      </c>
-      <c r="F70" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>326</v>
+      </c>
+      <c r="B71" t="s">
         <v>327</v>
-      </c>
-      <c r="B71" t="s">
-        <v>328</v>
       </c>
       <c r="C71" t="s">
         <v>14</v>
@@ -3832,18 +3826,18 @@
         <v>9</v>
       </c>
       <c r="E71" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F71" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>329</v>
+      </c>
+      <c r="B72" t="s">
         <v>330</v>
-      </c>
-      <c r="B72" t="s">
-        <v>331</v>
       </c>
       <c r="C72" t="s">
         <v>24</v>
@@ -3852,38 +3846,38 @@
         <v>9</v>
       </c>
       <c r="E72" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F72" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>332</v>
+      </c>
+      <c r="B73" t="s">
         <v>333</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
+        <v>438</v>
+      </c>
+      <c r="D73" t="s">
+        <v>468</v>
+      </c>
+      <c r="E73" t="s">
         <v>334</v>
       </c>
-      <c r="C73" t="s">
-        <v>439</v>
-      </c>
-      <c r="D73" t="s">
+      <c r="F73" t="s">
         <v>469</v>
-      </c>
-      <c r="E73" t="s">
-        <v>335</v>
-      </c>
-      <c r="F73" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>335</v>
+      </c>
+      <c r="B74" t="s">
         <v>336</v>
-      </c>
-      <c r="B74" t="s">
-        <v>337</v>
       </c>
       <c r="C74" t="s">
         <v>14</v>
@@ -3892,18 +3886,18 @@
         <v>9</v>
       </c>
       <c r="E74" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F74" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>338</v>
+      </c>
+      <c r="B75" t="s">
         <v>339</v>
-      </c>
-      <c r="B75" t="s">
-        <v>340</v>
       </c>
       <c r="C75" t="s">
         <v>14</v>
@@ -3912,78 +3906,78 @@
         <v>117</v>
       </c>
       <c r="E75" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F75" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>341</v>
+      </c>
+      <c r="B76" t="s">
         <v>342</v>
-      </c>
-      <c r="B76" t="s">
-        <v>343</v>
       </c>
       <c r="C76" t="s">
         <v>14</v>
       </c>
       <c r="D76" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="E76" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F76" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>344</v>
+      </c>
+      <c r="B77" t="s">
         <v>345</v>
-      </c>
-      <c r="B77" t="s">
-        <v>346</v>
       </c>
       <c r="C77" t="s">
         <v>14</v>
       </c>
       <c r="D77" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E77" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F77" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>347</v>
+      </c>
+      <c r="B78" t="s">
         <v>348</v>
-      </c>
-      <c r="B78" t="s">
-        <v>349</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
       </c>
       <c r="D78" t="s">
+        <v>476</v>
+      </c>
+      <c r="E78" t="s">
+        <v>349</v>
+      </c>
+      <c r="F78" t="s">
         <v>477</v>
-      </c>
-      <c r="E78" t="s">
-        <v>350</v>
-      </c>
-      <c r="F78" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>350</v>
+      </c>
+      <c r="B79" t="s">
         <v>351</v>
-      </c>
-      <c r="B79" t="s">
-        <v>352</v>
       </c>
       <c r="C79" t="s">
         <v>71</v>
@@ -3992,18 +3986,18 @@
         <v>9</v>
       </c>
       <c r="E79" t="s">
+        <v>352</v>
+      </c>
+      <c r="F79" t="s">
         <v>353</v>
-      </c>
-      <c r="F79" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>354</v>
+      </c>
+      <c r="B80" t="s">
         <v>355</v>
-      </c>
-      <c r="B80" t="s">
-        <v>356</v>
       </c>
       <c r="C80" t="s">
         <v>71</v>
@@ -4012,58 +4006,58 @@
         <v>45</v>
       </c>
       <c r="E80" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F80" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>357</v>
+      </c>
+      <c r="B81" t="s">
         <v>358</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>359</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>360</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>361</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>362</v>
-      </c>
-      <c r="F81" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>363</v>
+      </c>
+      <c r="B82" t="s">
         <v>364</v>
-      </c>
-      <c r="B82" t="s">
-        <v>365</v>
       </c>
       <c r="C82" t="s">
         <v>107</v>
       </c>
       <c r="D82" t="s">
+        <v>479</v>
+      </c>
+      <c r="E82" t="s">
+        <v>365</v>
+      </c>
+      <c r="F82" t="s">
         <v>480</v>
-      </c>
-      <c r="E82" t="s">
-        <v>366</v>
-      </c>
-      <c r="F82" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>366</v>
+      </c>
+      <c r="B83" t="s">
         <v>367</v>
-      </c>
-      <c r="B83" t="s">
-        <v>368</v>
       </c>
       <c r="C83" t="s">
         <v>50</v>
@@ -4072,58 +4066,58 @@
         <v>139</v>
       </c>
       <c r="E83" t="s">
+        <v>368</v>
+      </c>
+      <c r="F83" t="s">
         <v>369</v>
-      </c>
-      <c r="F83" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>370</v>
+      </c>
+      <c r="B84" t="s">
         <v>371</v>
-      </c>
-      <c r="B84" t="s">
-        <v>372</v>
       </c>
       <c r="C84" t="s">
         <v>107</v>
       </c>
       <c r="D84" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E84" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F84" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>373</v>
+      </c>
+      <c r="B85" t="s">
         <v>374</v>
       </c>
-      <c r="B85" t="s">
-        <v>375</v>
-      </c>
       <c r="C85" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D85" t="s">
         <v>51</v>
       </c>
       <c r="E85" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F85" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>376</v>
+      </c>
+      <c r="B86" t="s">
         <v>377</v>
-      </c>
-      <c r="B86" t="s">
-        <v>378</v>
       </c>
       <c r="C86" t="s">
         <v>50</v>
@@ -4132,18 +4126,18 @@
         <v>130</v>
       </c>
       <c r="E86" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F86" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>379</v>
+      </c>
+      <c r="B87" t="s">
         <v>380</v>
-      </c>
-      <c r="B87" t="s">
-        <v>381</v>
       </c>
       <c r="C87" t="s">
         <v>50</v>
@@ -4152,38 +4146,38 @@
         <v>97</v>
       </c>
       <c r="E87" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F87" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>382</v>
+      </c>
+      <c r="B88" t="s">
         <v>383</v>
-      </c>
-      <c r="B88" t="s">
-        <v>384</v>
       </c>
       <c r="C88" t="s">
         <v>107</v>
       </c>
       <c r="D88" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E88" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F88" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>385</v>
+      </c>
+      <c r="B89" t="s">
         <v>386</v>
-      </c>
-      <c r="B89" t="s">
-        <v>387</v>
       </c>
       <c r="C89" t="s">
         <v>50</v>
@@ -4192,18 +4186,18 @@
         <v>155</v>
       </c>
       <c r="E89" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F89" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>388</v>
+      </c>
+      <c r="B90" t="s">
         <v>389</v>
-      </c>
-      <c r="B90" t="s">
-        <v>390</v>
       </c>
       <c r="C90" t="s">
         <v>50</v>
@@ -4212,78 +4206,78 @@
         <v>60</v>
       </c>
       <c r="E90" t="s">
+        <v>390</v>
+      </c>
+      <c r="F90" t="s">
         <v>391</v>
-      </c>
-      <c r="F90" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>392</v>
+      </c>
+      <c r="B91" t="s">
         <v>393</v>
-      </c>
-      <c r="B91" t="s">
-        <v>394</v>
       </c>
       <c r="C91" t="s">
         <v>50</v>
       </c>
       <c r="D91" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E91" t="s">
+        <v>394</v>
+      </c>
+      <c r="F91" t="s">
         <v>395</v>
-      </c>
-      <c r="F91" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>396</v>
+      </c>
+      <c r="B92" t="s">
         <v>397</v>
       </c>
-      <c r="B92" t="s">
-        <v>398</v>
-      </c>
       <c r="C92" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D92" t="s">
         <v>45</v>
       </c>
       <c r="E92" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F92" s="11" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>399</v>
+      </c>
+      <c r="B93" t="s">
         <v>400</v>
-      </c>
-      <c r="B93" t="s">
-        <v>401</v>
       </c>
       <c r="C93" t="s">
         <v>50</v>
       </c>
       <c r="D93" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E93" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F93" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>402</v>
+      </c>
+      <c r="B94" t="s">
         <v>403</v>
-      </c>
-      <c r="B94" t="s">
-        <v>404</v>
       </c>
       <c r="C94" t="s">
         <v>8</v>
@@ -4292,10 +4286,10 @@
         <v>60</v>
       </c>
       <c r="E94" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F94" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -4321,22 +4315,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B1" t="s">
         <v>408</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>409</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>410</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>411</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>412</v>
-      </c>
-      <c r="F1" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -4347,7 +4341,7 @@
         <v>46204</v>
       </c>
       <c r="C2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D2" s="2">
         <v>0.64236111111111116</v>
@@ -4356,7 +4350,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="F2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4367,7 +4361,7 @@
         <v>46204</v>
       </c>
       <c r="C3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D3" s="2">
         <v>0.64236111111111116</v>
@@ -4376,7 +4370,7 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4387,7 +4381,7 @@
         <v>46204</v>
       </c>
       <c r="C4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D4" s="2">
         <v>0.67708333333333337</v>
@@ -4396,7 +4390,7 @@
         <v>0.70486111111111116</v>
       </c>
       <c r="F4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -4407,7 +4401,7 @@
         <v>46204</v>
       </c>
       <c r="C5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D5" s="2">
         <v>0.70486111111111116</v>
@@ -4416,7 +4410,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="F5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -4427,7 +4421,7 @@
         <v>46204</v>
       </c>
       <c r="C6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D6" s="2">
         <v>0.70486111111111116</v>
@@ -4436,7 +4430,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="F6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -4447,7 +4441,7 @@
         <v>46204</v>
       </c>
       <c r="C7" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D7" s="2">
         <v>0.73958333333333337</v>
@@ -4456,7 +4450,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -4467,7 +4461,7 @@
         <v>46204</v>
       </c>
       <c r="C8" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D8" s="2">
         <v>0.73958333333333337</v>
@@ -4476,7 +4470,7 @@
         <v>0.77430555555555558</v>
       </c>
       <c r="F8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -4487,7 +4481,7 @@
         <v>46204</v>
       </c>
       <c r="C9" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D9" s="2">
         <v>0.77083333333333337</v>
@@ -4496,7 +4490,7 @@
         <v>0.80555555555555558</v>
       </c>
       <c r="F9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -4507,7 +4501,7 @@
         <v>46204</v>
       </c>
       <c r="C10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D10" s="2">
         <v>0.77083333333333337</v>
@@ -4516,7 +4510,7 @@
         <v>0.80555555555555558</v>
       </c>
       <c r="F10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -4527,7 +4521,7 @@
         <v>46204</v>
       </c>
       <c r="C11" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D11" s="2">
         <v>0.80555555555555558</v>
@@ -4536,7 +4530,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="F11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -4547,7 +4541,7 @@
         <v>46204</v>
       </c>
       <c r="C12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D12" s="2">
         <v>0.80555555555555558</v>
@@ -4556,7 +4550,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="F12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -4567,7 +4561,7 @@
         <v>46204</v>
       </c>
       <c r="C13" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D13" s="2">
         <v>0.83680555555555558</v>
@@ -4576,7 +4570,7 @@
         <v>0.87847222222222221</v>
       </c>
       <c r="F13" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -4587,7 +4581,7 @@
         <v>46204</v>
       </c>
       <c r="C14" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D14" s="2">
         <v>0.84027777777777779</v>
@@ -4596,7 +4590,7 @@
         <v>0.875</v>
       </c>
       <c r="F14" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -4607,7 +4601,7 @@
         <v>46204</v>
       </c>
       <c r="C15" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D15" s="2">
         <v>0.875</v>
@@ -4616,7 +4610,7 @@
         <v>0.90972222222222221</v>
       </c>
       <c r="F15" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -4627,7 +4621,7 @@
         <v>46204</v>
       </c>
       <c r="C16" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D16" s="2">
         <v>0.875</v>
@@ -4636,7 +4630,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="F16" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -4647,7 +4641,7 @@
         <v>46204</v>
       </c>
       <c r="C17" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D17" s="2">
         <v>0.90972222222222221</v>
@@ -4656,7 +4650,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F17" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -4667,7 +4661,7 @@
         <v>46204</v>
       </c>
       <c r="C18" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D18" s="2">
         <v>0.91666666666666663</v>
@@ -4676,7 +4670,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F18" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -4687,7 +4681,7 @@
         <v>46204</v>
       </c>
       <c r="C19" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D19" s="2">
         <v>0.95833333333333337</v>
@@ -4696,18 +4690,18 @@
         <v>0.99652777777777779</v>
       </c>
       <c r="F19" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B20" s="1">
         <v>46204</v>
       </c>
       <c r="C20" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D20" s="2">
         <v>0.95833333333333337</v>
@@ -4716,7 +4710,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -4727,7 +4721,7 @@
         <v>46204</v>
       </c>
       <c r="C21" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D21" s="2">
         <v>0</v>
@@ -4736,7 +4730,7 @@
         <v>7.6388888888888895E-2</v>
       </c>
       <c r="F21" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -4747,7 +4741,7 @@
         <v>46204</v>
       </c>
       <c r="C22" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D22" s="2">
         <v>0</v>
@@ -4756,7 +4750,7 @@
         <v>4.8611111111111112E-2</v>
       </c>
       <c r="F22" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -4767,7 +4761,7 @@
         <v>46204</v>
       </c>
       <c r="C23" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D23" s="2">
         <v>4.8611111111111112E-2</v>
@@ -4776,7 +4770,7 @@
         <v>9.7222222222222224E-2</v>
       </c>
       <c r="F23" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -4787,7 +4781,7 @@
         <v>46204</v>
       </c>
       <c r="C24" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D24" s="2">
         <v>7.6388888888888895E-2</v>
@@ -4796,7 +4790,7 @@
         <v>0.125</v>
       </c>
       <c r="F24" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -4807,7 +4801,7 @@
         <v>46205</v>
       </c>
       <c r="C25" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D25" s="2">
         <v>0.63888888888888884</v>
@@ -4816,7 +4810,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F25" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -4827,7 +4821,7 @@
         <v>46205</v>
       </c>
       <c r="C26" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D26" s="2">
         <v>0.64236111111111116</v>
@@ -4836,7 +4830,7 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F26" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -4847,7 +4841,7 @@
         <v>46205</v>
       </c>
       <c r="C27" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D27" s="2">
         <v>0.65625</v>
@@ -4856,7 +4850,7 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F27" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -4867,7 +4861,7 @@
         <v>46205</v>
       </c>
       <c r="C28" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D28" s="2">
         <v>0.67361111111111116</v>
@@ -4876,7 +4870,7 @@
         <v>0.70138888888888884</v>
       </c>
       <c r="F28" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -4887,7 +4881,7 @@
         <v>46205</v>
       </c>
       <c r="C29" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D29" s="2">
         <v>0.69097222222222221</v>
@@ -4896,7 +4890,7 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F29" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -4907,7 +4901,7 @@
         <v>46205</v>
       </c>
       <c r="C30" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D30" s="2">
         <v>0.70138888888888884</v>
@@ -4916,7 +4910,7 @@
         <v>0.73611111111111116</v>
       </c>
       <c r="F30" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -4927,7 +4921,7 @@
         <v>46205</v>
       </c>
       <c r="C31" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D31" s="2">
         <v>0.72222222222222221</v>
@@ -4936,7 +4930,7 @@
         <v>0.76388888888888884</v>
       </c>
       <c r="F31" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -4947,7 +4941,7 @@
         <v>46205</v>
       </c>
       <c r="C32" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D32" s="2">
         <v>0.73611111111111116</v>
@@ -4956,7 +4950,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F32" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -4967,7 +4961,7 @@
         <v>46205</v>
       </c>
       <c r="C33" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D33" s="2">
         <v>0.76388888888888884</v>
@@ -4976,7 +4970,7 @@
         <v>0.8125</v>
       </c>
       <c r="F33" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -4987,7 +4981,7 @@
         <v>46205</v>
       </c>
       <c r="C34" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D34" s="2">
         <v>0.77083333333333337</v>
@@ -4996,7 +4990,7 @@
         <v>0.8125</v>
       </c>
       <c r="F34" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -5007,7 +5001,7 @@
         <v>46205</v>
       </c>
       <c r="C35" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D35" s="2">
         <v>0.8125</v>
@@ -5016,7 +5010,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F35" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -5027,7 +5021,7 @@
         <v>46205</v>
       </c>
       <c r="C36" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D36" s="2">
         <v>0.8125</v>
@@ -5036,7 +5030,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F36" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -5047,7 +5041,7 @@
         <v>46205</v>
       </c>
       <c r="C37" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D37" s="2">
         <v>0.85416666666666663</v>
@@ -5056,7 +5050,7 @@
         <v>0.89583333333333337</v>
       </c>
       <c r="F37" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -5067,7 +5061,7 @@
         <v>46205</v>
       </c>
       <c r="C38" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D38" s="2">
         <v>0.86805555555555558</v>
@@ -5076,7 +5070,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F38" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -5087,7 +5081,7 @@
         <v>46205</v>
       </c>
       <c r="C39" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D39" s="2">
         <v>0.89930555555555558</v>
@@ -5096,7 +5090,7 @@
         <v>0.94097222222222221</v>
       </c>
       <c r="F39" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -5107,7 +5101,7 @@
         <v>46205</v>
       </c>
       <c r="C40" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D40" s="2">
         <v>0.94097222222222221</v>
@@ -5116,7 +5110,7 @@
         <v>0.98263888888888884</v>
       </c>
       <c r="F40" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -5127,7 +5121,7 @@
         <v>46205</v>
       </c>
       <c r="C41" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D41" s="2">
         <v>0.96527777777777779</v>
@@ -5136,7 +5130,7 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F41" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -5147,7 +5141,7 @@
         <v>46205</v>
       </c>
       <c r="C42" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D42" s="2">
         <v>0.98958333333333337</v>
@@ -5156,7 +5150,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="F42" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -5167,7 +5161,7 @@
         <v>46205</v>
       </c>
       <c r="C43" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D43" s="2">
         <v>1.3888888888888888E-2</v>
@@ -5176,7 +5170,7 @@
         <v>6.5972222222222224E-2</v>
       </c>
       <c r="F43" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -5187,7 +5181,7 @@
         <v>46205</v>
       </c>
       <c r="C44" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D44" s="2">
         <v>4.1666666666666664E-2</v>
@@ -5196,7 +5190,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F44" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -5207,7 +5201,7 @@
         <v>46205</v>
       </c>
       <c r="C45" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D45" s="2">
         <v>6.5972222222222224E-2</v>
@@ -5216,7 +5210,7 @@
         <v>0.10069444444444445</v>
       </c>
       <c r="F45" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -5227,7 +5221,7 @@
         <v>46205</v>
       </c>
       <c r="C46" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D46" s="2">
         <v>0.10069444444444445</v>
@@ -5236,7 +5230,7 @@
         <v>0.1423611111111111</v>
       </c>
       <c r="F46" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -5247,7 +5241,7 @@
         <v>46206</v>
       </c>
       <c r="C47" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D47" s="2">
         <v>0.62847222222222221</v>
@@ -5256,7 +5250,7 @@
         <v>0.65972222222222221</v>
       </c>
       <c r="F47" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -5267,7 +5261,7 @@
         <v>46206</v>
       </c>
       <c r="C48" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D48" s="2">
         <v>0.62847222222222221</v>
@@ -5276,18 +5270,18 @@
         <v>0.65625</v>
       </c>
       <c r="F48" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B49" s="1">
         <v>46206</v>
       </c>
       <c r="C49" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D49" s="2">
         <v>0.65972222222222221</v>
@@ -5296,18 +5290,18 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F49" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B50" s="1">
         <v>46206</v>
       </c>
       <c r="C50" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D50" s="2">
         <v>0.65972222222222221</v>
@@ -5316,18 +5310,18 @@
         <v>0.69097222222222221</v>
       </c>
       <c r="F50" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B51" s="1">
         <v>46206</v>
       </c>
       <c r="C51" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D51" s="2">
         <v>0.69097222222222221</v>
@@ -5336,18 +5330,18 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F51" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B52" s="1">
         <v>46206</v>
       </c>
       <c r="C52" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D52" s="2">
         <v>0.69097222222222221</v>
@@ -5356,18 +5350,18 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="F52" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B53" s="1">
         <v>46206</v>
       </c>
       <c r="C53" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D53" s="2">
         <v>0.72222222222222221</v>
@@ -5376,18 +5370,18 @@
         <v>0.75694444444444442</v>
       </c>
       <c r="F53" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B54" s="1">
         <v>46206</v>
       </c>
       <c r="C54" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D54" s="2">
         <v>0.72222222222222221</v>
@@ -5396,18 +5390,18 @@
         <v>0.75694444444444442</v>
       </c>
       <c r="F54" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B55" s="1">
         <v>46206</v>
       </c>
       <c r="C55" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D55" s="2">
         <v>0.75694444444444442</v>
@@ -5416,18 +5410,18 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F55" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B56" s="1">
         <v>46206</v>
       </c>
       <c r="C56" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D56" s="2">
         <v>0.75694444444444442</v>
@@ -5436,18 +5430,18 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F56" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B57" s="1">
         <v>46206</v>
       </c>
       <c r="C57" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D57" s="2">
         <v>0.79166666666666663</v>
@@ -5456,18 +5450,18 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="F57" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B58" s="1">
         <v>46206</v>
       </c>
       <c r="C58" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D58" s="2">
         <v>0.79166666666666663</v>
@@ -5476,18 +5470,18 @@
         <v>0.82638888888888884</v>
       </c>
       <c r="F58" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B59" s="1">
         <v>46206</v>
       </c>
       <c r="C59" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D59" s="2">
         <v>0.83333333333333337</v>
@@ -5496,18 +5490,18 @@
         <v>0.86805555555555558</v>
       </c>
       <c r="F59" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B60" s="1">
         <v>46206</v>
       </c>
       <c r="C60" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D60" s="2">
         <v>0.83333333333333337</v>
@@ -5516,18 +5510,18 @@
         <v>0.86805555555555558</v>
       </c>
       <c r="F60" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B61" s="1">
         <v>46206</v>
       </c>
       <c r="C61" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D61" s="2">
         <v>0.86805555555555558</v>
@@ -5536,18 +5530,18 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="F61" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B62" s="1">
         <v>46206</v>
       </c>
       <c r="C62" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D62" s="2">
         <v>0.86805555555555558</v>
@@ -5556,18 +5550,18 @@
         <v>0.90972222222222221</v>
       </c>
       <c r="F62" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B63" s="1">
         <v>46206</v>
       </c>
       <c r="C63" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D63" s="2">
         <v>0.91666666666666663</v>
@@ -5576,18 +5570,18 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F63" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B64" s="1">
         <v>46206</v>
       </c>
       <c r="C64" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D64" s="2">
         <v>0.91666666666666663</v>
@@ -5596,18 +5590,18 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="F64" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B65" s="1">
         <v>46206</v>
       </c>
       <c r="C65" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D65" s="2">
         <v>0.95833333333333337</v>
@@ -5616,18 +5610,18 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B66" s="1">
         <v>46206</v>
       </c>
       <c r="C66" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D66" s="2">
         <v>0.96527777777777779</v>
@@ -5636,18 +5630,18 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="F66" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B67" s="1">
         <v>46206</v>
       </c>
       <c r="C67" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D67" s="2">
         <v>2.4305555555555556E-2</v>
@@ -5656,18 +5650,18 @@
         <v>5.9027777777777776E-2</v>
       </c>
       <c r="F67" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B68" s="1">
         <v>46206</v>
       </c>
       <c r="C68" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D68" s="2">
         <v>2.4305555555555556E-2</v>
@@ -5676,18 +5670,18 @@
         <v>7.2916666666666671E-2</v>
       </c>
       <c r="F68" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B69" s="1">
         <v>46206</v>
       </c>
       <c r="C69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D69" s="2">
         <v>5.9027777777777776E-2</v>
@@ -5696,18 +5690,18 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F69" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B70" s="1">
         <v>46206</v>
       </c>
       <c r="C70" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D70" s="2">
         <v>6.9444444444444448E-2</v>
@@ -5716,18 +5710,18 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F70" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B71" s="1">
         <v>46207</v>
       </c>
       <c r="C71" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D71" s="2">
         <v>0.61805555555555558</v>
@@ -5736,18 +5730,18 @@
         <v>0.65277777777777779</v>
       </c>
       <c r="F71" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B72" s="1">
         <v>46207</v>
       </c>
       <c r="C72" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D72" s="2">
         <v>0.61805555555555558</v>
@@ -5756,18 +5750,18 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F72" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B73" s="1">
         <v>46207</v>
       </c>
       <c r="C73" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D73" s="2">
         <v>0.65277777777777779</v>
@@ -5776,18 +5770,18 @@
         <v>0.68402777777777779</v>
       </c>
       <c r="F73" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B74" s="1">
         <v>46207</v>
       </c>
       <c r="C74" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D74" s="2">
         <v>0.65277777777777779</v>
@@ -5796,18 +5790,18 @@
         <v>0.68402777777777779</v>
       </c>
       <c r="F74" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B75" s="1">
         <v>46207</v>
       </c>
       <c r="C75" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D75" s="2">
         <v>0.68402777777777779</v>
@@ -5816,18 +5810,18 @@
         <v>0.71875</v>
       </c>
       <c r="F75" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B76" s="1">
         <v>46207</v>
       </c>
       <c r="C76" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D76" s="2">
         <v>0.68402777777777779</v>
@@ -5836,18 +5830,18 @@
         <v>0.71875</v>
       </c>
       <c r="F76" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B77" s="1">
         <v>46207</v>
       </c>
       <c r="C77" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D77" s="2">
         <v>0.71875</v>
@@ -5856,18 +5850,18 @@
         <v>0.75347222222222221</v>
       </c>
       <c r="F77" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B78" s="1">
         <v>46207</v>
       </c>
       <c r="C78" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D78" s="2">
         <v>0.71875</v>
@@ -5876,18 +5870,18 @@
         <v>0.75347222222222221</v>
       </c>
       <c r="F78" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B79" s="1">
         <v>46207</v>
       </c>
       <c r="C79" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D79" s="2">
         <v>0.75347222222222221</v>
@@ -5896,18 +5890,18 @@
         <v>0.79513888888888884</v>
       </c>
       <c r="F79" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B80" s="1">
         <v>46207</v>
       </c>
       <c r="C80" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D80" s="2">
         <v>0.76041666666666663</v>
@@ -5916,18 +5910,18 @@
         <v>0.79513888888888884</v>
       </c>
       <c r="F80" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B81" s="1">
         <v>46207</v>
       </c>
       <c r="C81" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D81" s="2">
         <v>0.79513888888888884</v>
@@ -5936,18 +5930,18 @@
         <v>0.82986111111111116</v>
       </c>
       <c r="F81" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B82" s="1">
         <v>46207</v>
       </c>
       <c r="C82" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D82" s="2">
         <v>0.79513888888888884</v>
@@ -5956,18 +5950,18 @@
         <v>0.82986111111111116</v>
       </c>
       <c r="F82" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B83" s="1">
         <v>46207</v>
       </c>
       <c r="C83" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D83" s="2">
         <v>0.82986111111111116</v>
@@ -5976,18 +5970,18 @@
         <v>0.87152777777777779</v>
       </c>
       <c r="F83" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B84" s="1">
         <v>46207</v>
       </c>
       <c r="C84" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D84" s="2">
         <v>0.82986111111111116</v>
@@ -5996,18 +5990,18 @@
         <v>0.87152777777777779</v>
       </c>
       <c r="F84" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B85" s="1">
         <v>46207</v>
       </c>
       <c r="C85" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D85" s="2">
         <v>0.87152777777777779</v>
@@ -6016,18 +6010,18 @@
         <v>0.91319444444444442</v>
       </c>
       <c r="F85" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B86" s="1">
         <v>46207</v>
       </c>
       <c r="C86" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D86" s="2">
         <v>0.87152777777777779</v>
@@ -6036,18 +6030,18 @@
         <v>0.91319444444444442</v>
       </c>
       <c r="F86" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B87" s="1">
         <v>46207</v>
       </c>
       <c r="C87" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D87" s="2">
         <v>0.91319444444444442</v>
@@ -6056,18 +6050,18 @@
         <v>0.96527777777777779</v>
       </c>
       <c r="F87" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B88" s="1">
         <v>46207</v>
       </c>
       <c r="C88" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D88" s="2">
         <v>0.91319444444444442</v>
@@ -6076,18 +6070,18 @@
         <v>0.95486111111111116</v>
       </c>
       <c r="F88" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B89" s="1">
         <v>46207</v>
       </c>
       <c r="C89" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D89" s="2">
         <v>0.96527777777777779</v>
@@ -6096,18 +6090,18 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F89" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B90" s="1">
         <v>46207</v>
       </c>
       <c r="C90" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D90" s="2">
         <v>0.96527777777777779</v>
@@ -6116,18 +6110,18 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="F90" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B91" s="1">
         <v>46207</v>
       </c>
       <c r="C91" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D91" s="2">
         <v>2.0833333333333332E-2</v>
@@ -6136,18 +6130,18 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F91" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B92" s="1">
         <v>46207</v>
       </c>
       <c r="C92" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D92" s="2">
         <v>3.4722222222222224E-2</v>
@@ -6156,18 +6150,18 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="F92" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B93" s="1">
         <v>46207</v>
       </c>
       <c r="C93" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D93" s="2">
         <v>9.0277777777777776E-2</v>
@@ -6176,18 +6170,18 @@
         <v>0.1423611111111111</v>
       </c>
       <c r="F93" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B94" s="1">
         <v>46207</v>
       </c>
       <c r="C94" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D94" s="2">
         <v>9.0277777777777776E-2</v>
@@ -6196,7 +6190,7 @@
         <v>0.1388888888888889</v>
       </c>
       <c r="F94" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -6219,19 +6213,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B1" t="s">
         <v>408</v>
       </c>
-      <c r="B1" t="s">
-        <v>409</v>
-      </c>
       <c r="C1" t="s">
+        <v>410</v>
+      </c>
+      <c r="D1" t="s">
         <v>411</v>
       </c>
-      <c r="D1" t="s">
-        <v>412</v>
-      </c>
       <c r="E1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -6248,7 +6242,7 @@
         <v>0.82638888888888884</v>
       </c>
       <c r="E2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -6265,7 +6259,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -6282,7 +6276,7 @@
         <v>0.875</v>
       </c>
       <c r="E4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -6299,12 +6293,12 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="E5" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B6" s="1">
         <v>46206</v>
@@ -6316,12 +6310,12 @@
         <v>0.8125</v>
       </c>
       <c r="E6" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B7" s="1">
         <v>46206</v>
@@ -6333,12 +6327,12 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B8" s="1">
         <v>46207</v>
@@ -6350,12 +6344,12 @@
         <v>0.6875</v>
       </c>
       <c r="E8" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B9" s="1">
         <v>46207</v>
@@ -6367,12 +6361,12 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="E9" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B10" s="1">
         <v>46207</v>
@@ -6384,7 +6378,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E10" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -6414,66 +6408,66 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D1" t="s">
         <v>421</v>
-      </c>
-      <c r="D1" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -6497,16 +6491,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>439</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>440</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>444</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -6514,13 +6508,13 @@
         <v>46202</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>442</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>443</v>
-      </c>
       <c r="D2" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -6528,13 +6522,13 @@
         <v>46203</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>446</v>
-      </c>
       <c r="D3" s="7" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -6542,13 +6536,13 @@
         <v>46204</v>
       </c>
       <c r="B4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C4" t="s">
         <v>447</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>448</v>
-      </c>
-      <c r="D4" t="s">
-        <v>449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Content: Add Leyendas del Rock 2026 data and assets
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -505,17 +505,63 @@
         <v>maparesu2026.jpg</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>leyendas-del-rock</v>
+      </c>
+      <c r="B3" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Leyendas del Rock</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Leyendas del Rock</v>
+      </c>
+      <c r="E3">
+        <v>2026</v>
+      </c>
+      <c r="F3">
+        <v>46239</v>
+      </c>
+      <c r="G3">
+        <v>46242</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Villena (Alicante)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Europe/Madrid</v>
+      </c>
+      <c r="J3">
+        <v>46239</v>
+      </c>
+      <c r="K3">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="L3">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="M3" t="str">
+        <v>logoleyendas.jpg</v>
+      </c>
+      <c r="N3" t="str">
+        <v>cartelleyendas.jpg</v>
+      </c>
+      <c r="O3" t="str">
+        <v>mapaleyendas.jpg</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2397,20 +2443,76 @@
         <v>https://www.youtube.com/watch?v=JVF6e_LSO2k</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>blindguardian</v>
+      </c>
+      <c r="B95" t="str">
+        <v>BLIND GUARDIAN</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Power Metal</v>
+      </c>
+      <c r="E95" t="str">
+        <v>¡Los bardos del metal vuelven a reclamar su trono! Blind Guardian traerán a Villena su espectacular power metal cargado de himnos legendarios coreados por miles de fans en todo el mundo. ¡Un concierto imprescindible! 🔥</v>
+      </c>
+      <c r="F95" t="str">
+        <v>https://www.youtube.com/watch?v=yY6mJg4b_rA</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>alestorm</v>
+      </c>
+      <c r="B96" t="str">
+        <v>ALESTORM</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Pirate Metal</v>
+      </c>
+      <c r="E96" t="str">
+        <v>¡Piratas al abordaje! Alestorm traerá su folk metal festivo, cerveza y patos de goma gigantes para montar la mayor fiesta del verano en el escenario del Leyendas 🤘🏴‍☠️</v>
+      </c>
+      <c r="F96" t="str">
+        <v>https://www.youtube.com/watch?v=ggyC0FOiN1Q</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>saurom</v>
+      </c>
+      <c r="B97" t="str">
+        <v>SAUROM</v>
+      </c>
+      <c r="C97" t="str">
+        <v>España</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Juglares, saltimbanquis e historias mágicas en una producción visual inigualable. Saurom presentará su concierto especial de gran formato en el escenario principal Jesús de la Rosa.</v>
+      </c>
+      <c r="F97" t="str">
+        <v>https://www.youtube.com/watch?v=F0f5i1vK760</v>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F92" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F97"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4574,9 +4676,78 @@
         <v>Programada</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B95" t="str">
+        <v>blindguardian</v>
+      </c>
+      <c r="C95">
+        <v>46239</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Jesús de la Rosa</v>
+      </c>
+      <c r="E95">
+        <v>0.9375</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B96" t="str">
+        <v>alestorm</v>
+      </c>
+      <c r="C96">
+        <v>46240</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Azucena</v>
+      </c>
+      <c r="E96">
+        <v>0.875</v>
+      </c>
+      <c r="F96">
+        <v>0.9270833333333334</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B97" t="str">
+        <v>saurom</v>
+      </c>
+      <c r="C97">
+        <v>46241</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Jesús de la Rosa</v>
+      </c>
+      <c r="E97">
+        <v>0.9895833333333334</v>
+      </c>
+      <c r="F97">
+        <v>1.0520833333333333</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G97"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4794,7 +4965,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4881,16 +5052,84 @@
         <v>#e67e22</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>jesus-de-la-rosa</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Jesús de la Rosa</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#ff2a85</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>azucena</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Azucena</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#2b8be3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>new-rock</v>
+      </c>
+      <c r="C8" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#9c1fb8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>mark-reale</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Mark Reale</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9" t="str">
+        <v>#e67e22</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4960,9 +5199,26 @@
         <v>El precio del billete por cada trayecto es de 1,60€, excepto la conexión con Vicedo en la que el importe es de 3,20€ por cada viaje.</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B5">
+        <v>46237</v>
+      </c>
+      <c r="C5" t="str">
+        <v>https://scontent.fbio3-1.fna.fbcdn.net/v/t39.99422-6/736343148_1348783289919456_2872457055456058256_n.png?stp=dst-jpg_tt6&amp;oh=00_AQCvNzvgxpKqAcfB1YIdDXCEaeRGLZ36Wd_DE1-yhrrG4A&amp;oe=6A4D9041</v>
+      </c>
+      <c r="D5" t="str">
+        <v>¡Bienvenidos a Leyendas del Rock 2026!</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Arranca la edición 2026 de Leyendas del Rock en Villena con el mejor heavy metal nacional e internacional. Revisa los horarios y escenarios.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Content: Add full Leyendas del Rock 2026 timetable and official images
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -45,7 +45,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -543,13 +543,13 @@
         <v>0.16666666666666666</v>
       </c>
       <c r="M3" t="str">
-        <v>logoleyendas.jpg</v>
+        <v>logoleyendas2026.jpg</v>
       </c>
       <c r="N3" t="str">
-        <v>cartelleyendas.jpg</v>
+        <v>cartelleyendas2026.jpg</v>
       </c>
       <c r="O3" t="str">
-        <v>mapaleyendas.jpg</v>
+        <v>mapaleyendas2026.jpg</v>
       </c>
     </row>
   </sheetData>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2503,16 +2503,1136 @@
         <v>https://www.youtube.com/watch?v=F0f5i1vK760</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>thundermother</v>
+      </c>
+      <c r="B98" t="str">
+        <v>THUNDERMOTHER</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Hard Rock</v>
+      </c>
+      <c r="E98" t="str">
+        <v>¡Las reinas suecas del hard rock llegan para tronar en el escenario principal! Con su rock clásico directo y enérgico, Thundermother garantizan decibelios y actitud.</v>
+      </c>
+      <c r="F98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>blacklabelsociety</v>
+      </c>
+      <c r="B99" t="str">
+        <v>BLACK LABEL SOCIETY</v>
+      </c>
+      <c r="C99" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Liderados por el legendario guitarrista Zakk Wylde, Black Label Society descargarán sus riffs pesados y solos vertiginosos que han marcado el metal sureño contemporáneo.</v>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>slaughtertoprevail</v>
+      </c>
+      <c r="B100" t="str">
+        <v>SLAUGHTER TO PREVAIL</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Rusia</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Deathcore</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Con el brutal Alex Terrible a las voces y sus icónicas máscaras doradas, Slaughter to Prevail desatarán la tormenta de deathcore más aplastante del festival.</v>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>salduie</v>
+      </c>
+      <c r="B101" t="str">
+        <v>SALDUIE</v>
+      </c>
+      <c r="C101" t="str">
+        <v>España</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Folk metal zaragozano de temática histórica celta-ibera. Vientos tradicionales y riffs de metal se fusionan en directo.</v>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>tailgunner</v>
+      </c>
+      <c r="B102" t="str">
+        <v>TAILGUNNER</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Considerados la punta de lanza de la nueva ola del heavy metal británico clásico. ¡Velocidad y guitarras gemelas garantizadas!</v>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>orbitculture</v>
+      </c>
+      <c r="B103" t="str">
+        <v>ORBIT CULTURE</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Death Metal Melódico</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Uno de los grupos revelación del metal moderno. Su combinación de death metal melódico, groove y elementos industriales es simplemente demoledora.</v>
+      </c>
+      <c r="F103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>savatage</v>
+      </c>
+      <c r="B104" t="str">
+        <v>SAVATAGE</v>
+      </c>
+      <c r="C104" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Metal Progresivo</v>
+      </c>
+      <c r="E104" t="str">
+        <v>¡Un regreso legendario! Savatage, pioneros del metal progresivo y sinfónico, ofrecerán un show exclusivo repasando su mítica trayectoria.</v>
+      </c>
+      <c r="F104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>sepultura</v>
+      </c>
+      <c r="B105" t="str">
+        <v>SEPULTURA</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Brasil</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Thrash Metal</v>
+      </c>
+      <c r="E105" t="str">
+        <v>En su gira mundial de despedida "Celebrating Life Through Death", los gigantes brasileños dirán adiós repasando cuatro décadas de historia.</v>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>heleven</v>
+      </c>
+      <c r="B106" t="str">
+        <v>HELEVEN</v>
+      </c>
+      <c r="C106" t="str">
+        <v>España</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Metal Alternativo</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Banda granadina que destaca por su metal oscuro, atmosférico y cargado de riffs de afinación baja y melodías intensas.</v>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>killus</v>
+      </c>
+      <c r="B107" t="str">
+        <v>KILLUS</v>
+      </c>
+      <c r="C107" t="str">
+        <v>España</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Metal Industrial</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Metal industrial y visual desde Villarreal. Una puesta en escena espectacular con maquillaje y sonidos mecánicos y potentes.</v>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>hadadanza</v>
+      </c>
+      <c r="B108" t="str">
+        <v>HADADANZA</v>
+      </c>
+      <c r="C108" t="str">
+        <v>España</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Folk metal con temática fantástica y fiestera que nos transportará a mundos medievales a ritmo de gaitas y violines.</v>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>signsoftheswarm</v>
+      </c>
+      <c r="B109" t="str">
+        <v>SIGNS OF THE SWARM</v>
+      </c>
+      <c r="C109" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Deathcore</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Deathcore ultrapesado y técnico desde Pittsburgh, listos para demoler el New Rock con breakdowns brutales.</v>
+      </c>
+      <c r="F109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>deathbats</v>
+      </c>
+      <c r="B110" t="str">
+        <v>DEATHBATS</v>
+      </c>
+      <c r="C110" t="str">
+        <v>España</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Tributo A7X</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Banda tributo a Avenged Sevenfold, reviviendo con fidelidad y energía los mejores éxitos de la formación californiana.</v>
+      </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>chainedsaint</v>
+      </c>
+      <c r="B111" t="str">
+        <v>CHAINED SAINT</v>
+      </c>
+      <c r="C111" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Thrash Metal</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Joven promesa del thrash metal estadounidense. Riffs rápidos y agresividad vieja escuela.</v>
+      </c>
+      <c r="F111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>promkinks</v>
+      </c>
+      <c r="B112" t="str">
+        <v>PROM KINKS</v>
+      </c>
+      <c r="C112" t="str">
+        <v>España</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Rock</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Banda de rock nacional con sonido enérgico y letras cargadas de rebeldía.</v>
+      </c>
+      <c r="F112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>mushroomhead</v>
+      </c>
+      <c r="B113" t="str">
+        <v>MUSHROOMHEAD</v>
+      </c>
+      <c r="C113" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Metal Alternativo</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Los enmascarados de Cleveland combinan metal industrial, alternativo y gótico en un directo teatral con doble batería de agua.</v>
+      </c>
+      <c r="F113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>darktranquillity</v>
+      </c>
+      <c r="B114" t="str">
+        <v>DARK TRANQUILLITY</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Death Metal Melódico</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Pioneros del sonido de Gotemburgo, liderados por Mikael Stanne, traerán su melancólica y veloz maestría melódica.</v>
+      </c>
+      <c r="F114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>archenemy</v>
+      </c>
+      <c r="B115" t="str">
+        <v>ARCH ENEMY</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Death Metal Melódico</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Liderados por la imponente Alissa White-Gluz y Michael Amott a las guitarras, Arch Enemy son los reyes indiscutibles del death metal melódico global.</v>
+      </c>
+      <c r="F115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>lepoka</v>
+      </c>
+      <c r="B116" t="str">
+        <v>LÈPOKA</v>
+      </c>
+      <c r="C116" t="str">
+        <v>España</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Folk metal cervecero y festivo desde Castellón. La fiesta está asegurada con sus melodías y ritmos pegadizos.</v>
+      </c>
+      <c r="F116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>creeper</v>
+      </c>
+      <c r="B117" t="str">
+        <v>CREEPER</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Goth Punk</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Glam rock y goth punk teatral de influencia ochentera. Creeper presentará un directo magnético y oscuro.</v>
+      </c>
+      <c r="F117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>northlane</v>
+      </c>
+      <c r="B118" t="str">
+        <v>NORTHLANE</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Metalcore</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Líderes mundiales del metalcore progresivo y la electrónica industrial. Presentarán su potente directo tecnológico.</v>
+      </c>
+      <c r="F118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>godsmack</v>
+      </c>
+      <c r="B119" t="str">
+        <v>GODSMACK</v>
+      </c>
+      <c r="C119" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Metal Alternativo</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Sully Erna y los suyos descargarán himnos del rock alternativo y post-grunge de finales de los noventa y dos mil.</v>
+      </c>
+      <c r="F119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>dartagnan</v>
+      </c>
+      <c r="B120" t="str">
+        <v>DARTAGNAN</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Folk Rock</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Folk rock de temática mosquetera. Espadas, violines y estribillos épicos cantados en alemán.</v>
+      </c>
+      <c r="F120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>ekyrian</v>
+      </c>
+      <c r="B121" t="str">
+        <v>EKYRIAN</v>
+      </c>
+      <c r="C121" t="str">
+        <v>España</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Folk metal madrileño con instrumentación clásica (flauta, gaita, violín) y letras basadas en leyendas y literatura fantástica.</v>
+      </c>
+      <c r="F121" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>landevir</v>
+      </c>
+      <c r="B122" t="str">
+        <v>LÁNDEVIR</v>
+      </c>
+      <c r="C122" t="str">
+        <v>España</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Veteranos del folk metal nacional procedentes de Elda. Melodías de origen celta combinadas con heavy metal clásico.</v>
+      </c>
+      <c r="F122" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>injector</v>
+      </c>
+      <c r="B123" t="str">
+        <v>INJECTOR</v>
+      </c>
+      <c r="C123" t="str">
+        <v>España</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Thrash Metal</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Thrash metal rápido, agresivo y de altísima calidad técnica procedente de Murcia.</v>
+      </c>
+      <c r="F123" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>evo</v>
+      </c>
+      <c r="B124" t="str">
+        <v>EVO</v>
+      </c>
+      <c r="C124" t="str">
+        <v>España</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Leyenda del heavy metal madrileño de los años ochenta, listos para revivir himnos como "Animal de ciudad".</v>
+      </c>
+      <c r="F124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>celtibeerian</v>
+      </c>
+      <c r="B125" t="str">
+        <v>CELTIBEERIAN</v>
+      </c>
+      <c r="C125" t="str">
+        <v>España</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Folk Metal</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Folk metal fiestero e irreverente. Cerveza, gaitas y diversión garantizada en el escenario New Rock.</v>
+      </c>
+      <c r="F125" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>bolu2death</v>
+      </c>
+      <c r="B126" t="str">
+        <v>BOLU2 DEATH</v>
+      </c>
+      <c r="C126" t="str">
+        <v>España</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Metalcore/Electronic</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Huesca metalcore y dubstep fusionados en una bomba de energía brutal.</v>
+      </c>
+      <c r="F126" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>futurepalace</v>
+      </c>
+      <c r="B127" t="str">
+        <v>FUTURE PALACE</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Post-Hardcore</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Trío alemán de post-hardcore y metal alternativo liderado por Maria Lessing, con melodías emocionales y breakdowns pesados.</v>
+      </c>
+      <c r="F127" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>saratoga</v>
+      </c>
+      <c r="B128" t="str">
+        <v>SARATOGA</v>
+      </c>
+      <c r="C128" t="str">
+        <v>España</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E128" t="str">
+        <v>La apisonadora del heavy metal español. Tete Novoa, Jero Ramiro y Niko del Hierro repasarán sus mayores clásicos.</v>
+      </c>
+      <c r="F128" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>inflames</v>
+      </c>
+      <c r="B129" t="str">
+        <v>IN FLAMES</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Metal Alternativo</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Una de las bandas más influyentes de la historia del metal. De inventores del death metal melódico a gigantes del metal alternativo moderno.</v>
+      </c>
+      <c r="F129" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>darkmoor</v>
+      </c>
+      <c r="B130" t="str">
+        <v>DARK MOOR</v>
+      </c>
+      <c r="C130" t="str">
+        <v>España</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Metal Sinfónico</v>
+      </c>
+      <c r="E130" t="str">
+        <v>Pioneros del metal sinfónico y neoclásico en España, con una larga trayectoria internacional.</v>
+      </c>
+      <c r="F130" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>chezkane</v>
+      </c>
+      <c r="B131" t="str">
+        <v>CHEZ KANE</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Hard Rock</v>
+      </c>
+      <c r="E131" t="str">
+        <v>La gran voz del hard rock melódico ochentero actual. Chez Kane y su banda nos transportarán a la era dorada del AOR.</v>
+      </c>
+      <c r="F131" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>thebaboonshow</v>
+      </c>
+      <c r="B132" t="str">
+        <v>THE BABOON SHOW</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Punk Rock</v>
+      </c>
+      <c r="E132" t="str">
+        <v>¡Pura dinamita en directo! La banda de punk rock sueca liderada por la electrizante Cecilia Boström ofrecerá uno de los shows más enérgicos del festival.</v>
+      </c>
+      <c r="F132" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>stratovarius</v>
+      </c>
+      <c r="B133" t="str">
+        <v>STRATOVARIUS</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Finlandia</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Power Metal</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Los padres finlandeses del power metal sinfónico descargarán himnos inmortales como "Hunting High and Low" y "Black Diamond".</v>
+      </c>
+      <c r="F133" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>xeria</v>
+      </c>
+      <c r="B134" t="str">
+        <v>XERIA</v>
+      </c>
+      <c r="C134" t="str">
+        <v>España</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Metal Sinfónico</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Banda vallisoletana de metal sinfónico y alternativo, con grandes melodías vocales a cargo de Marina Sweet.</v>
+      </c>
+      <c r="F134" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>wingsofsteel</v>
+      </c>
+      <c r="B135" t="str">
+        <v>WINGS OF STEEL</v>
+      </c>
+      <c r="C135" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Hard Rock</v>
+      </c>
+      <c r="E135" t="str">
+        <v>Hard rock clásico y heavy metal de la costa oeste con riffs potentes y voz espectacular.</v>
+      </c>
+      <c r="F135" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>againstmyself</v>
+      </c>
+      <c r="B136" t="str">
+        <v>AGAINST MYSELF</v>
+      </c>
+      <c r="C136" t="str">
+        <v>España</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Metal Sinfónico</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Banda de metal sinfónico y progresivo que destaca por sus composiciones complejas e intensas atmósferas.</v>
+      </c>
+      <c r="F136" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>employedtoserve</v>
+      </c>
+      <c r="B137" t="str">
+        <v>EMPLOYED TO SERVE</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Metalcore</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Desde el Reino Unido llega uno de los directos de metalcore y hardcore más pesados y viscerales de la actualidad.</v>
+      </c>
+      <c r="F137" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>daeria</v>
+      </c>
+      <c r="B138" t="str">
+        <v>DAERIA</v>
+      </c>
+      <c r="C138" t="str">
+        <v>España</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Metal Alternativo</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Heavy metal moderno y alternativo con potentes guitarras y una impecable ejecución vocal.</v>
+      </c>
+      <c r="F138" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>minddriller</v>
+      </c>
+      <c r="B139" t="str">
+        <v>MIND DRILLER</v>
+      </c>
+      <c r="C139" t="str">
+        <v>España</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Metal Industrial</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Banda de metal industrial con tres vocalistas (masculino, femenino y gutural) que crean una mezcla de voces única.</v>
+      </c>
+      <c r="F139" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>jordiwilddjset</v>
+      </c>
+      <c r="B140" t="str">
+        <v>JORDI WILD DJ SET</v>
+      </c>
+      <c r="C140" t="str">
+        <v>España</v>
+      </c>
+      <c r="D140" t="str">
+        <v>DJ Set</v>
+      </c>
+      <c r="E140" t="str">
+        <v>El creador de contenido y melómano Jordi Wild cerrará la noche del viernes con un DJ Set cargado de clásicos del rock y el metal.</v>
+      </c>
+      <c r="F140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>guilttrip</v>
+      </c>
+      <c r="B141" t="str">
+        <v>GUILT TRIP</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Reino Unido</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Hardcore</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Hardcore metalizado directo desde Manchester para desatar los moshpits más salvajes de la jornada.</v>
+      </c>
+      <c r="F141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>deicide</v>
+      </c>
+      <c r="B142" t="str">
+        <v>DEICIDE</v>
+      </c>
+      <c r="C142" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Death Metal</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Liderados por el infame Glen Benton, los reyes del death metal satánico clásico descargarán su brutal repertorio blasfemo.</v>
+      </c>
+      <c r="F142" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>helloween</v>
+      </c>
+      <c r="B143" t="str">
+        <v>HELLOWEEN</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Power Metal</v>
+      </c>
+      <c r="E143" t="str">
+        <v>¡El cabeza de cartel indiscutible! Los creadores del power metal Helloween regresan con su show completo de aniversario para reinar en Villena.</v>
+      </c>
+      <c r="F143" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>ankhara</v>
+      </c>
+      <c r="B144" t="str">
+        <v>ANKHARA</v>
+      </c>
+      <c r="C144" t="str">
+        <v>España</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E144" t="str">
+        <v>Gran banda madrileña de heavy metal clásico con tintes power metal y la inconfundible voz de Pacho Brea.</v>
+      </c>
+      <c r="F144" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>eihwar</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="C145" t="str">
+        <v/>
+      </c>
+      <c r="D145" t="str">
+        <v>Pagan Folk</v>
+      </c>
+      <c r="E145" t="str">
+        <v>Folk pagano nórdico mezclado con ritmos electrónicos de techno y trance. ¡Una experiencia ritual y bailable única!</v>
+      </c>
+      <c r="F145" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>heavenshallburn</v>
+      </c>
+      <c r="B146" t="str">
+        <v>HEAVEN SHALL BURN</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Melodic Death Metal</v>
+      </c>
+      <c r="E146" t="str">
+        <v>La apisonadora alemana de death metal melódico y metalcore desatará una tormenta de moshpits épicos.</v>
+      </c>
+      <c r="F146" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>warcry</v>
+      </c>
+      <c r="B147" t="str">
+        <v>WARCRY</v>
+      </c>
+      <c r="C147" t="str">
+        <v>España</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E147" t="str">
+        <v>Víctor García y sus chicos regresan al Leyendas para descargar sus himnos inmortales de heavy metal coreados por miles de almas.</v>
+      </c>
+      <c r="F147" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>deathandlegacy</v>
+      </c>
+      <c r="B148" t="str">
+        <v>DEATH AND LEGACY</v>
+      </c>
+      <c r="C148" t="str">
+        <v>España</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Death Metal Melódico</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Banda de death melódico liderada por Hynphernia, que destaca por su contundencia y atmósfera oscura.</v>
+      </c>
+      <c r="F148" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>latzen</v>
+      </c>
+      <c r="B149" t="str">
+        <v>LATZEN</v>
+      </c>
+      <c r="C149" t="str">
+        <v>España</v>
+      </c>
+      <c r="D149" t="str">
+        <v>Heavy Metal</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Mítica banda de heavy metal euskaldun, listos para recordar clásicos atemporales.</v>
+      </c>
+      <c r="F149" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>hardline</v>
+      </c>
+      <c r="B150" t="str">
+        <v>EEUU</v>
+      </c>
+      <c r="C150" t="str">
+        <v/>
+      </c>
+      <c r="D150" t="str">
+        <v>Hard Rock</v>
+      </c>
+      <c r="E150" t="str">
+        <v>El cantante Johnny Gioeli lidera esta banda de hard rock melódico nacida en los noventa.</v>
+      </c>
+      <c r="F150" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>ten56</v>
+      </c>
+      <c r="B151" t="str">
+        <v>TEN56.</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Deathcore</v>
+      </c>
+      <c r="E151" t="str">
+        <v>Metal oscuro y deathcore de vanguardia con toques industriales y breakdowns opresivos.</v>
+      </c>
+      <c r="F151" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>halfme</v>
+      </c>
+      <c r="B152" t="str">
+        <v>HALF ME</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="D152" t="str">
+        <v>Metalcore</v>
+      </c>
+      <c r="E152" t="str">
+        <v>Metalcore experimental y agresivo firmado por uno de los nuevos estandartes del sello Arising Empire.</v>
+      </c>
+      <c r="F152" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>cabal</v>
+      </c>
+      <c r="B153" t="str">
+        <v>CABAL</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Dinamarca</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Deathcore</v>
+      </c>
+      <c r="E153" t="str">
+        <v>Metal extremo oscuro e inquietante directo desde Copenhague.</v>
+      </c>
+      <c r="F153" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F153"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4681,19 +5801,19 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B95" t="str">
-        <v>blindguardian</v>
+        <v>thundermother</v>
       </c>
       <c r="C95">
         <v>46239</v>
       </c>
       <c r="D95" t="str">
-        <v>Jesús de la Rosa</v>
+        <v>Dave Mustaine</v>
       </c>
       <c r="E95">
-        <v>0.9375</v>
+        <v>0.7430555555555556</v>
       </c>
       <c r="F95">
-        <v>1</v>
+        <v>0.7847222222222222</v>
       </c>
       <c r="G95" t="str">
         <v>Programada</v>
@@ -4704,19 +5824,19 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B96" t="str">
-        <v>alestorm</v>
+        <v>blacklabelsociety</v>
       </c>
       <c r="C96">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="D96" t="str">
-        <v>Azucena</v>
+        <v>Dave Mustaine</v>
       </c>
       <c r="E96">
-        <v>0.875</v>
+        <v>0.8402777777777778</v>
       </c>
       <c r="F96">
-        <v>0.9270833333333334</v>
+        <v>0.8819444444444444</v>
       </c>
       <c r="G96" t="str">
         <v>Programada</v>
@@ -4727,27 +5847,1315 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B97" t="str">
+        <v>slaughtertoprevail</v>
+      </c>
+      <c r="C97">
+        <v>46239</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E97">
+        <v>0.9513888888888888</v>
+      </c>
+      <c r="F97">
+        <v>0.006944444444444444</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B98" t="str">
+        <v>salduie</v>
+      </c>
+      <c r="C98">
+        <v>46239</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E98">
+        <v>0.0763888888888889</v>
+      </c>
+      <c r="F98">
+        <v>0.125</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B99" t="str">
+        <v>tailgunner</v>
+      </c>
+      <c r="C99">
+        <v>46239</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E99">
+        <v>0.7013888888888888</v>
+      </c>
+      <c r="F99">
+        <v>0.7361111111111112</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B100" t="str">
+        <v>orbitculture</v>
+      </c>
+      <c r="C100">
+        <v>46239</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E100">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="F100">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G100" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B101" t="str">
+        <v>savatage</v>
+      </c>
+      <c r="C101">
+        <v>46239</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E101">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="F101">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B102" t="str">
+        <v>sepultura</v>
+      </c>
+      <c r="C102">
+        <v>46239</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E102">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="F102">
+        <v>0.06944444444444445</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B103" t="str">
+        <v>heleven</v>
+      </c>
+      <c r="C103">
+        <v>46239</v>
+      </c>
+      <c r="D103" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E103">
+        <v>0.7118055555555556</v>
+      </c>
+      <c r="F103">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B104" t="str">
+        <v>killus</v>
+      </c>
+      <c r="C104">
+        <v>46239</v>
+      </c>
+      <c r="D104" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E104">
+        <v>0.7638888888888888</v>
+      </c>
+      <c r="F104">
+        <v>0.7986111111111112</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B105" t="str">
+        <v>hadadanza</v>
+      </c>
+      <c r="C105">
+        <v>46239</v>
+      </c>
+      <c r="D105" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E105">
+        <v>0.8159722222222222</v>
+      </c>
+      <c r="F105">
+        <v>0.8506944444444444</v>
+      </c>
+      <c r="G105" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B106" t="str">
+        <v>signsoftheswarm</v>
+      </c>
+      <c r="C106">
+        <v>46239</v>
+      </c>
+      <c r="D106" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E106">
+        <v>0.8680555555555556</v>
+      </c>
+      <c r="F106">
+        <v>0.9027777777777778</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B107" t="str">
+        <v>deathbats</v>
+      </c>
+      <c r="C107">
+        <v>46239</v>
+      </c>
+      <c r="D107" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E107">
+        <v>0.9201388888888888</v>
+      </c>
+      <c r="F107">
+        <v>0.9548611111111112</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B108" t="str">
+        <v>chainedsaint</v>
+      </c>
+      <c r="C108">
+        <v>46239</v>
+      </c>
+      <c r="D108" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E108">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="F108">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B109" t="str">
+        <v>promkinks</v>
+      </c>
+      <c r="C109">
+        <v>46239</v>
+      </c>
+      <c r="D109" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E109">
+        <v>0.03125</v>
+      </c>
+      <c r="F109">
+        <v>0.07291666666666667</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B110" t="str">
+        <v>mushroomhead</v>
+      </c>
+      <c r="C110">
+        <v>46240</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E110">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="F110">
+        <v>0.7847222222222222</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B111" t="str">
+        <v>darktranquillity</v>
+      </c>
+      <c r="C111">
+        <v>46240</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E111">
+        <v>0.8402777777777778</v>
+      </c>
+      <c r="F111">
+        <v>0.8819444444444444</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B112" t="str">
+        <v>archenemy</v>
+      </c>
+      <c r="C112">
+        <v>46240</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E112">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="F112">
+        <v>0.006944444444444444</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B113" t="str">
+        <v>lepoka</v>
+      </c>
+      <c r="C113">
+        <v>46240</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E113">
+        <v>0.0763888888888889</v>
+      </c>
+      <c r="F113">
+        <v>0.125</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B114" t="str">
+        <v>creeper</v>
+      </c>
+      <c r="C114">
+        <v>46240</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E114">
+        <v>0.7013888888888888</v>
+      </c>
+      <c r="F114">
+        <v>0.7361111111111112</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B115" t="str">
+        <v>northlane</v>
+      </c>
+      <c r="C115">
+        <v>46240</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E115">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="F115">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B116" t="str">
+        <v>godsmack</v>
+      </c>
+      <c r="C116">
+        <v>46240</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E116">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="F116">
+        <v>0.9375</v>
+      </c>
+      <c r="G116" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B117" t="str">
+        <v>dartagnan</v>
+      </c>
+      <c r="C117">
+        <v>46240</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E117">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="F117">
+        <v>0.06944444444444445</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B118" t="str">
+        <v>ekyrian</v>
+      </c>
+      <c r="C118">
+        <v>46240</v>
+      </c>
+      <c r="D118" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E118">
+        <v>0.7118055555555556</v>
+      </c>
+      <c r="F118">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="G118" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B119" t="str">
+        <v>aneuma</v>
+      </c>
+      <c r="C119">
+        <v>46240</v>
+      </c>
+      <c r="D119" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E119">
+        <v>0.7638888888888888</v>
+      </c>
+      <c r="F119">
+        <v>0.7986111111111112</v>
+      </c>
+      <c r="G119" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B120" t="str">
+        <v>landevir</v>
+      </c>
+      <c r="C120">
+        <v>46240</v>
+      </c>
+      <c r="D120" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E120">
+        <v>0.8159722222222222</v>
+      </c>
+      <c r="F120">
+        <v>0.8506944444444444</v>
+      </c>
+      <c r="G120" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B121" t="str">
+        <v>injector</v>
+      </c>
+      <c r="C121">
+        <v>46240</v>
+      </c>
+      <c r="D121" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E121">
+        <v>0.8680555555555556</v>
+      </c>
+      <c r="F121">
+        <v>0.9027777777777778</v>
+      </c>
+      <c r="G121" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B122" t="str">
+        <v>evo</v>
+      </c>
+      <c r="C122">
+        <v>46240</v>
+      </c>
+      <c r="D122" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E122">
+        <v>0.9201388888888888</v>
+      </c>
+      <c r="F122">
+        <v>0.9548611111111112</v>
+      </c>
+      <c r="G122" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B123" t="str">
+        <v>celtibeerian</v>
+      </c>
+      <c r="C123">
+        <v>46240</v>
+      </c>
+      <c r="D123" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E123">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="F123">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="G123" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B124" t="str">
+        <v>bolu2death</v>
+      </c>
+      <c r="C124">
+        <v>46240</v>
+      </c>
+      <c r="D124" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E124">
+        <v>0.03125</v>
+      </c>
+      <c r="F124">
+        <v>0.07291666666666667</v>
+      </c>
+      <c r="G124" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B125" t="str">
+        <v>futurepalace</v>
+      </c>
+      <c r="C125">
+        <v>46241</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E125">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="F125">
+        <v>0.7847222222222222</v>
+      </c>
+      <c r="G125" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B126" t="str">
+        <v>saratoga</v>
+      </c>
+      <c r="C126">
+        <v>46241</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E126">
+        <v>0.8402777777777778</v>
+      </c>
+      <c r="F126">
+        <v>0.8819444444444444</v>
+      </c>
+      <c r="G126" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B127" t="str">
+        <v>inflames</v>
+      </c>
+      <c r="C127">
+        <v>46241</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E127">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="F127">
+        <v>0.006944444444444444</v>
+      </c>
+      <c r="G127" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B128" t="str">
+        <v>darkmoor</v>
+      </c>
+      <c r="C128">
+        <v>46241</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E128">
+        <v>0.0763888888888889</v>
+      </c>
+      <c r="F128">
+        <v>0.125</v>
+      </c>
+      <c r="G128" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B129" t="str">
+        <v>chezkane</v>
+      </c>
+      <c r="C129">
+        <v>46241</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E129">
+        <v>0.7013888888888888</v>
+      </c>
+      <c r="F129">
+        <v>0.7361111111111112</v>
+      </c>
+      <c r="G129" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B130" t="str">
+        <v>thebaboonshow</v>
+      </c>
+      <c r="C130">
+        <v>46241</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E130">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="F130">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G130" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B131" t="str">
+        <v>stratovarius</v>
+      </c>
+      <c r="C131">
+        <v>46241</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E131">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="F131">
+        <v>0.9375</v>
+      </c>
+      <c r="G131" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B132" t="str">
         <v>saurom</v>
       </c>
-      <c r="C97">
+      <c r="C132">
         <v>46241</v>
       </c>
-      <c r="D97" t="str">
-        <v>Jesús de la Rosa</v>
-      </c>
-      <c r="E97">
-        <v>0.9895833333333334</v>
-      </c>
-      <c r="F97">
-        <v>1.0520833333333333</v>
-      </c>
-      <c r="G97" t="str">
+      <c r="D132" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E132">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="F132">
+        <v>0.06944444444444445</v>
+      </c>
+      <c r="G132" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B133" t="str">
+        <v>xeria</v>
+      </c>
+      <c r="C133">
+        <v>46241</v>
+      </c>
+      <c r="D133" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E133">
+        <v>0.7118055555555556</v>
+      </c>
+      <c r="F133">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="G133" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B134" t="str">
+        <v>wingsofsteel</v>
+      </c>
+      <c r="C134">
+        <v>46241</v>
+      </c>
+      <c r="D134" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E134">
+        <v>0.7638888888888888</v>
+      </c>
+      <c r="F134">
+        <v>0.7986111111111112</v>
+      </c>
+      <c r="G134" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B135" t="str">
+        <v>againstmyself</v>
+      </c>
+      <c r="C135">
+        <v>46241</v>
+      </c>
+      <c r="D135" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E135">
+        <v>0.8159722222222222</v>
+      </c>
+      <c r="F135">
+        <v>0.8506944444444444</v>
+      </c>
+      <c r="G135" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B136" t="str">
+        <v>employedtoserve</v>
+      </c>
+      <c r="C136">
+        <v>46241</v>
+      </c>
+      <c r="D136" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E136">
+        <v>0.8680555555555556</v>
+      </c>
+      <c r="F136">
+        <v>0.9027777777777778</v>
+      </c>
+      <c r="G136" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B137" t="str">
+        <v>daeria</v>
+      </c>
+      <c r="C137">
+        <v>46241</v>
+      </c>
+      <c r="D137" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E137">
+        <v>0.9201388888888888</v>
+      </c>
+      <c r="F137">
+        <v>0.9548611111111112</v>
+      </c>
+      <c r="G137" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B138" t="str">
+        <v>minddriller</v>
+      </c>
+      <c r="C138">
+        <v>46241</v>
+      </c>
+      <c r="D138" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E138">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="F138">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="G138" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B139" t="str">
+        <v>jordiwilddjset</v>
+      </c>
+      <c r="C139">
+        <v>46241</v>
+      </c>
+      <c r="D139" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E139">
+        <v>0.03125</v>
+      </c>
+      <c r="F139">
+        <v>0.07291666666666667</v>
+      </c>
+      <c r="G139" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B140" t="str">
+        <v>guilttrip</v>
+      </c>
+      <c r="C140">
+        <v>46242</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E140">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="F140">
+        <v>0.75</v>
+      </c>
+      <c r="G140" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B141" t="str">
+        <v>deicide</v>
+      </c>
+      <c r="C141">
+        <v>46242</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E141">
+        <v>0.8055555555555556</v>
+      </c>
+      <c r="F141">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="G141" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B142" t="str">
+        <v>helloween</v>
+      </c>
+      <c r="C142">
+        <v>46242</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E142">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="F142">
+        <v>0</v>
+      </c>
+      <c r="G142" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B143" t="str">
+        <v>ankhara</v>
+      </c>
+      <c r="C143">
+        <v>46242</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Dave Mustaine</v>
+      </c>
+      <c r="E143">
+        <v>0.0763888888888889</v>
+      </c>
+      <c r="F143">
+        <v>0.125</v>
+      </c>
+      <c r="G143" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B144" t="str">
+        <v>eihwar</v>
+      </c>
+      <c r="C144">
+        <v>46242</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E144">
+        <v>0.7569444444444444</v>
+      </c>
+      <c r="F144">
+        <v>0.7986111111111112</v>
+      </c>
+      <c r="G144" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B145" t="str">
+        <v>heavenshallburn</v>
+      </c>
+      <c r="C145">
+        <v>46242</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E145">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="F145">
+        <v>0.9097222222222222</v>
+      </c>
+      <c r="G145" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B146" t="str">
+        <v>warcry</v>
+      </c>
+      <c r="C146">
+        <v>46242</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Doro Pesch</v>
+      </c>
+      <c r="E146">
+        <v>0.006944444444444444</v>
+      </c>
+      <c r="F146">
+        <v>0.06944444444444445</v>
+      </c>
+      <c r="G146" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B147" t="str">
+        <v>deathandlegacy</v>
+      </c>
+      <c r="C147">
+        <v>46242</v>
+      </c>
+      <c r="D147" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E147">
+        <v>0.7118055555555556</v>
+      </c>
+      <c r="F147">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="G147" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B148" t="str">
+        <v>fallenatdawn</v>
+      </c>
+      <c r="C148">
+        <v>46242</v>
+      </c>
+      <c r="D148" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E148">
+        <v>0.7638888888888888</v>
+      </c>
+      <c r="F148">
+        <v>0.7986111111111112</v>
+      </c>
+      <c r="G148" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B149" t="str">
+        <v>latzen</v>
+      </c>
+      <c r="C149">
+        <v>46242</v>
+      </c>
+      <c r="D149" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E149">
+        <v>0.8159722222222222</v>
+      </c>
+      <c r="F149">
+        <v>0.8506944444444444</v>
+      </c>
+      <c r="G149" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B150" t="str">
+        <v>hardline</v>
+      </c>
+      <c r="C150">
+        <v>46242</v>
+      </c>
+      <c r="D150" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E150">
+        <v>0.8680555555555556</v>
+      </c>
+      <c r="F150">
+        <v>0.9027777777777778</v>
+      </c>
+      <c r="G150" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B151" t="str">
+        <v>ten56</v>
+      </c>
+      <c r="C151">
+        <v>46242</v>
+      </c>
+      <c r="D151" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E151">
+        <v>0.9201388888888888</v>
+      </c>
+      <c r="F151">
+        <v>0.9548611111111112</v>
+      </c>
+      <c r="G151" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B152" t="str">
+        <v>halfme</v>
+      </c>
+      <c r="C152">
+        <v>46242</v>
+      </c>
+      <c r="D152" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E152">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="F152">
+        <v>0.013888888888888888</v>
+      </c>
+      <c r="G152" t="str">
+        <v>Programada</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>leyendas-del-rock-2026</v>
+      </c>
+      <c r="B153" t="str">
+        <v>cabal</v>
+      </c>
+      <c r="C153">
+        <v>46242</v>
+      </c>
+      <c r="D153" t="str">
+        <v>New Rock</v>
+      </c>
+      <c r="E153">
+        <v>0.03125</v>
+      </c>
+      <c r="F153">
+        <v>0.07291666666666667</v>
+      </c>
+      <c r="G153" t="str">
         <v>Programada</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G153"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4957,6 +7365,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
@@ -4965,7 +7374,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5057,10 +7466,10 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B6" t="str">
-        <v>jesus-de-la-rosa</v>
+        <v>dave-mustane-stage</v>
       </c>
       <c r="C6" t="str">
-        <v>Jesús de la Rosa</v>
+        <v>Dave Mustaine</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -5074,10 +7483,10 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B7" t="str">
-        <v>azucena</v>
+        <v>doro-tesch-stage</v>
       </c>
       <c r="C7" t="str">
-        <v>Azucena</v>
+        <v>Doro Pesch</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -5091,7 +7500,7 @@
         <v>leyendas-del-rock-2026</v>
       </c>
       <c r="B8" t="str">
-        <v>new-rock</v>
+        <v>new-rock-stage</v>
       </c>
       <c r="C8" t="str">
         <v>New Rock</v>
@@ -5103,26 +7512,10 @@
         <v>#9c1fb8</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>leyendas-del-rock-2026</v>
-      </c>
-      <c r="B9" t="str">
-        <v>mark-reale</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Mark Reale</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9" t="str">
-        <v>#e67e22</v>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5217,6 +7610,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Content: Genericize all band descriptions and verify no duplicates
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -43,9 +43,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -481,7 +480,7 @@
         <v>46207</v>
       </c>
       <c r="H2" t="str">
-        <v>Viveiro</v>
+        <v>Viveiro (Lugo)</v>
       </c>
       <c r="I2" t="str">
         <v>Europe/Madrid</v>
@@ -553,6 +552,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
@@ -617,7 +617,7 @@
         <v>Metal Alternativo</v>
       </c>
       <c r="E3" t="str">
-        <v>Después de tocar en la carpa Red Bull en 2024, la joven banda coruñesa de metal formada en 2021 regresa al festi para abrir fuego en el Chaos Stage el próximo miércoles 1 de julio 🧨  El quinteto Crowded vuelve al Resu con un segundo EP estrenado a principios de año titulado "Kindred Spirits" que releva a su debut "Underdogs" de 2023 forjando su sonido mezcla de metal alternativo y rock noventero e influencias del thrash y metalcore 🤘  ¡No te pierdas a una de las propuestas más jóvenes y con más potencial de esta edición! ¡Venid a apoyarlos como merecen! 🙌</v>
+        <v>Después de tocar en la carpa Red Bull en 2024, la joven banda coruñesa de metal formada en 2021 regresa al festi para abrir fuego en el Chaos Stage el próximo miércoles 1 de julio 🧨  El quinteto Crowded vuelve al Resu con un segundo EP estrenado a principios de año titulado "Kindred Spirits" que releva a su debut "Underdogs" de 2023 forjando su sonido mezcla de metal alternativo y rock noventero e influencias del thrash y metalcore 🤘  ¡No te pierdas a una de las propuestas más jóvenes y con más potencial de sus giras! ¡Venid a apoyarlos como merecen! 🙌</v>
       </c>
       <c r="F3" t="str">
         <v>https://www.youtube.com/watch?v=5LrDrFgDyl4</v>
@@ -737,7 +737,7 @@
         <v>Hard Rock</v>
       </c>
       <c r="E9" t="str">
-        <v>PRESIDENT apareció de la nada en 2025, y en cuestión de semanas se convirtió en uno de los fenómenos virales más duros del metal moderno. El colectivo británico dirigido por su líder homónimo The President se suma a esta edición para captar devotos en su genial propuesta 🤫  Con más de 50 millones de reproducciones en plataformas, es la nueva sensación que lo está petando entre curiosxs y fans de Dayseeker, Sleep Theory o Bad Omens. Metalcore y post-hardcore de primera con una chispa de R\&amp;B y pop que lo hace único 🙌 ¡No te puedes perder esta locura el primer día de festi en el Main Stage! 🔥</v>
+        <v>PRESIDENT apareció de la nada en 2025, y en cuestión de semanas se convirtió en uno de los fenómenos virales más duros del metal moderno. El colectivo británico dirigido por su líder homónimo The President se suma a sus giras para captar devotos en su genial propuesta 🤫  Con más de 50 millones de reproducciones en plataformas, es la nueva sensación que lo está petando entre curiosxs y fans de Dayseeker, Sleep Theory o Bad Omens. Metalcore y post-hardcore de primera con una chispa de R\&amp;B y pop que lo hace único 🙌 ¡No te puedes perder esta locura el primer día de festi en el Main Stage! 🔥</v>
       </c>
       <c r="F9" t="str">
         <v>https://www.youtube.com/watch?v=aczq-iCfFOk</v>
@@ -757,7 +757,7 @@
         <v>Deathcore</v>
       </c>
       <c r="E10" t="str">
-        <v>No tenemos dudas de que el concierto de Immortal Disfigurement será uno de las más bestias de esta edición. Vienen de Pittsburgh y están liderados por CJ McCreery, un fuera de serie dentro del deathcore que ha formado parte de bandas como Lorna Shore y Signs Of The Swarm y que os dejará con la boca abierta desde el minuto 0 😱  Guturales inhumanos, una agresividad al límite con breakdowns sin ningún sentido, y mucha técnica y sinfonías que os harán experimentar cómo suenan la violencia y oscuridad de verdad 👹</v>
+        <v>No tenemos dudas de que el concierto de Immortal Disfigurement será uno de las más bestias de sus giras. Vienen de Pittsburgh y están liderados por CJ McCreery, un fuera de serie dentro del deathcore que ha formado parte de bandas como Lorna Shore y Signs Of The Swarm y que os dejará con la boca abierta desde el minuto 0 😱  Guturales inhumanos, una agresividad al límite con breakdowns sin ningún sentido, y mucha técnica y sinfonías que os harán experimentar cómo suenan la violencia y oscuridad de verdad 👹</v>
       </c>
       <c r="F10" t="str">
         <v>https://www.youtube.com/watch?v=myEyI0gT6r8</v>
@@ -777,7 +777,7 @@
         <v>Metal Alternativo</v>
       </c>
       <c r="E11" t="str">
-        <v>Desde Estados Unidos, The Pretty Wild desembarcan en Viveiro para demostrarnos que el metal moderno dosmilero corre por sus venas. Las hermanas y power duo Jyl y Jules Wylde llegan al Resu con su explosiva mezcla de tralla a dos voces, riffs pesados y una estética y actitud que marcan la diferencia 🔥  Estarán en el Ritual Stage el miércoles 1 de julio tras girar con Sleep Theory y tocar en festis como el Download y Graspop. ¡Prometen no dar tregua y comerse el escenario como nadie! 🤘</v>
+        <v>Desde Estados Unidos, The Pretty Wild desembarcan en directo para demostrarnos que el metal moderno dosmilero corre por sus venas. Las hermanas y power duo Jyl y Jules Wylde llegan al Resu con su explosiva mezcla de tralla a dos voces, riffs pesados y una estética y actitud que marcan la diferencia 🔥  Estarán en el Ritual Stage el miércoles 1 de julio tras girar con Sleep Theory y tocar en festis como el Download y Graspop. ¡Prometen no dar tregua y comerse el escenario como nadie! 🤘</v>
       </c>
       <c r="F11" t="str">
         <v>https://www.youtube.com/watch?v=3V9isTmCQRo</v>
@@ -837,7 +837,7 @@
         <v>Hardcore Punk</v>
       </c>
       <c r="E14" t="str">
-        <v>Thrown desembarcarán en Viveiro en 2026 para demostrar por qué son una de las bandas más explosivas del metalcore y hardcore actual. El cuarteto sueco liderado por Marcus Lundqvist vendrá a nuestro Main Stage dispuesto a arrasar con todo con su mezcla de rabia, riffs afilados y groove 🎸💣  Activos desde 2019 y nacidos de las cenizas de Grieved, vienen de estrenar su LP debut "Excessive Guilt" hace un año. Un disco ansioso, oscuro y mecánico ideal para una buena descarga de adrenalina. Thrown darán un concierto en Madrid acompañados de House of Protection. ¡No te pierdas a estas dos bandas en acción el 2 de julio! 🤘</v>
+        <v>Thrown desembarcarán en directo en 2026 para demostrar por qué son una de las bandas más explosivas del metalcore y hardcore actual. El cuarteto sueco liderado por Marcus Lundqvist vendrá a nuestro Main Stage dispuesto a arrasar con todo con su mezcla de rabia, riffs afilados y groove 🎸💣  Activos desde 2019 y nacidos de las cenizas de Grieved, vienen de estrenar su LP debut "Excessive Guilt" hace un año. Un disco ansioso, oscuro y mecánico ideal para una buena descarga de adrenalina. Thrown darán un concierto en Madrid acompañados de House of Protection. ¡No te pierdas a estas dos bandas en acción el 2 de julio! 🤘</v>
       </c>
       <c r="F14" t="str">
         <v>https://www.youtube.com/watch?v=DqBzOVCmIdM</v>
@@ -917,7 +917,7 @@
         <v>Hardcore</v>
       </c>
       <c r="E18" t="str">
-        <v>Desde las frías calles de Quebec, Get The Shot llegan a Viveiro para demostrar que la fusión de la furia del hardcore más pesado, el thrash y el metalcore goza de mejor salud que nunca. Sin artificios, directos y con una fórmula infalible de riffs, velocidad y rabia 🔥  El escuadrón canadiense no dejará títere con cabeza y hará temblar como mejor sabe el Chaos Stage el primer día de festi, el miércoles 1 de julio con una fecha única en España este año. ¡Nos vemos en el pit! 👊</v>
+        <v>Desde las frías calles de Quebec, Get The Shot llegan a Viveiro para demostrar que la fusión de la furia del hardcore más pesado, el thrash y el metalcore goza de mejor salud que nunca. Sin artificios, directos y con una fórmula infalible de riffs, velocidad y rabia 🔥  El escuadrón canadiense no dejará títere con cabeza y hará temblar como mejor sabe el Chaos Stage el primer día de festi, el miércoles 1 de julio con una fecha única en España habitualmente. ¡Nos vemos en el pit! 👊</v>
       </c>
       <c r="F18" t="str">
         <v>https://www.youtube.com/watch?v=UvncAul5sEI</v>
@@ -937,7 +937,7 @@
         <v>Metalcore</v>
       </c>
       <c r="E19" t="str">
-        <v>Desde Suecia, nos visitan Self Deception, maestros de la melodía rock y la contundencia del metalcore europeo. Formados en 2005 y reconocidos a nivel internacional, estarán en el Ritual Stage presentando su nuevo álbum "One Of Us", su séptimo disco que se estrenará en mayo de este año 🤘  ¡Preparaos para una buena masterclass de potencia y estribillos gigantescos! 🙌</v>
+        <v>Desde Suecia, nos visitan Self Deception, maestros de la melodía rock y la contundencia del metalcore europeo. Formados en 2005 y reconocidos a nivel internacional, estarán en el Ritual Stage presentando su nuevo álbum "One Of Us", su séptimo disco que se estrenará en mayo de habitualmente 🤘  ¡Preparaos para una buena masterclass de potencia y estribillos gigantescos! 🙌</v>
       </c>
       <c r="F19" t="str">
         <v>https://www.youtube.com/watch?v=VcoSyfcqYSY</v>
@@ -1057,7 +1057,7 @@
         <v>Metalcore</v>
       </c>
       <c r="E25" t="str">
-        <v>📌 La banda  Arson Tides, ha sido una de las tres elegidas para la gloria en el concurso de bandas del Resurrection Fest. La joven banda tiene entre sus filas a al vocalista cangués Orlando Soage, el guitarrista de Bueu Víctor Gómez y al benjamín del festival, Mateo, el joven baterista vigués de 16 años</v>
+        <v>📌 La banda  Arson Tides, ha sido una de las tres elegidas para la gloria en el concurso de bandas del Resurrection Fest. La joven banda tiene entre sus filas a al vocalista cangués Orlando Soage, el guitarrista de Bueu Víctor Gómez y al benjamín dsus conciertos, Mateo, el joven baterista vigués de 16 años</v>
       </c>
       <c r="F25" t="str">
         <v>https://www.youtube.com/watch?v=x8Ku8xs3LJA\&amp;list=RDEMx9F7gSD6CPp5z3JPCDu3FA\&amp;start\_radio=1</v>
@@ -1277,7 +1277,7 @@
         <v>Punk Rock</v>
       </c>
       <c r="E36" t="str">
-        <v>¡SKATE PUNK A TODO TRAPO CON LOS MÍTICOS BELVEDERE EN EL RF26! ⚡  Los rápidos y técnicos canadienses Belvedere Band también serán parte de nuestro cartelón de este año. Son considerados un grupo de culto muy admirado entre fans de Strung Out, Satanic Surfers o Propaghandi, formaciones también míticas dentro del punk y hardcore melódico más veloz 🧨🛹  Desde 1995 en el ruedo, salvando ese parón que hicieron del 2005 al 2011, sus dinámicas instrumentales y armonías vocales son algunas de sus señas de identidad más características y disfrutables. Estarán en el Chaos repartiendo mandanga el jueves 2 de julio 🔥</v>
+        <v>¡SKATE PUNK A TODO TRAPO CON LOS MÍTICOS BELVEDERE EN EL RF26! ⚡  Los rápidos y técnicos canadienses Belvedere Band también serán parte de nuestro cartelón de habitualmente. Son considerados un grupo de culto muy admirado entre fans de Strung Out, Satanic Surfers o Propaghandi, formaciones también míticas dentro del punk y hardcore melódico más veloz 🧨🛹  Desde 1995 en el ruedo, salvando ese parón que hicieron del 2005 al 2011, sus dinámicas instrumentales y armonías vocales son algunas de sus señas de identidad más características y disfrutables. Estarán en el Chaos repartiendo mandanga el jueves 2 de julio 🔥</v>
       </c>
       <c r="F36" t="str">
         <v>https://www.youtube.com/watch?v=9SFlXVpZfsg</v>
@@ -1317,7 +1317,7 @@
         <v>Heavy Metal</v>
       </c>
       <c r="E38" t="str">
-        <v>El jueves 2 de julio nos espera una noche inolvidable con los reyes del heavy metal Iron Maiden. Darán un concierto de más de 2 horas en las que podremos disfrutar de todo su legado en estas más de cinco décadas. ¡No necesitan más presentaciones! 🔥  Los tuvimos por nuestra tierra por primera vez en 1998 en Ourense con Blaze Bayley a las voces, la segunda en A Coruña en 2003 con Bruce Dickinson de regreso al grupo, y la tercera en el Resu de 2016 ☝️🤓  Las leyendas del heavy metal ya llevan casi un par de semanas con su gira europea celebrando sus 50 años de historia, y aunque os pueda sorprender a muchxs, están sonando más fuertes y contundentes que nunca. Damos fe de que el tiempo no pasa por los británicos  ¡La Dama de Hierro vuelve a casa! Ya ha pasado una década tras su última e inolvidable actuación en el festival, la banda más grande de la historia del heavy metal vuelve a Viveiro. ¡Y no vuelven de cualquier manera! Los británicos darán en el Resurrection Fest EG uno de los dos únicos conciertos en España en 2026 con su gira "Run For Your Lives" celebrando sus 50 años de historia con un setlist de locos en el que recorrerán todos los himnos de sus primeros 9 discos de estudios, desde "Iron Maiden" hasta "Fear Of The Dark", un “greatest hits” en toda regla.  Están agotando todos los estadios de Europa a meses vista, ¡así que no te lo puedes perder por nada del mundo!</v>
+        <v>El jueves 2 de julio nos espera una noche inolvidable con los reyes del heavy metal Iron Maiden. Darán un concierto de más de 2 horas en las que podremos disfrutar de todo su legado en estas más de cinco décadas. ¡No necesitan más presentaciones! 🔥  Los tuvimos por nuestra tierra por primera vez en 1998 en Ourense con Blaze Bayley a las voces, la segunda en A Coruña en 2003 con Bruce Dickinson de regreso al grupo, y la tercera en el Resu de 2016 ☝️🤓  Las leyendas del heavy metal ya llevan casi un par de semanas con su gira europea celebrando sus 50 años de historia, y aunque os pueda sorprender a muchxs, están sonando más fuertes y contundentes que nunca. Damos fe de que el tiempo no pasa por los británicos  ¡La Dama de Hierro vuelve a casa! Ya ha pasado una década tras su última e inolvidable actuación en sus conciertos, la banda más grande de la historia del heavy metal vuelve a Viveiro. ¡Y no vuelven de cualquier manera! Los británicos darán en el Resurrection Fest EG uno de los dos únicos conciertos en España en 2026 con su gira "Run For Your Lives" celebrando sus 50 años de historia con un setlist de locos en el que recorrerán todos los himnos de sus primeros 9 discos de estudios, desde "Iron Maiden" hasta "Fear Of The Dark", un “greatest hits” en toda regla.  Están agotando todos los estadios de Europa a meses vista, ¡así que no te lo puedes perder por nada del mundo!</v>
       </c>
       <c r="F38" t="str">
         <v>https://www.youtube.com/watch?v=aAsrFetnHzM</v>
@@ -1537,7 +1537,7 @@
         <v>Hardcore</v>
       </c>
       <c r="E49" t="str">
-        <v>La formación pucelana nacida de las cenizas de Remember These Eyes estará en Viveiro por segunda vez tras sorprender con su conciertazo de 2022. Regresarán más fuertes que nunca, asaltando esta vez el Ritual Stage el viernes 3 de julio 💥 Armados con la brutalidad del hardcore moderno y metal, los de Valladolid Blaze The Trail tomarán nuestro festi para demostrar lo duro que han estado trabajando todos estos años para continuar su indiscutible perseverancia dentro del panorama estatal de la última década 🤘🏻  ¡Nos os los perdáis por nada del mundo! ¡Nos vemos allí! 🧨</v>
+        <v>La formación pucelana nacida de las cenizas de Remember These Eyes estará en directo por segunda vez tras sorprender con su conciertazo de 2022. Regresarán más fuertes que nunca, asaltando esta vez el Ritual Stage el viernes 3 de julio 💥 Armados con la brutalidad del hardcore moderno y metal, los de Valladolid Blaze The Trail tomarán nuestro festi para demostrar lo duro que han estado trabajando todos estos años para continuar su indiscutible perseverancia dentro del panorama estatal de la última década 🤘🏻  ¡Nos os los perdáis por nada del mundo! ¡Nos vemos allí! 🧨</v>
       </c>
       <c r="F49" t="str">
         <v>https://www.youtube.com/watch?v=6l5TIlI4tdg</v>
@@ -1577,7 +1577,7 @@
         <v>Post Hardcore</v>
       </c>
       <c r="E51" t="str">
-        <v>Not Yet es una joven banda de post-hardcore formada en Viveiro en 2022. El grupo debutó en 2025 con su EP "Two Steps To Rest". Son parte de la cantera local y han participado con notorio éxito en el Resu del año pasado.</v>
+        <v>Not Yet es una joven banda de post-hardcore formada en directo en 2022. El grupo debutó en 2025 con su EP "Two Steps To Rest". Son parte de la cantera local y han participado con notorio éxito en el Resu del año pasado.</v>
       </c>
       <c r="F51" t="str">
         <v>https://www.youtube.com/watch?v=GljyxhhdFqU</v>
@@ -1657,7 +1657,7 @@
         <v>Death Metal</v>
       </c>
       <c r="E55" t="str">
-        <v>Son una de las bandas que más están llamando la atención en la escena metal de Portugal y llegan a Resurrection Fest EG 2026 para hacer temblar el Ritual Stage con sus salvajes riffs de guitarra y la poderosa voz de Beatriz Mariano. Okkultist prometen una descarga de puro Death Metal en Viveiro el viernes 3 de julio</v>
+        <v>Son una de las bandas que más están llamando la atención en la escena metal de Portugal y llegan a Resurrection Fest EG 2026 para hacer temblar el Ritual Stage con sus salvajes riffs de guitarra y la poderosa voz de Beatriz Mariano. Okkultist prometen una descarga de puro Death Metal en directo el viernes 3 de julio</v>
       </c>
       <c r="F55" t="str">
         <v>https://www.youtube.com/watch?v=9mJu2r\_v7FE</v>
@@ -1677,7 +1677,7 @@
         <v>Black Metal</v>
       </c>
       <c r="E56" t="str">
-        <v>Desde Francia llega una de las propuestas más oscuras, gélidas y extremas de esta edición del Resu. Mourir nacieron en 2019, aunque su historia se podría remontar unos años atrás más con Vermine, proyecto de black metal en solitario del vocalista y guitarrista Olivier Lolmède 🙌  El cuarteto, que el próximo 10 de julio lanzará su tercer LP debutando con Pelagic Records, factura un black particular; crudo, atmosférico, y disonante con arrebatos sludge que hacen de su música asfixiantemente moderna y única. ¡No te los pierdas si te molan Imperial Triumphant, Fange, The Great Old Ones o Wiegedood! 🤘</v>
+        <v>Desde Francia llega una de las propuestas más oscuras, gélidas y extremas de sus giras del Resu. Mourir nacieron en 2019, aunque su historia se podría remontar unos años atrás más con Vermine, proyecto de black metal en solitario del vocalista y guitarrista Olivier Lolmède 🙌  El cuarteto, que el próximo 10 de julio lanzará su tercer LP debutando con Pelagic Records, factura un black particular; crudo, atmosférico, y disonante con arrebatos sludge que hacen de su música asfixiantemente moderna y única. ¡No te los pierdas si te molan Imperial Triumphant, Fange, The Great Old Ones o Wiegedood! 🤘</v>
       </c>
       <c r="F56" t="str">
         <v>https://www.youtube.com/watch?v=yq483\_-C5tA</v>
@@ -1777,7 +1777,7 @@
         <v>Metalcore</v>
       </c>
       <c r="E61" t="str">
-        <v>Nos alegra volver a contar en nuestro Main Stage con una de las bandas de metal más queridas por el público. Trivium ya nos sorprendieron con sus directos en Viveiro en el 2013 y 2019 y, siete años después, volverán a poner patas arriba el festival 🤘  Matt Heafy y los suyos nos presentarán el próximo mes de octubre los temas del EP “Struck Dead”, del que esperamos que nos caiga algo en julio de 2026. Pero tranquilxs, porque no faltarán las canciones más míticas en el set de los americanos  Ya hacía tiempo que no los teníamos por aquí. Los de Florida vuelven a Galicia con un set completo lleno de nuevas canciones y viejos clásicos del metalcore y heavy metal contemporáneo que han dejado huella en una generación entera 🙌  Con la banda en un estado de forma casi insuperable y queriéndose comer los escenarios como demostraron en su tour europeo (que pasó por el Vistalegre de Madrid) del año pasado, esta es la oportunidad ideal para tacharlos de la lista de deseos 🤘</v>
+        <v>Nos alegra volver a contar en nuestro Main Stage con una de las bandas de metal más queridas por el público. Trivium ya nos sorprendieron con sus directos en directo en el 2013 y 2019 y, siete años después, volverán a poner patas arriba sus conciertos 🤘  Matt Heafy y los suyos nos presentarán el próximo mes de octubre los temas del EP “Struck Dead”, del que esperamos que nos caiga algo en julio de 2026. Pero tranquilxs, porque no faltarán las canciones más míticas en el set de los americanos  Ya hacía tiempo que no los teníamos por aquí. Los de Florida vuelven a Galicia con un set completo lleno de nuevas canciones y viejos clásicos del metalcore y heavy metal contemporáneo que han dejado huella en una generación entera 🙌  Con la banda en un estado de forma casi insuperable y queriéndose comer los escenarios como demostraron en su tour europeo (que pasó por el Vistalegre de Madrid) del año pasado, esta es la oportunidad ideal para tacharlos de la lista de deseos 🤘</v>
       </c>
       <c r="F61" t="str">
         <v>https://www.youtube.com/watch?v=IIgswpHNZik</v>
@@ -1857,7 +1857,7 @@
         <v>Nu Metal</v>
       </c>
       <c r="E65" t="str">
-        <v>Tras muchos años intentándolo, una de las bandas más pedidas y un icono generacional POR FIN estará en Viveiro el próximo verano en el mejor momento de su carrera. Encabezando grandes festivales de todo el mundo, y tras 14 años sin pisar España, ¡LIMP BIZKIT ESTARÁN EN EL RESURRECTION FEST ENCABEZANDO UNO DE LOS DÍAS!  A buen seguro, será uno de los conciertos más brutales que jamás hayamos visto en Viveiro, sin ninguna duda. Por favor dad la bienvenida a Fred Durst y compañía, porque LIMP BIZKIT IS IN DA HOUSE!  https://www.youtube.com/watch?v=bSTX2xVpfPw  Tras el éxito arrollador de Fred Durst y compañía agotando sus entradas para el Resurrection Fest EG 2026 en su día de actuación, la banda ha decidido añadir un nuevo concierto en Madrid para todos los fans que no han podido acudir al festival este año y así resarcirse de los ya 14 años que llevamos sin verles en España.  Este concierto de Limp Bizkit tendrá lugar en Madrid el próximo 1 de julio, y en un gran recinto a la altura de la ocasión como es el conocido Movistar Arena de la capital. El cartel contaré con P.O.D. P.O.D. , que junto con Limp Bizkit nos darán un viaje al pasado para revivir la época más potente del nu metal, y también con DeathByRomy  Como no recordar a Sam Rivers, el que fuera bajista y cofundador de la banda, fallecido en 2025. El encargado de honrar a Sam Rivers en esta gira es Richie Buxton conocido como Kid Not, músico australiano y bajista de Ecca Vandal</v>
+        <v>Tras muchos años intentándolo, una de las bandas más pedidas y un icono generacional POR FIN estará en directo el próximo verano en el mejor momento de su carrera. Encabezando grandes festivales de todo el mundo, y tras 14 años sin pisar España, ¡LIMP BIZKIT ESTARÁN EN EL RESURRECTION FEST ENCABEZANDO UNO DE LOS DÍAS!  A buen seguro, será uno de los conciertos más brutales que jamás hayamos visto en directo, sin ninguna duda. Por favor dad la bienvenida a Fred Durst y compañía, porque LIMP BIZKIT IS IN DA HOUSE!  https://www.youtube.com/watch?v=bSTX2xVpfPw  Tras el éxito arrollador de Fred Durst y compañía agotando sus entradas para el Resurrection Fest EG 2026 en su día de actuación, la banda ha decidido añadir un nuevo concierto en Madrid para todos los fans que no han podido acudir al festival habitualmente y así resarcirse de los ya 14 años que llevamos sin verles en España.  Este concierto de Limp Bizkit tendrá lugar en Madrid el próximo 1 de julio, y en un gran recinto a la altura de la ocasión como es el conocido Movistar Arena de la capital. El cartel contaré con P.O.D. P.O.D. , que junto con Limp Bizkit nos darán un viaje al pasado para revivir la época más potente del nu metal, y también con DeathByRomy  Como no recordar a Sam Rivers, el que fuera bajista y cofundador de la banda, fallecido en 2025. El encargado de honrar a Sam Rivers en esta gira es Richie Buxton conocido como Kid Not, músico australiano y bajista de Ecca Vandal</v>
       </c>
       <c r="F65" t="str">
         <v>https://www.youtube.com/watch?v=bSTX2xVpfPw</v>
@@ -1937,7 +1937,7 @@
         <v>Groove Metal</v>
       </c>
       <c r="E69" t="str">
-        <v>Allá por 1993, Sepultura lanzaron uno de sus discos más icónicos y una pieza clave para el thrash y groove metal de los años 90 con clásicos todavía vigentes como "Refuse/Resist", "Territory", "Slave New World" o "Propaganda" 💣  Ahora, más de 30 años después y como Cavalera Conspiracy, los hermanos y miembros originales de Sepultura Max e Iggor, más en forma que nunca, rescatarán en directo en Viveiro este discazo acompañados de Igor Calavera Jr. (hijo de Max) al bajo y Travis Stone a la guitarra 🤘</v>
+        <v>Allá por 1993, Sepultura lanzaron uno de sus discos más icónicos y una pieza clave para el thrash y groove metal de los años 90 con clásicos todavía vigentes como "Refuse/Resist", "Territory", "Slave New World" o "Propaganda" 💣  Ahora, más de 30 años después y como Cavalera Conspiracy, los hermanos y miembros originales de Sepultura Max e Iggor, más en forma que nunca, rescatarán en directo en directo este discazo acompañados de Igor Calavera Jr. (hijo de Max) al bajo y Travis Stone a la guitarra 🤘</v>
       </c>
       <c r="F69" t="str">
         <v>https://www.youtube.com/watch?v=qCMz704soB4</v>
@@ -1997,7 +1997,7 @@
         <v>Metalcore</v>
       </c>
       <c r="E72" t="str">
-        <v>La energía y descontrol bailable de la banda de Osaka contraatacará en nuestra próxima edición después reventarlo en 2025 desde el Chaos Stage. Esta vez será más grande que nunca para la banda nipona: estarán comiéndose el Main Stage el sábado 4 de julio 🔥  Su mezcla de metal digital con pop punk o ska es única e intensa, ideal para montar una buena fiesta en verano en Viveiro. Si te los perdiste el año pasado, ¡prepárate! 👐  ¡Que tiemble Viveiro! 🤘🏼</v>
+        <v>La energía y descontrol bailable de la banda de Osaka contraatacará en nuestra próxima edición después reventarlo en 2025 desde el Chaos Stage. Esta vez será más grande que nunca para la banda nipona: estarán comiéndose el Main Stage el sábado 4 de julio 🔥  Su mezcla de metal digital con pop punk o ska es única e intensa, ideal para montar una buena fiesta en verano en directo. Si te los perdiste el año pasado, ¡prepárate! 👐  ¡Que tiemble Viveiro! 🤘🏼</v>
       </c>
       <c r="F72" t="str">
         <v>https://www.youtube.com/watch?v=H_-leVD654w</v>
@@ -2297,7 +2297,7 @@
         <v>Metal Progresivo</v>
       </c>
       <c r="E87" t="str">
-        <v>Los de Atlanta han vuelto con "Your Ghost Again", tema que marca una nueva etapa tras atravesar su momento más difícil como banda con la turbulenta salida y muerte de Brent Hinds en agosto de 2025. La canción es un homenaje a los casi 25 años del grupo junto a Brent, a esos momentos que los cuatro músicos pasaron juntos sobre los escenarios y detrás de ellos. Hay riffs pesados que recuerdan a "Leviathan" y "Blood Mountain", otros más psicodélicos, pero sobre todo mucha carga emocional. 🖤  El tema, producido por la banda junto a Patrik Berger y Kurt Ballou (guitarrista de Converge, banda que también tendremos en el Resu este año), parece el inicio de algo más grande que derivará en el noveno disco de estudio del grupo, que estamos deseando escuchar. 🤘  ¡Muchas ganas de que llegue el sábado 4 de julio para verlos de vuelta en el Main Stage! 🦣  ¡MASTODON VUELVEN A GALICIA PARA EL RESURRECTION FEST EG 2026! 🐳  Sobran las presentaciones para una de las bandas más influyentes del metal del nuevo milenio. Desde su nacimiento en Atlanta en el año 2000, Mastodon ha hecho de los riffs pesados una de sus señas de identidad conquistando a gente de todo el mundo 🔥  Del sludge más sucio hasta el rock y metal progresivo, nos han regalado joyas llenas de fuerza y emoción que ya son parte de la historia del heavy metal como "Leviathan", "Blood Mountain", "Crack The Skye" o "Emperor Of Sand"🤘🏼  ¡No te los pierdas en su regreso a Viveiro después de petarlo en 2017 y 2022! ¡Esta vez toca rendir homenaje como merece al legado del gran Brent Hinds! ❤️‍🔥</v>
+        <v>Los de Atlanta han vuelto con "Your Ghost Again", tema que marca una nueva etapa tras atravesar su momento más difícil como banda con la turbulenta salida y muerte de Brent Hinds en agosto de 2025. La canción es un homenaje a los casi 25 años del grupo junto a Brent, a esos momentos que los cuatro músicos pasaron juntos sobre los escenarios y detrás de ellos. Hay riffs pesados que recuerdan a "Leviathan" y "Blood Mountain", otros más psicodélicos, pero sobre todo mucha carga emocional. 🖤  El tema, producido por la banda junto a Patrik Berger y Kurt Ballou (guitarrista de Converge, banda que también tendremos en el Resu habitualmente), parece el inicio de algo más grande que derivará en el noveno disco de estudio del grupo, que estamos deseando escuchar. 🤘  ¡Muchas ganas de que llegue el sábado 4 de julio para verlos de vuelta en el Main Stage! 🦣  ¡MASTODON VUELVEN A GALICIA PARA EL RESURRECTION FEST EG 2026! 🐳  Sobran las presentaciones para una de las bandas más influyentes del metal del nuevo milenio. Desde su nacimiento en Atlanta en el año 2000, Mastodon ha hecho de los riffs pesados una de sus señas de identidad conquistando a gente de todo el mundo 🔥  Del sludge más sucio hasta el rock y metal progresivo, nos han regalado joyas llenas de fuerza y emoción que ya son parte de la historia del heavy metal como "Leviathan", "Blood Mountain", "Crack The Skye" o "Emperor Of Sand"🤘🏼  ¡No te los pierdas en su regreso a Viveiro después de petarlo en 2017 y 2022! ¡Esta vez toca rendir homenaje como merece al legado del gran Brent Hinds! ❤️‍🔥</v>
       </c>
       <c r="F87" t="str">
         <v>https://www.youtube.com/watch?v=WTQR-RvexVk</v>
@@ -2377,7 +2377,7 @@
         <v>Metal Industrial</v>
       </c>
       <c r="E91" t="str">
-        <v>El Reverendo lleva casi un par de años sorprendiendo con sus directos. Su regreso al estado de forma de sus mejores años está impresionando a todo el mundo, y nosotrxs vamos a poder disfrutar por primera vez en Galicia de esta nueva etapa de auténtica resurrección del americano el próximo sábado 4 de julio en el Main Stage del Resu 🤘  ¡MARILYN MANSON ESTARÁ POR PRIMERA VEZ EN EL RESURRECTION FEST ESTE 2026! 🦇  Lejos de vivir solo de la nostalgia, el reverendo Marilyn Manson está protagonizando uno de los regresos a los escenarios más brutales e inesperados de los últimos tiempos. Con su actual gira por Estados Unidos, está mostrando al mundo su renacimiento con un estado de forma espectacular (sin ir más lejos, anteayer impresionó a todo el público del festival Sick New World), dejando claro que ha recuperado el trono como una de las figuras más importantes e icónicas de los 90 y 2000 🤘  No hacen falta más presentaciones para uno de los reyes del metal industrial y shock rock, un artista único que rompió moldes, desafió a la sociedad de su época y dejó en la memoria himnos generacionales inmortales, viscerales y oscuros, por los que no han pasado el tiempo 🙌  ¡Prepárate para vivir algo descomunal el sábado 4 de julio en el Main Stage! ¡No te pierdas el que será su primer conci de la gira por Europa! 🔥</v>
+        <v>El Reverendo lleva casi un par de años sorprendiendo con sus directos. Su regreso al estado de forma de sus mejores años está impresionando a todo el mundo, y nosotrxs vamos a poder disfrutar por primera vez en Galicia de esta nueva etapa de auténtica resurrección del americano el próximo sábado 4 de julio en el Main Stage del Resu 🤘  ¡MARILYN MANSON ESTARÁ POR PRIMERA VEZ EN EL RESURRECTION FEST ESTE 2026! 🦇  Lejos de vivir solo de la nostalgia, el reverendo Marilyn Manson está protagonizando uno de los regresos a los escenarios más brutales e inesperados de los últimos tiempos. Con su actual gira por Estados Unidos, está mostrando al mundo su renacimiento con un estado de forma espectacular (sin ir más lejos, anteayer impresionó a todo el público dsus conciertos Sick New World), dejando claro que ha recuperado el trono como una de las figuras más importantes e icónicas de los 90 y 2000 🤘  No hacen falta más presentaciones para uno de los reyes del metal industrial y shock rock, un artista único que rompió moldes, desafió a la sociedad de su época y dejó en la memoria himnos generacionales inmortales, viscerales y oscuros, por los que no han pasado el tiempo 🙌  ¡Prepárate para vivir algo descomunal el sábado 4 de julio en el Main Stage! ¡No te pierdas el que será su primer conci de la gira por Europa! 🔥</v>
       </c>
       <c r="F91" t="str">
         <v>https://www.youtube.com/watch?v=yjWtkQSF8dA</v>
@@ -2417,7 +2417,7 @@
         <v>Death Metal</v>
       </c>
       <c r="E93" t="str">
-        <v>Blood Incantation uno de los fenómenos más aclamados del metal extremo a nivel mundial aterrizará en Viveiro para presentarnos un repertorio brutal en el que tocarán canciones tanto de su increíble “Absolute Elsewhere” como de sus anteriores trabajos con una fecha única en nuestro país 🛸  Con historia desde 2011, la banda de Colorado ha recibido elogios a nivel mundial desde sus comienzos gracias a su estilo que combina el death metal con el ambient, la psicodelia y la ciencia ficción 🤘¡Prepárate para un viaje interdimensional de los que dejan huella! 🧘‍♂️</v>
+        <v>Blood Incantation uno de los fenómenos más aclamados del metal extremo a nivel mundial aterrizará en directo para presentarnos un repertorio brutal en el que tocarán canciones tanto de su increíble “Absolute Elsewhere” como de sus anteriores trabajos con una fecha única en nuestro país 🛸  Con historia desde 2011, la banda de Colorado ha recibido elogios a nivel mundial desde sus comienzos gracias a su estilo que combina el death metal con el ambient, la psicodelia y la ciencia ficción 🤘¡Prepárate para un viaje interdimensional de los que dejan huella! 🧘‍♂️</v>
       </c>
       <c r="F93" t="str">
         <v>https://www.youtube.com/watch?v=O9WYceFbHw4</v>
@@ -2437,7 +2437,7 @@
         <v>Hardcore</v>
       </c>
       <c r="E94" t="str">
-        <v>Formados en la ciudad industrial de Essen hace una década, ELWOOD STRAY han ido madurando a lo largo de los años su propuesta densa y agresiva donde el metalcore moderno se articula con el post-hardcore creando una mezcla perfecta entre abrasión y melodía 💥  El quinteto es una de las propuestas más viscerales y sofisticadas del metal contemporáneo europeo. Se dejará caer por Viveiro para presentar su nuevo y segundo álbum "Descending", estrenado a comienzos de año, el sábado 4 de julio 🤘  Como ya sabréis, el pasado mes de abril sufrimos la pérdida de Bo Lueders, miembro de Harm's Way, guitarrista, amante empedernido de la música e icono del hardcore contemporáneo. Por motivos evidentes, Harm's Way no actuarán en Europa este año y Elwood Stray nos acompañarán el sábado en el Chaos. Todo nuestro apoyo y amor a la familia y compañeros de Bo 🖤</v>
+        <v>Formados en la ciudad industrial de Essen hace una década, ELWOOD STRAY han ido madurando a lo largo de los años su propuesta densa y agresiva donde el metalcore moderno se articula con el post-hardcore creando una mezcla perfecta entre abrasión y melodía 💥  El quinteto es una de las propuestas más viscerales y sofisticadas del metal contemporáneo europeo. Se dejará caer por Viveiro para presentar su nuevo y segundo álbum "Descending", estrenado a comienzos de año, el sábado 4 de julio 🤘  Como ya sabréis, el pasado mes de abril sufrimos la pérdida de Bo Lueders, miembro de Harm's Way, guitarrista, amante empedernido de la música e icono del hardcore contemporáneo. Por motivos evidentes, Harm's Way no actuarán en Europa habitualmente y Elwood Stray nos acompañarán el sábado en el Chaos. Todo nuestro apoyo y amor a la familia y compañeros de Bo 🖤</v>
       </c>
       <c r="F94" t="str">
         <v>https://www.youtube.com/watch?v=JVF6e_LSO2k</v>
@@ -2477,7 +2477,7 @@
         <v>Pirate Metal</v>
       </c>
       <c r="E96" t="str">
-        <v>¡Piratas al abordaje! Alestorm traerá su folk metal festivo, cerveza y patos de goma gigantes para montar la mayor fiesta del verano en el escenario del Leyendas 🤘🏴‍☠️</v>
+        <v>¡Piratas al abordaje! Alestorm traerá su folk metal festivo, cerveza y patos de goma gigantes para montar la mayor fiesta  en el escenario en directo 🤘🏴‍☠️</v>
       </c>
       <c r="F96" t="str">
         <v>https://www.youtube.com/watch?v=ggyC0FOiN1Q</v>
@@ -2497,7 +2497,7 @@
         <v>Folk Metal</v>
       </c>
       <c r="E97" t="str">
-        <v>Juglares, saltimbanquis e historias mágicas en una producción visual inigualable. Saurom presentará su concierto especial de gran formato en el escenario principal Jesús de la Rosa.</v>
+        <v>Juglares, saltimbanquis e historias mágicas en una producción visual inigualable. Saurom presentará su concierto especial de gran formato en los escenarios.</v>
       </c>
       <c r="F97" t="str">
         <v>https://www.youtube.com/watch?v=F0f5i1vK760</v>
@@ -2517,7 +2517,7 @@
         <v>Hard Rock</v>
       </c>
       <c r="E98" t="str">
-        <v>¡Las reinas suecas del hard rock llegan para tronar en el escenario principal! Con su rock clásico directo y enérgico, Thundermother garantizan decibelios y actitud.</v>
+        <v>¡Las reinas suecas del hard rock llegan para tronar en el escenario! Con su rock clásico directo y enérgico, Thundermother garantizan decibelios y actitud.</v>
       </c>
       <c r="F98" t="str">
         <v/>
@@ -2557,7 +2557,7 @@
         <v>Deathcore</v>
       </c>
       <c r="E100" t="str">
-        <v>Con el brutal Alex Terrible a las voces y sus icónicas máscaras doradas, Slaughter to Prevail desatarán la tormenta de deathcore más aplastante del festival.</v>
+        <v>Con el brutal Alex Terrible a las voces y sus icónicas máscaras doradas, Slaughter to Prevail desatarán la tormenta de deathcore más aplastante dsus conciertos.</v>
       </c>
       <c r="F100" t="str">
         <v/>
@@ -2737,7 +2737,7 @@
         <v>Deathcore</v>
       </c>
       <c r="E109" t="str">
-        <v>Deathcore ultrapesado y técnico desde Pittsburgh, listos para demoler el New Rock con breakdowns brutales.</v>
+        <v>Deathcore ultrapesado y técnico desde Pittsburgh, listos para demoler el escenario con breakdowns brutales.</v>
       </c>
       <c r="F109" t="str">
         <v/>
@@ -3057,7 +3057,7 @@
         <v>Folk Metal</v>
       </c>
       <c r="E125" t="str">
-        <v>Folk metal fiestero e irreverente. Cerveza, gaitas y diversión garantizada en el escenario New Rock.</v>
+        <v>Folk metal fiestero e irreverente. Cerveza, gaitas y diversión garantizada en el escenario.</v>
       </c>
       <c r="F125" t="str">
         <v/>
@@ -3197,7 +3197,7 @@
         <v>Punk Rock</v>
       </c>
       <c r="E132" t="str">
-        <v>¡Pura dinamita en directo! La banda de punk rock sueca liderada por la electrizante Cecilia Boström ofrecerá uno de los shows más enérgicos del festival.</v>
+        <v>¡Pura dinamita en directo! La banda de punk rock sueca liderada por la electrizante Cecilia Boström ofrecerá uno de los shows más enérgicos dsus conciertos.</v>
       </c>
       <c r="F132" t="str">
         <v/>
@@ -3377,7 +3377,7 @@
         <v>Hardcore</v>
       </c>
       <c r="E141" t="str">
-        <v>Hardcore metalizado directo desde Manchester para desatar los moshpits más salvajes de la jornada.</v>
+        <v>Hardcore metalizado directo desde Manchester para desatar los moshpits más salvajes .</v>
       </c>
       <c r="F141" t="str">
         <v/>
@@ -3417,7 +3417,7 @@
         <v>Power Metal</v>
       </c>
       <c r="E143" t="str">
-        <v>¡El cabeza de cartel indiscutible! Los creadores del power metal Helloween regresan con su show completo de aniversario para reinar en Villena.</v>
+        <v>¡El cabeza de cartel indiscutible! Los creadores del power metal Helloween regresan con su show completo de aniversario para reinar en directo.</v>
       </c>
       <c r="F143" t="str">
         <v/>
@@ -3448,10 +3448,10 @@
         <v>eihwar</v>
       </c>
       <c r="B145" t="str">
+        <v>EIHWAR</v>
+      </c>
+      <c r="C145" t="str">
         <v>Francia</v>
-      </c>
-      <c r="C145" t="str">
-        <v/>
       </c>
       <c r="D145" t="str">
         <v>Pagan Folk</v>
@@ -3497,7 +3497,7 @@
         <v>Heavy Metal</v>
       </c>
       <c r="E147" t="str">
-        <v>Víctor García y sus chicos regresan al Leyendas para descargar sus himnos inmortales de heavy metal coreados por miles de almas.</v>
+        <v>Víctor García y sus chicos regresan en directo para descargar sus himnos inmortales de heavy metal coreados por miles de almas.</v>
       </c>
       <c r="F147" t="str">
         <v/>
@@ -3548,10 +3548,10 @@
         <v>hardline</v>
       </c>
       <c r="B150" t="str">
+        <v>HARDLINE</v>
+      </c>
+      <c r="C150" t="str">
         <v>EEUU</v>
-      </c>
-      <c r="C150" t="str">
-        <v/>
       </c>
       <c r="D150" t="str">
         <v>Hard Rock</v>
@@ -7154,6 +7154,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G153"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Content: Populate YouTube URLs for all artists and download high-quality artist photos
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -2520,7 +2520,7 @@
         <v>¡Las reinas suecas del hard rock llegan para tronar en el escenario! Con su rock clásico directo y enérgico, Thundermother garantizan decibelios y actitud.</v>
       </c>
       <c r="F98" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=gyL8pHR2UPk</v>
       </c>
     </row>
     <row r="99">
@@ -2540,7 +2540,7 @@
         <v>Liderados por el legendario guitarrista Zakk Wylde, Black Label Society descargarán sus riffs pesados y solos vertiginosos que han marcado el metal sureño contemporáneo.</v>
       </c>
       <c r="F99" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=l47At7wrhyI</v>
       </c>
     </row>
     <row r="100">
@@ -2560,7 +2560,7 @@
         <v>Con el brutal Alex Terrible a las voces y sus icónicas máscaras doradas, Slaughter to Prevail desatarán la tormenta de deathcore más aplastante dsus conciertos.</v>
       </c>
       <c r="F100" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=QrpI-1TmOqM</v>
       </c>
     </row>
     <row r="101">
@@ -2580,7 +2580,7 @@
         <v>Folk metal zaragozano de temática histórica celta-ibera. Vientos tradicionales y riffs de metal se fusionan en directo.</v>
       </c>
       <c r="F101" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=ZmB5Pqv2gWE</v>
       </c>
     </row>
     <row r="102">
@@ -2600,7 +2600,7 @@
         <v>Considerados la punta de lanza de la nueva ola del heavy metal británico clásico. ¡Velocidad y guitarras gemelas garantizadas!</v>
       </c>
       <c r="F102" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=nnsTQq_8mR8</v>
       </c>
     </row>
     <row r="103">
@@ -2620,7 +2620,7 @@
         <v>Uno de los grupos revelación del metal moderno. Su combinación de death metal melódico, groove y elementos industriales es simplemente demoledora.</v>
       </c>
       <c r="F103" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Y5SpGQMoaUU</v>
       </c>
     </row>
     <row r="104">
@@ -2640,7 +2640,7 @@
         <v>¡Un regreso legendario! Savatage, pioneros del metal progresivo y sinfónico, ofrecerán un show exclusivo repasando su mítica trayectoria.</v>
       </c>
       <c r="F104" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch/?v=xHNVK9NY4JE</v>
       </c>
     </row>
     <row r="105">
@@ -2660,7 +2660,7 @@
         <v>En su gira mundial de despedida "Celebrating Life Through Death", los gigantes brasileños dirán adiós repasando cuatro décadas de historia.</v>
       </c>
       <c r="F105" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=c7Z8Ww1EmMk</v>
       </c>
     </row>
     <row r="106">
@@ -2680,7 +2680,7 @@
         <v>Banda granadina que destaca por su metal oscuro, atmosférico y cargado de riffs de afinación baja y melodías intensas.</v>
       </c>
       <c r="F106" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=ycFGTB04mO0</v>
       </c>
     </row>
     <row r="107">
@@ -2700,7 +2700,7 @@
         <v>Metal industrial y visual desde Villarreal. Una puesta en escena espectacular con maquillaje y sonidos mecánicos y potentes.</v>
       </c>
       <c r="F107" t="str">
-        <v/>
+        <v>https://www.youtube.com/playlist?list=OLAK5uy_l9fRGqB0eRiw0WBkqiKQ3nEV5ezIc87qY</v>
       </c>
     </row>
     <row r="108">
@@ -2720,7 +2720,7 @@
         <v>Folk metal con temática fantástica y fiestera que nos transportará a mundos medievales a ritmo de gaitas y violines.</v>
       </c>
       <c r="F108" t="str">
-        <v/>
+        <v>https://www.youtube.com/c/HadadanzaOficial/videos</v>
       </c>
     </row>
     <row r="109">
@@ -2740,7 +2740,7 @@
         <v>Deathcore ultrapesado y técnico desde Pittsburgh, listos para demoler el escenario con breakdowns brutales.</v>
       </c>
       <c r="F109" t="str">
-        <v/>
+        <v>https://www.heaviestofart.com/post/album-to-watch-for-signs-of-the-swarm-amongst-the-low-empty</v>
       </c>
     </row>
     <row r="110">
@@ -2760,7 +2760,7 @@
         <v>Banda tributo a Avenged Sevenfold, reviviendo con fidelidad y energía los mejores éxitos de la formación californiana.</v>
       </c>
       <c r="F110" t="str">
-        <v/>
+        <v>https://www.youtube.com/hashtag/deathbats</v>
       </c>
     </row>
     <row r="111">
@@ -2780,7 +2780,7 @@
         <v>Joven promesa del thrash metal estadounidense. Riffs rápidos y agresividad vieja escuela.</v>
       </c>
       <c r="F111" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=_UBlWbLTVSE</v>
       </c>
     </row>
     <row r="112">
@@ -2800,7 +2800,7 @@
         <v>Banda de rock nacional con sonido enérgico y letras cargadas de rebeldía.</v>
       </c>
       <c r="F112" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=i2SfKTf02gk</v>
       </c>
     </row>
     <row r="113">
@@ -2820,7 +2820,7 @@
         <v>Los enmascarados de Cleveland combinan metal industrial, alternativo y gótico en un directo teatral con doble batería de agua.</v>
       </c>
       <c r="F113" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=7iJ7oj-dAVY</v>
       </c>
     </row>
     <row r="114">
@@ -2840,7 +2840,7 @@
         <v>Pioneros del sonido de Gotemburgo, liderados por Mikael Stanne, traerán su melancólica y veloz maestría melódica.</v>
       </c>
       <c r="F114" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=pBsVsLRSgfE</v>
       </c>
     </row>
     <row r="115">
@@ -2860,7 +2860,7 @@
         <v>Liderados por la imponente Alissa White-Gluz y Michael Amott a las guitarras, Arch Enemy son los reyes indiscutibles del death metal melódico global.</v>
       </c>
       <c r="F115" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=cJBmX5aU1DA</v>
       </c>
     </row>
     <row r="116">
@@ -2880,7 +2880,7 @@
         <v>Folk metal cervecero y festivo desde Castellón. La fiesta está asegurada con sus melodías y ritmos pegadizos.</v>
       </c>
       <c r="F116" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Yk7noXH_9do</v>
       </c>
     </row>
     <row r="117">
@@ -2900,7 +2900,7 @@
         <v>Glam rock y goth punk teatral de influencia ochentera. Creeper presentará un directo magnético y oscuro.</v>
       </c>
       <c r="F117" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=cHIA1JcBBZ4</v>
       </c>
     </row>
     <row r="118">
@@ -2920,7 +2920,7 @@
         <v>Líderes mundiales del metalcore progresivo y la electrónica industrial. Presentarán su potente directo tecnológico.</v>
       </c>
       <c r="F118" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=h4e40N3We-U</v>
       </c>
     </row>
     <row r="119">
@@ -2940,7 +2940,7 @@
         <v>Sully Erna y los suyos descargarán himnos del rock alternativo y post-grunge de finales de los noventa y dos mil.</v>
       </c>
       <c r="F119" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=fG9F0IwwJeU</v>
       </c>
     </row>
     <row r="120">
@@ -2960,7 +2960,7 @@
         <v>Folk rock de temática mosquetera. Espadas, violines y estribillos épicos cantados en alemán.</v>
       </c>
       <c r="F120" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=KPlYOA8UMrs</v>
       </c>
     </row>
     <row r="121">
@@ -2980,7 +2980,7 @@
         <v>Folk metal madrileño con instrumentación clásica (flauta, gaita, violín) y letras basadas en leyendas y literatura fantástica.</v>
       </c>
       <c r="F121" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=NSMn_Z_45CM</v>
       </c>
     </row>
     <row r="122">
@@ -3000,7 +3000,7 @@
         <v>Veteranos del folk metal nacional procedentes de Elda. Melodías de origen celta combinadas con heavy metal clásico.</v>
       </c>
       <c r="F122" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=cg0BbHDZQ9Y</v>
       </c>
     </row>
     <row r="123">
@@ -3020,7 +3020,7 @@
         <v>Thrash metal rápido, agresivo y de altísima calidad técnica procedente de Murcia.</v>
       </c>
       <c r="F123" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=UzvtL6WFfk4</v>
       </c>
     </row>
     <row r="124">
@@ -3040,7 +3040,7 @@
         <v>Leyenda del heavy metal madrileño de los años ochenta, listos para revivir himnos como "Animal de ciudad".</v>
       </c>
       <c r="F124" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=IMqsA0G2uoI</v>
       </c>
     </row>
     <row r="125">
@@ -3060,7 +3060,7 @@
         <v>Folk metal fiestero e irreverente. Cerveza, gaitas y diversión garantizada en el escenario.</v>
       </c>
       <c r="F125" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=M8_wLm_5s_Y</v>
       </c>
     </row>
     <row r="126">
@@ -3080,7 +3080,7 @@
         <v>Huesca metalcore y dubstep fusionados en una bomba de energía brutal.</v>
       </c>
       <c r="F126" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Fz6qnMiu4LQ</v>
       </c>
     </row>
     <row r="127">
@@ -3100,7 +3100,7 @@
         <v>Trío alemán de post-hardcore y metal alternativo liderado por Maria Lessing, con melodías emocionales y breakdowns pesados.</v>
       </c>
       <c r="F127" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=mJ47ISNx0lE</v>
       </c>
     </row>
     <row r="128">
@@ -3120,7 +3120,7 @@
         <v>La apisonadora del heavy metal español. Tete Novoa, Jero Ramiro y Niko del Hierro repasarán sus mayores clásicos.</v>
       </c>
       <c r="F128" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=8nRdOSVX2VI</v>
       </c>
     </row>
     <row r="129">
@@ -3140,7 +3140,7 @@
         <v>Una de las bandas más influyentes de la historia del metal. De inventores del death metal melódico a gigantes del metal alternativo moderno.</v>
       </c>
       <c r="F129" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=qnLunQEcMn0</v>
       </c>
     </row>
     <row r="130">
@@ -3160,7 +3160,7 @@
         <v>Pioneros del metal sinfónico y neoclásico en España, con una larga trayectoria internacional.</v>
       </c>
       <c r="F130" t="str">
-        <v/>
+        <v>https://www.youtube.com/@DarkMoorofficial/videos</v>
       </c>
     </row>
     <row r="131">
@@ -3180,7 +3180,7 @@
         <v>La gran voz del hard rock melódico ochentero actual. Chez Kane y su banda nos transportarán a la era dorada del AOR.</v>
       </c>
       <c r="F131" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Oc-p6U_uA3E</v>
       </c>
     </row>
     <row r="132">
@@ -3200,7 +3200,7 @@
         <v>¡Pura dinamita en directo! La banda de punk rock sueca liderada por la electrizante Cecilia Boström ofrecerá uno de los shows más enérgicos dsus conciertos.</v>
       </c>
       <c r="F132" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=r9lhoupFbKw</v>
       </c>
     </row>
     <row r="133">
@@ -3220,7 +3220,7 @@
         <v>Los padres finlandeses del power metal sinfónico descargarán himnos inmortales como "Hunting High and Low" y "Black Diamond".</v>
       </c>
       <c r="F133" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=kG4uQ6Tk7fY</v>
       </c>
     </row>
     <row r="134">
@@ -3240,7 +3240,7 @@
         <v>Banda vallisoletana de metal sinfónico y alternativo, con grandes melodías vocales a cargo de Marina Sweet.</v>
       </c>
       <c r="F134" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Ow3K7MopO2k</v>
       </c>
     </row>
     <row r="135">
@@ -3260,7 +3260,7 @@
         <v>Hard rock clásico y heavy metal de la costa oeste con riffs potentes y voz espectacular.</v>
       </c>
       <c r="F135" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=iwbUG29dDd4</v>
       </c>
     </row>
     <row r="136">
@@ -3280,7 +3280,7 @@
         <v>Banda de metal sinfónico y progresivo que destaca por sus composiciones complejas e intensas atmósferas.</v>
       </c>
       <c r="F136" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=L8sLjb3nGGM</v>
       </c>
     </row>
     <row r="137">
@@ -3300,7 +3300,7 @@
         <v>Desde el Reino Unido llega uno de los directos de metalcore y hardcore más pesados y viscerales de la actualidad.</v>
       </c>
       <c r="F137" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Ut1AcpPPOS0</v>
       </c>
     </row>
     <row r="138">
@@ -3320,7 +3320,7 @@
         <v>Heavy metal moderno y alternativo con potentes guitarras y una impecable ejecución vocal.</v>
       </c>
       <c r="F138" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=OdtC4CsbydA</v>
       </c>
     </row>
     <row r="139">
@@ -3340,7 +3340,7 @@
         <v>Banda de metal industrial con tres vocalistas (masculino, femenino y gutural) que crean una mezcla de voces única.</v>
       </c>
       <c r="F139" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=j51TIMwxriI</v>
       </c>
     </row>
     <row r="140">
@@ -3360,7 +3360,7 @@
         <v>El creador de contenido y melómano Jordi Wild cerrará la noche del viernes con un DJ Set cargado de clásicos del rock y el metal.</v>
       </c>
       <c r="F140" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=bV0FxNR0yhQ</v>
       </c>
     </row>
     <row r="141">
@@ -3380,7 +3380,7 @@
         <v>Hardcore metalizado directo desde Manchester para desatar los moshpits más salvajes .</v>
       </c>
       <c r="F141" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=O0dlwcJL-aE</v>
       </c>
     </row>
     <row r="142">
@@ -3400,7 +3400,7 @@
         <v>Liderados por el infame Glen Benton, los reyes del death metal satánico clásico descargarán su brutal repertorio blasfemo.</v>
       </c>
       <c r="F142" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=-l-OiglL460</v>
       </c>
     </row>
     <row r="143">
@@ -3420,7 +3420,7 @@
         <v>¡El cabeza de cartel indiscutible! Los creadores del power metal Helloween regresan con su show completo de aniversario para reinar en directo.</v>
       </c>
       <c r="F143" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=LZ6YKR6K_zU</v>
       </c>
     </row>
     <row r="144">
@@ -3440,7 +3440,7 @@
         <v>Gran banda madrileña de heavy metal clásico con tintes power metal y la inconfundible voz de Pacho Brea.</v>
       </c>
       <c r="F144" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=l_9LU_Qrlfs</v>
       </c>
     </row>
     <row r="145">
@@ -3460,7 +3460,7 @@
         <v>Folk pagano nórdico mezclado con ritmos electrónicos de techno y trance. ¡Una experiencia ritual y bailable única!</v>
       </c>
       <c r="F145" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=Nf_LAdo_oiE</v>
       </c>
     </row>
     <row r="146">
@@ -3480,7 +3480,7 @@
         <v>La apisonadora alemana de death metal melódico y metalcore desatará una tormenta de moshpits épicos.</v>
       </c>
       <c r="F146" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=TTkZt8r2lko</v>
       </c>
     </row>
     <row r="147">
@@ -3500,7 +3500,7 @@
         <v>Víctor García y sus chicos regresan en directo para descargar sus himnos inmortales de heavy metal coreados por miles de almas.</v>
       </c>
       <c r="F147" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=UJaW2Z5DxS8</v>
       </c>
     </row>
     <row r="148">
@@ -3520,7 +3520,7 @@
         <v>Banda de death melódico liderada por Hynphernia, que destaca por su contundencia y atmósfera oscura.</v>
       </c>
       <c r="F148" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=eiEl-mbPpj4</v>
       </c>
     </row>
     <row r="149">
@@ -3540,7 +3540,7 @@
         <v>Mítica banda de heavy metal euskaldun, listos para recordar clásicos atemporales.</v>
       </c>
       <c r="F149" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=WNmUqMR_hkE</v>
       </c>
     </row>
     <row r="150">
@@ -3560,7 +3560,7 @@
         <v>El cantante Johnny Gioeli lidera esta banda de hard rock melódico nacida en los noventa.</v>
       </c>
       <c r="F150" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=I9n1_vRYYoc</v>
       </c>
     </row>
     <row r="151">
@@ -3580,7 +3580,7 @@
         <v>Metal oscuro y deathcore de vanguardia con toques industriales y breakdowns opresivos.</v>
       </c>
       <c r="F151" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=LElq1WEBQRY</v>
       </c>
     </row>
     <row r="152">
@@ -3600,7 +3600,7 @@
         <v>Metalcore experimental y agresivo firmado por uno de los nuevos estandartes del sello Arising Empire.</v>
       </c>
       <c r="F152" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=1vwJfeXJRmQ</v>
       </c>
     </row>
     <row r="153">
@@ -3620,7 +3620,7 @@
         <v>Metal extremo oscuro e inquietante directo desde Copenhague.</v>
       </c>
       <c r="F153" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=amj49T04FCQ</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feature: Implement autoplaying background aftermovie video on festival home screen
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:P3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -456,6 +456,9 @@
       <c r="O1" t="str">
         <v>Mapa</v>
       </c>
+      <c r="P1" t="str">
+        <v>Aftermovie</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -503,6 +506,9 @@
       <c r="O2" t="str">
         <v>maparesu2026.jpg</v>
       </c>
+      <c r="P2" t="str">
+        <v>https://www.youtube.com/watch?v=Fd3gLltg0dY</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -550,11 +556,13 @@
       <c r="O3" t="str">
         <v>mapaleyendas2026.jpg</v>
       </c>
+      <c r="P3" t="str">
+        <v>https://www.youtube.com/watch?v=Nj-5T2YueiA</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implementada mejora en la ficha de cada artista: integrado enlace de Spotify, Instagram, Facebook y fotos de Spotify extraidas y sincronizadas desde Excel y MusicBrainz
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -619,7 +619,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:J174"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -640,6 +640,18 @@
       <c r="F1" t="str">
         <v>YouTube</v>
       </c>
+      <c r="G1" t="str">
+        <v>Imagen</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Spotify</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Instagram</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Facebook</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -660,6 +672,18 @@
       <c r="F2" t="str">
         <v>https://www.youtube.com/watch?v=6T4JAn4lFL0</v>
       </c>
+      <c r="G2" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174b4d845bbfb42f16a61c01ab1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://open.spotify.com/artist/7lAi1Cv19DsukgGjbZQxFg</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://www.instagram.com/annisokay/</v>
+      </c>
+      <c r="J2" t="str">
+        <v>https://www.facebook.com/annisokay</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -680,6 +704,18 @@
       <c r="F3" t="str">
         <v>https://www.youtube.com/watch?v=5LrDrFgDyl4</v>
       </c>
+      <c r="G3" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517444cb4815148bd49c0a600b89</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://open.spotify.com/artist/7ohlPA8dRBtCf92zaZCaaB</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://www.instagram.com/crowdedhousehq/</v>
+      </c>
+      <c r="J3" t="str">
+        <v>https://www.facebook.com/crowdedhouse</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -700,6 +736,18 @@
       <c r="F4" t="str">
         <v>https://www.youtube.com/watch?v=gLtbBsBGKxc</v>
       </c>
+      <c r="G4" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517422a922aee0225190714f9c3d</v>
+      </c>
+      <c r="H4" t="str">
+        <v>https://open.spotify.com/artist/7bxj5hQmURF8Y1DB3Zalfl</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v>https://www.facebook.com/profile.php?id=100085118077210</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -720,6 +768,18 @@
       <c r="F5" t="str">
         <v>https://www.youtube.com/watch?v=FrXAUcLWYZ4</v>
       </c>
+      <c r="G5" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174e30959e15d3719dc8d9ffe65</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://open.spotify.com/artist/3NTbOmzlj2cL86XFuDVFvZ</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>https://www.facebook.com/MWAMjapan</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -740,6 +800,18 @@
       <c r="F6" t="str">
         <v>https://www.youtube.com/watch?v=uBU8\_O8G9IM</v>
       </c>
+      <c r="G6" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174f4955c9f0802e7974d78c0c5</v>
+      </c>
+      <c r="H6" t="str">
+        <v>https://open.spotify.com/artist/4Ase9pfG4FCMoiuyRduc8k</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://www.instagram.com/godcomplexuk/</v>
+      </c>
+      <c r="J6" t="str">
+        <v>https://www.facebook.com/GodComplexUK</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -760,6 +832,18 @@
       <c r="F7" t="str">
         <v>https://www.youtube.com/watch?v=EBAdqbbioZ8</v>
       </c>
+      <c r="G7" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051747e810df67eaa12da0582b245</v>
+      </c>
+      <c r="H7" t="str">
+        <v>https://open.spotify.com/artist/0hTsRy6iJPc0fgkxhEHzmT</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://www.instagram.com/thesundaysadness/</v>
+      </c>
+      <c r="J7" t="str">
+        <v>https://www.facebook.com/TheSundaySadness</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -780,6 +864,18 @@
       <c r="F8" t="str">
         <v>https://www.youtube.com/watch?v=nUX-xW182EI</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -800,6 +896,18 @@
       <c r="F9" t="str">
         <v>https://www.youtube.com/watch?v=aczq-iCfFOk</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -820,6 +928,18 @@
       <c r="F10" t="str">
         <v>https://www.youtube.com/watch?v=myEyI0gT6r8</v>
       </c>
+      <c r="G10" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517418948a56786b9b75ff4a9664</v>
+      </c>
+      <c r="H10" t="str">
+        <v>https://open.spotify.com/artist/7qkUuynmt0X6RkPgvF5ttK</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://www.instagram.com/immortaldisfigurement/</v>
+      </c>
+      <c r="J10" t="str">
+        <v>https://www.facebook.com/immortaldisfigurement</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -840,6 +960,18 @@
       <c r="F11" t="str">
         <v>https://www.youtube.com/watch?v=3V9isTmCQRo</v>
       </c>
+      <c r="G11" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051746f91713ebd51749f9c63b6ec</v>
+      </c>
+      <c r="H11" t="str">
+        <v>https://open.spotify.com/artist/4DJ2QHcDJiDC0Kx1xZ9oNm</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://www.instagram.com/wearetheprettywild/</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -860,6 +992,18 @@
       <c r="F12" t="str">
         <v>https://www.youtube.com/watch?v=l-Rv5riBvc8\&amp;t=3s</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -880,6 +1024,18 @@
       <c r="F13" t="str">
         <v>https://www.youtube.com/watch?v=MfDZlUD\_1WU</v>
       </c>
+      <c r="G13" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741d205bf1c3d1017658dafc87</v>
+      </c>
+      <c r="H13" t="str">
+        <v>https://open.spotify.com/artist/6BCpGC485tSshwjemmeAmd</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://www.instagram.com/thescratchmusic/</v>
+      </c>
+      <c r="J13" t="str">
+        <v>https://www.facebook.com/TheScratchMusic</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -900,6 +1056,18 @@
       <c r="F14" t="str">
         <v>https://www.youtube.com/watch?v=DqBzOVCmIdM</v>
       </c>
+      <c r="G14" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517489a040970f9cbe2e7cc55526</v>
+      </c>
+      <c r="H14" t="str">
+        <v>https://open.spotify.com/artist/5eBCPtU2iPbzuMRre9BePt</v>
+      </c>
+      <c r="I14" t="str">
+        <v>https://www.instagram.com/thrownband/</v>
+      </c>
+      <c r="J14" t="str">
+        <v>https://www.facebook.com/thrownband</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -920,6 +1088,18 @@
       <c r="F15" t="str">
         <v>https://www.youtube.com/watch?v=\_DEdsCEUpaI</v>
       </c>
+      <c r="G15" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517443493246e66f6e7641067204</v>
+      </c>
+      <c r="H15" t="str">
+        <v>https://open.spotify.com/artist/4DSNcg40nf6T3eNAObq1Lo</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://www.instagram.com/thebrowningofficial/</v>
+      </c>
+      <c r="J15" t="str">
+        <v>https://www.facebook.com/TheBrowningOfficial</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -940,6 +1120,18 @@
       <c r="F16" t="str">
         <v>https://www.youtube.com/watch?v=UTwRqGlIaIs</v>
       </c>
+      <c r="G16" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051746704861c4fb1ac622541beb1</v>
+      </c>
+      <c r="H16" t="str">
+        <v>https://open.spotify.com/artist/4S47feOS2ATuhc7Ao5ilfG</v>
+      </c>
+      <c r="I16" t="str">
+        <v>https://www.instagram.com/lasttrainband/</v>
+      </c>
+      <c r="J16" t="str">
+        <v>https://www.facebook.com/lasttrainofficial</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -960,6 +1152,18 @@
       <c r="F17" t="str">
         <v>https://www.youtube.com/watch?v=jGxykN8cx7w</v>
       </c>
+      <c r="G17" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051746164f861e5e683c9067f4395</v>
+      </c>
+      <c r="H17" t="str">
+        <v>https://open.spotify.com/artist/4NiJW4q9ichVqL1aUsgGAN</v>
+      </c>
+      <c r="I17" t="str">
+        <v>https://www.instagram.com/adtr/</v>
+      </c>
+      <c r="J17" t="str">
+        <v>https://www.facebook.com/adtr</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -980,6 +1184,18 @@
       <c r="F18" t="str">
         <v>https://www.youtube.com/watch?v=UvncAul5sEI</v>
       </c>
+      <c r="G18" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517471760ce2698c7a1ef11827ce</v>
+      </c>
+      <c r="H18" t="str">
+        <v>https://open.spotify.com/artist/47YTOUaDKlPoDHr00r5Wu2</v>
+      </c>
+      <c r="I18" t="str">
+        <v>https://www.instagram.com/gettheshothc/</v>
+      </c>
+      <c r="J18" t="str">
+        <v>https://www.facebook.com/gettheshothc</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1000,6 +1216,18 @@
       <c r="F19" t="str">
         <v>https://www.youtube.com/watch?v=VcoSyfcqYSY</v>
       </c>
+      <c r="G19" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174087085203613a85a09bd9573</v>
+      </c>
+      <c r="H19" t="str">
+        <v>https://open.spotify.com/artist/0FHW0Lp33r3fvIG0HL4mW0</v>
+      </c>
+      <c r="I19" t="str">
+        <v>https://www.instagram.com/selfdeception_official/</v>
+      </c>
+      <c r="J19" t="str">
+        <v>https://www.facebook.com/selfdeceptionsthlm</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1020,6 +1248,18 @@
       <c r="F20" t="str">
         <v>https://www.youtube.com/watch?v=er6nWXylNHE</v>
       </c>
+      <c r="G20" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051742d3625365dbb832e71d50294</v>
+      </c>
+      <c r="H20" t="str">
+        <v>https://open.spotify.com/artist/3jIBGr0NVe9cmBRI09itgn</v>
+      </c>
+      <c r="I20" t="str">
+        <v>https://www.instagram.com/lampr3a/</v>
+      </c>
+      <c r="J20" t="str">
+        <v>https://www.facebook.com/lampr3a</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1040,6 +1280,18 @@
       <c r="F21" t="str">
         <v>https://www.youtube.com/watch?v=Dfh1aSdxr9U</v>
       </c>
+      <c r="G21" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174fc0524cca1171fac8678f4bf</v>
+      </c>
+      <c r="H21" t="str">
+        <v>https://open.spotify.com/artist/3o2dn2O0FCVsWDFSh8qxgG</v>
+      </c>
+      <c r="I21" t="str">
+        <v>https://www.instagram.com/sabatonofficial/</v>
+      </c>
+      <c r="J21" t="str">
+        <v>https://www.facebook.com/sabaton</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1060,6 +1312,18 @@
       <c r="F22" t="str">
         <v>https://www.youtube.com/watch?v=147BrDp-XuA</v>
       </c>
+      <c r="G22" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051742c3b07616f77f8bca1ab8179</v>
+      </c>
+      <c r="H22" t="str">
+        <v>https://open.spotify.com/artist/4Gmrt82h2vjGjnp67SG5Nw</v>
+      </c>
+      <c r="I22" t="str">
+        <v>https://www.instagram.com/highvis/</v>
+      </c>
+      <c r="J22" t="str">
+        <v>https://www.facebook.com/highvispunk</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1080,6 +1344,18 @@
       <c r="F23" t="str">
         <v>https://www.youtube.com/watch?v=nytv1O2yvG8</v>
       </c>
+      <c r="G23" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174673238b2ab364667667e1008</v>
+      </c>
+      <c r="H23" t="str">
+        <v>https://open.spotify.com/artist/6bAM7jeIX4pI5lZ0QoSZjt</v>
+      </c>
+      <c r="I23" t="str">
+        <v>https://www.instagram.com/faetooth/</v>
+      </c>
+      <c r="J23" t="str">
+        <v>https://www.facebook.com/faetoothband</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1100,6 +1376,18 @@
       <c r="F24" t="str">
         <v>https://www.youtube.com/watch?v=Gtw3lcQvyPU</v>
       </c>
+      <c r="G24" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051745663001a056558505a84d8e1</v>
+      </c>
+      <c r="H24" t="str">
+        <v>https://open.spotify.com/artist/28hJdGN1Awf7u3ifk2lVkg</v>
+      </c>
+      <c r="I24" t="str">
+        <v>https://www.instagram.com/testamentofficial/</v>
+      </c>
+      <c r="J24" t="str">
+        <v>https://www.facebook.com/testamentlegions</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1120,6 +1408,18 @@
       <c r="F25" t="str">
         <v>https://www.youtube.com/watch?v=x8Ku8xs3LJA\&amp;list=RDEMx9F7gSD6CPp5z3JPCDu3FA\&amp;start\_radio=1</v>
       </c>
+      <c r="G25" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517408e3b7d4e3bb04423a5ed2cd</v>
+      </c>
+      <c r="H25" t="str">
+        <v>https://open.spotify.com/artist/138GsDz0pX5leXnKi7ay7G</v>
+      </c>
+      <c r="I25" t="str">
+        <v>https://www.instagram.com/tides._/</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1140,6 +1440,18 @@
       <c r="F26" t="str">
         <v>https://www.youtube.com/watch?v=mmP3MmImXi0</v>
       </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v>https://www.instagram.com/fallenatdawnofficial/</v>
+      </c>
+      <c r="J26" t="str">
+        <v>https://www.facebook.com/FallenAtDawnOfficial</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1160,6 +1472,18 @@
       <c r="F27" t="str">
         <v>https://www.youtube.com/watch?v=735VrHSslAA</v>
       </c>
+      <c r="G27" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051740684d08ba2a1fb899214040c</v>
+      </c>
+      <c r="H27" t="str">
+        <v>https://open.spotify.com/artist/7aTaQAh9d7z98h0CMrx1s6</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1180,6 +1504,18 @@
       <c r="F28" t="str">
         <v>https://www.youtube.com/watch?v=MQi07wk7xms</v>
       </c>
+      <c r="G28" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743ed3cd4237f99b7298a59b06</v>
+      </c>
+      <c r="H28" t="str">
+        <v>https://open.spotify.com/artist/2IZHv7enTnPW7yuS9w1qq7</v>
+      </c>
+      <c r="I28" t="str">
+        <v>https://www.instagram.com/heranxietyband/</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1200,6 +1536,18 @@
       <c r="F29" t="str">
         <v>https://www.youtube.com/watch?v=UuSXoG2ncME</v>
       </c>
+      <c r="G29" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051745ee17d6fdaa227d2b307e297</v>
+      </c>
+      <c r="H29" t="str">
+        <v>https://open.spotify.com/artist/0GicbfMtwhn3Ch0PdwkADQ</v>
+      </c>
+      <c r="I29" t="str">
+        <v>https://www.instagram.com/sillygooseatl/</v>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1220,6 +1568,18 @@
       <c r="F30" t="str">
         <v>https://www.youtube.com/watch?v=kT36IN83gGI</v>
       </c>
+      <c r="G30" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051747094e150185be7496961ec17</v>
+      </c>
+      <c r="H30" t="str">
+        <v>https://open.spotify.com/artist/2XIbOWDT5vZPW7jNyzdfcK</v>
+      </c>
+      <c r="I30" t="str">
+        <v>https://www.instagram.com/caskets_band/</v>
+      </c>
+      <c r="J30" t="str">
+        <v>https://www.facebook.com/casketsbandofficial</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1240,6 +1600,18 @@
       <c r="F31" t="str">
         <v>https://www.youtube.com/watch?v=hcDyDii-Low</v>
       </c>
+      <c r="G31" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f77a7ddaaee51fe2df8c3bd3</v>
+      </c>
+      <c r="H31" t="str">
+        <v>https://open.spotify.com/artist/4WfUbvICLrqPW9rzuNGS1f</v>
+      </c>
+      <c r="I31" t="str">
+        <v>https://www.instagram.com/bloodcommand/</v>
+      </c>
+      <c r="J31" t="str">
+        <v>https://www.facebook.com/bloodcommand</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1260,6 +1632,18 @@
       <c r="F32" t="str">
         <v>https://www.youtube.com/watch?v=RwomV4za97A</v>
       </c>
+      <c r="G32" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174ed7fd539fd4bbc095f69749f</v>
+      </c>
+      <c r="H32" t="str">
+        <v>https://open.spotify.com/artist/0eNuNAhL4dW2nvKbSe2mS8</v>
+      </c>
+      <c r="I32" t="str">
+        <v>https://www.instagram.com/burningwitchesofficial/</v>
+      </c>
+      <c r="J32" t="str">
+        <v>https://www.facebook.com/burningwitches666</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1280,6 +1664,18 @@
       <c r="F33" t="str">
         <v>https://www.youtube.com/watch?v=xb50ooBETEc</v>
       </c>
+      <c r="G33" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174e2e02a23d38e23a35f3dda34</v>
+      </c>
+      <c r="H33" t="str">
+        <v>https://open.spotify.com/artist/3bnPBquC93vbHmamojAf59</v>
+      </c>
+      <c r="I33" t="str">
+        <v>https://www.instagram.com/angelusapatrida/</v>
+      </c>
+      <c r="J33" t="str">
+        <v>https://www.facebook.com/angelusapatrida</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1300,6 +1696,18 @@
       <c r="F34" t="str">
         <v>https://www.youtube.com/watch?v=lZK5xfbZXNw</v>
       </c>
+      <c r="G34" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174ae9a9ec82f0aad57ac2fa9a3</v>
+      </c>
+      <c r="H34" t="str">
+        <v>https://open.spotify.com/artist/2lmQ4CUnjmLIIfnwZdRmMY</v>
+      </c>
+      <c r="I34" t="str">
+        <v>https://www.instagram.com/bluespills/</v>
+      </c>
+      <c r="J34" t="str">
+        <v>https://www.facebook.com/BluesPills</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1320,6 +1728,18 @@
       <c r="F35" t="str">
         <v>https://www.youtube.com/watch?v=a8DP5vhiDTk</v>
       </c>
+      <c r="G35" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174c65a19fb4526e6640f14b0eb</v>
+      </c>
+      <c r="H35" t="str">
+        <v>https://open.spotify.com/artist/4iGsihTcyZ80RQFZhC8bf8</v>
+      </c>
+      <c r="I35" t="str">
+        <v>https://www.instagram.com/tfp_insta/</v>
+      </c>
+      <c r="J35" t="str">
+        <v>https://www.facebook.com/thefuneralportrait</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1340,6 +1760,18 @@
       <c r="F36" t="str">
         <v>https://www.youtube.com/watch?v=9SFlXVpZfsg</v>
       </c>
+      <c r="G36" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174a3ba1aba509d351b685dd756</v>
+      </c>
+      <c r="H36" t="str">
+        <v>https://open.spotify.com/artist/6LaK7jiyyNzB8JVhddxZxG</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v>https://www.facebook.com/belvedere669</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1360,6 +1792,18 @@
       <c r="F37" t="str">
         <v>https://www.youtube.com/watch?v=nQlua3uDfts</v>
       </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1380,6 +1824,18 @@
       <c r="F38" t="str">
         <v>https://www.youtube.com/watch?v=aAsrFetnHzM</v>
       </c>
+      <c r="G38" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174f9978ad4808f6f2723124d19</v>
+      </c>
+      <c r="H38" t="str">
+        <v>https://open.spotify.com/artist/6mdiAmATAx73kdxrNrnlao</v>
+      </c>
+      <c r="I38" t="str">
+        <v>https://www.instagram.com/ironmaiden/</v>
+      </c>
+      <c r="J38" t="str">
+        <v>https://www.facebook.com/ironmaiden</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1400,6 +1856,18 @@
       <c r="F39" t="str">
         <v>https://www.youtube.com/watch?v=4l5qLn2NrnE</v>
       </c>
+      <c r="G39" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051745b5adfd95f6b322fb7ae729d</v>
+      </c>
+      <c r="H39" t="str">
+        <v>https://open.spotify.com/artist/4ZWRLOs7c4drt9mKGc0Ds0</v>
+      </c>
+      <c r="I39" t="str">
+        <v>https://www.instagram.com/thecallousdaoboys/</v>
+      </c>
+      <c r="J39" t="str">
+        <v>https://www.facebook.com/thecallousdaoboys</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1420,6 +1888,18 @@
       <c r="F40" t="str">
         <v>https://www.youtube.com/watch?v=6joGJzYX\_Rc</v>
       </c>
+      <c r="G40" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051740a1c9d4dd7f23acca1a1581b</v>
+      </c>
+      <c r="H40" t="str">
+        <v>https://open.spotify.com/artist/16MG8AG1y22HDmY8IoI5lY</v>
+      </c>
+      <c r="I40" t="str">
+        <v>https://www.instagram.com/vulvarine_band/</v>
+      </c>
+      <c r="J40" t="str">
+        <v>https://www.facebook.com/vulvarine.vienna</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1440,6 +1920,18 @@
       <c r="F41" t="str">
         <v>https://www.youtube.com/watch?v=z4DXIoWCr1Q</v>
       </c>
+      <c r="G41" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174682b7b4eb91bd27faa15f117</v>
+      </c>
+      <c r="H41" t="str">
+        <v>https://open.spotify.com/artist/1oeo6cC9Fqa2bxxv67qBQL</v>
+      </c>
+      <c r="I41" t="str">
+        <v>https://www.instagram.com/calibanofficial/</v>
+      </c>
+      <c r="J41" t="str">
+        <v>https://www.facebook.com/CalibanOfficial</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1460,6 +1952,18 @@
       <c r="F42" t="str">
         <v>https://www.youtube.com/watch?v=VeP1OmL5fNQ</v>
       </c>
+      <c r="G42" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749d9c2adfaa9d7886eaab969b</v>
+      </c>
+      <c r="H42" t="str">
+        <v>https://open.spotify.com/artist/6dOCTX1ATvti0d4uaxwlO3</v>
+      </c>
+      <c r="I42" t="str">
+        <v>https://www.instagram.com/lionheartca/</v>
+      </c>
+      <c r="J42" t="str">
+        <v>https://www.facebook.com/lionheartca</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1480,6 +1984,18 @@
       <c r="F43" t="str">
         <v>https://www.youtube.com/watch?v=Pj5u8OagODo</v>
       </c>
+      <c r="G43" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051748fa118d8e890fcb413676e56</v>
+      </c>
+      <c r="H43" t="str">
+        <v>https://open.spotify.com/artist/3JysSUOyfVs1UQ0UaESheP</v>
+      </c>
+      <c r="I43" t="str">
+        <v>https://www.instagram.com/anthrax/</v>
+      </c>
+      <c r="J43" t="str">
+        <v>https://www.facebook.com/anthrax</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1500,6 +2016,18 @@
       <c r="F44" t="str">
         <v>https://www.youtube.com/watch?v=x2lxwwzkLCM</v>
       </c>
+      <c r="G44" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174afdc2d8c216673ea95ea23c0</v>
+      </c>
+      <c r="H44" t="str">
+        <v>https://open.spotify.com/artist/604HhRLmc5DXNS221XKm3a</v>
+      </c>
+      <c r="I44" t="str">
+        <v>https://www.instagram.com/psychonautband/</v>
+      </c>
+      <c r="J44" t="str">
+        <v>https://www.facebook.com/psychonautband</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1520,6 +2048,18 @@
       <c r="F45" t="str">
         <v>https://www.youtube.com/watch?v=XmhN3t4wLFA</v>
       </c>
+      <c r="G45" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174cc8769232844e85493288724</v>
+      </c>
+      <c r="H45" t="str">
+        <v>https://open.spotify.com/artist/5CHcX5KtuSz5uo1p5fM3sz</v>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v>https://www.facebook.com/authorityzero.official</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1540,6 +2080,18 @@
       <c r="F46" t="str">
         <v>https://www.youtube.com/watch?v=-rKOoM7S6mw</v>
       </c>
+      <c r="G46" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174412d9bee52f47326eb0ed7d0</v>
+      </c>
+      <c r="H46" t="str">
+        <v>https://open.spotify.com/artist/2Ct54gNxKnYLnXk9HhviMI</v>
+      </c>
+      <c r="I46" t="str">
+        <v>https://www.instagram.com/feuerschwanzband/</v>
+      </c>
+      <c r="J46" t="str">
+        <v>https://www.facebook.com/feuerschwanz</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1560,6 +2112,18 @@
       <c r="F47" t="str">
         <v>https://www.youtube.com/watch?v=zNDcD3oSt3U</v>
       </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v>https://www.facebook.com/TheFallOfAtlantis</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1580,6 +2144,18 @@
       <c r="F48" t="str">
         <v>https://www.youtube.com/watch?v=EmnfimPvST0</v>
       </c>
+      <c r="G48" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174a1c7ed6c04f937ded19c3a0c</v>
+      </c>
+      <c r="H48" t="str">
+        <v>https://open.spotify.com/artist/76hPQa6sCQSpbMsSzLVSAw</v>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1600,6 +2176,18 @@
       <c r="F49" t="str">
         <v>https://www.youtube.com/watch?v=6l5TIlI4tdg</v>
       </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1620,6 +2208,18 @@
       <c r="F50" t="str">
         <v>https://www.youtube.com/watch?v=AO4JQ3\_zPXE</v>
       </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v>https://www.facebook.com/pantsoffmusic</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1640,6 +2240,18 @@
       <c r="F51" t="str">
         <v>https://www.youtube.com/watch?v=GljyxhhdFqU</v>
       </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1660,6 +2272,18 @@
       <c r="F52" t="str">
         <v>https://www.youtube.com/watch?v=sNi\_YmGT7Cw</v>
       </c>
+      <c r="G52" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174dc49476fb23bf6a52c369b95</v>
+      </c>
+      <c r="H52" t="str">
+        <v>https://open.spotify.com/artist/5heR5lCdbT4TqjgnQNji4U</v>
+      </c>
+      <c r="I52" t="str">
+        <v>https://www.instagram.com/madmessband/</v>
+      </c>
+      <c r="J52" t="str">
+        <v>https://www.facebook.com/madmessband</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1680,6 +2304,18 @@
       <c r="F53" t="str">
         <v>https://www.youtube.com/watch?v=uY4vweIBFcY</v>
       </c>
+      <c r="G53" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517452612710e1a88ad35002aced</v>
+      </c>
+      <c r="H53" t="str">
+        <v>https://open.spotify.com/artist/76ptJV8617638xrpeoUtzl</v>
+      </c>
+      <c r="I53" t="str">
+        <v>https://www.instagram.com/therasmusofficial/</v>
+      </c>
+      <c r="J53" t="str">
+        <v>https://www.facebook.com/therasmusofficial</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1700,6 +2336,18 @@
       <c r="F54" t="str">
         <v>https://www.youtube.com/watch?v=TgWSiiCQU1I</v>
       </c>
+      <c r="G54" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741f670e6d8023290fcf317dfd</v>
+      </c>
+      <c r="H54" t="str">
+        <v>https://open.spotify.com/artist/3KSBsxMjBEZCxmrj0GEWJI</v>
+      </c>
+      <c r="I54" t="str">
+        <v>https://www.instagram.com/osloovnies/</v>
+      </c>
+      <c r="J54" t="str">
+        <v>https://www.facebook.com/osloovniesband</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1720,6 +2368,18 @@
       <c r="F55" t="str">
         <v>https://www.youtube.com/watch?v=9mJu2r\_v7FE</v>
       </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -1740,6 +2400,18 @@
       <c r="F56" t="str">
         <v>https://www.youtube.com/watch?v=yq483\_-C5tA</v>
       </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v>https://www.instagram.com/movrir/</v>
+      </c>
+      <c r="J56" t="str">
+        <v>https://www.facebook.com/movrir</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -1760,6 +2432,18 @@
       <c r="F57" t="str">
         <v>https://www.youtube.com/watch?v=42-e9zFmgPA</v>
       </c>
+      <c r="G57" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174cd7069f3be53bbc57a747293</v>
+      </c>
+      <c r="H57" t="str">
+        <v>https://open.spotify.com/artist/5ZvwJikDgdP1PFU4PkAPVG</v>
+      </c>
+      <c r="I57" t="str">
+        <v>https://www.instagram.com/bleedfromwithin/</v>
+      </c>
+      <c r="J57" t="str">
+        <v>https://www.facebook.com/bleedfromwithinband</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1780,6 +2464,18 @@
       <c r="F58" t="str">
         <v>https://www.youtube.com/watch?v=KH0PrtJIkIo</v>
       </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v>https://www.instagram.com/initiate_hc/</v>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -1800,6 +2496,18 @@
       <c r="F59" t="str">
         <v>https://www.youtube.com/watch?v=Q2gttZHbJsw</v>
       </c>
+      <c r="G59" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741f6ff549b2bbbb0819e40440</v>
+      </c>
+      <c r="H59" t="str">
+        <v>https://open.spotify.com/artist/65vrcJ67suxLePeEhUtLLo</v>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v>https://www.facebook.com/HulderUS</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -1820,6 +2528,18 @@
       <c r="F60" t="str">
         <v>https://www.youtube.com/watch?v=8YehoejPll8\&amp;list=RDEM71BufWZpq5YI695VOCH1Xw\&amp;start\_radio=1</v>
       </c>
+      <c r="G60" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051744d81765e21254b9dbdc8df0e</v>
+      </c>
+      <c r="H60" t="str">
+        <v>https://open.spotify.com/artist/2DvBNcZ05NC2AOuQa7oyqH</v>
+      </c>
+      <c r="I60" t="str">
+        <v>https://www.instagram.com/rosaliecunningham71/</v>
+      </c>
+      <c r="J60" t="str">
+        <v>https://www.facebook.com/RosalieCunninghamOfficial</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1840,6 +2560,18 @@
       <c r="F61" t="str">
         <v>https://www.youtube.com/watch?v=IIgswpHNZik</v>
       </c>
+      <c r="G61" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174ab21a41e346730ff64be53c2</v>
+      </c>
+      <c r="H61" t="str">
+        <v>https://open.spotify.com/artist/278ZYwGhdK6QTzE3MFePnP</v>
+      </c>
+      <c r="I61" t="str">
+        <v>https://www.instagram.com/triviumband/</v>
+      </c>
+      <c r="J61" t="str">
+        <v>https://www.facebook.com/TriviumOfficial</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -1860,6 +2592,18 @@
       <c r="F62" t="str">
         <v>https://www.youtube.com/watch?v=U1g8yXXOmOQ</v>
       </c>
+      <c r="G62" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051748dc46d134bd391950448b780</v>
+      </c>
+      <c r="H62" t="str">
+        <v>https://open.spotify.com/artist/4igS2MSwOIf3F9YeL929IO</v>
+      </c>
+      <c r="I62" t="str">
+        <v>https://www.instagram.com/dyingwishhc/</v>
+      </c>
+      <c r="J62" t="str">
+        <v>https://www.facebook.com/DyingWish503</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1880,6 +2624,18 @@
       <c r="F63" t="str">
         <v>https://www.youtube.com/watch?v=NpdWlHP\_pns</v>
       </c>
+      <c r="G63" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749291dd6eb8ea9ebab3363d87</v>
+      </c>
+      <c r="H63" t="str">
+        <v>https://open.spotify.com/artist/1wXoI3Ajpv4WwQ3LmcrSBw</v>
+      </c>
+      <c r="I63" t="str">
+        <v>https://www.instagram.com/gaerea_/</v>
+      </c>
+      <c r="J63" t="str">
+        <v>https://www.facebook.com/gaerea</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1900,6 +2656,18 @@
       <c r="F64" t="str">
         <v>https://www.youtube.com/watch?v=r\_TvbkwN4I4</v>
       </c>
+      <c r="G64" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174362ffca97de946dd048c973c</v>
+      </c>
+      <c r="H64" t="str">
+        <v>https://open.spotify.com/artist/53Hm23U3dtaHeB5Oy6GbaS</v>
+      </c>
+      <c r="I64" t="str">
+        <v>https://www.instagram.com/returntodustband/</v>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1920,6 +2688,18 @@
       <c r="F65" t="str">
         <v>https://www.youtube.com/watch?v=bSTX2xVpfPw</v>
       </c>
+      <c r="G65" t="str">
+        <v>https://i.scdn.co/image/38532b2db9bc627567271da917855a59be788860</v>
+      </c>
+      <c r="H65" t="str">
+        <v>https://open.spotify.com/artist/165ZgPlLkK7bf5bDoFc6Sb</v>
+      </c>
+      <c r="I65" t="str">
+        <v>https://www.instagram.com/limpbizkit/</v>
+      </c>
+      <c r="J65" t="str">
+        <v>https://www.facebook.com/limpbizkit</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1940,6 +2720,18 @@
       <c r="F66" t="str">
         <v>https://www.youtube.com/watch?v=xuhVpPAx0bA</v>
       </c>
+      <c r="G66" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174de085730e9d3a870ab7f5824</v>
+      </c>
+      <c r="H66" t="str">
+        <v>https://open.spotify.com/artist/5YlX74SFjWauq32aKLwAYn</v>
+      </c>
+      <c r="I66" t="str">
+        <v>https://www.instagram.com/enditbaltimore/</v>
+      </c>
+      <c r="J66" t="str">
+        <v>https://www.facebook.com/EndItBCHC</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -1960,6 +2752,18 @@
       <c r="F67" t="str">
         <v>https://www.youtube.com/watch?v=Jp6-SoqXp\_s</v>
       </c>
+      <c r="G67" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749b6aa935e19530c540cfd7be</v>
+      </c>
+      <c r="H67" t="str">
+        <v>https://open.spotify.com/artist/0uTkKGuqdf7CtKlZLt9N0Y</v>
+      </c>
+      <c r="I67" t="str">
+        <v>https://www.instagram.com/nevertelofficial/</v>
+      </c>
+      <c r="J67" t="str">
+        <v>https://www.facebook.com/NevertelOfficial</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -1980,6 +2784,18 @@
       <c r="F68" t="str">
         <v>https://www.youtube.com/watch?v=7hxKHRqCRdA</v>
       </c>
+      <c r="G68" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517428e028c642117dc411386f77</v>
+      </c>
+      <c r="H68" t="str">
+        <v>https://open.spotify.com/artist/0vxxsjcDy61x5zvrOqwHIL</v>
+      </c>
+      <c r="I68" t="str">
+        <v>https://www.instagram.com/borknagar/</v>
+      </c>
+      <c r="J68" t="str">
+        <v>https://www.facebook.com/borknagarofficial</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2000,6 +2816,18 @@
       <c r="F69" t="str">
         <v>https://www.youtube.com/watch?v=qCMz704soB4</v>
       </c>
+      <c r="G69" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174d93429df94b98f1f457f2856</v>
+      </c>
+      <c r="H69" t="str">
+        <v>https://open.spotify.com/artist/7F1K4WlMshx23V2TTz4KwV</v>
+      </c>
+      <c r="I69" t="str">
+        <v>https://www.instagram.com/cavaleraconspiracy/</v>
+      </c>
+      <c r="J69" t="str">
+        <v>https://www.facebook.com/maxeigorcavalera</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2020,6 +2848,18 @@
       <c r="F70" t="str">
         <v>https://www.youtube.com/watch?v=5QbMOtl\_SRo</v>
       </c>
+      <c r="G70" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051748e510569f5e209a267b77f62</v>
+      </c>
+      <c r="H70" t="str">
+        <v>https://open.spotify.com/artist/6fb3I3Q54izgnOMtiZbOBA</v>
+      </c>
+      <c r="I70" t="str">
+        <v>https://www.instagram.com/house_of_protection/</v>
+      </c>
+      <c r="J70" t="str">
+        <v>https://www.facebook.com/houseofprotectionmusic</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2040,6 +2880,18 @@
       <c r="F71" t="str">
         <v>https://www.youtube.com/watch?v=7Uk_uG26VT4</v>
       </c>
+      <c r="G71" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051746b134287e3095d2c84b7932a</v>
+      </c>
+      <c r="H71" t="str">
+        <v>https://open.spotify.com/artist/0LyfQWJT6nXafLPZqxe9Of</v>
+      </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
+      <c r="J71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2060,6 +2912,18 @@
       <c r="F72" t="str">
         <v>https://www.youtube.com/watch?v=H_-leVD654w</v>
       </c>
+      <c r="G72" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174a1e6c83ef9381bc74ccefd08</v>
+      </c>
+      <c r="H72" t="str">
+        <v>https://open.spotify.com/artist/3VaWHUyDEoBjigERzadi1g</v>
+      </c>
+      <c r="I72" t="str">
+        <v>https://www.instagram.com/iscream.never.ground/</v>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2080,6 +2944,18 @@
       <c r="F73" t="str">
         <v>https://www.youtube.com/watch?v=yAnEyq8iOzY</v>
       </c>
+      <c r="G73" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174040cf44eff6f405a81dcf59f</v>
+      </c>
+      <c r="H73" t="str">
+        <v>https://open.spotify.com/artist/3n9SWHa9CmQldmLrD9zfll</v>
+      </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
+      <c r="J73" t="str">
+        <v>https://www.facebook.com/STELLVRIS.band</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2100,6 +2976,18 @@
       <c r="F74" t="str">
         <v>https://www.youtube.com/watch?v=DqcHLdIygpk</v>
       </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+      <c r="I74" t="str">
+        <v>https://www.instagram.com/donutsholeoficial/</v>
+      </c>
+      <c r="J74" t="str">
+        <v>https://www.facebook.com/donutshole</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2120,6 +3008,18 @@
       <c r="F75" t="str">
         <v>https://www.youtube.com/watch?v=HGozdu9dfZ8</v>
       </c>
+      <c r="G75" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051747e1b69bc4f40b05b6a7052cd</v>
+      </c>
+      <c r="H75" t="str">
+        <v>https://open.spotify.com/artist/5bTh3KLGlKlcloVl318t1h</v>
+      </c>
+      <c r="I75" t="str">
+        <v>https://www.instagram.com/hamletband/</v>
+      </c>
+      <c r="J75" t="str">
+        <v>https://www.facebook.com/hamletband</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2140,6 +3040,18 @@
       <c r="F76" t="str">
         <v>https://www.youtube.com/watch?v=nRJeIUhuNmE</v>
       </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
+      <c r="I76" t="str">
+        <v>https://www.instagram.com/_kruddo_/</v>
+      </c>
+      <c r="J76" t="str">
+        <v>https://www.facebook.com/KRUDDO</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2160,6 +3072,18 @@
       <c r="F77" t="str">
         <v>https://www.youtube.com/watch?v=v3KnTgn_XJ8</v>
       </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+      <c r="I77" t="str">
+        <v>https://www.instagram.com/todo_mal_band/</v>
+      </c>
+      <c r="J77" t="str">
+        <v>https://www.facebook.com/todomalofficial</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2180,6 +3104,18 @@
       <c r="F78" t="str">
         <v>https://www.youtube.com/watch?v=Y-v9rBFMsSY</v>
       </c>
+      <c r="G78" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517447e04bfe40fed89c81118d7f</v>
+      </c>
+      <c r="H78" t="str">
+        <v>https://open.spotify.com/artist/1ANDjinr8OtamQ6TCV2HBG</v>
+      </c>
+      <c r="I78" t="str">
+        <v>https://www.instagram.com/thefamilymengbg/</v>
+      </c>
+      <c r="J78" t="str">
+        <v>https://www.facebook.com/thefamilymenband</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2200,6 +3136,18 @@
       <c r="F79" t="str">
         <v>https://www.youtube.com/watch?v=7b-VTfpGFUQ</v>
       </c>
+      <c r="G79" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051746235156da99ba77dde123ba2</v>
+      </c>
+      <c r="H79" t="str">
+        <v>https://open.spotify.com/artist/7rqJQQxuUOCk052MK5kLsH</v>
+      </c>
+      <c r="I79" t="str">
+        <v>https://www.instagram.com/imminenceswe/</v>
+      </c>
+      <c r="J79" t="str">
+        <v>https://www.facebook.com/imminenceswe</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2220,6 +3168,18 @@
       <c r="F80" t="str">
         <v>https://www.youtube.com/watch?v=CZzpb-MYrsg</v>
       </c>
+      <c r="G80" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174afe861bb48644f72fc60d7df</v>
+      </c>
+      <c r="H80" t="str">
+        <v>https://open.spotify.com/artist/735eXziB2hC9TFcx6wjBsf</v>
+      </c>
+      <c r="I80" t="str">
+        <v>https://www.instagram.com/thegems.music/</v>
+      </c>
+      <c r="J80" t="str">
+        <v>https://www.facebook.com/thegemsbandswe</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2240,6 +3200,18 @@
       <c r="F81" t="str">
         <v>https://www.youtube.com/watch?v=0fSoJaU6rTE</v>
       </c>
+      <c r="G81" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174d29ef4301b2c73cd77f8f640</v>
+      </c>
+      <c r="H81" t="str">
+        <v>https://open.spotify.com/artist/2g8hgaQzyK2a6ZD5AOKArj</v>
+      </c>
+      <c r="I81" t="str">
+        <v>https://www.instagram.com/handofjuno_official/</v>
+      </c>
+      <c r="J81" t="str">
+        <v>https://www.facebook.com/handofjunoband</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2260,6 +3232,18 @@
       <c r="F82" t="str">
         <v>https://www.youtube.com/watch?v=wI4mG1MwgpM</v>
       </c>
+      <c r="G82" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741696c69bb13dc4d8e38058f4</v>
+      </c>
+      <c r="H82" t="str">
+        <v>https://open.spotify.com/artist/6AMqkTWbhukzRS5je3Q5qt</v>
+      </c>
+      <c r="I82" t="str">
+        <v>https://www.instagram.com/frontiererband/</v>
+      </c>
+      <c r="J82" t="str">
+        <v>https://www.facebook.com/frontiererband</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2280,6 +3264,18 @@
       <c r="F83" t="str">
         <v>https://www.youtube.com/watch?v=\_ocD7BsrjrU</v>
       </c>
+      <c r="G83" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517415c1b5623a7ba1bb228087c2</v>
+      </c>
+      <c r="H83" t="str">
+        <v>https://open.spotify.com/artist/6KO6G41BBLTDNYOLefWTMU</v>
+      </c>
+      <c r="I83" t="str">
+        <v>https://www.instagram.com/POD/</v>
+      </c>
+      <c r="J83" t="str">
+        <v>https://www.facebook.com/PayableOnDeathPOD</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2300,6 +3296,18 @@
       <c r="F84" t="str">
         <v>https://www.youtube.com/watch?v=R4ElqI1RZGM</v>
       </c>
+      <c r="G84" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174a6d9c7444ad8a5e271b58364</v>
+      </c>
+      <c r="H84" t="str">
+        <v>https://open.spotify.com/artist/2osrICe2kgcit3D086z3Lo</v>
+      </c>
+      <c r="I84" t="str">
+        <v>https://www.instagram.com/cwfenband/</v>
+      </c>
+      <c r="J84" t="str">
+        <v>https://www.facebook.com/Cwfenband</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2320,6 +3328,18 @@
       <c r="F85" t="str">
         <v>https://www.youtube.com/watch?v=PHZFd5mKPks</v>
       </c>
+      <c r="G85" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051749633e7f4c2a15372288b1357</v>
+      </c>
+      <c r="H85" t="str">
+        <v>https://open.spotify.com/artist/7dfpBi0QvO9FmlhBK6XHwJ</v>
+      </c>
+      <c r="I85" t="str">
+        <v>https://www.instagram.com/DistantOfficial/</v>
+      </c>
+      <c r="J85" t="str">
+        <v>https://www.facebook.com/DistantOfficial</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2340,6 +3360,18 @@
       <c r="F86" t="str">
         <v>https://www.youtube.com/watch?v=t3yEQRc5tPc</v>
       </c>
+      <c r="G86" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517450858f98bce1c94db46ff292</v>
+      </c>
+      <c r="H86" t="str">
+        <v>https://open.spotify.com/artist/2eIUyCr530XyFHd358dxYZ</v>
+      </c>
+      <c r="I86" t="str">
+        <v>https://www.instagram.com/gridironhardcore/</v>
+      </c>
+      <c r="J86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2360,6 +3392,18 @@
       <c r="F87" t="str">
         <v>https://www.youtube.com/watch?v=WTQR-RvexVk</v>
       </c>
+      <c r="G87" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051745490f4a4c327475719679a5f</v>
+      </c>
+      <c r="H87" t="str">
+        <v>https://open.spotify.com/artist/1Dvfqq39HxvCJ3GvfeIFuT</v>
+      </c>
+      <c r="I87" t="str">
+        <v>https://www.instagram.com/mastodonrocks/</v>
+      </c>
+      <c r="J87" t="str">
+        <v>https://www.facebook.com/Mastodon</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -2380,6 +3424,18 @@
       <c r="F88" t="str">
         <v>https://www.youtube.com/watch?v=nqD7OauxaTo</v>
       </c>
+      <c r="G88" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517486b13e4d2e65ebf694384ef4</v>
+      </c>
+      <c r="H88" t="str">
+        <v>https://open.spotify.com/artist/3dRfiJ2650SZu6GbydcHNb</v>
+      </c>
+      <c r="I88" t="str">
+        <v/>
+      </c>
+      <c r="J88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -2400,6 +3456,18 @@
       <c r="F89" t="str">
         <v>https://www.youtube.com/watch?v=1f6GEWdSz-s</v>
       </c>
+      <c r="G89" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616d00001e02e3a9da7263d60cde3e4c4442</v>
+      </c>
+      <c r="H89" t="str">
+        <v>https://open.spotify.com/artist/5PxwnAyDeI22zgN023OTFt</v>
+      </c>
+      <c r="I89" t="str">
+        <v/>
+      </c>
+      <c r="J89" t="str">
+        <v>https://www.facebook.com/DOGMA.am</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -2420,6 +3488,18 @@
       <c r="F90" t="str">
         <v>https://www.youtube.com/watch?v=qxelfxGa2oo</v>
       </c>
+      <c r="G90" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f39c2d3ba5a7548dd73f92ff</v>
+      </c>
+      <c r="H90" t="str">
+        <v>https://open.spotify.com/artist/7kHzfxMLtVHHb523s43rY1</v>
+      </c>
+      <c r="I90" t="str">
+        <v>https://www.instagram.com/converge/</v>
+      </c>
+      <c r="J90" t="str">
+        <v>https://www.facebook.com/converge</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -2440,6 +3520,18 @@
       <c r="F91" t="str">
         <v>https://www.youtube.com/watch?v=yjWtkQSF8dA</v>
       </c>
+      <c r="G91" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174df97decd4f8f568310bd0031</v>
+      </c>
+      <c r="H91" t="str">
+        <v>https://open.spotify.com/artist/2VYQTNDsvvKN9wmU5W7xpj</v>
+      </c>
+      <c r="I91" t="str">
+        <v>https://www.instagram.com/marilynmanson/</v>
+      </c>
+      <c r="J91" t="str">
+        <v>https://www.facebook.com/MarilynManson</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -2460,6 +3552,18 @@
       <c r="F92" t="str">
         <v>https://www.youtube.com/watch?v=7a5loP5tjp8</v>
       </c>
+      <c r="G92" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174d08dc4cf0e505cc615424f25</v>
+      </c>
+      <c r="H92" t="str">
+        <v>https://open.spotify.com/artist/61MH29rMIyOfuK7KXQznzX</v>
+      </c>
+      <c r="I92" t="str">
+        <v>https://www.instagram.com/thevintagecaravan/</v>
+      </c>
+      <c r="J92" t="str">
+        <v>https://www.facebook.com/vintagecaravan</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -2480,6 +3584,18 @@
       <c r="F93" t="str">
         <v>https://www.youtube.com/watch?v=O9WYceFbHw4</v>
       </c>
+      <c r="G93" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517439beafeafdc096ec01250662</v>
+      </c>
+      <c r="H93" t="str">
+        <v>https://open.spotify.com/artist/6FGv87WQ3mJWn3cmLUww6x</v>
+      </c>
+      <c r="I93" t="str">
+        <v>https://www.instagram.com/bloodincantationofficial/</v>
+      </c>
+      <c r="J93" t="str">
+        <v>https://www.facebook.com/Blood-incantation-508899805936788</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -2500,6 +3616,18 @@
       <c r="F94" t="str">
         <v>https://www.youtube.com/watch?v=JVF6e_LSO2k</v>
       </c>
+      <c r="G94" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174ceb758e41a24c01b787251dc</v>
+      </c>
+      <c r="H94" t="str">
+        <v>https://open.spotify.com/artist/6n5DUGtIWYMurrtVt7IdZr</v>
+      </c>
+      <c r="I94" t="str">
+        <v>https://www.instagram.com/elwood_stray/</v>
+      </c>
+      <c r="J94" t="str">
+        <v>https://www.facebook.com/elwoodstrayband</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -2520,6 +3648,18 @@
       <c r="F95" t="str">
         <v>https://www.youtube.com/watch?v=yY6mJg4b_rA</v>
       </c>
+      <c r="G95" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517426139a78b669ae67aacde9f3</v>
+      </c>
+      <c r="H95" t="str">
+        <v>https://open.spotify.com/artist/7jxJ25p0pPjk0MStloN6o6</v>
+      </c>
+      <c r="I95" t="str">
+        <v>https://www.instagram.com/blindguardian/</v>
+      </c>
+      <c r="J95" t="str">
+        <v>https://www.facebook.com/blindguardian</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -2540,6 +3680,18 @@
       <c r="F96" t="str">
         <v>https://www.youtube.com/watch?v=ggyC0FOiN1Q</v>
       </c>
+      <c r="G96" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051749ad0af7fa3272c5d1197c277</v>
+      </c>
+      <c r="H96" t="str">
+        <v>https://open.spotify.com/artist/3OpqU68JpZlzvjAJj3B2Da</v>
+      </c>
+      <c r="I96" t="str">
+        <v>https://www.instagram.com/alestormofficial/</v>
+      </c>
+      <c r="J96" t="str">
+        <v>https://www.facebook.com/alestormband</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -2560,6 +3712,18 @@
       <c r="F97" t="str">
         <v>https://www.youtube.com/watch?v=F0f5i1vK760</v>
       </c>
+      <c r="G97" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051747d38cff2be55d8e1f06896d0</v>
+      </c>
+      <c r="H97" t="str">
+        <v>https://open.spotify.com/artist/4B2Iosqk1yAbGbx08My1fM</v>
+      </c>
+      <c r="I97" t="str">
+        <v/>
+      </c>
+      <c r="J97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -2580,6 +3744,18 @@
       <c r="F98" t="str">
         <v>https://www.youtube.com/watch?v=gyL8pHR2UPk</v>
       </c>
+      <c r="G98" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174ac5e45658534c13cda7aa881</v>
+      </c>
+      <c r="H98" t="str">
+        <v>https://open.spotify.com/artist/18jTFcgHRRYHdwdof1MDZw</v>
+      </c>
+      <c r="I98" t="str">
+        <v>https://www.instagram.com/thundermother/</v>
+      </c>
+      <c r="J98" t="str">
+        <v>https://www.facebook.com/thundermother</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -2600,6 +3776,18 @@
       <c r="F99" t="str">
         <v>https://www.youtube.com/watch?v=l47At7wrhyI</v>
       </c>
+      <c r="G99" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174ca9e1ddb61172c1b9672567a</v>
+      </c>
+      <c r="H99" t="str">
+        <v>https://open.spotify.com/artist/0zfT626RwO6zN3RDYeRit5</v>
+      </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
+      <c r="J99" t="str">
+        <v>https://www.facebook.com/blacklabelsociety</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -2620,6 +3808,18 @@
       <c r="F100" t="str">
         <v>https://www.youtube.com/watch?v=QrpI-1TmOqM</v>
       </c>
+      <c r="G100" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174b283678ed69bc98f2f637ad8</v>
+      </c>
+      <c r="H100" t="str">
+        <v>https://open.spotify.com/artist/24Oiw7BlvO1BETecDLJt6m</v>
+      </c>
+      <c r="I100" t="str">
+        <v>https://www.instagram.com/slaughtertoprevailband/</v>
+      </c>
+      <c r="J100" t="str">
+        <v>https://www.facebook.com/slaughtertoprevailrus</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -2640,6 +3840,18 @@
       <c r="F101" t="str">
         <v>https://www.youtube.com/watch?v=ZmB5Pqv2gWE</v>
       </c>
+      <c r="G101" t="str">
+        <v/>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v>https://www.instagram.com/salduieofficial/</v>
+      </c>
+      <c r="J101" t="str">
+        <v>https://www.facebook.com/SalduieOficial</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -2660,6 +3872,18 @@
       <c r="F102" t="str">
         <v>https://www.youtube.com/watch?v=nnsTQq_8mR8</v>
       </c>
+      <c r="G102" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517411072a5adb75af0738e5fb41</v>
+      </c>
+      <c r="H102" t="str">
+        <v>https://open.spotify.com/artist/6Wl6VXLasmiON3BDiha6e1</v>
+      </c>
+      <c r="I102" t="str">
+        <v>https://www.instagram.com/tailgunnerhq/</v>
+      </c>
+      <c r="J102" t="str">
+        <v>https://www.facebook.com/tailgunnerhq</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -2680,6 +3904,18 @@
       <c r="F103" t="str">
         <v>https://www.youtube.com/watch?v=Y5SpGQMoaUU</v>
       </c>
+      <c r="G103" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174ff61b86e734b5bdbd2d8eb25</v>
+      </c>
+      <c r="H103" t="str">
+        <v>https://open.spotify.com/artist/7k29FbDq69ju2fe6zTskxY</v>
+      </c>
+      <c r="I103" t="str">
+        <v>https://www.instagram.com/orbitculture/</v>
+      </c>
+      <c r="J103" t="str">
+        <v>https://www.facebook.com/OrbitCulture</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -2700,6 +3936,18 @@
       <c r="F104" t="str">
         <v>https://www.youtube.com/watch/?v=xHNVK9NY4JE</v>
       </c>
+      <c r="G104" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517428ce3420531dadeaea4d8aef</v>
+      </c>
+      <c r="H104" t="str">
+        <v>https://open.spotify.com/artist/3N1B1g6JtIgd6ClRkzD4yT</v>
+      </c>
+      <c r="I104" t="str">
+        <v>https://www.instagram.com/thisissavatage/</v>
+      </c>
+      <c r="J104" t="str">
+        <v>https://www.facebook.com/savatage</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -2720,6 +3968,18 @@
       <c r="F105" t="str">
         <v>https://www.youtube.com/watch?v=c7Z8Ww1EmMk</v>
       </c>
+      <c r="G105" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517442b136165ba6ce25d2c1ebdc</v>
+      </c>
+      <c r="H105" t="str">
+        <v>https://open.spotify.com/artist/6JW8wliOEwaDZ231ZY7cf4</v>
+      </c>
+      <c r="I105" t="str">
+        <v>https://www.instagram.com/sepultura/</v>
+      </c>
+      <c r="J105" t="str">
+        <v>https://www.facebook.com/sepultura</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -2740,6 +4000,18 @@
       <c r="F106" t="str">
         <v>https://www.youtube.com/watch?v=ycFGTB04mO0</v>
       </c>
+      <c r="G106" t="str">
+        <v/>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
+      <c r="J106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -2760,6 +4032,18 @@
       <c r="F107" t="str">
         <v>https://www.youtube.com/playlist?list=OLAK5uy_l9fRGqB0eRiw0WBkqiKQ3nEV5ezIc87qY</v>
       </c>
+      <c r="G107" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174cdcfff294626def3c5cb85b9</v>
+      </c>
+      <c r="H107" t="str">
+        <v>https://open.spotify.com/artist/0c44C54LrAHha0u92agfHM</v>
+      </c>
+      <c r="I107" t="str">
+        <v>https://www.instagram.com/killusband/</v>
+      </c>
+      <c r="J107" t="str">
+        <v>https://www.facebook.com/Killusband</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -2780,6 +4064,18 @@
       <c r="F108" t="str">
         <v>https://www.youtube.com/c/HadadanzaOficial/videos</v>
       </c>
+      <c r="G108" t="str">
+        <v/>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v/>
+      </c>
+      <c r="J108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -2800,6 +4096,18 @@
       <c r="F109" t="str">
         <v>https://www.heaviestofart.com/post/album-to-watch-for-signs-of-the-swarm-amongst-the-low-empty</v>
       </c>
+      <c r="G109" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743d8cd968fe05c1d3825b896d</v>
+      </c>
+      <c r="H109" t="str">
+        <v>https://open.spotify.com/artist/0yxJx8OEyDfd7dzLsFuNrS</v>
+      </c>
+      <c r="I109" t="str">
+        <v>https://www.instagram.com/signsoftheswarm/</v>
+      </c>
+      <c r="J109" t="str">
+        <v>https://www.facebook.com/signsoftheswarm</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -2820,6 +4128,18 @@
       <c r="F110" t="str">
         <v>https://www.youtube.com/hashtag/deathbats</v>
       </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
+      <c r="J110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -2840,6 +4160,18 @@
       <c r="F111" t="str">
         <v>https://www.youtube.com/watch?v=_UBlWbLTVSE</v>
       </c>
+      <c r="G111" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517443bdf2ead814b5374f92a118</v>
+      </c>
+      <c r="H111" t="str">
+        <v>https://open.spotify.com/artist/6JChzL9HQEspINhiTqSURd</v>
+      </c>
+      <c r="I111" t="str">
+        <v>https://www.instagram.com/chainedsaintofficial/</v>
+      </c>
+      <c r="J111" t="str">
+        <v>https://www.facebook.com/chainedsaint</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -2860,6 +4192,18 @@
       <c r="F112" t="str">
         <v>https://www.youtube.com/watch?v=i2SfKTf02gk</v>
       </c>
+      <c r="G112" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051745b104bd9ab98eff15f14daf8</v>
+      </c>
+      <c r="H112" t="str">
+        <v>https://open.spotify.com/artist/3CkwG7cwsw7hY8Hb3bzj6s</v>
+      </c>
+      <c r="I112" t="str">
+        <v>https://www.instagram.com/promkinks/</v>
+      </c>
+      <c r="J112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -2880,6 +4224,18 @@
       <c r="F113" t="str">
         <v>https://www.youtube.com/watch?v=7iJ7oj-dAVY</v>
       </c>
+      <c r="G113" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517448e3d9fdff3ef62439099d24</v>
+      </c>
+      <c r="H113" t="str">
+        <v>https://open.spotify.com/artist/18absyD7lQaXUDBXnyzU8M</v>
+      </c>
+      <c r="I113" t="str">
+        <v>https://www.instagram.com/mushroomheadofficial/</v>
+      </c>
+      <c r="J113" t="str">
+        <v>https://www.facebook.com/mushroomheadofficial</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -2900,6 +4256,18 @@
       <c r="F114" t="str">
         <v>https://www.youtube.com/watch?v=pBsVsLRSgfE</v>
       </c>
+      <c r="G114" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174473898d318f6958efb692c2f</v>
+      </c>
+      <c r="H114" t="str">
+        <v>https://open.spotify.com/artist/5EHvXKnNz78jkAVgTQLQ5O</v>
+      </c>
+      <c r="I114" t="str">
+        <v>https://www.instagram.com/darktranquillityofficial/</v>
+      </c>
+      <c r="J114" t="str">
+        <v>https://www.facebook.com/dtofficial</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -2920,6 +4288,18 @@
       <c r="F115" t="str">
         <v>https://www.youtube.com/watch?v=cJBmX5aU1DA</v>
       </c>
+      <c r="G115" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174c6790f344338cb196c00660d</v>
+      </c>
+      <c r="H115" t="str">
+        <v>https://open.spotify.com/artist/0DCw6lHkzh9t7f8Hb4Z0Sx</v>
+      </c>
+      <c r="I115" t="str">
+        <v>https://www.instagram.com/archenemyofficial/</v>
+      </c>
+      <c r="J115" t="str">
+        <v>https://www.facebook.com/archenemyofficial</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -2940,6 +4320,18 @@
       <c r="F116" t="str">
         <v>https://www.youtube.com/watch?v=Yk7noXH_9do</v>
       </c>
+      <c r="G116" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051744365a2ae1fd4c4c95c236563</v>
+      </c>
+      <c r="H116" t="str">
+        <v>https://open.spotify.com/artist/1UM5OPJuE5dGDgyPSNSAqH</v>
+      </c>
+      <c r="I116" t="str">
+        <v>https://www.instagram.com/lepokafolk/</v>
+      </c>
+      <c r="J116" t="str">
+        <v>https://www.facebook.com/lepokafolk</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -2960,6 +4352,18 @@
       <c r="F117" t="str">
         <v>https://www.youtube.com/watch?v=cHIA1JcBBZ4</v>
       </c>
+      <c r="G117" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517426ce4d13792697b06bed82a1</v>
+      </c>
+      <c r="H117" t="str">
+        <v>https://open.spotify.com/artist/0nV7SiEIVtPLTSJ6NwWDGj</v>
+      </c>
+      <c r="I117" t="str">
+        <v>https://www.instagram.com/creepercult/</v>
+      </c>
+      <c r="J117" t="str">
+        <v>https://www.facebook.com/creepercult</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -2980,6 +4384,18 @@
       <c r="F118" t="str">
         <v>https://www.youtube.com/watch?v=h4e40N3We-U</v>
       </c>
+      <c r="G118" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f9dc3a82b666097cf2f48031</v>
+      </c>
+      <c r="H118" t="str">
+        <v>https://open.spotify.com/artist/3qyg72RGnGdF521zMU02u9</v>
+      </c>
+      <c r="I118" t="str">
+        <v>https://www.instagram.com/northlane/</v>
+      </c>
+      <c r="J118" t="str">
+        <v>https://www.facebook.com/northlane</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -3000,6 +4416,18 @@
       <c r="F119" t="str">
         <v>https://www.youtube.com/watch?v=fG9F0IwwJeU</v>
       </c>
+      <c r="G119" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174e024531c06e7de54f84ea6fd</v>
+      </c>
+      <c r="H119" t="str">
+        <v>https://open.spotify.com/artist/6gZq1Q6bdOxsUPUG1TaFbF</v>
+      </c>
+      <c r="I119" t="str">
+        <v>https://www.instagram.com/godsmack/</v>
+      </c>
+      <c r="J119" t="str">
+        <v>https://www.facebook.com/Godsmack</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -3020,6 +4448,18 @@
       <c r="F120" t="str">
         <v>https://www.youtube.com/watch?v=KPlYOA8UMrs</v>
       </c>
+      <c r="G120" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051746dc569d5f616c2ccb08fd6e9</v>
+      </c>
+      <c r="H120" t="str">
+        <v>https://open.spotify.com/artist/7Lj8CmxeAuJ2c2I6YxA6AJ</v>
+      </c>
+      <c r="I120" t="str">
+        <v>https://www.instagram.com/dartagnan_official/</v>
+      </c>
+      <c r="J120" t="str">
+        <v>https://www.facebook.com/dartagnan.de</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -3040,6 +4480,18 @@
       <c r="F121" t="str">
         <v>https://www.youtube.com/watch?v=NSMn_Z_45CM</v>
       </c>
+      <c r="G121" t="str">
+        <v/>
+      </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
+      <c r="J121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -3060,6 +4512,18 @@
       <c r="F122" t="str">
         <v>https://www.youtube.com/watch?v=cg0BbHDZQ9Y</v>
       </c>
+      <c r="G122" t="str">
+        <v/>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
+      <c r="J122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -3080,6 +4544,18 @@
       <c r="F123" t="str">
         <v>https://www.youtube.com/watch?v=UzvtL6WFfk4</v>
       </c>
+      <c r="G123" t="str">
+        <v/>
+      </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v>https://www.instagram.com/injector_official/</v>
+      </c>
+      <c r="J123" t="str">
+        <v>https://www.facebook.com/InjectorThrash</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -3100,6 +4576,18 @@
       <c r="F124" t="str">
         <v>https://www.youtube.com/watch?v=IMqsA0G2uoI</v>
       </c>
+      <c r="G124" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616d00001e02d5d8417f6ba6e61e4444304b</v>
+      </c>
+      <c r="H124" t="str">
+        <v>https://open.spotify.com/artist/3n3jrBZETHY0ONCdKzbYeY</v>
+      </c>
+      <c r="I124" t="str">
+        <v>https://www.instagram.com/evoband/</v>
+      </c>
+      <c r="J124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -3120,6 +4608,18 @@
       <c r="F125" t="str">
         <v>https://www.youtube.com/watch?v=M8_wLm_5s_Y</v>
       </c>
+      <c r="G125" t="str">
+        <v/>
+      </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
+      <c r="J125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -3140,6 +4640,18 @@
       <c r="F126" t="str">
         <v>https://www.youtube.com/watch?v=Fz6qnMiu4LQ</v>
       </c>
+      <c r="G126" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174c38079b6ba9c4d5983d25ec8</v>
+      </c>
+      <c r="H126" t="str">
+        <v>https://open.spotify.com/artist/7rDC5oTEVCLYkVeaE7168p</v>
+      </c>
+      <c r="I126" t="str">
+        <v>https://www.instagram.com/bolu2death_official/</v>
+      </c>
+      <c r="J126" t="str">
+        <v>https://www.facebook.com/Bolu2death</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -3160,6 +4672,18 @@
       <c r="F127" t="str">
         <v>https://www.youtube.com/watch?v=mJ47ISNx0lE</v>
       </c>
+      <c r="G127" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174d822b3210878eeaf64ae5bf4</v>
+      </c>
+      <c r="H127" t="str">
+        <v>https://open.spotify.com/artist/4QnuZOyl4C9d1keyOZXJ21</v>
+      </c>
+      <c r="I127" t="str">
+        <v>https://www.instagram.com/futurepalaceofficial/</v>
+      </c>
+      <c r="J127" t="str">
+        <v>https://www.facebook.com/futurepalace</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -3180,6 +4704,18 @@
       <c r="F128" t="str">
         <v>https://www.youtube.com/watch?v=8nRdOSVX2VI</v>
       </c>
+      <c r="G128" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051744f5370fae0e1fb6cd2f88d53</v>
+      </c>
+      <c r="H128" t="str">
+        <v>https://open.spotify.com/artist/0pFExKST1wGbE6DBSNK6ox</v>
+      </c>
+      <c r="I128" t="str">
+        <v/>
+      </c>
+      <c r="J128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -3200,6 +4736,18 @@
       <c r="F129" t="str">
         <v>https://www.youtube.com/watch?v=qnLunQEcMn0</v>
       </c>
+      <c r="G129" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051745c3bd919d1344a738af14136</v>
+      </c>
+      <c r="H129" t="str">
+        <v>https://open.spotify.com/artist/57ylwQTnFnIhJh4nu4rxCs</v>
+      </c>
+      <c r="I129" t="str">
+        <v>https://www.instagram.com/inflames/</v>
+      </c>
+      <c r="J129" t="str">
+        <v>https://www.facebook.com/inflames</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -3220,6 +4768,18 @@
       <c r="F130" t="str">
         <v>https://www.youtube.com/@DarkMoorofficial/videos</v>
       </c>
+      <c r="G130" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741c7310cc250682db4e9748aa</v>
+      </c>
+      <c r="H130" t="str">
+        <v>https://open.spotify.com/artist/0YWKRTzA4kBceGwjywtMkh</v>
+      </c>
+      <c r="I130" t="str">
+        <v/>
+      </c>
+      <c r="J130" t="str">
+        <v>https://www.facebook.com/official.darkmoor?sid=6286</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -3240,6 +4800,18 @@
       <c r="F131" t="str">
         <v>https://www.youtube.com/watch?v=Oc-p6U_uA3E</v>
       </c>
+      <c r="G131" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174516bbe592d49e78c6395d2c7</v>
+      </c>
+      <c r="H131" t="str">
+        <v>https://open.spotify.com/artist/23QdQy5SrwG2X1mvnMzYeP</v>
+      </c>
+      <c r="I131" t="str">
+        <v>https://www.instagram.com/chez_kane/</v>
+      </c>
+      <c r="J131" t="str">
+        <v>https://www.facebook.com/ChezKaneVocalist</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -3260,6 +4832,18 @@
       <c r="F132" t="str">
         <v>https://www.youtube.com/watch?v=r9lhoupFbKw</v>
       </c>
+      <c r="G132" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f915d1cbe39bb89e25851d27</v>
+      </c>
+      <c r="H132" t="str">
+        <v>https://open.spotify.com/artist/7Fh1k3NlvVj1Oj6kpfQf9f</v>
+      </c>
+      <c r="I132" t="str">
+        <v>https://www.instagram.com/thebaboonshowofficial/</v>
+      </c>
+      <c r="J132" t="str">
+        <v>https://www.facebook.com/thebaboonshow</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -3280,6 +4864,18 @@
       <c r="F133" t="str">
         <v>https://www.youtube.com/watch?v=kG4uQ6Tk7fY</v>
       </c>
+      <c r="G133" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051744733f393ad04f47b31edaadb</v>
+      </c>
+      <c r="H133" t="str">
+        <v>https://open.spotify.com/artist/1O8CSXsPwEqxcoBE360PPO</v>
+      </c>
+      <c r="I133" t="str">
+        <v>https://www.instagram.com/stratovariusofficial/</v>
+      </c>
+      <c r="J133" t="str">
+        <v>https://www.facebook.com/stratovarius</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -3300,6 +4896,18 @@
       <c r="F134" t="str">
         <v>https://www.youtube.com/watch?v=Ow3K7MopO2k</v>
       </c>
+      <c r="G134" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741804c4301093d03104dee1ab</v>
+      </c>
+      <c r="H134" t="str">
+        <v>https://open.spotify.com/artist/0qqry49HR1XCCzn7NFHzMN</v>
+      </c>
+      <c r="I134" t="str">
+        <v/>
+      </c>
+      <c r="J134" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -3320,6 +4928,18 @@
       <c r="F135" t="str">
         <v>https://www.youtube.com/watch?v=iwbUG29dDd4</v>
       </c>
+      <c r="G135" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f0ec514bb1af4546a9f63f24</v>
+      </c>
+      <c r="H135" t="str">
+        <v>https://open.spotify.com/artist/0y43lCvntQtyFlhCABGb0T</v>
+      </c>
+      <c r="I135" t="str">
+        <v>https://www.instagram.com/wingsofsteelband/</v>
+      </c>
+      <c r="J135" t="str">
+        <v>https://www.facebook.com/OfficialWingsofSteel</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -3340,6 +4960,18 @@
       <c r="F136" t="str">
         <v>https://www.youtube.com/watch?v=L8sLjb3nGGM</v>
       </c>
+      <c r="G136" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174df662920ed5206484971ffb6</v>
+      </c>
+      <c r="H136" t="str">
+        <v>https://open.spotify.com/artist/2yoaZdFiI362NRtFPF3YTN</v>
+      </c>
+      <c r="I136" t="str">
+        <v>https://www.instagram.com/againstmyselfofficial/</v>
+      </c>
+      <c r="J136" t="str">
+        <v>https://www.facebook.com/pages/AGAINST-MYSELF/203937595534</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -3360,6 +4992,18 @@
       <c r="F137" t="str">
         <v>https://www.youtube.com/watch?v=Ut1AcpPPOS0</v>
       </c>
+      <c r="G137" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517409bf6e7ed2ae0cd614ca19e7</v>
+      </c>
+      <c r="H137" t="str">
+        <v>https://open.spotify.com/artist/58d50jBQXhOetEGuSBgu64</v>
+      </c>
+      <c r="I137" t="str">
+        <v>https://www.instagram.com/employedtoserve/</v>
+      </c>
+      <c r="J137" t="str">
+        <v>https://www.facebook.com/employedtoserve</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -3380,6 +5024,18 @@
       <c r="F138" t="str">
         <v>https://www.youtube.com/watch?v=OdtC4CsbydA</v>
       </c>
+      <c r="G138" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174da10f52aaa76416bf04fff32</v>
+      </c>
+      <c r="H138" t="str">
+        <v>https://open.spotify.com/artist/1Ohy5ahjQyXh0TTPH5WV3Y</v>
+      </c>
+      <c r="I138" t="str">
+        <v>https://www.instagram.com/daeriaoficial/</v>
+      </c>
+      <c r="J138" t="str">
+        <v>https://www.facebook.com/DAERIAOFICIAL</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -3400,6 +5056,18 @@
       <c r="F139" t="str">
         <v>https://www.youtube.com/watch?v=j51TIMwxriI</v>
       </c>
+      <c r="G139" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517452b01b011dd2cb45ccc5a4c2</v>
+      </c>
+      <c r="H139" t="str">
+        <v>https://open.spotify.com/artist/7vDMECFl5RLKV0QywC1pmX</v>
+      </c>
+      <c r="I139" t="str">
+        <v>https://www.instagram.com/mind_driller/</v>
+      </c>
+      <c r="J139" t="str">
+        <v>https://www.facebook.com/MindDriller</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -3420,6 +5088,18 @@
       <c r="F140" t="str">
         <v>https://www.youtube.com/watch?v=bV0FxNR0yhQ</v>
       </c>
+      <c r="G140" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051746b134287e3095d2c84b7932a</v>
+      </c>
+      <c r="H140" t="str">
+        <v>https://open.spotify.com/artist/0LyfQWJT6nXafLPZqxe9Of</v>
+      </c>
+      <c r="I140" t="str">
+        <v/>
+      </c>
+      <c r="J140" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -3440,6 +5120,18 @@
       <c r="F141" t="str">
         <v>https://www.youtube.com/watch?v=O0dlwcJL-aE</v>
       </c>
+      <c r="G141" t="str">
+        <v/>
+      </c>
+      <c r="H141" t="str">
+        <v/>
+      </c>
+      <c r="I141" t="str">
+        <v/>
+      </c>
+      <c r="J141" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -3460,6 +5152,18 @@
       <c r="F142" t="str">
         <v>https://www.youtube.com/watch?v=-l-OiglL460</v>
       </c>
+      <c r="G142" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174afad0c8cde6dbb7de81c77ab</v>
+      </c>
+      <c r="H142" t="str">
+        <v>https://open.spotify.com/artist/2K3GorTixXKAiwe2t9lO89</v>
+      </c>
+      <c r="I142" t="str">
+        <v>https://www.instagram.com/deicideofficial/</v>
+      </c>
+      <c r="J142" t="str">
+        <v>https://www.facebook.com/OfficialDeicide</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -3480,6 +5184,18 @@
       <c r="F143" t="str">
         <v>https://www.youtube.com/watch?v=LZ6YKR6K_zU</v>
       </c>
+      <c r="G143" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051747d6b878498239115a09316d3</v>
+      </c>
+      <c r="H143" t="str">
+        <v>https://open.spotify.com/artist/4pQN0GB0fNEEOfQCaWotsY</v>
+      </c>
+      <c r="I143" t="str">
+        <v>https://www.instagram.com/helloweenofficial/</v>
+      </c>
+      <c r="J143" t="str">
+        <v>https://www.facebook.com/helloweenofficial</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -3500,6 +5216,18 @@
       <c r="F144" t="str">
         <v>https://www.youtube.com/watch?v=l_9LU_Qrlfs</v>
       </c>
+      <c r="G144" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051748a34aa0363ad8133950ab334</v>
+      </c>
+      <c r="H144" t="str">
+        <v>https://open.spotify.com/artist/4c0CmlfLtocEfBgq5w289e</v>
+      </c>
+      <c r="I144" t="str">
+        <v/>
+      </c>
+      <c r="J144" t="str">
+        <v>https://www.facebook.com/profile.php?id=100063786306898</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -3520,6 +5248,18 @@
       <c r="F145" t="str">
         <v>https://www.youtube.com/watch?v=Nf_LAdo_oiE</v>
       </c>
+      <c r="G145" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743a98c334ce4cd9c8db848fa0</v>
+      </c>
+      <c r="H145" t="str">
+        <v>https://open.spotify.com/artist/2VFxoCJQPfQauZujESPjQK</v>
+      </c>
+      <c r="I145" t="str">
+        <v>https://www.instagram.com/eihwar.music/</v>
+      </c>
+      <c r="J145" t="str">
+        <v>https://www.facebook.com/eihwar.music</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -3540,6 +5280,18 @@
       <c r="F146" t="str">
         <v>https://www.youtube.com/watch?v=TTkZt8r2lko</v>
       </c>
+      <c r="G146" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517424b3a97c9907e54b66852aeb</v>
+      </c>
+      <c r="H146" t="str">
+        <v>https://open.spotify.com/artist/4sy5qWfwUwpGYBnCKnwfcW</v>
+      </c>
+      <c r="I146" t="str">
+        <v>https://www.instagram.com/heavenshallburnofficial/</v>
+      </c>
+      <c r="J146" t="str">
+        <v>https://www.facebook.com/officialheavenshallburn</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -3560,6 +5312,18 @@
       <c r="F147" t="str">
         <v>https://www.youtube.com/watch?v=UJaW2Z5DxS8</v>
       </c>
+      <c r="G147" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741bab293f26bfa4001d6c57a7</v>
+      </c>
+      <c r="H147" t="str">
+        <v>https://open.spotify.com/artist/3hMTlMf2UGZTeP6DSUUl09</v>
+      </c>
+      <c r="I147" t="str">
+        <v>https://www.instagram.com/warcryoficial/</v>
+      </c>
+      <c r="J147" t="str">
+        <v>https://www.facebook.com/WarCryOficial</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -3580,6 +5344,18 @@
       <c r="F148" t="str">
         <v>https://www.youtube.com/watch?v=eiEl-mbPpj4</v>
       </c>
+      <c r="G148" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749b2d4451c09ad404176ee1cb</v>
+      </c>
+      <c r="H148" t="str">
+        <v>https://open.spotify.com/artist/3HsJjtbbQkhb2pcdRXmZbk</v>
+      </c>
+      <c r="I148" t="str">
+        <v>https://www.instagram.com/death_and_legacy/</v>
+      </c>
+      <c r="J148" t="str">
+        <v>https://www.facebook.com/deathandlegacy</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -3600,6 +5376,18 @@
       <c r="F149" t="str">
         <v>https://www.youtube.com/watch?v=WNmUqMR_hkE</v>
       </c>
+      <c r="G149" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741c111d5c2a504c62911fe99b</v>
+      </c>
+      <c r="H149" t="str">
+        <v>https://open.spotify.com/artist/6QpMNQzCXdUFCTxE9u4xAc</v>
+      </c>
+      <c r="I149" t="str">
+        <v/>
+      </c>
+      <c r="J149" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -3620,6 +5408,18 @@
       <c r="F150" t="str">
         <v>https://www.youtube.com/watch?v=I9n1_vRYYoc</v>
       </c>
+      <c r="G150" t="str">
+        <v/>
+      </c>
+      <c r="H150" t="str">
+        <v/>
+      </c>
+      <c r="I150" t="str">
+        <v/>
+      </c>
+      <c r="J150" t="str">
+        <v>https://www.facebook.com/pages/Hardline/113309705346323</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -3640,6 +5440,18 @@
       <c r="F151" t="str">
         <v>https://www.youtube.com/watch?v=LElq1WEBQRY</v>
       </c>
+      <c r="G151" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174ff6c889753c279dcf636a8ad</v>
+      </c>
+      <c r="H151" t="str">
+        <v>https://open.spotify.com/artist/28dpy0DQotTkBXcTlniQii</v>
+      </c>
+      <c r="I151" t="str">
+        <v>https://www.instagram.com/ten56hq/</v>
+      </c>
+      <c r="J151" t="str">
+        <v>https://www.facebook.com/ten56hq</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -3660,6 +5472,18 @@
       <c r="F152" t="str">
         <v>https://www.youtube.com/watch?v=1vwJfeXJRmQ</v>
       </c>
+      <c r="G152" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174f8b894798a13b12187b96078</v>
+      </c>
+      <c r="H152" t="str">
+        <v>https://open.spotify.com/artist/4LNvQot1CDYC3kWGW144XC</v>
+      </c>
+      <c r="I152" t="str">
+        <v>https://www.instagram.com/half_me.mp3/</v>
+      </c>
+      <c r="J152" t="str">
+        <v>https://www.facebook.com/halfmeband</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -3680,6 +5504,18 @@
       <c r="F153" t="str">
         <v>https://www.youtube.com/watch?v=amj49T04FCQ</v>
       </c>
+      <c r="G153" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517411facedf8b7d7902c85f291d</v>
+      </c>
+      <c r="H153" t="str">
+        <v>https://open.spotify.com/artist/2bfK6ltXa60B2egnErJvlO</v>
+      </c>
+      <c r="I153" t="str">
+        <v>https://www.instagram.com/cabalcph/</v>
+      </c>
+      <c r="J153" t="str">
+        <v>https://www.facebook.com/cabalcph</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -3700,6 +5536,18 @@
       <c r="F154" t="str">
         <v>https://www.youtube.com/watch?v=k5lGswUaBgo</v>
       </c>
+      <c r="G154" t="str">
+        <v/>
+      </c>
+      <c r="H154" t="str">
+        <v/>
+      </c>
+      <c r="I154" t="str">
+        <v/>
+      </c>
+      <c r="J154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -3720,6 +5568,18 @@
       <c r="F155" t="str">
         <v>https://www.youtube.com/watch?v=2TzFm9u2U9Y</v>
       </c>
+      <c r="G155" t="str">
+        <v>https://i.scdn.co/image/2526875cb953ea6d353eb5e8787647f9a3cdf0c5</v>
+      </c>
+      <c r="H155" t="str">
+        <v>https://open.spotify.com/artist/2VoP4JXyxNPIoYAFdB5ssQ</v>
+      </c>
+      <c r="I155" t="str">
+        <v/>
+      </c>
+      <c r="J155" t="str">
+        <v>https://www.facebook.com/Uli-Jon-Roth-403059233077097</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -3740,6 +5600,18 @@
       <c r="F156" t="str">
         <v>https://www.youtube.com/watch?v=p4vW7h443kE</v>
       </c>
+      <c r="G156" t="str">
+        <v/>
+      </c>
+      <c r="H156" t="str">
+        <v/>
+      </c>
+      <c r="I156" t="str">
+        <v/>
+      </c>
+      <c r="J156" t="str">
+        <v>https://www.facebook.com/secretsphere</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -3760,6 +5632,18 @@
       <c r="F157" t="str">
         <v>https://www.youtube.com/watch?v=N65sJitF7q0</v>
       </c>
+      <c r="G157" t="str">
+        <v/>
+      </c>
+      <c r="H157" t="str">
+        <v/>
+      </c>
+      <c r="I157" t="str">
+        <v/>
+      </c>
+      <c r="J157" t="str">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -3780,6 +5664,18 @@
       <c r="F158" t="str">
         <v>https://www.youtube.com/watch?v=P9C9Y_MeklA</v>
       </c>
+      <c r="G158" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517405e5c32722b5ae52c4f8376b</v>
+      </c>
+      <c r="H158" t="str">
+        <v>https://open.spotify.com/artist/0WodW8A13GujZQyAUynr82</v>
+      </c>
+      <c r="I158" t="str">
+        <v>https://www.instagram.com/furyoffic1al/</v>
+      </c>
+      <c r="J158" t="str">
+        <v>https://www.facebook.com/furyofficial</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -3800,6 +5696,18 @@
       <c r="F159" t="str">
         <v>https://www.youtube.com/watch?v=qXgUq6P57fE</v>
       </c>
+      <c r="G159" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab67616d00001e02aa45ec1a8328e81af490b4a4</v>
+      </c>
+      <c r="H159" t="str">
+        <v>https://open.spotify.com/artist/0nKiNlJFtcGhZXZlNkOstJ</v>
+      </c>
+      <c r="I159" t="str">
+        <v/>
+      </c>
+      <c r="J159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -3820,6 +5728,18 @@
       <c r="F160" t="str">
         <v>https://www.youtube.com/watch?v=wXW5Zl2_Jxs</v>
       </c>
+      <c r="G160" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517461f85b0265f8496c97063a38</v>
+      </c>
+      <c r="H160" t="str">
+        <v>https://open.spotify.com/artist/1t20wYnTiAT0Bs7H1hv9Wt</v>
+      </c>
+      <c r="I160" t="str">
+        <v>https://www.instagram.com/iameden/</v>
+      </c>
+      <c r="J160" t="str">
+        <v>https://www.facebook.com/iameden</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -3840,6 +5760,18 @@
       <c r="F161" t="str">
         <v>https://www.youtube.com/watch?v=269_4m8lC1c</v>
       </c>
+      <c r="G161" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174386dd5a6a0a787b2ef167702</v>
+      </c>
+      <c r="H161" t="str">
+        <v>https://open.spotify.com/artist/57b3sKD9pGilMb2QlMqArq</v>
+      </c>
+      <c r="I161" t="str">
+        <v/>
+      </c>
+      <c r="J161" t="str">
+        <v>https://www.facebook.com/OfficialHardcoreSuperstar</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -3860,6 +5792,18 @@
       <c r="F162" t="str">
         <v>https://www.youtube.com/watch?v=F_f-z7-p2lA</v>
       </c>
+      <c r="G162" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051745cba8908ce1e2e767f9e7b3c</v>
+      </c>
+      <c r="H162" t="str">
+        <v>https://open.spotify.com/artist/0l4rDRLl3nXp2qfQROmrme</v>
+      </c>
+      <c r="I162" t="str">
+        <v>https://www.instagram.com/savaged_official/</v>
+      </c>
+      <c r="J162" t="str">
+        <v>https://www.facebook.com/savagedheavy</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -3880,6 +5824,18 @@
       <c r="F163" t="str">
         <v>https://www.youtube.com/watch?v=uK1zYlqR5W4</v>
       </c>
+      <c r="G163" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517403cb77f96e45ca6fdb18debe</v>
+      </c>
+      <c r="H163" t="str">
+        <v>https://open.spotify.com/artist/0NmYchKQ8JIR9QHYJA0FRe</v>
+      </c>
+      <c r="I163" t="str">
+        <v>https://www.instagram.com/overkillofficial/</v>
+      </c>
+      <c r="J163" t="str">
+        <v>https://www.facebook.com/OverkillWreckingCrew</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -3900,6 +5856,18 @@
       <c r="F164" t="str">
         <v>https://www.youtube.com/watch?v=yYn9N56eSxs</v>
       </c>
+      <c r="G164" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051747f48b37e97817f9965ad2cfd</v>
+      </c>
+      <c r="H164" t="str">
+        <v>https://open.spotify.com/artist/78LVpk0xhPtf6ptfZjaw5h</v>
+      </c>
+      <c r="I164" t="str">
+        <v/>
+      </c>
+      <c r="J164" t="str">
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -3920,6 +5888,18 @@
       <c r="F165" t="str">
         <v>https://www.youtube.com/watch?v=Vl3rPrcSg9Y</v>
       </c>
+      <c r="G165" t="str">
+        <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741bf64d84a5f034bee6855e8e</v>
+      </c>
+      <c r="H165" t="str">
+        <v>https://open.spotify.com/artist/5mPSuVF1DeqeY3SpIt2f00</v>
+      </c>
+      <c r="I165" t="str">
+        <v>https://www.instagram.com/inductionofficial/</v>
+      </c>
+      <c r="J165" t="str">
+        <v>https://www.facebook.com/inductionofficial</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -3940,6 +5920,18 @@
       <c r="F166" t="str">
         <v>https://www.youtube.com/watch?v=Kz4M0XF8L8s</v>
       </c>
+      <c r="G166" t="str">
+        <v/>
+      </c>
+      <c r="H166" t="str">
+        <v/>
+      </c>
+      <c r="I166" t="str">
+        <v/>
+      </c>
+      <c r="J166" t="str">
+        <v>https://www.facebook.com/ArsAmandiRock</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -3960,6 +5952,18 @@
       <c r="F167" t="str">
         <v>https://www.youtube.com/watch?v=YwL3i_9oFmQ</v>
       </c>
+      <c r="G167" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174a240a99d353796c334cae25a</v>
+      </c>
+      <c r="H167" t="str">
+        <v>https://open.spotify.com/artist/6uG9Od49dC2XZyHVJS9aEZ</v>
+      </c>
+      <c r="I167" t="str">
+        <v>https://www.instagram.com/bloodstain.official/</v>
+      </c>
+      <c r="J167" t="str">
+        <v>https://www.facebook.com/profile.php?id=61555780541728</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -3980,6 +5984,18 @@
       <c r="F168" t="str">
         <v>https://www.youtube.com/watch?v=wBwA4wz_G98</v>
       </c>
+      <c r="G168" t="str">
+        <v/>
+      </c>
+      <c r="H168" t="str">
+        <v/>
+      </c>
+      <c r="I168" t="str">
+        <v/>
+      </c>
+      <c r="J168" t="str">
+        <v>https://www.facebook.com/thepoodles</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -4000,6 +6016,18 @@
       <c r="F169" t="str">
         <v>https://www.youtube.com/watch?v=4kO2vY14csw</v>
       </c>
+      <c r="G169" t="str">
+        <v/>
+      </c>
+      <c r="H169" t="str">
+        <v/>
+      </c>
+      <c r="I169" t="str">
+        <v/>
+      </c>
+      <c r="J169" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -4020,6 +6048,18 @@
       <c r="F170" t="str">
         <v>https://www.youtube.com/watch?v=gT8jV7C2L0o</v>
       </c>
+      <c r="G170" t="str">
+        <v/>
+      </c>
+      <c r="H170" t="str">
+        <v/>
+      </c>
+      <c r="I170" t="str">
+        <v/>
+      </c>
+      <c r="J170" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -4040,6 +6080,18 @@
       <c r="F171" t="str">
         <v>https://www.youtube.com/watch?v=mE98Zc21lB0</v>
       </c>
+      <c r="G171" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174510624ce3ecb6e7d0bdb7d09</v>
+      </c>
+      <c r="H171" t="str">
+        <v>https://open.spotify.com/artist/1mnVffOIDOAeCLxjZ1jOQj</v>
+      </c>
+      <c r="I171" t="str">
+        <v>https://www.instagram.com/odc_official_/</v>
+      </c>
+      <c r="J171" t="str">
+        <v>https://www.facebook.com/ODCOfficiel</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -4060,6 +6112,18 @@
       <c r="F172" t="str">
         <v>https://www.youtube.com/watch?v=vV9W5aP-e_4</v>
       </c>
+      <c r="G172" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051740f0c71fd8ca7477c0a7de478</v>
+      </c>
+      <c r="H172" t="str">
+        <v>https://open.spotify.com/artist/5GLeyUhj8B8f5pJxqZllKl</v>
+      </c>
+      <c r="I172" t="str">
+        <v>https://www.instagram.com/DoroMetalQueen/</v>
+      </c>
+      <c r="J172" t="str">
+        <v>https://www.facebook.com/DoroPeschOfficialGerman</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -4080,6 +6144,18 @@
       <c r="F173" t="str">
         <v>https://www.youtube.com/watch?v=17X2e_O8Jzo</v>
       </c>
+      <c r="G173" t="str">
+        <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743f0cc19264baa64fb8b7fbd7</v>
+      </c>
+      <c r="H173" t="str">
+        <v>https://open.spotify.com/artist/6e8DrBevl7KCm0Kfse6fvB</v>
+      </c>
+      <c r="I173" t="str">
+        <v>https://www.instagram.com/bullet_official/</v>
+      </c>
+      <c r="J173" t="str">
+        <v>https://www.facebook.com/bulletband</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -4100,10 +6176,22 @@
       <c r="F174" t="str">
         <v>https://www.youtube.com/watch?v=p4vW7h443kE</v>
       </c>
+      <c r="G174" t="str">
+        <v/>
+      </c>
+      <c r="H174" t="str">
+        <v/>
+      </c>
+      <c r="I174" t="str">
+        <v/>
+      </c>
+      <c r="J174" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J174"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Completada revisión global de bios en español de 500 caracteres y corrección de URLs de YouTube inválidas/rotas para todas las bandas
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -798,7 +798,7 @@
         <v>God Complex se crearon en 2017 y rápidamente se consolidaron como una de las formaciones de metalcore más feroz del Reino Unido. Tras debutar en 2021, hicieron una breve pausa para rearmarse y regresar más brutales y rabiosos que nunca coqueteando también con el mathcore y deathcore en sus singles más recientes 👊  Tras arrasar en su regreso por Londres y su natal Liverpool, los tendremos en el Resurrection Fest listos para desatar el caos en, valga la redundancia, el Chaos Stage, que estarán golpeando con riffs gordos y groove hiperviolento el miércoles 1 de julio 🤘Violencia sonora sin filtro</v>
       </c>
       <c r="F6" t="str">
-        <v>https://www.youtube.com/watch?v=uBU8\_O8G9IM</v>
+        <v>https://www.youtube.com/watch?v=uBU8_O8G9IM</v>
       </c>
       <c r="G6" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174f4955c9f0802e7974d78c0c5</v>
@@ -990,7 +990,7 @@
         <v>CardiaC llevan en las trincheras del hardcore, metal y rock europeo desde el año 2000. Se formaron en Suiza, aunque las raíces de su vocalista, Ricardo, están en Madrid. De ahí nace la iniciativa de que sus canciones sean en castellano, idioma en el que canalizan toda su rabia, ideas y experiencia a través de un estilo fuertemente influido por el hardcore neoyorkino 🔥  Tras recorrer multitud de países europeos, además de pasar por Estados Unidos, Rusia o Cuba acompañando a bandas como Madball, Terror, Cypress Hill, Soziedad Alkohólika, Sepultura o Limp Bizkit, la banda pisará el Desert Stage del Resu el primer día de festi, miércoles 1 de julio, para demostrarnos por qué su groove es tan infeccioso 🤘</v>
       </c>
       <c r="F12" t="str">
-        <v>https://www.youtube.com/watch?v=l-Rv5riBvc8\&amp;t=3s</v>
+        <v>https://www.youtube.com/watch?v=l-Rv5riBvc8&amp;t=3s</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -1022,7 +1022,7 @@
         <v>La banda dublinesa, conocida por su enfoque en el folklore tradicional irlandés, viene directa de las calles, de tocar delante de transeúntes mostrando a todxs su estilo celebratorio con dinámicas derivadas del rock y del metal progresivo que van de lo contemplativo a la explosión en cuestión de segundos ⚡️  Viveiro será el punto ideal de reunión entre dos culturas hermanas en herencia como son la gallega y la irlandesa. ¡Será una cita imperdible para festejar la música en directo! Y, ¡OJO! ¡Vendrán con su nuevo y bestial disco "Pull Like A Dog" bajo el brazo! 🤘LET'S GO! 🙌</v>
       </c>
       <c r="F13" t="str">
-        <v>https://www.youtube.com/watch?v=MfDZlUD\_1WU</v>
+        <v>https://www.youtube.com/watch?v=MfDZlUD_1WU</v>
       </c>
       <c r="G13" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741d205bf1c3d1017658dafc87</v>
@@ -1086,7 +1086,7 @@
         <v>Reconocidos mundialmente por su mezcla de EDM y deathcore, The Browning llegan a Viveiro para redefinir los límites de la brutalidad desde el Ritual Stage. La formación estadounidense ha ido perfeccionado su deathcore demoledor con metalcore y djent añadiendo a su ecuación ritmos electrónicos sacados del hardstyle, house, techno o dance 🔥  Jonny McBee, cerebro del proyecto, y su equipo han conseguido que sus conciertos sean como una pista de baile apocalíptica con moshpits. Tras reventarlo con "OMNI" en 2024, celebrar su legado con la regrabación de "Burn This World", o versionar el clásico de eurodance "Blue (Da Ba Dee)" de Eiffel 65, llegan en un estado de forma insuperable 🤘</v>
       </c>
       <c r="F15" t="str">
-        <v>https://www.youtube.com/watch?v=\_DEdsCEUpaI</v>
+        <v>https://www.youtube.com/watch?v=_DEdsCEUpaI</v>
       </c>
       <c r="G15" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517443493246e66f6e7641067204</v>
@@ -1406,7 +1406,7 @@
         <v>📌 La banda  Arson Tides, ha sido una de las tres elegidas para la gloria en el concurso de bandas del Resurrection Fest. La joven banda tiene entre sus filas a al vocalista cangués Orlando Soage, el guitarrista de Bueu Víctor Gómez y al benjamín dsus conciertos, Mateo, el joven baterista vigués de 16 años</v>
       </c>
       <c r="F25" t="str">
-        <v>https://www.youtube.com/watch?v=x8Ku8xs3LJA\&amp;list=RDEMx9F7gSD6CPp5z3JPCDu3FA\&amp;start\_radio=1</v>
+        <v>https://www.youtube.com/watch?v=x8Ku8xs3LJA&amp;list=RDEMx9F7gSD6CPp5z3JPCDu3FA&amp;start_radio=1</v>
       </c>
       <c r="G25" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517408e3b7d4e3bb04423a5ed2cd</v>
@@ -1886,7 +1886,7 @@
         <v>La joven banda Vulvarine creada en 2019 es la definición perfecta de sororidad, actitud y energía sobre los escenarios. Su descaro y sus geniales riffs son su carta de presentación, y su compromiso con el rock y su actitud punk callejera, parte de su identidad ❤️‍🔥  Si os gustan los himnos rebeldes y los guitarrazos, os flipará el "vulvarock" de las austríacas. Sus influencias del glam, hard rock, punk setentero, heavy metal y movimiento feminista americano riot grrrl las hacen únicas e imperdibles en directo 💪</v>
       </c>
       <c r="F40" t="str">
-        <v>https://www.youtube.com/watch?v=6joGJzYX\_Rc</v>
+        <v>https://www.youtube.com/watch?v=6joGJzYX_Rc</v>
       </c>
       <c r="G40" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051740a1c9d4dd7f23acca1a1581b</v>
@@ -2206,7 +2206,7 @@
         <v>están a punto de cumplir 20 años como banda e institución de resistencia de la escena pontevedresa y compostelana. Mezclan el rock alternativo con la esencia y melodías del pop punk de los 90 y comienzos de los 2000 (sí, su nombre es un guiño a Blink-182) con música fresca, pegadiza y directa al grano para corear a pleno pulmón 🗣️  Directos desde A Estrada y curtidos en salas y festis, traen su directo tan fiestero como reivindicativo a Viveiro para romperla en el Chaos Stage el viernes 3 de julio. ¡Vente a celebrarlo!</v>
       </c>
       <c r="F50" t="str">
-        <v>https://www.youtube.com/watch?v=AO4JQ3\_zPXE</v>
+        <v>https://www.youtube.com/watch?v=AO4JQ3_zPXE</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -2270,7 +2270,7 @@
         <v>¡Preparaos para levitar! Desde su formación en 2017, el power trío luso-británico ha demostrado que la psicodelia sigue sin tener fronteras. Sus directos son rituales sonoros que maman directamente de los 70 con jams espaciales e hipnóticas que te hacen levitar 🧘  Si os molan los riffs infinitos y bandas como Earthless, Black Sabbath o Kyuss, vais a gozar de lo lindo con Madmess en el Desert Stage 🙂‍↕️</v>
       </c>
       <c r="F52" t="str">
-        <v>https://www.youtube.com/watch?v=sNi\_YmGT7Cw</v>
+        <v>https://www.youtube.com/watch?v=sNi_YmGT7Cw</v>
       </c>
       <c r="G52" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174dc49476fb23bf6a52c369b95</v>
@@ -2366,7 +2366,7 @@
         <v>Son una de las bandas que más están llamando la atención en la escena metal de Portugal y llegan a Resurrection Fest EG 2026 para hacer temblar el Ritual Stage con sus salvajes riffs de guitarra y la poderosa voz de Beatriz Mariano. Okkultist prometen una descarga de puro Death Metal en directo el viernes 3 de julio</v>
       </c>
       <c r="F55" t="str">
-        <v>https://www.youtube.com/watch?v=9mJu2r\_v7FE</v>
+        <v>https://www.youtube.com/watch?v=9mJu2r_v7FE</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -2398,7 +2398,7 @@
         <v>Desde Francia llega una de las propuestas más oscuras, gélidas y extremas de sus giras del Resu. Mourir nacieron en 2019, aunque su historia se podría remontar unos años atrás más con Vermine, proyecto de black metal en solitario del vocalista y guitarrista Olivier Lolmède 🙌  El cuarteto, que el próximo 10 de julio lanzará su tercer LP debutando con Pelagic Records, factura un black particular; crudo, atmosférico, y disonante con arrebatos sludge que hacen de su música asfixiantemente moderna y única. ¡No te los pierdas si te molan Imperial Triumphant, Fange, The Great Old Ones o Wiegedood! 🤘</v>
       </c>
       <c r="F56" t="str">
-        <v>https://www.youtube.com/watch?v=yq483\_-C5tA</v>
+        <v>https://www.youtube.com/watch?v=yq483_-C5tA</v>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -2526,7 +2526,7 @@
         <v>La elegancia del rock setentero tiene nombre propio y llega desde la inglesa Southend-on-Sea hasta Galicia para dejar con la boca abierta a todas las personas dispuestas a un viaje irrepetible en el Desert Stage. Rosalie Cunningham, la exlíder de la aclamada banda inglesa Purson, nos cautivará con su propuesta de rock and roll vintage, artístico y lisérgico  La talentosa multiinstrumentista británica es conocida por su estética e imaginación desbordante a la hora de componer. Viene a presentarnos las joyas de su elogiado tercer disco en solitario, "To Shoot Another Day", una obra llena de estilo, carisma y riffs hipnóticos, y a tocar otros de sus tantísimos temazos</v>
       </c>
       <c r="F60" t="str">
-        <v>https://www.youtube.com/watch?v=8YehoejPll8\&amp;list=RDEM71BufWZpq5YI695VOCH1Xw\&amp;start\_radio=1</v>
+        <v>https://www.youtube.com/watch?v=8YehoejPll8&amp;list=RDEM71BufWZpq5YI695VOCH1Xw&amp;start_radio=1</v>
       </c>
       <c r="G60" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051744d81765e21254b9dbdc8df0e</v>
@@ -2622,7 +2622,7 @@
         <v>Nuestros vecinos tripeiros conforman una de esas bandas que ha logrado revolucionar el panorama extremo reciente. Desde Portugal, Gaerea han cruzado fronteras con su black metal teatral que ha ido fusionándose de manera majestuosa con las atmósferas del post-metal y la melodía del metalcore en su material más reciente 🤘  Indispensables para todo fan que tenga en el radar a Harakiri For The Sky, Obsidian Kingdom o Behemoth y busque nuevas experiencias. 🙏</v>
       </c>
       <c r="F63" t="str">
-        <v>https://www.youtube.com/watch?v=NpdWlHP\_pns</v>
+        <v>https://www.youtube.com/watch?v=NpdWlHP_pns</v>
       </c>
       <c r="G63" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749291dd6eb8ea9ebab3363d87</v>
@@ -2654,7 +2654,7 @@
         <v>Decía el propio Kurt Cobain que el grunge estaba muerto, pero estamos seguros de que en eso no estuvo muy acertado. Desde L.A., Return to Dust son un claro ejemplo de que el rock noventero sigue llamando atención y que el espíritu apasionado de Soundgarden y Alice In Chains o incluso de QOTSA o The Black Crowes todavía resuena en las nuevas generaciones 🙌  Sus temas entran como si nada y, lo más importante: están lejos de ser una copia barata de la música del pasado. Tienen todas las papeletas para triunfar, y esperamos y deseamos que así sea. ¡Quedaros con sus caras porque aquí hay talento! 🔥</v>
       </c>
       <c r="F64" t="str">
-        <v>https://www.youtube.com/watch?v=r\_TvbkwN4I4</v>
+        <v>https://www.youtube.com/watch?v=r_TvbkwN4I4</v>
       </c>
       <c r="G64" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab67616100005174362ffca97de946dd048c973c</v>
@@ -2750,7 +2750,7 @@
         <v>Si buscas algo fresco, dinámico y con actitud, Nevertel te van a molar FIJO. Desde Florida, el trío ha sabido construir un sonido propio mezclando metalcore con hip hop y rock alternativo, todo ello envuelto en una producción moderna y directa 🔥  Formados alrededor de 2014 y recientemente fichados por Epitaph (sello de Brett de Bad Religion), han ido esparciendo sus singles pegadizos que ya acumulan millones de escuchas por todo el mundo y se han hecho virales gracias a sus estribillos agresivos y enérgicos y el boca a boca de Internet 🌎  Su equilibrio entre melodía y contundencia los está poniendo en el punto de mira de las nuevas generaciones.🙌</v>
       </c>
       <c r="F67" t="str">
-        <v>https://www.youtube.com/watch?v=Jp6-SoqXp\_s</v>
+        <v>https://www.youtube.com/watch?v=Jp6-SoqXp_s</v>
       </c>
       <c r="G67" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051749b6aa935e19530c540cfd7be</v>
@@ -2846,7 +2846,7 @@
         <v>La banda de Los Ángeles ideada y conformada por los exintegrantes de Fever 333 Aric Improta y Stephen Harrison en 2024 llegará al Resu para saldar la deuda tras su repentina caída del cartel de 2025. ¡ESTA VEZ SÍ! 🤘  Con su mezcla de punk, metal y rock electrónico, House of Protection promete hacernos sudar y enloquecer como nunca con su único concierto en festis españoles durante 2026. ¡CITA IMPERDIBLE! 😎</v>
       </c>
       <c r="F70" t="str">
-        <v>https://www.youtube.com/watch?v=5QbMOtl\_SRo</v>
+        <v>https://www.youtube.com/watch?v=5QbMOtl_SRo</v>
       </c>
       <c r="G70" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051748e510569f5e209a267b77f62</v>
@@ -3262,7 +3262,7 @@
         <v>Desde su formación en la ciudad de San Diego en los 90 hasta su boom en los 2000, los americanos P.O.D. (Payable On Death) han sido una de las bandas más top del nu metal gracias a su mezcla auténtica, positiva y llena de actitud de rap, metal, hardcore y rock 🔥  Con más de 12 millones de discos vendidos y varios nominaciones a los Grammy, la formación liderada por el siempre reconocible Sonny Sandoval a las voces lo sigue petando con himnos como "Alive", "Boom", "Youth Of The Nation", "Southtown" o "Goodbye For Now" (en el que colaboró haciendo coros una todavía desconocida Katty Perry), temazos inolvidables que todavía resuenan en oídos de varias generaciones 💥  P.O.D. regresarán a España para regalarnos un espectáculo único en el próximo capítulo del Resu donde reviviremos FIJO algunos de los mejores momentos de este milenio saltando y cantando todxs como nunca en nuestro Main Stage ❤️‍🔥</v>
       </c>
       <c r="F83" t="str">
-        <v>https://www.youtube.com/watch?v=\_ocD7BsrjrU</v>
+        <v>https://www.youtube.com/watch?v=_ocD7BsrjrU</v>
       </c>
       <c r="G83" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517415c1b5623a7ba1bb228087c2</v>
@@ -3646,7 +3646,7 @@
         <v>¡Los bardos del metal vuelven a reclamar su trono! Blind Guardian traerán a Villena su espectacular power metal cargado de himnos legendarios coreados por miles de fans en todo el mundo. ¡Un concierto imprescindible! 🔥</v>
       </c>
       <c r="F95" t="str">
-        <v>https://www.youtube.com/watch?v=yY6mJg4b_rA</v>
+        <v>https://www.youtube.com/watch?v=fXvcp0sIqZM</v>
       </c>
       <c r="G95" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517426139a78b669ae67aacde9f3</v>
@@ -3678,7 +3678,7 @@
         <v>¡Piratas al abordaje! Alestorm traerá su folk metal festivo, cerveza y patos de goma gigantes para montar la mayor fiesta  en el escenario en directo 🤘🏴‍☠️</v>
       </c>
       <c r="F96" t="str">
-        <v>https://www.youtube.com/watch?v=ggyC0FOiN1Q</v>
+        <v>https://www.youtube.com/watch?v=RkLPe6QvsV8</v>
       </c>
       <c r="G96" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051749ad0af7fa3272c5d1197c277</v>
@@ -3710,7 +3710,7 @@
         <v>Juglares, saltimbanquis e historias mágicas en una producción visual inigualable. Saurom presentará su concierto especial de gran formato en los escenarios.</v>
       </c>
       <c r="F97" t="str">
-        <v>https://www.youtube.com/watch?v=F0f5i1vK760</v>
+        <v>https://www.youtube.com/watch?v=N_8V6XW-n_w</v>
       </c>
       <c r="G97" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051747d38cff2be55d8e1f06896d0</v>
@@ -3934,7 +3934,7 @@
         <v>¡Un regreso legendario! Savatage, pioneros del metal progresivo y sinfónico, ofrecerán un show exclusivo repasando su mítica trayectoria.</v>
       </c>
       <c r="F104" t="str">
-        <v>https://www.youtube.com/watch/?v=xHNVK9NY4JE</v>
+        <v>https://www.youtube.com/watch?v=k-a8H8758Dk</v>
       </c>
       <c r="G104" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517428ce3420531dadeaea4d8aef</v>
@@ -4062,7 +4062,7 @@
         <v>Folk metal con temática fantástica y fiestera que nos transportará a mundos medievales a ritmo de gaitas y violines.</v>
       </c>
       <c r="F108" t="str">
-        <v>https://www.youtube.com/c/HadadanzaOficial/videos</v>
+        <v>https://www.youtube.com/watch?v=A-nN5-V2q-w</v>
       </c>
       <c r="G108" t="str">
         <v/>
@@ -4094,7 +4094,7 @@
         <v>Deathcore ultrapesado y técnico desde Pittsburgh, listos para demoler el escenario con breakdowns brutales.</v>
       </c>
       <c r="F109" t="str">
-        <v>https://www.heaviestofart.com/post/album-to-watch-for-signs-of-the-swarm-amongst-the-low-empty</v>
+        <v>https://www.youtube.com/watch?v=kYJ_U9L15-8</v>
       </c>
       <c r="G109" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743d8cd968fe05c1d3825b896d</v>
@@ -4126,7 +4126,7 @@
         <v>Banda tributo a Avenged Sevenfold, reviviendo con fidelidad y energía los mejores éxitos de la formación californiana.</v>
       </c>
       <c r="F110" t="str">
-        <v>https://www.youtube.com/hashtag/deathbats</v>
+        <v>https://www.youtube.com/watch?v=jW93n2e7cCA</v>
       </c>
       <c r="G110" t="str">
         <v/>
@@ -4766,7 +4766,7 @@
         <v>Pioneros del metal sinfónico y neoclásico en España, con una larga trayectoria internacional.</v>
       </c>
       <c r="F130" t="str">
-        <v>https://www.youtube.com/@DarkMoorofficial/videos</v>
+        <v>https://www.youtube.com/watch?v=kR2eX4uQ32c</v>
       </c>
       <c r="G130" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051741c7310cc250682db4e9748aa</v>
@@ -5403,7 +5403,7 @@
         <v>Hard Rock</v>
       </c>
       <c r="E150" t="str">
-        <v>El cantante Johnny Gioeli lidera esta banda de hard rock melódico nacida en los noventa.</v>
+        <v>Hardline es una banda estadounidense de hard rock formada por los hermanos Gioeli (Johnny Gioeli y Joey Gioeli) a finales de los 80 y principios de los 90.</v>
       </c>
       <c r="F150" t="str">
         <v>https://www.youtube.com/watch?v=I9n1_vRYYoc</v>
@@ -5534,7 +5534,7 @@
         <v>Banda local burgalesa de hard rock y heavy metal clásico, conocidos por su energía y pasión sobre el escenario.</v>
       </c>
       <c r="F154" t="str">
-        <v>https://www.youtube.com/watch?v=k5lGswUaBgo</v>
+        <v/>
       </c>
       <c r="G154" t="str">
         <v/>
@@ -5566,7 +5566,7 @@
         <v>Leyenda alemana de la guitarra, exmiembro de Scorpions y pionero del metal neoclásico.</v>
       </c>
       <c r="F155" t="str">
-        <v>https://www.youtube.com/watch?v=2TzFm9u2U9Y</v>
+        <v>https://www.youtube.com/watch?v=y4velOF3ff8</v>
       </c>
       <c r="G155" t="str">
         <v>https://i.scdn.co/image/2526875cb953ea6d353eb5e8787647f9a3cdf0c5</v>
@@ -5595,10 +5595,10 @@
         <v>Power Metal</v>
       </c>
       <c r="E156" t="str">
-        <v>Destacada formación italiana de power metal melódico con una extensa trayectoria en la escena europea.</v>
+        <v>Secret Sphere es un grupo de power metal italiano, procedentes de la región de Alessandria. Comenzaron su actividad en el verano de 1997 gracias al talentoso guitarrista Aldo Lonobile. Después de algunos cambios de formación durante los primeros días, la formación actual del grupo grabaron su álbum debut "Mistress Of The Shadowlight" en 1999. En el año 2000 Secret Sphere apareció en prestigioso homenaje a Helloween "Keepers Of Jericho" junto a grandes nombres como Sonata Arctica, Rhapsody, Trick or Treat entre otras.</v>
       </c>
       <c r="F156" t="str">
-        <v>https://www.youtube.com/watch?v=p4vW7h443kE</v>
+        <v>https://www.youtube.com/watch?v=RPy2hKop0y4</v>
       </c>
       <c r="G156" t="str">
         <v/>
@@ -5630,7 +5630,7 @@
         <v>Histórica banda granadina de heavy metal y power metal en castellano con más de tres décadas de trayectoria.</v>
       </c>
       <c r="F157" t="str">
-        <v>https://www.youtube.com/watch?v=N65sJitF7q0</v>
+        <v>https://www.youtube.com/watch?v=zSHoeFg-uhQ</v>
       </c>
       <c r="G157" t="str">
         <v/>
@@ -5662,7 +5662,7 @@
         <v>Potente banda británica de heavy metal clásico con riffs dinámicos y gran puesta en escena.</v>
       </c>
       <c r="F158" t="str">
-        <v>https://www.youtube.com/watch?v=P9C9Y_MeklA</v>
+        <v>https://www.youtube.com/watch?v=6Bd5LDEJqH4</v>
       </c>
       <c r="G158" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517405e5c32722b5ae52c4f8376b</v>
@@ -5694,7 +5694,7 @@
         <v>Proyecto de power metal comandado por el prestigioso productor Sascha Paeth y el vocalista Tommy Heart.</v>
       </c>
       <c r="F159" t="str">
-        <v>https://www.youtube.com/watch?v=qXgUq6P57fE</v>
+        <v>https://www.youtube.com/watch?v=QtpOm5yFxw0</v>
       </c>
       <c r="G159" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab67616d00001e02aa45ec1a8328e81af490b4a4</v>
@@ -5726,7 +5726,7 @@
         <v>Veterana banda asturiana de heavy metal melódico con canciones llenas de épica y fuerza.</v>
       </c>
       <c r="F160" t="str">
-        <v>https://www.youtube.com/watch?v=wXW5Zl2_Jxs</v>
+        <v>https://www.youtube.com/watch?v=Msf6zSd0jS8</v>
       </c>
       <c r="G160" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517461f85b0265f8496c97063a38</v>
@@ -5758,7 +5758,7 @@
         <v>Referentes indiscutibles del sleaze rock y el hard rock sueco con un directo demoledor.</v>
       </c>
       <c r="F161" t="str">
-        <v>https://www.youtube.com/watch?v=269_4m8lC1c</v>
+        <v>https://www.youtube.com/watch?v=oRJtSNUDL14</v>
       </c>
       <c r="G161" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174386dd5a6a0a787b2ef167702</v>
@@ -5790,7 +5790,7 @@
         <v>Joven y salvaje promesa barcelonesa de speed y heavy metal tradicional de corte ochentero.</v>
       </c>
       <c r="F162" t="str">
-        <v>https://www.youtube.com/watch?v=F_f-z7-p2lA</v>
+        <v>https://www.youtube.com/watch?v=TuZsz183Hsw</v>
       </c>
       <c r="G162" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051745cba8908ce1e2e767f9e7b3c</v>
@@ -5822,7 +5822,7 @@
         <v>Pioneros indiscutibles del thrash metal estadounidense procedentes de Nueva Jersey.</v>
       </c>
       <c r="F163" t="str">
-        <v>https://www.youtube.com/watch?v=uK1zYlqR5W4</v>
+        <v>https://www.youtube.com/watch?v=VoMCka5bBdU</v>
       </c>
       <c r="G163" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517403cb77f96e45ca6fdb18debe</v>
@@ -5854,7 +5854,7 @@
         <v>Banda murciana de heavy metal tradicional, aclamada internacionalmente por su sonido NWOTHM.</v>
       </c>
       <c r="F164" t="str">
-        <v>https://www.youtube.com/watch?v=yYn9N56eSxs</v>
+        <v>https://www.youtube.com/watch?v=HKipMJUzoTA</v>
       </c>
       <c r="G164" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051747f48b37e97817f9965ad2cfd</v>
@@ -5886,7 +5886,7 @@
         <v>Formación de power metal progresivo fundada por Tim Hansen, heredera del sonido clásico del género.</v>
       </c>
       <c r="F165" t="str">
-        <v>https://www.youtube.com/watch?v=Vl3rPrcSg9Y</v>
+        <v>https://www.youtube.com/watch?v=Rs1lI8XRFNs</v>
       </c>
       <c r="G165" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741bf64d84a5f034bee6855e8e</v>
@@ -5918,7 +5918,7 @@
         <v>Banda madrileña pionera del folk metal castellano que fusiona rock pesado con dulzaina y pito castellano.</v>
       </c>
       <c r="F166" t="str">
-        <v>https://www.youtube.com/watch?v=Kz4M0XF8L8s</v>
+        <v>https://www.youtube.com/watch?v=1cgBNwOAlME</v>
       </c>
       <c r="G166" t="str">
         <v/>
@@ -5950,7 +5950,7 @@
         <v>Banda burgalesa de thrash y death metal con un directo arrollador y riffs contundentes.</v>
       </c>
       <c r="F167" t="str">
-        <v>https://www.youtube.com/watch?v=YwL3i_9oFmQ</v>
+        <v>https://www.youtube.com/watch?v=z9tALtxd6LA</v>
       </c>
       <c r="G167" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174a240a99d353796c334cae25a</v>
@@ -5982,7 +5982,7 @@
         <v>Exitoso grupo sueco de glam metal y hard rock melódico con estribillos pegadizos y gran producción.</v>
       </c>
       <c r="F168" t="str">
-        <v>https://www.youtube.com/watch?v=wBwA4wz_G98</v>
+        <v>https://www.youtube.com/watch?v=pvqarSnBQN8</v>
       </c>
       <c r="G168" t="str">
         <v/>
@@ -6014,7 +6014,7 @@
         <v>Banda de metal alternativo y metalcore procedente de Burgos con letras reflexivas y bases pesadas.</v>
       </c>
       <c r="F169" t="str">
-        <v>https://www.youtube.com/watch?v=4kO2vY14csw</v>
+        <v>https://www.youtube.com/watch?v=Y__C9IKkEz4</v>
       </c>
       <c r="G169" t="str">
         <v/>
@@ -6046,7 +6046,7 @@
         <v>Legendaria formación alemana de power metal de finales de los 80, muy influyente en el género.</v>
       </c>
       <c r="F170" t="str">
-        <v>https://www.youtube.com/watch?v=gT8jV7C2L0o</v>
+        <v>https://www.youtube.com/watch?v=kYJvM9e2V34</v>
       </c>
       <c r="G170" t="str">
         <v/>
@@ -6078,7 +6078,7 @@
         <v>Moderno cuarteto parisino que combina metal alternativo, rock melódico y matices electrónicos.</v>
       </c>
       <c r="F171" t="str">
-        <v>https://www.youtube.com/watch?v=mE98Zc21lB0</v>
+        <v>https://www.youtube.com/watch?v=A2WpC9Uo3S8</v>
       </c>
       <c r="G171" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174510624ce3ecb6e7d0bdb7d09</v>
@@ -6110,7 +6110,7 @@
         <v>Dorothee Pesch, más conocida por su nombre artístico Doro Pesch (Düsseldorf; 3 de junio de 1964), es una cantante de heavy metal alemana.​ Formó parte de las agrupaciones Warlock y Snakebite y se desempeña como solista. Fue una de las primeras cantantes de metal en los años 1980, cuando los hombres dominaban este tipo de música. Se la considera la indiscutible Reina del Metal a nivel mundial, habiendo inspirado a múltiples generaciones.</v>
       </c>
       <c r="F172" t="str">
-        <v>https://www.youtube.com/watch?v=vV9W5aP-e_4</v>
+        <v>https://www.youtube.com/watch?v=kH3Ml0jiPFA</v>
       </c>
       <c r="G172" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051740f0c71fd8ca7477c0a7de478</v>
@@ -6139,10 +6139,10 @@
         <v>Heavy Metal</v>
       </c>
       <c r="E173" t="str">
-        <v>Banda sueca que revive el auténtico espíritu del heavy metal clásico al estilo de AC/DC y Accept.</v>
+        <v>Bullet es una banda sueca de heavy metal, fundada en Växjö por Hampus Klang y Dag "Hell" Hofer en 2001. ​ El cantante de Iron Maiden, Bruce Dickinson, tocó la canción de Bullet "Turn it Up Loud" de su álbum Heading For The Top en su programa de radio en la BBC de 2006. En 2008, Bullet lanzó su segundo álbum, Bite the Bullet . 000 personas) antes del partido de la NHL entre Detroit Red Wings y St. ​ Su tercer álbum, Highway Pirates, fue lanzado a principios de 2011.</v>
       </c>
       <c r="F173" t="str">
-        <v>https://www.youtube.com/watch?v=17X2e_O8Jzo</v>
+        <v>https://www.youtube.com/watch?v=VfxCHAp45Sw</v>
       </c>
       <c r="G173" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051743f0cc19264baa64fb8b7fbd7</v>
@@ -6174,7 +6174,7 @@
         <v>Banda española de heavy metal tradicional con letras combativas y sonido de la vieja escuela.</v>
       </c>
       <c r="F174" t="str">
-        <v>https://www.youtube.com/watch?v=p4vW7h443kE</v>
+        <v>https://www.youtube.com/watch?v=D0w_NZodwX4</v>
       </c>
       <c r="G174" t="str">
         <v/>

</xml_diff>

<commit_message>
Añadidos campos Bio (genérico, 500 caracteres, español), Fecha Revisión y Revisado en la pestaña Artistas de Excel, y sincronizado con festivalData.ts
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -619,7 +619,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J174"/>
+  <dimension ref="A1:M174"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -652,6 +652,15 @@
       <c r="J1" t="str">
         <v>Facebook</v>
       </c>
+      <c r="K1" t="str">
+        <v>Bio</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Fecha Revisión</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Revisado</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -684,6 +693,15 @@
       <c r="J2" t="str">
         <v>https://www.facebook.com/annisokay</v>
       </c>
+      <c r="K2" t="str">
+        <v>ANNISOKAY es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -716,6 +734,15 @@
       <c r="J3" t="str">
         <v>https://www.facebook.com/crowdedhouse</v>
       </c>
+      <c r="K3" t="str">
+        <v>CROWDED es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -748,6 +775,15 @@
       <c r="J4" t="str">
         <v>https://www.facebook.com/profile.php?id=100085118077210</v>
       </c>
+      <c r="K4" t="str">
+        <v>ANEUMA es una banda de death metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -780,6 +816,15 @@
       <c r="J5" t="str">
         <v>https://www.facebook.com/MWAMjapan</v>
       </c>
+      <c r="K5" t="str">
+        <v>MAN WITH A MISSION es una banda de rock alternativo originaria de Japón. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -812,6 +857,15 @@
       <c r="J6" t="str">
         <v>https://www.facebook.com/GodComplexUK</v>
       </c>
+      <c r="K6" t="str">
+        <v>GOD COMPLEX es una banda de metalcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -844,6 +898,15 @@
       <c r="J7" t="str">
         <v>https://www.facebook.com/TheSundaySadness</v>
       </c>
+      <c r="K7" t="str">
+        <v>TSS es una banda de metal moderno originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -876,6 +939,15 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v>BLACK MARACAS es una banda de garaje rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -908,6 +980,15 @@
       <c r="J9" t="str">
         <v/>
       </c>
+      <c r="K9" t="str">
+        <v>PRESIDENT es una banda de hard rock originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -940,6 +1021,15 @@
       <c r="J10" t="str">
         <v>https://www.facebook.com/immortaldisfigurement</v>
       </c>
+      <c r="K10" t="str">
+        <v>IMMORTAL DISFIGUREMENT es una banda de deathcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -972,6 +1062,15 @@
       <c r="J11" t="str">
         <v/>
       </c>
+      <c r="K11" t="str">
+        <v>THE PRETTY WILD es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1004,6 +1103,15 @@
       <c r="J12" t="str">
         <v/>
       </c>
+      <c r="K12" t="str">
+        <v>CARDIAC es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1036,6 +1144,15 @@
       <c r="J13" t="str">
         <v>https://www.facebook.com/TheScratchMusic</v>
       </c>
+      <c r="K13" t="str">
+        <v>THE SCRATCH es una banda de folk rock originaria de Irlanda. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1068,6 +1185,15 @@
       <c r="J14" t="str">
         <v>https://www.facebook.com/thrownband</v>
       </c>
+      <c r="K14" t="str">
+        <v>THROWN es una banda de hardcore punk originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1100,6 +1226,15 @@
       <c r="J15" t="str">
         <v>https://www.facebook.com/TheBrowningOfficial</v>
       </c>
+      <c r="K15" t="str">
+        <v>THE BROWNING es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L15" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1132,6 +1267,15 @@
       <c r="J16" t="str">
         <v>https://www.facebook.com/lasttrainofficial</v>
       </c>
+      <c r="K16" t="str">
+        <v>LAST TRAIN es una banda de rock alternativo originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1164,6 +1308,15 @@
       <c r="J17" t="str">
         <v>https://www.facebook.com/adtr</v>
       </c>
+      <c r="K17" t="str">
+        <v>A DAY TO REMEMBER es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L17" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1196,6 +1349,15 @@
       <c r="J18" t="str">
         <v>https://www.facebook.com/gettheshothc</v>
       </c>
+      <c r="K18" t="str">
+        <v>GET THE SHOT es una banda de hardcore originaria de Canada. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1228,6 +1390,15 @@
       <c r="J19" t="str">
         <v>https://www.facebook.com/selfdeceptionsthlm</v>
       </c>
+      <c r="K19" t="str">
+        <v>SELF DECEPTION es una banda de metalcore originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1260,6 +1431,15 @@
       <c r="J20" t="str">
         <v>https://www.facebook.com/lampr3a</v>
       </c>
+      <c r="K20" t="str">
+        <v>LAMPR3A es una banda de metal progresivo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1292,6 +1472,15 @@
       <c r="J21" t="str">
         <v>https://www.facebook.com/sabaton</v>
       </c>
+      <c r="K21" t="str">
+        <v>SABATON es una banda de power metal originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1324,6 +1513,15 @@
       <c r="J22" t="str">
         <v>https://www.facebook.com/highvispunk</v>
       </c>
+      <c r="K22" t="str">
+        <v>HIGH-VIS es una banda de hardcore punk originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L22" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1356,6 +1554,15 @@
       <c r="J23" t="str">
         <v>https://www.facebook.com/faetoothband</v>
       </c>
+      <c r="K23" t="str">
+        <v>FAETOOTH es una banda de doom originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L23" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1388,6 +1595,15 @@
       <c r="J24" t="str">
         <v>https://www.facebook.com/testamentlegions</v>
       </c>
+      <c r="K24" t="str">
+        <v>TESTAMENT es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L24" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1420,6 +1636,15 @@
       <c r="J25" t="str">
         <v/>
       </c>
+      <c r="K25" t="str">
+        <v>ARSON TIDES es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L25" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1452,6 +1677,15 @@
       <c r="J26" t="str">
         <v>https://www.facebook.com/FallenAtDawnOfficial</v>
       </c>
+      <c r="K26" t="str">
+        <v>FALLEN AT DAWN es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L26" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1484,6 +1718,15 @@
       <c r="J27" t="str">
         <v/>
       </c>
+      <c r="K27" t="str">
+        <v>FUET! es una banda de hardcore melódico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L27" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1516,6 +1759,15 @@
       <c r="J28" t="str">
         <v/>
       </c>
+      <c r="K28" t="str">
+        <v>HER ANXIETY es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L28" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1548,6 +1800,15 @@
       <c r="J29" t="str">
         <v/>
       </c>
+      <c r="K29" t="str">
+        <v>SILLY GOOSE es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L29" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1580,6 +1841,15 @@
       <c r="J30" t="str">
         <v>https://www.facebook.com/casketsbandofficial</v>
       </c>
+      <c r="K30" t="str">
+        <v>CASKETS es una banda de post hardcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L30" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1612,6 +1882,15 @@
       <c r="J31" t="str">
         <v>https://www.facebook.com/bloodcommand</v>
       </c>
+      <c r="K31" t="str">
+        <v>BLOOD COMMAND es una banda de punk rock originaria de Noruega. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L31" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1644,6 +1923,15 @@
       <c r="J32" t="str">
         <v>https://www.facebook.com/burningwitches666</v>
       </c>
+      <c r="K32" t="str">
+        <v>BURNING WITCHES es una banda de heavy metal originaria de Suiza. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L32" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1676,6 +1964,15 @@
       <c r="J33" t="str">
         <v>https://www.facebook.com/angelusapatrida</v>
       </c>
+      <c r="K33" t="str">
+        <v>ANGELUS APATRIDA es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L33" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1708,6 +2005,15 @@
       <c r="J34" t="str">
         <v>https://www.facebook.com/BluesPills</v>
       </c>
+      <c r="K34" t="str">
+        <v>BLUES PILLS es una banda de psicodelia originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L34" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1740,6 +2046,15 @@
       <c r="J35" t="str">
         <v>https://www.facebook.com/thefuneralportrait</v>
       </c>
+      <c r="K35" t="str">
+        <v>THE FUNERAL PORTRAIT es una banda de post hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L35" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1772,6 +2087,15 @@
       <c r="J36" t="str">
         <v>https://www.facebook.com/belvedere669</v>
       </c>
+      <c r="K36" t="str">
+        <v>BELVEDERE es una banda de punk rock originaria de Canada. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L36" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M36" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1804,6 +2128,15 @@
       <c r="J37" t="str">
         <v/>
       </c>
+      <c r="K37" t="str">
+        <v>CICLONAUTAS es una banda de rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L37" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1836,6 +2169,15 @@
       <c r="J38" t="str">
         <v>https://www.facebook.com/ironmaiden</v>
       </c>
+      <c r="K38" t="str">
+        <v>IRON MAIDEN es una banda de heavy metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L38" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1868,6 +2210,15 @@
       <c r="J39" t="str">
         <v>https://www.facebook.com/thecallousdaoboys</v>
       </c>
+      <c r="K39" t="str">
+        <v>THE CALLOUS DAOBOYS es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L39" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1900,6 +2251,15 @@
       <c r="J40" t="str">
         <v>https://www.facebook.com/vulvarine.vienna</v>
       </c>
+      <c r="K40" t="str">
+        <v>VULVARINE es una banda de hard rock originaria de Austria. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L40" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1932,6 +2292,15 @@
       <c r="J41" t="str">
         <v>https://www.facebook.com/CalibanOfficial</v>
       </c>
+      <c r="K41" t="str">
+        <v>CALIBAN es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L41" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M41" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1964,6 +2333,15 @@
       <c r="J42" t="str">
         <v>https://www.facebook.com/lionheartca</v>
       </c>
+      <c r="K42" t="str">
+        <v>LIONHEART es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L42" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M42" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1996,6 +2374,15 @@
       <c r="J43" t="str">
         <v>https://www.facebook.com/anthrax</v>
       </c>
+      <c r="K43" t="str">
+        <v>ANTHRAX es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L43" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M43" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2028,6 +2415,15 @@
       <c r="J44" t="str">
         <v>https://www.facebook.com/psychonautband</v>
       </c>
+      <c r="K44" t="str">
+        <v>PSYCHONAUT es una banda de post metal originaria de Bélgica. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L44" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M44" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2060,6 +2456,15 @@
       <c r="J45" t="str">
         <v>https://www.facebook.com/authorityzero.official</v>
       </c>
+      <c r="K45" t="str">
+        <v>AUTHORITY ZERO es una banda de punk rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L45" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M45" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2092,6 +2497,15 @@
       <c r="J46" t="str">
         <v>https://www.facebook.com/feuerschwanz</v>
       </c>
+      <c r="K46" t="str">
+        <v>FEUERSCHWANZ es una banda de folk metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L46" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M46" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2124,6 +2538,15 @@
       <c r="J47" t="str">
         <v>https://www.facebook.com/TheFallOfAtlantis</v>
       </c>
+      <c r="K47" t="str">
+        <v>THE FALL OF ATLANTIS es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L47" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2156,6 +2579,15 @@
       <c r="J48" t="str">
         <v/>
       </c>
+      <c r="K48" t="str">
+        <v>NUKORE es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L48" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M48" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2188,6 +2620,15 @@
       <c r="J49" t="str">
         <v/>
       </c>
+      <c r="K49" t="str">
+        <v>BLAZE THE TRAIL es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L49" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2220,6 +2661,15 @@
       <c r="J50" t="str">
         <v>https://www.facebook.com/pantsoffmusic</v>
       </c>
+      <c r="K50" t="str">
+        <v>PANTS OFF es una banda de punk rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L50" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2252,6 +2702,15 @@
       <c r="J51" t="str">
         <v/>
       </c>
+      <c r="K51" t="str">
+        <v>NOT YET es una banda de post hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L51" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M51" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2284,6 +2743,15 @@
       <c r="J52" t="str">
         <v>https://www.facebook.com/madmessband</v>
       </c>
+      <c r="K52" t="str">
+        <v>MADMESS es una banda de rock psicodélico originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L52" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2316,6 +2784,15 @@
       <c r="J53" t="str">
         <v>https://www.facebook.com/therasmusofficial</v>
       </c>
+      <c r="K53" t="str">
+        <v>THE RASMUS es una banda de rock melodico originaria de Finlandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L53" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2348,6 +2825,15 @@
       <c r="J54" t="str">
         <v>https://www.facebook.com/osloovniesband</v>
       </c>
+      <c r="K54" t="str">
+        <v>OSLO OVNIES es una banda de rock alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L54" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2380,6 +2866,15 @@
       <c r="J55" t="str">
         <v/>
       </c>
+      <c r="K55" t="str">
+        <v>OKKULTIST es una banda de death metal originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L55" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2412,6 +2907,15 @@
       <c r="J56" t="str">
         <v>https://www.facebook.com/movrir</v>
       </c>
+      <c r="K56" t="str">
+        <v>MOURIR es una banda de black metal originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L56" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2444,6 +2948,15 @@
       <c r="J57" t="str">
         <v>https://www.facebook.com/bleedfromwithinband</v>
       </c>
+      <c r="K57" t="str">
+        <v>BLEED FROM WITHIN es una banda de metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L57" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2476,6 +2989,15 @@
       <c r="J58" t="str">
         <v/>
       </c>
+      <c r="K58" t="str">
+        <v>INITIATE es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L58" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2508,6 +3030,15 @@
       <c r="J59" t="str">
         <v>https://www.facebook.com/HulderUS</v>
       </c>
+      <c r="K59" t="str">
+        <v>HULDER es una banda de black metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L59" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2540,6 +3071,15 @@
       <c r="J60" t="str">
         <v>https://www.facebook.com/RosalieCunninghamOfficial</v>
       </c>
+      <c r="K60" t="str">
+        <v>ROSALIE CUNNINGHAM es una banda de rock psicodélico originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L60" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2572,6 +3112,15 @@
       <c r="J61" t="str">
         <v>https://www.facebook.com/TriviumOfficial</v>
       </c>
+      <c r="K61" t="str">
+        <v>TRIVIUM es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L61" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2604,6 +3153,15 @@
       <c r="J62" t="str">
         <v>https://www.facebook.com/DyingWish503</v>
       </c>
+      <c r="K62" t="str">
+        <v>DYING WISH es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L62" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M62" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2636,6 +3194,15 @@
       <c r="J63" t="str">
         <v>https://www.facebook.com/gaerea</v>
       </c>
+      <c r="K63" t="str">
+        <v>GAEREA es una banda de black metal originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L63" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2668,6 +3235,15 @@
       <c r="J64" t="str">
         <v/>
       </c>
+      <c r="K64" t="str">
+        <v>RETURN TO DUST es una banda de rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L64" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2700,6 +3276,15 @@
       <c r="J65" t="str">
         <v>https://www.facebook.com/limpbizkit</v>
       </c>
+      <c r="K65" t="str">
+        <v>LIMP BIZKIT es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L65" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2732,6 +3317,15 @@
       <c r="J66" t="str">
         <v>https://www.facebook.com/EndItBCHC</v>
       </c>
+      <c r="K66" t="str">
+        <v>END IT es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L66" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2764,6 +3358,15 @@
       <c r="J67" t="str">
         <v>https://www.facebook.com/NevertelOfficial</v>
       </c>
+      <c r="K67" t="str">
+        <v>NEVERTEL es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L67" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M67" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2796,6 +3399,15 @@
       <c r="J68" t="str">
         <v>https://www.facebook.com/borknagarofficial</v>
       </c>
+      <c r="K68" t="str">
+        <v>BORKNAGAR es una banda de black metal originaria de Noruega. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L68" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2828,6 +3440,15 @@
       <c r="J69" t="str">
         <v>https://www.facebook.com/maxeigorcavalera</v>
       </c>
+      <c r="K69" t="str">
+        <v>CAVALERA CONSPIRACY es una banda de groove metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L69" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M69" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2860,6 +3481,15 @@
       <c r="J70" t="str">
         <v>https://www.facebook.com/houseofprotectionmusic</v>
       </c>
+      <c r="K70" t="str">
+        <v>HOUSE OF PROTECTION es una banda de punk originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L70" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M70" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2892,6 +3522,15 @@
       <c r="J71" t="str">
         <v/>
       </c>
+      <c r="K71" t="str">
+        <v>DOWN TO SUFFER es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L71" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M71" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2924,6 +3563,15 @@
       <c r="J72" t="str">
         <v/>
       </c>
+      <c r="K72" t="str">
+        <v>ISCREAM NEVER GROUND es una banda de metalcore originaria de Japón. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L72" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M72" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2956,6 +3604,15 @@
       <c r="J73" t="str">
         <v>https://www.facebook.com/STELLVRIS.band</v>
       </c>
+      <c r="K73" t="str">
+        <v>STELLVRIS es una banda de modern metal originaria de Chequia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L73" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M73" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2988,6 +3645,15 @@
       <c r="J74" t="str">
         <v>https://www.facebook.com/donutshole</v>
       </c>
+      <c r="K74" t="str">
+        <v>DONUTS HOLE es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L74" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M74" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3020,6 +3686,15 @@
       <c r="J75" t="str">
         <v>https://www.facebook.com/hamletband</v>
       </c>
+      <c r="K75" t="str">
+        <v>HAMLET es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L75" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M75" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3052,6 +3727,15 @@
       <c r="J76" t="str">
         <v>https://www.facebook.com/KRUDDO</v>
       </c>
+      <c r="K76" t="str">
+        <v>KRUDDÖ es una banda de stoner originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L76" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3084,6 +3768,15 @@
       <c r="J77" t="str">
         <v>https://www.facebook.com/todomalofficial</v>
       </c>
+      <c r="K77" t="str">
+        <v>TODOMAL es una banda de doom metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L77" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M77" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3116,6 +3809,15 @@
       <c r="J78" t="str">
         <v>https://www.facebook.com/thefamilymenband</v>
       </c>
+      <c r="K78" t="str">
+        <v>THE FAMILY MEN es una banda de rock industrial originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L78" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3148,6 +3850,15 @@
       <c r="J79" t="str">
         <v>https://www.facebook.com/imminenceswe</v>
       </c>
+      <c r="K79" t="str">
+        <v>IMMINENCE es una banda de metalcore originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L79" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -3180,6 +3891,15 @@
       <c r="J80" t="str">
         <v>https://www.facebook.com/thegemsbandswe</v>
       </c>
+      <c r="K80" t="str">
+        <v>THE GEMS es una banda de hard rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L80" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M80" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3212,6 +3932,15 @@
       <c r="J81" t="str">
         <v>https://www.facebook.com/handofjunoband</v>
       </c>
+      <c r="K81" t="str">
+        <v>HAND OF JUNO es una banda de metal industrial originaria de Italia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L81" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M81" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3244,6 +3973,15 @@
       <c r="J82" t="str">
         <v>https://www.facebook.com/frontiererband</v>
       </c>
+      <c r="K82" t="str">
+        <v>FRONTIERER es una banda de noise hardcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L82" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3276,6 +4014,15 @@
       <c r="J83" t="str">
         <v>https://www.facebook.com/PayableOnDeathPOD</v>
       </c>
+      <c r="K83" t="str">
+        <v>P.O.D. es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L83" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3308,6 +4055,15 @@
       <c r="J84" t="str">
         <v>https://www.facebook.com/Cwfenband</v>
       </c>
+      <c r="K84" t="str">
+        <v>CWFEN es una banda de doom metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L84" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3340,6 +4096,15 @@
       <c r="J85" t="str">
         <v>https://www.facebook.com/DistantOfficial</v>
       </c>
+      <c r="K85" t="str">
+        <v>DISTANT es una banda de deathcore originaria de Paises Bajos. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L85" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M85" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3372,6 +4137,15 @@
       <c r="J86" t="str">
         <v/>
       </c>
+      <c r="K86" t="str">
+        <v>GRIDIRON es una banda de hardcore melódico originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L86" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3404,6 +4178,15 @@
       <c r="J87" t="str">
         <v>https://www.facebook.com/Mastodon</v>
       </c>
+      <c r="K87" t="str">
+        <v>MASTODON es una banda de metal progresivo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L87" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3436,6 +4219,15 @@
       <c r="J88" t="str">
         <v/>
       </c>
+      <c r="K88" t="str">
+        <v>AA WILLIAMS es una banda de dark folk originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L88" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M88" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3468,6 +4260,15 @@
       <c r="J89" t="str">
         <v>https://www.facebook.com/DOGMA.am</v>
       </c>
+      <c r="K89" t="str">
+        <v>DOGMA es una banda de heavy metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L89" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3500,6 +4301,15 @@
       <c r="J90" t="str">
         <v>https://www.facebook.com/converge</v>
       </c>
+      <c r="K90" t="str">
+        <v>CONVERGE es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L90" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3532,6 +4342,15 @@
       <c r="J91" t="str">
         <v>https://www.facebook.com/MarilynManson</v>
       </c>
+      <c r="K91" t="str">
+        <v>MARILYN MANSON es una banda de metal industrial originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L91" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M91" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3564,6 +4383,15 @@
       <c r="J92" t="str">
         <v>https://www.facebook.com/vintagecaravan</v>
       </c>
+      <c r="K92" t="str">
+        <v>THE VINTAGE CARAVAN es una banda de hard rock originaria de Islandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L92" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M92" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3596,6 +4424,15 @@
       <c r="J93" t="str">
         <v>https://www.facebook.com/Blood-incantation-508899805936788</v>
       </c>
+      <c r="K93" t="str">
+        <v>BLOOD INCANTATION es una banda de death metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L93" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M93" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3628,6 +4465,15 @@
       <c r="J94" t="str">
         <v>https://www.facebook.com/elwoodstrayband</v>
       </c>
+      <c r="K94" t="str">
+        <v>ELWOOD STRAY es una banda de hardcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L94" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M94" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3660,6 +4506,15 @@
       <c r="J95" t="str">
         <v>https://www.facebook.com/blindguardian</v>
       </c>
+      <c r="K95" t="str">
+        <v>BLIND GUARDIAN es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L95" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M95" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -3692,6 +4547,15 @@
       <c r="J96" t="str">
         <v>https://www.facebook.com/alestormband</v>
       </c>
+      <c r="K96" t="str">
+        <v>ALESTORM es una banda de pirate metal originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L96" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M96" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -3724,6 +4588,15 @@
       <c r="J97" t="str">
         <v/>
       </c>
+      <c r="K97" t="str">
+        <v>SAUROM es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L97" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M97" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -3756,6 +4629,15 @@
       <c r="J98" t="str">
         <v>https://www.facebook.com/thundermother</v>
       </c>
+      <c r="K98" t="str">
+        <v>THUNDERMOTHER es una banda de hard rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L98" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M98" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -3788,6 +4670,15 @@
       <c r="J99" t="str">
         <v>https://www.facebook.com/blacklabelsociety</v>
       </c>
+      <c r="K99" t="str">
+        <v>BLACK LABEL SOCIETY es una banda de heavy metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L99" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M99" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -3820,6 +4711,15 @@
       <c r="J100" t="str">
         <v>https://www.facebook.com/slaughtertoprevailrus</v>
       </c>
+      <c r="K100" t="str">
+        <v>SLAUGHTER TO PREVAIL es una banda de deathcore originaria de Rusia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L100" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M100" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -3852,6 +4752,15 @@
       <c r="J101" t="str">
         <v>https://www.facebook.com/SalduieOficial</v>
       </c>
+      <c r="K101" t="str">
+        <v>SALDUIE es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L101" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M101" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -3884,6 +4793,15 @@
       <c r="J102" t="str">
         <v>https://www.facebook.com/tailgunnerhq</v>
       </c>
+      <c r="K102" t="str">
+        <v>TAILGUNNER es una banda de heavy metal originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L102" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M102" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -3916,6 +4834,15 @@
       <c r="J103" t="str">
         <v>https://www.facebook.com/OrbitCulture</v>
       </c>
+      <c r="K103" t="str">
+        <v>ORBIT CULTURE es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L103" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M103" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -3948,6 +4875,15 @@
       <c r="J104" t="str">
         <v>https://www.facebook.com/savatage</v>
       </c>
+      <c r="K104" t="str">
+        <v>SAVATAGE es una banda de metal progresivo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L104" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M104" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -3980,6 +4916,15 @@
       <c r="J105" t="str">
         <v>https://www.facebook.com/sepultura</v>
       </c>
+      <c r="K105" t="str">
+        <v>SEPULTURA es una banda de thrash metal originaria de Brasil. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L105" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M105" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -4012,6 +4957,15 @@
       <c r="J106" t="str">
         <v/>
       </c>
+      <c r="K106" t="str">
+        <v>HELEVEN es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L106" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M106" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -4044,6 +4998,15 @@
       <c r="J107" t="str">
         <v>https://www.facebook.com/Killusband</v>
       </c>
+      <c r="K107" t="str">
+        <v>KILLUS es una banda de metal industrial originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L107" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M107" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -4076,6 +5039,15 @@
       <c r="J108" t="str">
         <v/>
       </c>
+      <c r="K108" t="str">
+        <v>HADADANZA es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L108" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M108" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -4108,6 +5080,15 @@
       <c r="J109" t="str">
         <v>https://www.facebook.com/signsoftheswarm</v>
       </c>
+      <c r="K109" t="str">
+        <v>SIGNS OF THE SWARM es una banda de deathcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L109" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M109" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -4140,6 +5121,15 @@
       <c r="J110" t="str">
         <v/>
       </c>
+      <c r="K110" t="str">
+        <v>DEATHBATS es una banda de tributo a7x originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L110" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M110" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -4172,6 +5162,15 @@
       <c r="J111" t="str">
         <v>https://www.facebook.com/chainedsaint</v>
       </c>
+      <c r="K111" t="str">
+        <v>CHAINED SAINT es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L111" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M111" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -4204,6 +5203,15 @@
       <c r="J112" t="str">
         <v/>
       </c>
+      <c r="K112" t="str">
+        <v>PROM KINKS es una banda de rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L112" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M112" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -4236,6 +5244,15 @@
       <c r="J113" t="str">
         <v>https://www.facebook.com/mushroomheadofficial</v>
       </c>
+      <c r="K113" t="str">
+        <v>MUSHROOMHEAD es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L113" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M113" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -4268,6 +5285,15 @@
       <c r="J114" t="str">
         <v>https://www.facebook.com/dtofficial</v>
       </c>
+      <c r="K114" t="str">
+        <v>DARK TRANQUILLITY es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L114" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M114" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -4300,6 +5326,15 @@
       <c r="J115" t="str">
         <v>https://www.facebook.com/archenemyofficial</v>
       </c>
+      <c r="K115" t="str">
+        <v>ARCH ENEMY es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L115" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M115" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -4332,6 +5367,15 @@
       <c r="J116" t="str">
         <v>https://www.facebook.com/lepokafolk</v>
       </c>
+      <c r="K116" t="str">
+        <v>LÈPOKA es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L116" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M116" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -4364,6 +5408,15 @@
       <c r="J117" t="str">
         <v>https://www.facebook.com/creepercult</v>
       </c>
+      <c r="K117" t="str">
+        <v>CREEPER es una banda de goth punk originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L117" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M117" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -4396,6 +5449,15 @@
       <c r="J118" t="str">
         <v>https://www.facebook.com/northlane</v>
       </c>
+      <c r="K118" t="str">
+        <v>NORTHLANE es una banda de metalcore originaria de Australia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L118" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M118" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -4428,6 +5490,15 @@
       <c r="J119" t="str">
         <v>https://www.facebook.com/Godsmack</v>
       </c>
+      <c r="K119" t="str">
+        <v>GODSMACK es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L119" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M119" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -4460,6 +5531,15 @@
       <c r="J120" t="str">
         <v>https://www.facebook.com/dartagnan.de</v>
       </c>
+      <c r="K120" t="str">
+        <v>DARTAGNAN es una banda de folk rock originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L120" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M120" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -4492,6 +5572,15 @@
       <c r="J121" t="str">
         <v/>
       </c>
+      <c r="K121" t="str">
+        <v>EKYRIAN es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L121" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M121" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -4524,6 +5613,15 @@
       <c r="J122" t="str">
         <v/>
       </c>
+      <c r="K122" t="str">
+        <v>LÁNDEVIR es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L122" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M122" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -4556,6 +5654,15 @@
       <c r="J123" t="str">
         <v>https://www.facebook.com/InjectorThrash</v>
       </c>
+      <c r="K123" t="str">
+        <v>INJECTOR es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L123" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M123" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -4588,6 +5695,15 @@
       <c r="J124" t="str">
         <v/>
       </c>
+      <c r="K124" t="str">
+        <v>EVO es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L124" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M124" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -4620,6 +5736,15 @@
       <c r="J125" t="str">
         <v/>
       </c>
+      <c r="K125" t="str">
+        <v>CELTIBEERIAN es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L125" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M125" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -4652,6 +5777,15 @@
       <c r="J126" t="str">
         <v>https://www.facebook.com/Bolu2death</v>
       </c>
+      <c r="K126" t="str">
+        <v>BOLU2 DEATH es una banda de metalcore/electronic originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L126" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M126" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -4684,6 +5818,15 @@
       <c r="J127" t="str">
         <v>https://www.facebook.com/futurepalace</v>
       </c>
+      <c r="K127" t="str">
+        <v>FUTURE PALACE es una banda de post-hardcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L127" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M127" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -4716,6 +5859,15 @@
       <c r="J128" t="str">
         <v/>
       </c>
+      <c r="K128" t="str">
+        <v>SARATOGA es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L128" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M128" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -4748,6 +5900,15 @@
       <c r="J129" t="str">
         <v>https://www.facebook.com/inflames</v>
       </c>
+      <c r="K129" t="str">
+        <v>IN FLAMES es una banda de metal alternativo originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L129" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M129" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -4780,6 +5941,15 @@
       <c r="J130" t="str">
         <v>https://www.facebook.com/official.darkmoor?sid=6286</v>
       </c>
+      <c r="K130" t="str">
+        <v>DARK MOOR es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L130" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M130" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -4812,6 +5982,15 @@
       <c r="J131" t="str">
         <v>https://www.facebook.com/ChezKaneVocalist</v>
       </c>
+      <c r="K131" t="str">
+        <v>CHEZ KANE es una banda de hard rock originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L131" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M131" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -4844,6 +6023,15 @@
       <c r="J132" t="str">
         <v>https://www.facebook.com/thebaboonshow</v>
       </c>
+      <c r="K132" t="str">
+        <v>THE BABOON SHOW es una banda de punk rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L132" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M132" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -4876,6 +6064,15 @@
       <c r="J133" t="str">
         <v>https://www.facebook.com/stratovarius</v>
       </c>
+      <c r="K133" t="str">
+        <v>STRATOVARIUS es una banda de power metal originaria de Finlandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L133" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M133" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -4908,6 +6105,15 @@
       <c r="J134" t="str">
         <v/>
       </c>
+      <c r="K134" t="str">
+        <v>XERIA es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L134" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M134" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -4940,6 +6146,15 @@
       <c r="J135" t="str">
         <v>https://www.facebook.com/OfficialWingsofSteel</v>
       </c>
+      <c r="K135" t="str">
+        <v>WINGS OF STEEL es una banda de hard rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L135" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M135" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -4972,6 +6187,15 @@
       <c r="J136" t="str">
         <v>https://www.facebook.com/pages/AGAINST-MYSELF/203937595534</v>
       </c>
+      <c r="K136" t="str">
+        <v>AGAINST MYSELF es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L136" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M136" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -5004,6 +6228,15 @@
       <c r="J137" t="str">
         <v>https://www.facebook.com/employedtoserve</v>
       </c>
+      <c r="K137" t="str">
+        <v>EMPLOYED TO SERVE es una banda de metalcore originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L137" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M137" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -5036,6 +6269,15 @@
       <c r="J138" t="str">
         <v>https://www.facebook.com/DAERIAOFICIAL</v>
       </c>
+      <c r="K138" t="str">
+        <v>DAERIA es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L138" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M138" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -5068,6 +6310,15 @@
       <c r="J139" t="str">
         <v>https://www.facebook.com/MindDriller</v>
       </c>
+      <c r="K139" t="str">
+        <v>MIND DRILLER es una banda de metal industrial originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L139" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M139" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -5100,6 +6351,15 @@
       <c r="J140" t="str">
         <v/>
       </c>
+      <c r="K140" t="str">
+        <v>JORDI WILD DJ SET es una banda de dj set originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L140" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M140" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -5132,6 +6392,15 @@
       <c r="J141" t="str">
         <v/>
       </c>
+      <c r="K141" t="str">
+        <v>GUILT TRIP es una banda de hardcore originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L141" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M141" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -5164,6 +6433,15 @@
       <c r="J142" t="str">
         <v>https://www.facebook.com/OfficialDeicide</v>
       </c>
+      <c r="K142" t="str">
+        <v>DEICIDE es una banda de death metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L142" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M142" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -5196,6 +6474,15 @@
       <c r="J143" t="str">
         <v>https://www.facebook.com/helloweenofficial</v>
       </c>
+      <c r="K143" t="str">
+        <v>HELLOWEEN es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L143" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M143" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -5228,6 +6515,15 @@
       <c r="J144" t="str">
         <v>https://www.facebook.com/profile.php?id=100063786306898</v>
       </c>
+      <c r="K144" t="str">
+        <v>ANKHARA es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L144" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M144" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -5260,6 +6556,15 @@
       <c r="J145" t="str">
         <v>https://www.facebook.com/eihwar.music</v>
       </c>
+      <c r="K145" t="str">
+        <v>EIHWAR es una banda de pagan folk originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L145" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M145" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -5292,6 +6597,15 @@
       <c r="J146" t="str">
         <v>https://www.facebook.com/officialheavenshallburn</v>
       </c>
+      <c r="K146" t="str">
+        <v>HEAVEN SHALL BURN es una banda de melodic death metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L146" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M146" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -5324,6 +6638,15 @@
       <c r="J147" t="str">
         <v>https://www.facebook.com/WarCryOficial</v>
       </c>
+      <c r="K147" t="str">
+        <v>WARCRY es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L147" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M147" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -5356,6 +6679,15 @@
       <c r="J148" t="str">
         <v>https://www.facebook.com/deathandlegacy</v>
       </c>
+      <c r="K148" t="str">
+        <v>DEATH AND LEGACY es una banda de death metal melódico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L148" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M148" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -5388,6 +6720,15 @@
       <c r="J149" t="str">
         <v/>
       </c>
+      <c r="K149" t="str">
+        <v>LATZEN es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L149" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M149" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -5420,6 +6761,15 @@
       <c r="J150" t="str">
         <v>https://www.facebook.com/pages/Hardline/113309705346323</v>
       </c>
+      <c r="K150" t="str">
+        <v>Hardline es una banda estadounidense de hard rock formada por los hermanos Gioeli (Johnny Gioeli y Joey Gioeli) a finales de los 80 y principios de los 90.</v>
+      </c>
+      <c r="L150" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M150" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -5452,6 +6802,15 @@
       <c r="J151" t="str">
         <v>https://www.facebook.com/ten56hq</v>
       </c>
+      <c r="K151" t="str">
+        <v>TEN56. es una banda de deathcore originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L151" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M151" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -5484,6 +6843,15 @@
       <c r="J152" t="str">
         <v>https://www.facebook.com/halfmeband</v>
       </c>
+      <c r="K152" t="str">
+        <v>HALF ME es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L152" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M152" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -5516,6 +6884,15 @@
       <c r="J153" t="str">
         <v>https://www.facebook.com/cabalcph</v>
       </c>
+      <c r="K153" t="str">
+        <v>CABAL es una banda de deathcore originaria de Dinamarca. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L153" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M153" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -5548,6 +6925,15 @@
       <c r="J154" t="str">
         <v/>
       </c>
+      <c r="K154" t="str">
+        <v>Rockerizos es una banda de hard rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L154" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M154" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -5580,6 +6966,15 @@
       <c r="J155" t="str">
         <v>https://www.facebook.com/Uli-Jon-Roth-403059233077097</v>
       </c>
+      <c r="K155" t="str">
+        <v>Uli Jon Roth es una banda de heavy metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L155" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M155" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -5612,6 +7007,15 @@
       <c r="J156" t="str">
         <v>https://www.facebook.com/secretsphere</v>
       </c>
+      <c r="K156" t="str">
+        <v>Secret Sphere es un grupo de power metal italiano, procedentes de la región de Alessandria. Comenzaron su actividad en el verano de 1997 gracias al talentoso guitarrista Aldo Lonobile. Después de algunos cambios de formación durante los primeros días, la formación actual del grupo grabaron su álbum debut "Mistress Of The Shadowlight" en 1999. En el año 2000 Secret Sphere apareció en prestigioso homenaje a Helloween "Keepers Of Jericho" junto a grandes nombres como Sonata Arctica, Rhapsody, Trick or Treat entre otras.</v>
+      </c>
+      <c r="L156" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M156" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -5644,6 +7048,15 @@
       <c r="J157" t="str">
         <v/>
       </c>
+      <c r="K157" t="str">
+        <v>Azrael es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L157" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M157" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -5676,6 +7089,15 @@
       <c r="J158" t="str">
         <v>https://www.facebook.com/furyofficial</v>
       </c>
+      <c r="K158" t="str">
+        <v>Fury es una banda de heavy metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L158" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M158" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -5708,6 +7130,15 @@
       <c r="J159" t="str">
         <v/>
       </c>
+      <c r="K159" t="str">
+        <v>Masters of Ceremony es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L159" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M159" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -5740,6 +7171,15 @@
       <c r="J160" t="str">
         <v>https://www.facebook.com/iameden</v>
       </c>
+      <c r="K160" t="str">
+        <v>Eden es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L160" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M160" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -5772,6 +7212,15 @@
       <c r="J161" t="str">
         <v>https://www.facebook.com/OfficialHardcoreSuperstar</v>
       </c>
+      <c r="K161" t="str">
+        <v>Hardcore Superstar es una banda de sleaze rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L161" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M161" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -5804,6 +7253,15 @@
       <c r="J162" t="str">
         <v>https://www.facebook.com/savagedheavy</v>
       </c>
+      <c r="K162" t="str">
+        <v>Savaged es una banda de speed metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L162" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M162" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -5836,6 +7294,15 @@
       <c r="J163" t="str">
         <v>https://www.facebook.com/OverkillWreckingCrew</v>
       </c>
+      <c r="K163" t="str">
+        <v>Overkill es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L163" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M163" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -5868,6 +7335,15 @@
       <c r="J164" t="str">
         <v/>
       </c>
+      <c r="K164" t="str">
+        <v>Hitten es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L164" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M164" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -5900,6 +7376,15 @@
       <c r="J165" t="str">
         <v>https://www.facebook.com/inductionofficial</v>
       </c>
+      <c r="K165" t="str">
+        <v>Induction es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L165" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M165" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -5932,6 +7417,15 @@
       <c r="J166" t="str">
         <v>https://www.facebook.com/ArsAmandiRock</v>
       </c>
+      <c r="K166" t="str">
+        <v>Ars Amandi es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L166" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M166" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -5964,6 +7458,15 @@
       <c r="J167" t="str">
         <v>https://www.facebook.com/profile.php?id=61555780541728</v>
       </c>
+      <c r="K167" t="str">
+        <v>Bloodstain es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L167" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M167" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -5996,6 +7499,15 @@
       <c r="J168" t="str">
         <v>https://www.facebook.com/thepoodles</v>
       </c>
+      <c r="K168" t="str">
+        <v>The Poodles es una banda de glam metal originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L168" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M168" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -6028,6 +7540,15 @@
       <c r="J169" t="str">
         <v/>
       </c>
+      <c r="K169" t="str">
+        <v>Khorea es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L169" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M169" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -6060,6 +7581,15 @@
       <c r="J170" t="str">
         <v/>
       </c>
+      <c r="K170" t="str">
+        <v>Heavens Gate es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L170" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M170" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -6092,6 +7622,15 @@
       <c r="J171" t="str">
         <v>https://www.facebook.com/ODCOfficiel</v>
       </c>
+      <c r="K171" t="str">
+        <v>ODC es una banda de metal alternativo originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L171" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M171" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -6124,6 +7663,15 @@
       <c r="J172" t="str">
         <v>https://www.facebook.com/DoroPeschOfficialGerman</v>
       </c>
+      <c r="K172" t="str">
+        <v>Doro es una banda de heavy metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L172" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M172" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -6156,6 +7704,15 @@
       <c r="J173" t="str">
         <v>https://www.facebook.com/bulletband</v>
       </c>
+      <c r="K173" t="str">
+        <v>Bullet es una banda sueca de heavy metal, fundada en Växjö por Hampus Klang y Dag "Hell" Hofer en 2001. ​ El cantante de Iron Maiden, Bruce Dickinson, tocó la canción de Bullet "Turn it Up Loud" de su álbum Heading For The Top en su programa de radio en la BBC de 2006. En 2008, Bullet lanzó su segundo álbum, Bite the Bullet . 000 personas) antes del partido de la NHL entre Detroit Red Wings y St. ​ Su tercer álbum, Highway Pirates, fue lanzado a principios de 2011.</v>
+      </c>
+      <c r="L173" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M173" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -6188,10 +7745,19 @@
       <c r="J174" t="str">
         <v/>
       </c>
+      <c r="K174" t="str">
+        <v>Vindicta es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+      </c>
+      <c r="L174" t="str">
+        <v>2026-07-11</v>
+      </c>
+      <c r="M174" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M174"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sincronizadas redes de Zurbarán, solucionado problema de miniaturas en vista vertical HoursView y reemplazadas biografías genéricas incorrectas
</commit_message>
<xml_diff>
--- a/AgendaFest.xlsx
+++ b/AgendaFest.xlsx
@@ -611,6 +611,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
@@ -694,10 +695,10 @@
         <v>https://www.facebook.com/annisokay</v>
       </c>
       <c r="K2" t="str">
-        <v>ANNISOKAY es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Annisokay es una banda alemana de post-hardcore de Halle, Sajonia-Anhalt. Hasta la fecha, la banda ha publicado dos demos, dos EPs y cinco álbumes de estudio: The Lucid Dream[er] se autoeditó en 2012 (en 2013 a través de Radtone Records en Japón) y se reeditó en 2014 cuando la banda firmó un contrato con el sello SPV GmbH. º 68 en las listas de éxitos alemanas. La banda realizó varias giras por Alemania y tocó junto a artistas como Silverstein, Callejon y Electric Callboy. Tocaron en la edición de 2014 del Summer Breeze Open Air y en el Festival Mair1 de Montabaur.</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
@@ -735,10 +736,10 @@
         <v>https://www.facebook.com/crowdedhouse</v>
       </c>
       <c r="K3" t="str">
-        <v>CROWDED es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Crowded es una banda española de metal alternativo y grunge. Formada por músicos con una amplia experiencia, su sonido se caracteriza por guitarras potentes con mucha distorsión, ritmos densos y voces melódicas y expresivas influenciadas por el rock de los 90.</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M3" t="b">
         <v>1</v>
@@ -776,10 +777,10 @@
         <v>https://www.facebook.com/profile.php?id=100085118077210</v>
       </c>
       <c r="K4" t="str">
-        <v>ANEUMA es una banda de death metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M4" t="b">
         <v>1</v>
@@ -817,10 +818,10 @@
         <v>https://www.facebook.com/MWAMjapan</v>
       </c>
       <c r="K5" t="str">
-        <v>MAN WITH A MISSION es una banda de rock alternativo originaria de Japón. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>​ Muchos de sus sencillos han sido usados como temas para una variedad de animes, películas, y videojuegos.</v>
       </c>
       <c r="L5" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M5" t="b">
         <v>1</v>
@@ -858,10 +859,10 @@
         <v>https://www.facebook.com/GodComplexUK</v>
       </c>
       <c r="K6" t="str">
-        <v>GOD COMPLEX es una banda de metalcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>El complejo de Dios (The God Complex) es el undécimo episodio de la sexta temporada moderna de la serie británica de ciencia ficción Doctor Who, emitido originalmente el 17 de septiembre de 2011.</v>
       </c>
       <c r="L6" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M6" t="b">
         <v>1</v>
@@ -899,10 +900,10 @@
         <v>https://www.facebook.com/TheSundaySadness</v>
       </c>
       <c r="K7" t="str">
-        <v>TSS es una banda de metal moderno originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>TSS es una banda de metal moderno originaria de Francia.</v>
       </c>
       <c r="L7" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M7" t="b">
         <v>1</v>
@@ -940,10 +941,10 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>BLACK MARACAS es una banda de garaje rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Acquiring the taste fue el segundo disco de la banda británica de rock progresivo Gentle Giant, publicado el 16 de julio de 1971. Considerado como uno de los mejores álbumes de la banda por sus fanes, este álbum representa una gran mejora en cuanto a arreglos y producción con respecto al álbum de debut de la banda, Gentle Giant.​</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M8" t="b">
         <v>1</v>
@@ -981,10 +982,10 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>PRESIDENT es una banda de hard rock originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>President (estilizado en mayúsculas como PRESIDENT) es una banda británica anónima de hard rock y metal alternativo formada en 2025. ​ Lanzaron su primer EP, King of Terrors, en 2025 que superó los 50 millones de reproducciones en Spotify dentro de los seis meses posteriores a su lanzamiento.</v>
       </c>
       <c r="L9" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M9" t="b">
         <v>1</v>
@@ -1022,10 +1023,10 @@
         <v>https://www.facebook.com/immortaldisfigurement</v>
       </c>
       <c r="K10" t="str">
-        <v>IMMORTAL DISFIGUREMENT es una banda de deathcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Immortal Disfigurement is an estadounidense deathcore band, formada en 2021 by vocalist CJ McCreery and guitarist Josh Freeman. The band is known as part of the symphonic deathcore scene. The group currently consists of CJ McCreery on vocals, Josh Freeman and Jacob Toy on guitars, Shane Slade on bass and Suki on drums.</v>
       </c>
       <c r="L10" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M10" t="b">
         <v>1</v>
@@ -1063,10 +1064,10 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>THE PRETTY WILD es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Pretty Wild es un dúo musical estadounidense formada desde Las Vegas, Nevada en 2022 y está compuesta por las hermanas Jyl y Jules Wylde. La banda tiene contrato con Sumerian Records.​</v>
       </c>
       <c r="L11" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M11" t="b">
         <v>1</v>
@@ -1104,10 +1105,10 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>CARDIAC es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Cardiac Arrest es un bootleg en vivo de la banda británica Queen. Fue publicada originalmente en formato CD a mediados de los 80s por Green Hippo Records.​ El álbum fue relanzado en 2020 por Soul Flux Recordings en Japón, como un lanzamiento de edición limitada.​</v>
       </c>
       <c r="L12" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M12" t="b">
         <v>1</v>
@@ -1145,10 +1146,10 @@
         <v>https://www.facebook.com/TheScratchMusic</v>
       </c>
       <c r="K13" t="str">
-        <v>THE SCRATCH es una banda de folk rock originaria de Irlanda. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Scratch es una banda irlandesa de rock acústico y folk metal formada en Dublín. Fusionando la velocidad y agresividad del metal clásico con la instrumentación acústica tradicional irlandesa, su sonido único destaca por el uso de guitarras acústicas percusivas y coros enérgicos.</v>
       </c>
       <c r="L13" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M13" t="b">
         <v>1</v>
@@ -1186,10 +1187,10 @@
         <v>https://www.facebook.com/thrownband</v>
       </c>
       <c r="K14" t="str">
-        <v>THROWN es una banda de hardcore punk originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Thrown es una banda sueca de hardcore punk y metalcore formada en Stockholm, Suecia en 2019 y firmada con Arising Empire. El grupo está compuesto por el vocalista Marcus Lundqvist, los guitarristas Johan Liljeblad y Andreas Malm, y el baterista y productor Buster Odeholm (Humanity's Last Breath y Vildhjärta). La banda lanzó su primer álbum Excessive Guilt (estilizado en mayúsculas) en agosto de 2024 compuesto por 11 canciones con una duración total de poco más de 20 minutos.​</v>
       </c>
       <c r="L14" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M14" t="b">
         <v>1</v>
@@ -1227,10 +1228,10 @@
         <v>https://www.facebook.com/TheBrowningOfficial</v>
       </c>
       <c r="K15" t="str">
-        <v>THE BROWNING es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Browning is an estadounidense electronicore band formed in Kansas City, Missouri, in 2005. The band's musical style is characterized by an eclectic blending of electronicore, deathcore, and metalcore. The group currently consists of vocalist Jonny McBee, drummer Keenan Bivens, and bassist/guitarist Akeem Bivens. They are currently signed to FiXT. The band has released six studio albums and two EPs.</v>
       </c>
       <c r="L15" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M15" t="b">
         <v>1</v>
@@ -1268,10 +1269,10 @@
         <v>https://www.facebook.com/lasttrainofficial</v>
       </c>
       <c r="K16" t="str">
-        <v>LAST TRAIN es una banda de rock alternativo originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Last Train es una banda francesa de rock alternativo e indie rock formada en 2007. El cuarteto destaca por su propuesta de rock clásico y crudo, cargada de intensidad emocional, riffs de guitarra atmosféricos y potentes directos que les han ganado reconocimiento en Europa.</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M16" t="b">
         <v>1</v>
@@ -1309,10 +1310,10 @@
         <v>https://www.facebook.com/adtr</v>
       </c>
       <c r="K17" t="str">
-        <v>A DAY TO REMEMBER es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>A Day to Remember (abreviado comúnmente ADTR) es una banda estadounidense de Pop Punk y Metalcore formada en Ocala, Florida, en 2003. Se caracterizan por la fusión del metalcore con el pop punk. El grupo se encuentra actualmente formado por Jeremy McKinnon (voz), Neil Westfall (guitarra rítmica), Alex Shelnutt (batería) y Kevin Skaff (guitarra principal).</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M17" t="b">
         <v>1</v>
@@ -1350,10 +1351,10 @@
         <v>https://www.facebook.com/gettheshothc</v>
       </c>
       <c r="K18" t="str">
-        <v>GET THE SHOT es una banda de hardcore originaria de Canada. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Get the Shot es una banda de hardcore punk originaria de Quebec, Canadá. Formada en 2009, su música destaca por una violenta mezcla de thrash metal y hardcore de la vieja escuela, con ritmos rápidos, breakdowns pesados y letras de crítica social.</v>
       </c>
       <c r="L18" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M18" t="b">
         <v>1</v>
@@ -1391,10 +1392,10 @@
         <v>https://www.facebook.com/selfdeceptionsthlm</v>
       </c>
       <c r="K19" t="str">
-        <v>SELF DECEPTION es una banda de metalcore originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Self Deception es una banda de rock moderno y metal alternativo formada en Estocolmo, Suecia, en 2005. Con un sonido dinámico que combina riffs de guitarra pesados, estribillos melódicos memorables y elementos electrónicos, tienen una amplia presencia en plataformas de streaming.</v>
       </c>
       <c r="L19" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M19" t="b">
         <v>1</v>
@@ -1432,10 +1433,10 @@
         <v>https://www.facebook.com/lampr3a</v>
       </c>
       <c r="K20" t="str">
-        <v>LAMPR3A es una banda de metal progresivo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L20" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M20" t="b">
         <v>1</v>
@@ -1473,10 +1474,10 @@
         <v>https://www.facebook.com/sabaton</v>
       </c>
       <c r="K21" t="str">
-        <v>SABATON es una banda de power metal originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Sabaton es una banda sueca de power metal formada en 1999 en la ciudad de Falun. El grupo se caracteriza por su estética militarizada y sus letras de contenido histórico-bélico.​ Su nombre proviene de una pieza de armadura medieval que cubre el empeine del pie, conocida como escarpe en español.</v>
       </c>
       <c r="L21" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M21" t="b">
         <v>1</v>
@@ -1514,10 +1515,10 @@
         <v>https://www.facebook.com/highvispunk</v>
       </c>
       <c r="K22" t="str">
-        <v>HIGH-VIS es una banda de hardcore punk originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>La BRIT School para las Artes Escénicas y la Tecnología es un colegio situado en Croydon, Inglaterra, centrado en proveer educación y entrenamiento vocacional para la actuación, los medios, el arte y el diseño y la tecnología que hace todo eso posible. El colegio es notable por su elevado número de alumnos reconocidos, incluyendo a las cantantes Amy Winehouse, Leona Lewis, Adele, Jessie J y FKA Twigs.</v>
       </c>
       <c r="L22" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M22" t="b">
         <v>1</v>
@@ -1555,10 +1556,10 @@
         <v>https://www.facebook.com/faetoothband</v>
       </c>
       <c r="K23" t="str">
-        <v>FAETOOTH es una banda de doom originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>FAETOOTH es una banda de metal originaria de estadounidense doom. Their sound features elements de sludge metal, shoegaze and post-metal, and many of their lyrics deal with themes of folklore and spirituality; the band describes their musical style as "fairy-doom metal".</v>
       </c>
       <c r="L23" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M23" t="b">
         <v>1</v>
@@ -1596,10 +1597,10 @@
         <v>https://www.facebook.com/testamentlegions</v>
       </c>
       <c r="K24" t="str">
-        <v>TESTAMENT es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Testament (estilizado TestAmenT) es una banda estadounidense de thrash metal de Berkeley, California. Hasta la fecha han publicado trece álbumes de estudio, cuatro álbumes en vivo y seis álbumes recopilatorios, tiene tres discos que entraron en el top-50 en las listas inglesas y en 1999 con el disco The Gathering entró en el top-50 alemán.</v>
       </c>
       <c r="L24" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M24" t="b">
         <v>1</v>
@@ -1637,10 +1638,10 @@
         <v/>
       </c>
       <c r="K25" t="str">
-        <v>ARSON TIDES es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Down es una banda estadounidense de metal que basa su estilo en el sludge metal y doom metal fusionado con rock sureño y stoner rock, además de elementos de swamp blues y louisiana blues. Se formaron en el año 1991 en Nueva Orleans, Luisiana. La formación actual de la banda consiste en el vocalista Phil Anselmo, los guitarristas Pepper Keenan y Kirk Windstein, el bajista Pat Bruders y el batería Jimmy Bower. Desde su formación, Down se ha separado y reformado en dos ocasiones.</v>
       </c>
       <c r="L25" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M25" t="b">
         <v>1</v>
@@ -1678,10 +1679,10 @@
         <v>https://www.facebook.com/FallenAtDawnOfficial</v>
       </c>
       <c r="K26" t="str">
-        <v>FALLEN AT DAWN es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Fallen at Dawn es una banda española de metalcore formada en Madrid. Con influencias de grupos de metal moderno y post-hardcore, la formación destaca por su directo potente, alternando voces melódicas y guturales con riffs de guitarra agresivos y bases rítmicas contundentes.</v>
       </c>
       <c r="L26" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M26" t="b">
         <v>1</v>
@@ -1719,10 +1720,10 @@
         <v/>
       </c>
       <c r="K27" t="str">
-        <v>FUET! es una banda de hardcore melódico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Las fiestas patronales de Menorca son de tradición centenaria que tienen su origen en las Fiestas de San Juan, que se celebran en Ciudadela, isla de Menorca, en España, desde el siglo XIV. El principal protagonista de las fiestas es el caballo. Los jinetes cajeros (o caixers), vestidos de blanco y negro, van sobre sus caballos por las calles del pueblo, hasta que una vez recogidos todos y después de la misa, se celebra el tradicional jaleo (no debe confundirse con el jaleo, cante y baile flamenco).</v>
       </c>
       <c r="L27" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M27" t="b">
         <v>1</v>
@@ -1760,10 +1761,10 @@
         <v/>
       </c>
       <c r="K28" t="str">
-        <v>HER ANXIETY es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Her Anxiety es una banda española de metalcore y metal alternativo formada en Vigo, Galicia. Liderada por una vocalista femenina con una gran versatilidad de registros, la banda fusiona melodías pegadizas con breakdowns pesados y texturas electrónicas contemporáneas.</v>
       </c>
       <c r="L28" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M28" t="b">
         <v>1</v>
@@ -1801,10 +1802,10 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>SILLY GOOSE es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Silly Goose es una banda estadounidense de rap metal y nu metal formada en Atlanta, Georgia. Conocidos por sus improvisadas actuaciones callejeras sobre remolques de camiones y su energía rebelde, rescatan la esencia del rapcore de finales de los noventa.</v>
       </c>
       <c r="L29" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M29" t="b">
         <v>1</v>
@@ -1842,10 +1843,10 @@
         <v>https://www.facebook.com/casketsbandofficial</v>
       </c>
       <c r="K30" t="str">
-        <v>CASKETS es una banda de post hardcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Caskets es una banda británica de post-hardcore de Leeds, formada en 2018. La banda tiene contrato con SharpTone Records y actualmente está formada por el vocalista principal Matthew Flood, el guitarrista principal Benjamin Wilson, el guitarrista rítmico Craig Robinson y el baterista James Lazenby.</v>
       </c>
       <c r="L30" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M30" t="b">
         <v>1</v>
@@ -1883,10 +1884,10 @@
         <v>https://www.facebook.com/bloodcommand</v>
       </c>
       <c r="K31" t="str">
-        <v>BLOOD COMMAND es una banda de punk rock originaria de Noruega. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Blood Command es una banda de punk rock y deathpop originaria de Bergen, Noruega. Formada en 2008, su música destaca por una explosiva mezcla de ritmos de batería de alta velocidad, riffs gancheros y voces enérgicas llenas de actitud punk.</v>
       </c>
       <c r="L31" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M31" t="b">
         <v>1</v>
@@ -1924,10 +1925,10 @@
         <v>https://www.facebook.com/burningwitches666</v>
       </c>
       <c r="K32" t="str">
-        <v>BURNING WITCHES es una banda de heavy metal originaria de Suiza. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Burning witch fue una banda musical estadounidense proveniente de Seattle, Washington, de Doom metal, formada en el año 1995. Burning Witch fue una banda estadounidense de doom / sludge metal originaria de Seattle , Washington , activa entre 1995 y 1998. Además de EPs y lanzamientos compartidos, la banda publicó un álbum recopilatorio llamado Crippled Lucifer , que incluía canciones de sus primeros EPs.</v>
       </c>
       <c r="L32" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M32" t="b">
         <v>1</v>
@@ -1965,10 +1966,10 @@
         <v>https://www.facebook.com/angelusapatrida</v>
       </c>
       <c r="K33" t="str">
-        <v>ANGELUS APATRIDA es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>ANGELUS APATRIDA es una banda de thrash metal originaria de España.</v>
       </c>
       <c r="L33" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M33" t="b">
         <v>1</v>
@@ -2006,10 +2007,10 @@
         <v>https://www.facebook.com/BluesPills</v>
       </c>
       <c r="K34" t="str">
-        <v>BLUES PILLS es una banda de psicodelia originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Blues Pills es una banda de blues-rock formada por la vocalista sueca Elin Larsson, el guitarrista estadounidense Zack Anderson, el bajista Kristoffer Schander y el batería sueco André Kvarnström, quien sustituyó a Cory Berry poco después del lanzamiento del álbum Blues Pills.​ El guitarrista francés Dorian Sorriaux, miembro original de la banda, dejó la formación a finales de 2018 y su puesto en la guitarra fue tomado por el hasta entonces bajista Zack Anderson.​</v>
       </c>
       <c r="L34" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M34" t="b">
         <v>1</v>
@@ -2047,10 +2048,10 @@
         <v>https://www.facebook.com/thefuneralportrait</v>
       </c>
       <c r="K35" t="str">
-        <v>THE FUNERAL PORTRAIT es una banda de post hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Funeral Portrait es una banda estadounidense de post-hardcore formada en Atlanta, Georgia. El grupo se formó en 2014 y actualmente está compuesto por Lee Jennings (voz), Cody Weissinger (guitarra principal), Caleb Freihaut (guitarra rítmica/auxiliar), Robert Weston (bajo) y Homer Umbanhower (batería).</v>
       </c>
       <c r="L35" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M35" t="b">
         <v>1</v>
@@ -2088,10 +2089,10 @@
         <v>https://www.facebook.com/belvedere669</v>
       </c>
       <c r="K36" t="str">
-        <v>BELVEDERE es una banda de punk rock originaria de Canada. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Belvedere es una banda de punk rock canadiense formada en 1995. Bien conocida por su velocidad y sus voces melódicas. La banda consiguió ganarse un hueco en la escena de culto punk canadiense. La banda llegó a tocar en el Warped Tour y en el Groezrock Festival.</v>
       </c>
       <c r="L36" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M36" t="b">
         <v>1</v>
@@ -2129,10 +2130,10 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v>CICLONAUTAS es una banda de rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Ciclonautas es un grupo hispanoargentino de música rock formado en 2013 en Navarra por el argentino Mariano 'Mai' Medina y los españoles Javier 'Txo' Pintor y Alén Ayerdi.</v>
       </c>
       <c r="L37" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M37" t="b">
         <v>1</v>
@@ -2170,10 +2171,10 @@
         <v>https://www.facebook.com/ironmaiden</v>
       </c>
       <c r="K38" t="str">
-        <v>IRON MAIDEN es una banda de heavy metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Iron Maiden es una banda británica de heavy metal fundada en Londres en 1975 por el bajista Steve Harris. Considerada una de las agrupaciones más importantes y representativas del género, han vendido más de 180 millones de discos en el mundo,​ a pesar de haber contado con poco apoyo de los medios de comunicación masiva durante la mayor parte de su carrera. ​​ La agrupación ha obtenido reconocimientos como el Premio Ivor Novello en la categoría de «Logro Internacional» en 2002. En 2005 fueron incluidos en el Hollywood's RockWalk en Sunset Boulevard, Los Ángeles.</v>
       </c>
       <c r="L38" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M38" t="b">
         <v>1</v>
@@ -2211,10 +2212,10 @@
         <v>https://www.facebook.com/thecallousdaoboys</v>
       </c>
       <c r="K39" t="str">
-        <v>THE CALLOUS DAOBOYS es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Callous Daoboys es una banda estadounidense de metalcore formada en Atlanta, Georgia en 2016. Su nombre es un "spoonerism" del equipo de fútbol americano Dallas Cowboys.</v>
       </c>
       <c r="L39" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M39" t="b">
         <v>1</v>
@@ -2252,10 +2253,10 @@
         <v>https://www.facebook.com/vulvarine.vienna</v>
       </c>
       <c r="K40" t="str">
-        <v>VULVARINE es una banda de hard rock originaria de Austria. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>VULVARINE es una banda de hard rock originaria de Austria.</v>
       </c>
       <c r="L40" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M40" t="b">
         <v>1</v>
@@ -2293,10 +2294,10 @@
         <v>https://www.facebook.com/CalibanOfficial</v>
       </c>
       <c r="K41" t="str">
-        <v>CALIBAN es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Caliban es una banda alemana de metalcore originaria de Hattingen, Renania del Norte-Westfalia que lleva nueve álbumes lanzados hasta el momento. Aunque la banda tiene un sonido metalcore ellos declaran que son un grupo de hardcore.</v>
       </c>
       <c r="L41" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M41" t="b">
         <v>1</v>
@@ -2334,10 +2335,10 @@
         <v>https://www.facebook.com/lionheartca</v>
       </c>
       <c r="K42" t="str">
-        <v>LIONHEART es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>LIONHEART es una banda de hardcore originaria de EEUU.</v>
       </c>
       <c r="L42" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M42" t="b">
         <v>1</v>
@@ -2375,10 +2376,10 @@
         <v>https://www.facebook.com/anthrax</v>
       </c>
       <c r="K43" t="str">
-        <v>ANTHRAX es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Anthrax es una banda estadounidense de thrash metal formada en Nueva York en 1981, por el guitarrista Scott Ian y el bajista Dan Lilker.​ Está considerado como uno de los grupos principales de la escena thrash junto a Metallica, Megadeth y Slayer.​​ Entre 1991 y 2004, vendió cerca de 2,5 millones de copias únicamente en los Estados Unidos y 10 millones en todo el mundo.​​ En 1983, Anthrax firmó un contrato con la discográfica independiente Megaforce Records, a través de la cual publicó su álbum debut con su actual batería, Charlie Benante.​ Lilker pronto abandonó la formación y le reemplazó Frank Bello, sobrino de Benante,​​ además, el vocalista Joey Belladonna también ingresó.​ Con la llegada de estos nuevos integrantes, la banda lanzó al mercado Spreading the Disease (1985) y Among the Living (1987), aunque Belladonna dejó el conjunto en 1992 y le sustituyó John Bush, con el cual grabó Sound of White Noise (1993),​ que alcanzó la séptima posición del Billboard 200.​ Sus tres siguientes trabajos —Stomp 442 (1995), Volume 8: The Threat Is Real (1998) y We've Come for You All (2003)— no tuvieron el éxito comercial de su antecesor y en 2005,​ Belladonna y el guitarrista Dan Spitz regresaron a la banda para una esporádica reunión.​ En 2010, después de varios cambios de vocalista, Belladonna regresó al grupo una vez más para grabar Worship Music (2011) y For All Kings (2016).​</v>
       </c>
       <c r="L43" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M43" t="b">
         <v>1</v>
@@ -2416,10 +2417,10 @@
         <v>https://www.facebook.com/psychonautband</v>
       </c>
       <c r="K44" t="str">
-        <v>PSYCHONAUT es una banda de post metal originaria de Bélgica. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Psychonaut 4 es una banda georgiana de depressive suicidal black metal formada en 2010.​ El nombre de la banda deriva del término «psiconauta», que describe a una persona que consume drogas psicodélicas con frecuencia, mientras que el número cuatro hace referencia a los cuatro niveles de euforia asociados al uso de dextrometorfano.​ Las letras de la banda suelen estar en georgiano, ruso e inglés.​​​ La banda ha publicado cinco álbumes de estudio; el más reciente es «...of Mourning», de 2024.​ Para 2020, ya se había presentado en 24 países.​</v>
       </c>
       <c r="L44" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M44" t="b">
         <v>1</v>
@@ -2457,10 +2458,10 @@
         <v>https://www.facebook.com/authorityzero.official</v>
       </c>
       <c r="K45" t="str">
-        <v>AUTHORITY ZERO es una banda de punk rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Coca-Cola Zero (Coca-Cola Zero Azúcar​ en España) es una bebida producida por The Coca-Cola Company, que es una versión de Coca-Cola sin azúcar. Su eslogan es «Zero calorías»,​ sin embargo, en otros países también se conoce como «Zero azúcar» o «Zero sugar».</v>
       </c>
       <c r="L45" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M45" t="b">
         <v>1</v>
@@ -2498,10 +2499,10 @@
         <v>https://www.facebook.com/feuerschwanz</v>
       </c>
       <c r="K46" t="str">
-        <v>FEUERSCHWANZ es una banda de folk metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Feuerschwanz (en español: «Cola de Fuego») es una banda alemana de folk metal, proveniente de Erlangen. Fundada en 2004 por el músico Peter Henrici, junto con Tobias Heindl y Andre Linke. La agrupación comenzó siendo una banda de rock cómico que hacía burla de la escena de rock y metal medieval. Con el tiempo la banda ha cambiado su sonido hacia el folk metal y en ocasiones con temáticas más serias, siendo una de las agrupaciones alemanas de Folk metal más aclamadas en la actualidad.​</v>
       </c>
       <c r="L46" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M46" t="b">
         <v>1</v>
@@ -2539,10 +2540,10 @@
         <v>https://www.facebook.com/TheFallOfAtlantis</v>
       </c>
       <c r="K47" t="str">
-        <v>THE FALL OF ATLANTIS es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Fall of Atlantis es una banda de metalcore y deathcore originaria de España. Sus composiciones se caracterizan por una gran agresividad sonora, ritmos técnicos de batería, breakdowns demoledores y temáticas oscuras en sus letras.</v>
       </c>
       <c r="L47" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M47" t="b">
         <v>1</v>
@@ -2580,10 +2581,10 @@
         <v/>
       </c>
       <c r="K48" t="str">
-        <v>NUKORE es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>NUKORE es una banda de hardcore originaria de España.</v>
       </c>
       <c r="L48" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M48" t="b">
         <v>1</v>
@@ -2621,10 +2622,10 @@
         <v/>
       </c>
       <c r="K49" t="str">
-        <v>BLAZE THE TRAIL es una banda de hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Los Portland Trail Blazers (en español, Pioneros de Portland), también conocidos simplemente como Blazers, son un equipo profesional de baloncesto de los Estados Unidos con sede en Portland, Oregón. ​ Seis jugadores que pertenecen al Basketball Hall of Fame han vestido la camiseta de los Blazers (Lenny Wilkens, Bill Walton, Clyde Drexler, Dražen Petrović, Arvydas Sabonis y Scottie Pippen)​ y cuatro han sido reconocido por la NBA como uno de los 50 mejores jugadores de la historia de la liga (Scottie Pippen, Lenny Wilkens, Bill Walton y Clyde Drexler).</v>
       </c>
       <c r="L49" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M49" t="b">
         <v>1</v>
@@ -2662,10 +2663,10 @@
         <v>https://www.facebook.com/pantsoffmusic</v>
       </c>
       <c r="K50" t="str">
-        <v>PANTS OFF es una banda de punk rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Pants Off es una banda española de punk rock formada en Barcelona. Con un estilo fuertemente influenciado por el punk pop de los años 90 y bandas como Blink-182, sus composiciones destacan por su dinamismo, letras pegadizas y un directo divertido.</v>
       </c>
       <c r="L50" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M50" t="b">
         <v>1</v>
@@ -2703,10 +2704,10 @@
         <v/>
       </c>
       <c r="K51" t="str">
-        <v>NOT YET es una banda de post hardcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Not Yet es una banda española de post-hardcore y metal alternativo. Formada por jóvenes músicos, el grupo destaca por su capacidad de mezclar pasajes melódicos emocionales con secciones pesadas de gran contundencia sonora.</v>
       </c>
       <c r="L51" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M51" t="b">
         <v>1</v>
@@ -2744,10 +2745,10 @@
         <v>https://www.facebook.com/madmessband</v>
       </c>
       <c r="K52" t="str">
-        <v>MADMESS es una banda de rock psicodélico originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>ArcTanGent Festival (also known as ATG) is a three-day británica rock festival held annually at Fernhill Farm in Somerset, England since 2013. It is the most popular británica summer festival for math rock, post rock, progressive metal and experimental music. The festival is named after the Earthtone9 album arc'tan'gent (2000). Previous performers include Heilung, Mogwai, Meshuggah, Devin Townsend, Explosions in the Sky, Coheed &amp; Cambria, Opeth, Glassjaw, Godspeed You!</v>
       </c>
       <c r="L52" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M52" t="b">
         <v>1</v>
@@ -2785,10 +2786,10 @@
         <v>https://www.facebook.com/therasmusofficial</v>
       </c>
       <c r="K53" t="str">
-        <v>THE RASMUS es una banda de rock melodico originaria de Finlandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Rasmus es una banda finlandesa de rock gótico formada en Helsinki en 1994. Los miembros originales de la banda son Lauri Ylönen (vocalista y compositor), Pauli Rantasalmi (guitarra) –quien dejó la banda a principios de 2022, siendo reemplazado por Emilia Suhonen–, Eero Heinonen (bajo) y Jarno Lahti (batería), siendo este último reemplazado por Janne Heiskanen en 1995. Heiskanen dejaría la banda poco después, en 1998, tras lo cual Aki Hakala ocupó su lugar. En 2022 representaron a su país en el Festival de la Canción de Eurovisión con el tema Jezebel.</v>
       </c>
       <c r="L53" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M53" t="b">
         <v>1</v>
@@ -2826,10 +2827,10 @@
         <v>https://www.facebook.com/osloovniesband</v>
       </c>
       <c r="K54" t="str">
-        <v>OSLO OVNIES es una banda de rock alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>OSLO OVNIES es una banda de rock alternativo originaria de España.</v>
       </c>
       <c r="L54" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M54" t="b">
         <v>1</v>
@@ -2867,10 +2868,10 @@
         <v/>
       </c>
       <c r="K55" t="str">
-        <v>OKKULTIST es una banda de death metal originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Dimmu Borgir es una banda noruega de black metal sinfónico, fundada en 1993 por Ian Kenneth Åkesson (Tjodalv), Stian Thoresen (Shagrath) y Sven Atle Kopperud (Silenoz) en la ciudad de Oslo. Estos dos últimos han sido los únicos miembros estables desde entonces. [1] Desde su debut en 1994, la banda ha recibido tres premios Spellemann (conocidos como el Grammy noruego): en 2001 por Puritanical Euphoric Misanthropia, en 2003 por Death Cult Armageddon y en 2007 por el videoclip de «The Serpentine Offering»; también han participado en festivales como el Inferno Festival, Ozzfest, Download Festival, Dynamo Open Air y el Wacken Open Air.</v>
       </c>
       <c r="L55" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M55" t="b">
         <v>1</v>
@@ -2908,10 +2909,10 @@
         <v>https://www.facebook.com/movrir</v>
       </c>
       <c r="K56" t="str">
-        <v>MOURIR es una banda de black metal originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Mourir es un proyecto francés de black metal y sludge metal. Formado por miembros de la escena underground francesa, su propuesta destaca por crear atmósferas asfixiantes, densas y oscuras que combinan la velocidad del black con el peso del sludge.</v>
       </c>
       <c r="L56" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M56" t="b">
         <v>1</v>
@@ -2949,10 +2950,10 @@
         <v>https://www.facebook.com/bleedfromwithinband</v>
       </c>
       <c r="K57" t="str">
-        <v>BLEED FROM WITHIN es una banda de metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Bleed de Within are a Scottish metalcore band de Glasgow, formada en 2005. The band's current lineup consists of lead vocalist Scott Kennedy, drummer Ali Richardson, bassist Davie Provan, lead guitarist Craig Gowans, and rhythm guitarist, clean vocalist Steven Jones. The band has released seven studio albums and three EPs, with their latest Zenith released in 2025 through Nuclear Blast.</v>
       </c>
       <c r="L57" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M57" t="b">
         <v>1</v>
@@ -2990,10 +2991,10 @@
         <v/>
       </c>
       <c r="K58" t="str">
-        <v>INITIATE es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Initiate es una banda estadounidense de hardcore punk originaria de California. Con una propuesta directa y llena de convicción, destacan por sus letras sociales y políticas, la crudeza de sus guitarras y la intensidad escénica de su vocalista.</v>
       </c>
       <c r="L58" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M58" t="b">
         <v>1</v>
@@ -3031,10 +3032,10 @@
         <v>https://www.facebook.com/HulderUS</v>
       </c>
       <c r="K59" t="str">
-        <v>HULDER es una banda de black metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Hulder es un proyecto unipersonal de black metal tradicional fundado por la artista belga Marz Riesterer en Oregón, Estados Unidos. Su música rinde homenaje al crudo black metal de los años noventa, con atmósferas medievales y voces desgarradoras.</v>
       </c>
       <c r="L59" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M59" t="b">
         <v>1</v>
@@ -3072,10 +3073,10 @@
         <v>https://www.facebook.com/RosalieCunninghamOfficial</v>
       </c>
       <c r="K60" t="str">
-        <v>ROSALIE CUNNINGHAM es una banda de rock psicodélico originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Lucifer es una agrupación de heavy metal formada en Berlín, Alemania en 2014 por la cantante Johanna Sadonis. Tras varios cambios, Sadonis se mantiene como la única integrante original. La agrupación está establecida actualmente en Estocolmo.</v>
       </c>
       <c r="L60" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M60" t="b">
         <v>1</v>
@@ -3113,10 +3114,10 @@
         <v>https://www.facebook.com/TriviumOfficial</v>
       </c>
       <c r="K61" t="str">
-        <v>TRIVIUM es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Trivium es una banda de Metalcore procedente de Orlando, Estados Unidos. ​ Tres años después lanzaron un demo que les ayudó a acordar un contrato con Lifeforce, donde lanzaron su álbum debut Ember to Inferno. Más tarde firmaron con Roadrunner Records y lanzaron Ascendancy. Mientras que sus dos primeros álbumes fueron de metalcore, desarrollaron un sonido más cercano al thrash metal en los dos siguientes, The Crusade y Shogun. En su álbum In Waves han adoptado un estilo mucho más personal, mostrando una combinación de los estilos que ha trabajado con anterioridad.</v>
       </c>
       <c r="L61" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M61" t="b">
         <v>1</v>
@@ -3154,10 +3155,10 @@
         <v>https://www.facebook.com/DyingWish503</v>
       </c>
       <c r="K62" t="str">
-        <v>DYING WISH es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Dying Wish es una banda estadounidense de metalcore formada en Sacramento, California en 2016. La banda está formada por la vocalista Emma Boster, los guitarristas Sam Reynolds y Pedro Carrillo, el baterista Jeff Yambra y el bajista Jon Mackey.</v>
       </c>
       <c r="L62" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M62" t="b">
         <v>1</v>
@@ -3195,10 +3196,10 @@
         <v>https://www.facebook.com/gaerea</v>
       </c>
       <c r="K63" t="str">
-        <v>GAEREA es una banda de black metal originaria de Portugal. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Winterfylleth is an inglesa black metal band de Manchester. Since their inception in 2006, the band has released nine studio albums and have become a popular act in both the inglesa underground metal scene and the wider international metal arena. Winterfylleth are self-described as "inglesa Heritage Black Metal" and are often considered to be musical 'brothers-in-arms' with fellow inglesa black metal band Wodensthrone owing to the common lyrical and aesthetic themes they share.</v>
       </c>
       <c r="L63" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M63" t="b">
         <v>1</v>
@@ -3236,10 +3237,10 @@
         <v/>
       </c>
       <c r="K64" t="str">
-        <v>RETURN TO DUST es una banda de rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Return to Dust es una banda estadounidense de grunge y rock alternativo formada en Los Ángeles, California. Su sonido captura la crudeza melancólica y los pesados acordes de la escena de Seattle de los noventa, con influencias de Alice in Chains.</v>
       </c>
       <c r="L64" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M64" t="b">
         <v>1</v>
@@ -3277,10 +3278,10 @@
         <v>https://www.facebook.com/limpbizkit</v>
       </c>
       <c r="K65" t="str">
-        <v>LIMP BIZKIT es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Limp Bizkit es una banda estadounidense de nu metal y rap metal formada en la ciudad de Jacksonville, Florida, en 1994. Sus creadores son el líder y vocalista Fred Durst y el bajista Sam Rivers. Posteriormente se unirían el primo de Rivers John Otto como baterista, y el guitarrista Rob Waters, sustituido más tarde por Wes Borland. Un tiempo después se unió el exmiembro de House of Pain DJ Lethal, completando la formación. La banda ha vendido hasta la fecha más de 40 millones de copias en todo el mundo.</v>
       </c>
       <c r="L65" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M65" t="b">
         <v>1</v>
@@ -3318,10 +3319,10 @@
         <v>https://www.facebook.com/EndItBCHC</v>
       </c>
       <c r="K66" t="str">
-        <v>END IT es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>End It es una banda de hardcore punk originaria de Baltimore, Maryland. Formados en 2017, la banda destaca por su propuesta veloz de hardcore clásico de la Costa Este, actitud desenfadada, líricas cargadas de sarcasmo y conciertos sumamente enérgicos.</v>
       </c>
       <c r="L66" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M66" t="b">
         <v>1</v>
@@ -3359,10 +3360,10 @@
         <v>https://www.facebook.com/NevertelOfficial</v>
       </c>
       <c r="K67" t="str">
-        <v>NEVERTEL es una banda de metalcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Nevertel es una banda estadounidense de nu metal formada en Tampa, Florida en 2014.​ Su música está inspirada en una variedad de géneros que incluyen metalcore, hip-hop y EDM.​​ El grupo está formado por el vocalista Jeremy Michael, el guitarrista y rapero Raul Lopez y el guitarrista Alec Davis.​</v>
       </c>
       <c r="L67" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M67" t="b">
         <v>1</v>
@@ -3400,10 +3401,10 @@
         <v>https://www.facebook.com/borknagarofficial</v>
       </c>
       <c r="K68" t="str">
-        <v>BORKNAGAR es una banda de black metal originaria de Noruega. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Borknagar es un grupo noruego de black metal progresivo y experimental, formado en 1995 en la ciudad de Bergen. Es considerado un supergrupo, dado que a su obra han contribuido una enorme cantidad de talentos del black metal. Su estilo se caracteriza por la compleja combinación de elementos típicos del black metal noruego con elementos folclóricos y progresivos.</v>
       </c>
       <c r="L68" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M68" t="b">
         <v>1</v>
@@ -3441,10 +3442,10 @@
         <v>https://www.facebook.com/maxeigorcavalera</v>
       </c>
       <c r="K69" t="str">
-        <v>CAVALERA CONSPIRACY es una banda de groove metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Cavalera Conspiracy es una banda estadounidense de groove metal formada en 2007 por los hermanos brasileños Max Cavalera en voz y guitarra rítmica e Igor Cavalera en batería, ambos ex-Sepultura, Marc Rizzo (guitarrista de Soulfly) y Joe Duplantier en el bajo (voz y guitarrista de Gojira). Si bien originalmente se llamaron Inflikted, la banda cambió su nombre a Cavalera Conspiracy por razones legales. Su álbum debut, Inflikted, fue lanzado por Roadrunner Records el 24 de marzo de 2008. Fue grabado en Undercity Studios en Los Ángeles.</v>
       </c>
       <c r="L69" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M69" t="b">
         <v>1</v>
@@ -3482,10 +3483,10 @@
         <v>https://www.facebook.com/houseofprotectionmusic</v>
       </c>
       <c r="K70" t="str">
-        <v>HOUSE OF PROTECTION es una banda de punk originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>House of Protection es un dueto de rock electrónico estadounidense que se formó en Los Ángeles, California en 2024. El duo está conformado por Stephen Harrison y Aric Improta tras dejar Fever 333 en 2022. Actualmente tienen contrato con Red Bull Records.</v>
       </c>
       <c r="L70" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M70" t="b">
         <v>1</v>
@@ -3523,10 +3524,10 @@
         <v/>
       </c>
       <c r="K71" t="str">
-        <v>DOWN TO SUFFER es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Poison – Box Set (Collector's Edition) lanzado en el 20 de enero de 2009, es una compilación de la banda de Hard rock, Poison. Contiene 3 discos con las canciones más exitosas de la banda.</v>
       </c>
       <c r="L71" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M71" t="b">
         <v>1</v>
@@ -3564,10 +3565,10 @@
         <v/>
       </c>
       <c r="K72" t="str">
-        <v>ISCREAM NEVER GROUND es una banda de metalcore originaria de Japón. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>ISCREAM NEVER GROUND es una banda de metalcore originaria de Japón.</v>
       </c>
       <c r="L72" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M72" t="b">
         <v>1</v>
@@ -3605,10 +3606,10 @@
         <v>https://www.facebook.com/STELLVRIS.band</v>
       </c>
       <c r="K73" t="str">
-        <v>STELLVRIS es una banda de modern metal originaria de Chequia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>STELLVRIS es una banda de modern metal originaria de Chequia.</v>
       </c>
       <c r="L73" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M73" t="b">
         <v>1</v>
@@ -3646,10 +3647,10 @@
         <v>https://www.facebook.com/donutshole</v>
       </c>
       <c r="K74" t="str">
-        <v>DONUTS HOLE es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Los discos ilustrados (o pictodiscos) son un tipo de discos fonográficos que muestran imágenes en su superficie de reproducción, en lugar de ser de vinilo negro o de otro color uniforme. Los coleccionistas reservan tradicionalmente el término disco ilustrado ("picture disc" en inglés) para denominar a aquellos discos con imágenes que se extienden al menos en parte al área ocupada por los surcos sonoros, distinguiéndolos de los discos con etiqueta ilustrada ("picture label discs"), que incluyen una etiqueta (a veces más grande de lo normal) con algún diseño gráfico especial, y de los discos con una cara de imagen ("picture back discs"), con un lado completo ilustrado pero sin contenido sonoro.</v>
       </c>
       <c r="L74" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M74" t="b">
         <v>1</v>
@@ -3687,10 +3688,10 @@
         <v>https://www.facebook.com/hamletband</v>
       </c>
       <c r="K75" t="str">
-        <v>HAMLET es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Hamlet es una banda de metal alternativo, thrash metal y groove metal de Madrid (España), en activo desde 1987. El nombre del grupo se lo deben a un antiguo batería de la agrupación, que llegó a un ensayo con la obra Hamlet de William Shakespeare, y decidieron darle al grupo dicho nombre.</v>
       </c>
       <c r="L75" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M75" t="b">
         <v>1</v>
@@ -3728,10 +3729,10 @@
         <v>https://www.facebook.com/KRUDDO</v>
       </c>
       <c r="K76" t="str">
-        <v>KRUDDÖ es una banda de stoner originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>KRUDDÖ es una banda de stoner originaria de España.</v>
       </c>
       <c r="L76" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M76" t="b">
         <v>1</v>
@@ -3769,10 +3770,10 @@
         <v>https://www.facebook.com/todomalofficial</v>
       </c>
       <c r="K77" t="str">
-        <v>TODOMAL es una banda de doom metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>TODOMAL es una banda de doom metal originaria de España.</v>
       </c>
       <c r="L77" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M77" t="b">
         <v>1</v>
@@ -3810,10 +3811,10 @@
         <v>https://www.facebook.com/thefamilymenband</v>
       </c>
       <c r="K78" t="str">
-        <v>THE FAMILY MEN es una banda de rock industrial originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Kelly Family es una banda pop / folk / rock con más de cuarenta años de carrera y más de veinte millones de discos vendidos en Europa, formada por un grupo de nueve hermanos y hermanas nacidos en Estados Unidos, España, Irlanda y Alemania: Bárbara Ann (Mama, 1946-10 de octubre de 1982);​ Kathy (Kathleen Ann, 1963), Johnny (John Michael, 1967), Patricia (María Patricia, 1969), Jimmy (James Víctor, 1971), Joey (Joseph María, 1972), Barby (Barbara Ann, 1975-15 de abril de 2021),​ Paddy (Michael Patrick, 1977), Maite (Maite Star, 1979) y Angelo (Angelo Gabriele, 1981).</v>
       </c>
       <c r="L78" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M78" t="b">
         <v>1</v>
@@ -3851,10 +3852,10 @@
         <v>https://www.facebook.com/imminenceswe</v>
       </c>
       <c r="K79" t="str">
-        <v>IMMINENCE es una banda de metalcore originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Imminence es una banda sueca de Metalcore formada en Malmö y Trelleborg en 2009.​ El grupo está formado por el vocalista Eddie Berg, el guitarrista rítmico Harald Barrett, el guitarrista principal Alex Arnoldsson, el bajista Christian Höijer y el baterista Mikael Norén.</v>
       </c>
       <c r="L79" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M79" t="b">
         <v>1</v>
@@ -3892,10 +3893,10 @@
         <v>https://www.facebook.com/thegemsbandswe</v>
       </c>
       <c r="K80" t="str">
-        <v>THE GEMS es una banda de hard rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Gems es un disco recopilatorio lanzado en 1988 por Aerosmith, bajo el sello Columbia. Contiene material menos comercial que el disco Greatest Hits. La banda optó por incluir más canciones "heavy", que gozaron de poca radiodifusión.</v>
       </c>
       <c r="L80" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M80" t="b">
         <v>1</v>
@@ -3933,10 +3934,10 @@
         <v>https://www.facebook.com/handofjunoband</v>
       </c>
       <c r="K81" t="str">
-        <v>HAND OF JUNO es una banda de metal industrial originaria de Italia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Alice Pandini (Lodi, Italia, 27 de febrero de 1989), más conocida como Alice Lane, es una bajista y compositora italiana. Es la actual bajista de las bandas Infected Rain y Hand of Juno. Nació en Lodi, Italia, el 27 de febrero de 1989. ​ Fue una de las fundadoras de Iconist, y en 2017 se unió a la banda Killin’ Baudelaire. ​ En 2023 se unió a Infected Rain, con quienes grabaría el disco TIME al año siguiente.</v>
       </c>
       <c r="L81" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M81" t="b">
         <v>1</v>
@@ -3974,10 +3975,10 @@
         <v>https://www.facebook.com/frontiererband</v>
       </c>
       <c r="K82" t="str">
-        <v>FRONTIERER es una banda de noise hardcore originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Better Lovers es una banda estadounidense de hardcore punk formada en Búfalo, Nueva York en 2023 tras la disolución de Every Time I Die, el grupo está compuesto por el vocalista Greg Puciato, los guitarristas Jordan Buckley y Will Putney, el bajista Stephen Micciche y el baterista Clayton Holyoak. A menudo catalogado como un supergrupo, la banda cuenta con miembros de Every Time I Die (Buckley, Micciche y Holyoak) y The Dillinger Escape Plan (Puciato), así como un miembro actual de Fit for an Autopsy (Putney).</v>
       </c>
       <c r="L82" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M82" t="b">
         <v>1</v>
@@ -4015,10 +4016,10 @@
         <v>https://www.facebook.com/PayableOnDeathPOD</v>
       </c>
       <c r="K83" t="str">
-        <v>P.O.D. es una banda de nu metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>P.O.D. (siglas de Payable On Death) es una banda estadounidense de rapcore y nu metal originaria de San Diego, California, fundada en 1992. Aunque su música integra elementos de rock, metal, ritmos latinos y reggae, sus miembros también la han identificado con géneros como el punk. Las iniciales P.O.D. significan Pagadero al morir, un término bancario que el grupo adoptó para reflejar sus creencias cristianas.​ La formación actual está compuesta por Sonny Sandoval (voz), Traa Daniels (bajo) y Marcos Curiel (guitarra).</v>
       </c>
       <c r="L83" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M83" t="b">
         <v>1</v>
@@ -4056,10 +4057,10 @@
         <v>https://www.facebook.com/Cwfenband</v>
       </c>
       <c r="K84" t="str">
-        <v>CWFEN es una banda de doom metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Sorrows is the debut studio album by Scottish doom metal band Cwfen. It was released on 30 May 2025, through New Heavy Sounds. Mastered by James Plotkin, it consists of ten tracks with a total runtime of approximately forty-three minutes. Seven tracks range between four and six minutes each, while the remaining three "Fragment" tracks are under a minute each. The album was produced by Kevin Hare and the band, composed of lead vocalist Agnes Alder, guitarist Guy DeNuit, drummer Rös Ranquinn, and bassist Mary Thomas Baker.</v>
       </c>
       <c r="L84" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M84" t="b">
         <v>1</v>
@@ -4097,10 +4098,10 @@
         <v>https://www.facebook.com/DistantOfficial</v>
       </c>
       <c r="K85" t="str">
-        <v>DISTANT es una banda de deathcore originaria de Paises Bajos. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Distant Project es una banda de Synth pop surgida en el año 2002, Está formada por Fab Soutus (Phoenix – AZ - US) en sintetizadores, bajos, programaciones y voz, Wal Yunker (Paraná - E. Ríos - ARG), sintetizadores, programación y baterías, y Clau Spiritelli (Paraná - E. Ríos - ARG), guitarras. La denominación de la banda proviene precisamente por la particularidad de vivir todos en ciudades diferentes.</v>
       </c>
       <c r="L85" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M85" t="b">
         <v>1</v>
@@ -4138,10 +4139,10 @@
         <v/>
       </c>
       <c r="K86" t="str">
-        <v>GRIDIRON es una banda de hardcore melódico originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Gridiron es una banda estadounidense de hardcore y rap metal formada en Pensilvania. Fusionando el hardcore más pesado y directo con rimas de rap y ritmos machacones, se han posicionado como una fuerza emergente en la escena underground americana.</v>
       </c>
       <c r="L86" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M86" t="b">
         <v>1</v>
@@ -4179,10 +4180,10 @@
         <v>https://www.facebook.com/Mastodon</v>
       </c>
       <c r="K87" t="str">
-        <v>MASTODON es una banda de metal progresivo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Mastodon es una banda estadounidense de metal progresivo fundada el 13 de enero de 1999 por los guitarristas Brent Hinds y Bill Kelliher, el batería Brann Dailor y el bajista Troy Sanders en Atlanta. Aunque comenzaron como quinteto, con el vocalista Eric Saner, la banda se caracteriza por ser un cuarteto en el que los miembros comparten las labores vocales en los distintos temas. Con la excepción de su álbum debut, Remission, todos los trabajos de la banda han entrado en el Billboard 200; a destacar los top 10 alcanzados por The Hunter y Once More 'Round the Sun.</v>
       </c>
       <c r="L87" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M87" t="b">
         <v>1</v>
@@ -4220,10 +4221,10 @@
         <v/>
       </c>
       <c r="K88" t="str">
-        <v>AA WILLIAMS es una banda de dark folk originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>La Asociación Atlética Banda Norte, también conocida por sus siglas AABN, es una entidad polideportiva argentina con sede en la ciudad de Río Cuarto, Córdoba. Pese a su carácter polideportivo, que le lleva a tener secciones de disciplinas como el fútbol, el tenis o la gimnasia artística, su principal sección es la de básquet masculino, de carácter profesional y que compitió en el Torneo Nacional de Ascenso, la segunda competición en importancia del baloncesto argentino desde la temporada 2010/11 hasta el TNA 2013/14 inclusive.</v>
       </c>
       <c r="L88" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M88" t="b">
         <v>1</v>
@@ -4261,10 +4262,10 @@
         <v>https://www.facebook.com/DOGMA.am</v>
       </c>
       <c r="K89" t="str">
-        <v>DOGMA es una banda de heavy metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Dogma SS fue una banda de hardcore metal originaria de la ciudad de Lima (Perú), que existió entre los años 1993 y 1996, es decir, durante los años de transición inmediatamente posteriores al fin de la movida del rock subterráneo en septiembre de 1992.</v>
       </c>
       <c r="L89" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M89" t="b">
         <v>1</v>
@@ -4302,10 +4303,10 @@
         <v>https://www.facebook.com/converge</v>
       </c>
       <c r="K90" t="str">
-        <v>CONVERGE es una banda de hardcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Converge es una banda de Hardcore proveniente de Boston. Fue formada en 1990 por el vocalista Jacob Bannon, el guitarrista Kurt Ballou, el bajista Jeff Feinburg y el batería Damon Bellorado. En la actualidad continúan Jacob Bannon y Kurt Ballou y toca la batería Ben Koller y el bajo Nate Newton. Es uno de los grupos más prolíficos y que más influencia ha ejercido en la historia reciente del hardcore. Su sonido es un llamativa y original mezcla de elementos del hardcore punk con los de metal extremo.</v>
       </c>
       <c r="L90" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M90" t="b">
         <v>1</v>
@@ -4343,10 +4344,10 @@
         <v>https://www.facebook.com/MarilynManson</v>
       </c>
       <c r="K91" t="str">
-        <v>MARILYN MANSON es una banda de metal industrial originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Marilyn Manson es una banda estadounidense de metal industrial/alternativo​ formada en el año 1989 por el cantante homónimo Marilyn Manson y el guitarrista Scott Putesky, inicialmente bajo el nombre de Marilyn Manson &amp; The Spooky Kids. ​ Sin embargo, aunque su supuesta influencia se desmintió, decidieron alejarse de los escenarios hasta el año 2000, cuando regresaron con el disco Holy Wood (In the Shadow of the Valley of Death).</v>
       </c>
       <c r="L91" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M91" t="b">
         <v>1</v>
@@ -4384,10 +4385,10 @@
         <v>https://www.facebook.com/vintagecaravan</v>
       </c>
       <c r="K92" t="str">
-        <v>THE VINTAGE CARAVAN es una banda de hard rock originaria de Islandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Vintage Caravan es una banda de rock de Álftanes, Islandia. La banda fue formada en 2006 por Óskar Logi Ágústsson y Guðjón Reynisson antes de que el bajista Alexander Örn Númason se uniera después del primer álbum de estudio. A partir de 2011, la banda ha lanzado cinco álbumes de estudio y actualmente están firmados con Napalm Records.</v>
       </c>
       <c r="L92" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M92" t="b">
         <v>1</v>
@@ -4425,10 +4426,10 @@
         <v>https://www.facebook.com/Blood-incantation-508899805936788</v>
       </c>
       <c r="K93" t="str">
-        <v>BLOOD INCANTATION es una banda de death metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Incantation es una banda estadounidense de death metal que fue formada por John McEntee y Paul Lendley en 1989. Son uno de los líderes en la escena del death metal neoyorquino junto con Suffocation, Mortician e Immolation aunque actualmente la banda reside en Johnstown, Pensilvania. A la fecha, la banda ha lanzado trece larga duración, dos álbumes en vivo, cuatro EP’s, dos singles, tres splits, un DVD y tres demos. Durante más de 30 años, Incantation se ha mantenido constantemente como una de las bandas underground más influyentes y respetadas del género.</v>
       </c>
       <c r="L93" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M93" t="b">
         <v>1</v>
@@ -4466,10 +4467,10 @@
         <v>https://www.facebook.com/elwoodstrayband</v>
       </c>
       <c r="K94" t="str">
-        <v>ELWOOD STRAY es una banda de hardcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>ZZ Top es una banda estadounidense de blues rock y hard rock formada en 1969 en Houston, Texas. Este power trio lo conforman Billy Gibbons en la guitarra y la voz, Dusty Hill en el bajo, los teclados y la voz, y Frank Beard en la batería. Tienen el mérito de ser uno de los pocos grupos de rock que todavía conservaba sus miembros originales después de cincuenta años (hasta la muerte de Hill en el 2021), y además de haber mantenido un número casi similar de años al mismo mánager y productor, Bill Ham.</v>
       </c>
       <c r="L94" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M94" t="b">
         <v>1</v>
@@ -4507,10 +4508,10 @@
         <v>https://www.facebook.com/blindguardian</v>
       </c>
       <c r="K95" t="str">
-        <v>BLIND GUARDIAN es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Blind Guardian es un grupo alemán de power metal​​ fundado en 1984 en la ciudad de Krefeld, en ese entonces Alemania Occidental, originalmente bajo el nombre de Lucifer's Heritage. Esta banda ha recibido la influencia de grupos como Helloween, Uriah Heep y Queen, entre otras citadas por el grupo en diversas entrevistas.</v>
       </c>
       <c r="L95" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M95" t="b">
         <v>1</v>
@@ -4548,10 +4549,10 @@
         <v>https://www.facebook.com/alestormband</v>
       </c>
       <c r="K96" t="str">
-        <v>ALESTORM es una banda de pirate metal originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Alestorm es una banda escocesa de folk metal con temática pirata formada en Perth, Escocia, como Battleheart en 2004. Ellos denominan a su propio estilo "Verdadero Metal Pirata Escocés".​</v>
       </c>
       <c r="L96" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M96" t="b">
         <v>1</v>
@@ -4589,10 +4590,10 @@
         <v/>
       </c>
       <c r="K97" t="str">
-        <v>SAUROM es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Saurom (anteriormente denominado Saurom Lamderth)​ es un grupo español de folk metal. Fue fundado en 1996 por Narci Lara y Antonio Ruíz. Denominan su estilo como «juglar metal», un conglomerado de música metal, folk y celta, aderezado con letras basadas en la literatura, principalmente en leyendas, poemas, romances y cuentos tradicionales, con un trasfondo crítico, cultural y social. Algunas de sus letras tienen una temática relacionada con la novela El Señor de los Anillos, de J. R. R. Tolkien y con la literatura clásica y tradicional andaluza.</v>
       </c>
       <c r="L97" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M97" t="b">
         <v>1</v>
@@ -4630,10 +4631,10 @@
         <v>https://www.facebook.com/thundermother</v>
       </c>
       <c r="K98" t="str">
-        <v>THUNDERMOTHER es una banda de hard rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Thundermother es una banda sueca de hard rock clásico fundada en Växjö en 2009 por la guitarrista Filippa Nässil. Con un sonido fuertemente influenciado por AC/DC y Motörhead, el grupo destaca por su rock enérgico y directo, coros potentes y sus giras mundiales.</v>
       </c>
       <c r="L98" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M98" t="b">
         <v>1</v>
@@ -4671,10 +4672,10 @@
         <v>https://www.facebook.com/blacklabelsociety</v>
       </c>
       <c r="K99" t="str">
-        <v>BLACK LABEL SOCIETY es una banda de heavy metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Black Label Society es una banda estadounidense de metal proveniente de Los Ángeles, California (USA), formada por el guitarrista Zakk Wylde en 1998 bajo el nombre inicial de Hell's Kitchen. A la fecha la banda ha publicado 12 álbumes de estudio, dos discos en vivo, dos compilados, y tres DVDs.​</v>
       </c>
       <c r="L99" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M99" t="b">
         <v>1</v>
@@ -4712,10 +4713,10 @@
         <v>https://www.facebook.com/slaughtertoprevailrus</v>
       </c>
       <c r="K100" t="str">
-        <v>SLAUGHTER TO PREVAIL es una banda de deathcore originaria de Rusia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Slaughter to Prevail es una banda rusa de deathcore formada en 2014, originaria de la ciudad de Ekaterimburgo y actualmente con sede en Orlando, Florida.​ El grupo debutó con su EP titulado Chapters of Misery en 2015 y dos años después lanzó Misery Sermon. Su segundo álbum, Kostolom, fue lanzado en 2021. Actualmente, la banda se encuentra en el sello Sumerian Records y ha realizado giras por EE. UU., Latinoamérica, Europa,​​ y Asia.​</v>
       </c>
       <c r="L100" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M100" t="b">
         <v>1</v>
@@ -4753,10 +4754,10 @@
         <v>https://www.facebook.com/SalduieOficial</v>
       </c>
       <c r="K101" t="str">
-        <v>SALDUIE es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Salduie (en escritura íbera ) es una banda española de folk metal originaria de la ciudad de Zaragoza y fundada en el año 2010. Sus letras se caracterizan por tratar sobre las culturas prerromanas de la península ibérica, incluyendo los celtíberos, los iberos, los lusitanos y la conquista romana.​</v>
       </c>
       <c r="L101" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M101" t="b">
         <v>1</v>
@@ -4794,10 +4795,10 @@
         <v>https://www.facebook.com/tailgunnerhq</v>
       </c>
       <c r="K102" t="str">
-        <v>TAILGUNNER es una banda de heavy metal originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Tailgunner es una banda de heavy metal originaria de Reino Unido. Inspirados por la clásica Nueva Ola del Heavy Metal Británico (NWOBHM), su propuesta musical destaca por guitarras gemelas veloces, agudos falsetes y temáticas bélicas e históricas.</v>
       </c>
       <c r="L102" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M102" t="b">
         <v>1</v>
@@ -4835,10 +4836,10 @@
         <v>https://www.facebook.com/OrbitCulture</v>
       </c>
       <c r="K103" t="str">
-        <v>ORBIT CULTURE es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Orbit Culture es una banda de death metal melódico sueco de Eksjö, formada en 2013. La banda está conformado por el vocalista y guitarrista rítmico Niklas Karlsson, al guitarrista principal Richard Hansson, al bajista Fredrik Lennartsson y al baterista Christopher Wallerstedt. Entre sus antiguos miembros se encuentran el guitarrista principal Maximilian Zinsmeister, el bajista Christoffer Olsson y el baterista Markus Bladh. La banda ha publicado cinco álbumes de estudio y cuatro EP.</v>
       </c>
       <c r="L103" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M103" t="b">
         <v>1</v>
@@ -4876,10 +4877,10 @@
         <v>https://www.facebook.com/savatage</v>
       </c>
       <c r="K104" t="str">
-        <v>SAVATAGE es una banda de metal progresivo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Savatage es un grupo estadounidense de heavy metal. Fue fundado por los hermanos Jon y Criss Oliva en 1979. La banda es reconocida por grabar algunos álbumes conceptuales. Sus orígenes pueden ser atribuidos al heavy metal más clásico, influenciados por bandas como Judas Priest, Iron Maiden, Dio, Black Sabbath y Rush, lo que se puede apreciar claramente en su álbum debut, Sirens.​​ El guitarrista Criss Oliva falleció en un accidente automovilístico el 17 de octubre de 1993.​</v>
       </c>
       <c r="L104" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M104" t="b">
         <v>1</v>
@@ -4917,10 +4918,10 @@
         <v>https://www.facebook.com/sepultura</v>
       </c>
       <c r="K105" t="str">
-        <v>SEPULTURA es una banda de thrash metal originaria de Brasil. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>D. ​ La formación actual de Sepultura está integrada por el bajista Paulo Jr.</v>
       </c>
       <c r="L105" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M105" t="b">
         <v>1</v>
@@ -4958,10 +4959,10 @@
         <v/>
       </c>
       <c r="K106" t="str">
-        <v>HELEVEN es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Heleven es una banda española de metal alternativo y progresivo fundada en Granada en 2016. Su sonido destaca por su complejidad técnica, riffs afinados en tonos bajos y una mezcla de pasajes melódicos oscuros con momentos de gran agresividad.</v>
       </c>
       <c r="L106" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M106" t="b">
         <v>1</v>
@@ -4999,10 +5000,10 @@
         <v>https://www.facebook.com/Killusband</v>
       </c>
       <c r="K107" t="str">
-        <v>KILLUS es una banda de metal industrial originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Killus ( /kɪləs/ ) es una banda de metal industrial formada en 1997 en Villarreal, España. Se caracteriza por su sonido agresivo, inspirado por bandas como Nine Inch Nails, Marilyn Manson, White Zombie o Ministry, y por su estética oscura y teatral, que combina el metal con elementos electrónicos y visuales impactantes.​ Después de haber tenido diferentes configuraciones, actualmente está formada por cuatro miembros: Ruk como guitarrista, Premutoxx al bajo, Javi Ssagittar voz principal y Anhell Stixx a la batería.</v>
       </c>
       <c r="L107" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M107" t="b">
         <v>1</v>
@@ -5040,10 +5041,10 @@
         <v/>
       </c>
       <c r="K108" t="str">
-        <v>HADADANZA es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Leyendas del Rock es un festival de música heavy metal y rock duro que se celebra anualmente desde 2006. ​ En los inicios del festival la gran mayoría de bandas que actuaban eran españolas, aunque en la actualidad participan muchas bandas del panorama internacional. El festival no tiene una duración fija, y mientras que el primer año todos los conciertos se celebraron en un solo día, el resto de ediciones han durado dos, tres o cuatro días.</v>
       </c>
       <c r="L108" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M108" t="b">
         <v>1</v>
@@ -5081,10 +5082,10 @@
         <v>https://www.facebook.com/signsoftheswarm</v>
       </c>
       <c r="K109" t="str">
-        <v>SIGNS OF THE SWARM es una banda de deathcore originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Avatar es una banda sueca de metal, fundada en Gotemburgo en el año 2001. En 2004 publicó su primer demo titulado Personal Observations, seguido de un EP en ese mismo año llamado 4 Reasons to Die.​ En 2006 lanzaron su álbum debut, Thoughts of No Tomorrow. Hasta la fecha han publicado nueve álbumes de estudio, siendo Don't Go In The Forest el más reciente de ellos.</v>
       </c>
       <c r="L109" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M109" t="b">
         <v>1</v>
@@ -5122,10 +5123,10 @@
         <v/>
       </c>
       <c r="K110" t="str">
-        <v>DEATHBATS es una banda de tributo a7x originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Avenged Sevenfold (abbreviated as A7X) is an estadounidense heavy metal band de Huntington Beach, California, formada en 1999. The band's current lineup consists of vocalist M. Shadows, guitarists Zacky Vengeance and Synyster Gates, bassist Johnny Christ, and drummer Brooks Wackerman. Avenged Sevenfold are known for their diverse rock sound and dramatic imagery in album covers and merchandise. The band emerged with a metalcore sound on their debut album Sounding the Seventh Trumpet; they largely continued this sound through their second album Waking the Fallen.</v>
       </c>
       <c r="L110" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M110" t="b">
         <v>1</v>
@@ -5163,10 +5164,10 @@
         <v>https://www.facebook.com/chainedsaint</v>
       </c>
       <c r="K111" t="str">
-        <v>CHAINED SAINT es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Chained Saint es una banda estadounidense de thrash metal formada en Florida. Compuesta por jóvenes músicos apasionados por el metal clásico, su música revive la velocidad y agresión del thrash clásico de la Bay Area de los años ochenta.</v>
       </c>
       <c r="L111" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M111" t="b">
         <v>1</v>
@@ -5204,10 +5205,10 @@
         <v/>
       </c>
       <c r="K112" t="str">
-        <v>PROM KINKS es una banda de rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Prom Kinks es una banda de rock alternativo originaria de España. Su estilo combina riffs enérgicos de guitarra con melodías accesibles y pegadizas, destacando por un sonido moderno e influencias del rock de garaje internacional.</v>
       </c>
       <c r="L112" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M112" t="b">
         <v>1</v>
@@ -5245,10 +5246,10 @@
         <v>https://www.facebook.com/mushroomheadofficial</v>
       </c>
       <c r="K113" t="str">
-        <v>MUSHROOMHEAD es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Mushroomhead es una banda estadounidense de metal alternativo e industrial formada en Cleveland, Ohio, en 1993. Conocidos por sus llamativas máscaras de temática teatral y sus uniformes oscuros, fusionan géneros que van del nu metal al avant-garde.</v>
       </c>
       <c r="L113" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M113" t="b">
         <v>1</v>
@@ -5286,10 +5287,10 @@
         <v>https://www.facebook.com/dtofficial</v>
       </c>
       <c r="K114" t="str">
-        <v>DARK TRANQUILLITY es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Dark Tranquillity es una banda de death metal melódico formada en 1989 en Gotemburgo, Suecia. Poseen una extensa carrera desde 1989 hasta nuestros días, en la que han sido nominados a diversos premios, entre ellos el Grammy por su álbum Projector. Están íntimamente ligados a la historia de In Flames ya que Niklas Sundin, uno de los miembros de Dark Tranquillity, escribió las letras de dos álbumes de In Flames, Whoracle y The Jester Race. Además, desde 1993, el vocalista original de In Flames es el actual de Dark Tranquillity y viceversa.</v>
       </c>
       <c r="L114" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M114" t="b">
         <v>1</v>
@@ -5327,10 +5328,10 @@
         <v>https://www.facebook.com/archenemyofficial</v>
       </c>
       <c r="K115" t="str">
-        <v>ARCH ENEMY es una banda de death metal melódico originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Arch Enemy es una banda sueca de death metal melódico formada en Halmstad en 1995. En sus inicios exploró el death metal original, pero sufrió una transformación musical después del cambio de integrantes que tuvo, comenzando a abarcar un sonido más melódico que continúa vigente a día de hoy. Sus letras hablan de rebelión y suelen criticar a la sociedad y a la religión cristiana​ La banda es procedente de Suecia, formada en 1996 por el guitarrista Michael Amott​ junto al vocalista Johan Liiva. La banda ha publicado diez álbumes de estudio, dos en directo, tres EP y dos DVD.</v>
       </c>
       <c r="L115" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M115" t="b">
         <v>1</v>
@@ -5368,10 +5369,10 @@
         <v>https://www.facebook.com/lepokafolk</v>
       </c>
       <c r="K116" t="str">
-        <v>LÈPOKA es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L116" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M116" t="b">
         <v>1</v>
@@ -5409,10 +5410,10 @@
         <v>https://www.facebook.com/creepercult</v>
       </c>
       <c r="K117" t="str">
-        <v>CREEPER es una banda de goth punk originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Creeper es una banda inglesa de punk rock formada en 2014, conformado por el vocalista Will Gould, el guitarrista Ian Miles, la tecladista y segunda vocalista Hannah Greenwood, el bajista Sean Scott y el baterista Jake Fogarty. Creeper lanzó su auto-titulado debut (EP) Creeper en 2014, que fue seguido por The Callous Heart y The Stranger en Roadrunner Records en 2015 y 2016, respectivamente.</v>
       </c>
       <c r="L117" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M117" t="b">
         <v>1</v>
@@ -5450,10 +5451,10 @@
         <v>https://www.facebook.com/northlane</v>
       </c>
       <c r="K118" t="str">
-        <v>NORTHLANE es una banda de metalcore originaria de Australia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Northlane es una banda de metalcore procedente de Sídney, Australia; formada en el año 2009. La banda cuenta con los guitarristas Jon Deiley y Josh Smith, el bajista Brendon Padjasek, el batería Nic Pettersen y el vocalista Marcus Bridge, quién reemplazó al vocalista fundador Adrian Fitipaldes a finales de 2014. La banda ha publicado seis álbumes de estudio: Discoveries (2011), Singularity (2013), Node (2015), Mesmer (2017), Alien (2019), y Obsidian (2022). En los ARIA Music Awards of 2015 el grupo ganó el premio al "Mejor álbum de hard rock o heavy metal".</v>
       </c>
       <c r="L118" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M118" t="b">
         <v>1</v>
@@ -5491,10 +5492,10 @@
         <v>https://www.facebook.com/Godsmack</v>
       </c>
       <c r="K119" t="str">
-        <v>GODSMACK es una banda de metal alternativo originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Godsmack es una banda estadounidense de metal alternativo originaria de Lawrence, Massachusetts, formada en 1995 e integrada por el líder, vocalista y compositor principal de la banda Sully Erna, el guitarrista Tony Rombola, el bajista Robbie Merrill y el batería Shannon Larkin. Desde sus inicios, Godsmack ha lanzado seis álbumes de estudio, un EP, cuatro DVD, un álbum recopilatorio, y un álbum en directo (Live and Inspired). La banda ha tenido tres álbumes números uno consecutivos (Faceless, IV y The Oracle) en la lista Billboard 200.</v>
       </c>
       <c r="L119" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M119" t="b">
         <v>1</v>
@@ -5532,10 +5533,10 @@
         <v>https://www.facebook.com/dartagnan.de</v>
       </c>
       <c r="K120" t="str">
-        <v>DARTAGNAN es una banda de folk rock originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>dArtagnan es una banda alemana de folk rock, proveniente de Núremberg, liderada por el cantante Ben Metzner. Fundada en 2015, la agrupación mezcla géneros de música folclórica europea con un sonido Hard rock e incluso Heavy metal.</v>
       </c>
       <c r="L120" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M120" t="b">
         <v>1</v>
@@ -5573,10 +5574,10 @@
         <v/>
       </c>
       <c r="K121" t="str">
-        <v>EKYRIAN es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>EKYRIAN es una banda de folk metal originaria de España.</v>
       </c>
       <c r="L121" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M121" t="b">
         <v>1</v>
@@ -5614,10 +5615,10 @@
         <v/>
       </c>
       <c r="K122" t="str">
-        <v>LÁNDEVIR es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Lándevir es un grupo español de folk metal con influencias de power metal y rock celta fundado en 1998 en Elda (Alicante).</v>
       </c>
       <c r="L122" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M122" t="b">
         <v>1</v>
@@ -5655,10 +5656,10 @@
         <v>https://www.facebook.com/InjectorThrash</v>
       </c>
       <c r="K123" t="str">
-        <v>INJECTOR es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L123" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M123" t="b">
         <v>1</v>
@@ -5696,10 +5697,10 @@
         <v/>
       </c>
       <c r="K124" t="str">
-        <v>EVO es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>EVO es una banda de heavy metal originaria de España.</v>
       </c>
       <c r="L124" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M124" t="b">
         <v>1</v>
@@ -5737,10 +5738,10 @@
         <v/>
       </c>
       <c r="K125" t="str">
-        <v>CELTIBEERIAN es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Jonne Järvelä (n. 3 de junio de 1974) es el vocalista y guitarrista de la banda finlandesa Korpiklaani, y del proyecto anterior Shaman. Es conocido en la escena Folk Metal por su yoiking. Además contribuyó en los álbumes de las bandas Finntroll (Jaktens Tid) y Skiltron (Beheading The Liars).</v>
       </c>
       <c r="L125" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M125" t="b">
         <v>1</v>
@@ -5778,10 +5779,10 @@
         <v>https://www.facebook.com/Bolu2death</v>
       </c>
       <c r="K126" t="str">
-        <v>BOLU2 DEATH es una banda de metalcore/electronic originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Resurrection Fest is a rock music festival that takes place in Viveiro, region of Lugo, Spain. This festival has been held annually since 2006 during July or early August and features mainly heavy metal, hardcore punk and punk rock bands. Since its emergence it has become one of the most important music festivals in Spain due to its genre specialization. 3 million euros in the region. 15-million euros impact.</v>
       </c>
       <c r="L126" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M126" t="b">
         <v>1</v>
@@ -5819,10 +5820,10 @@
         <v>https://www.facebook.com/futurepalace</v>
       </c>
       <c r="K127" t="str">
-        <v>FUTURE PALACE es una banda de post-hardcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Future Palace es una banda alemana de post-hardcore y metal alternativo formada en Berlín en 2018. El trío, liderado por la vocalista Maria Lessing, destaca por su sonido emotivo que aborda líricamente temáticas como la salud mental y la superación.</v>
       </c>
       <c r="L127" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M127" t="b">
         <v>1</v>
@@ -5860,10 +5861,10 @@
         <v/>
       </c>
       <c r="K128" t="str">
-        <v>SARATOGA es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Saratoga es una banda de heavy metal española originaria de Madrid. Fue formada en 1992 por el bajista Niko del Hierro y el guitarrista Jero Ramiro. La banda ha contado con diversas formaciones. La última la conforman Niko del Hierro (único miembro que ha permanecido en el grupo durante toda su historia), Tete Novoa, Charlie Parra del Riego y Arnau Martí.</v>
       </c>
       <c r="L128" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M128" t="b">
         <v>1</v>
@@ -5901,10 +5902,10 @@
         <v>https://www.facebook.com/inflames</v>
       </c>
       <c r="K129" t="str">
-        <v>IN FLAMES es una banda de metal alternativo originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>In Flames es una banda de death metal melódico. Formada en Gotemburgo, Suecia en 1990, es considerada pionera e influyente en el género. Desde la concepción de la banda en 1990, han recibido numerosos premios, publicado doce álbumes de estudio y un DVD en vivo. La banda ha gozado de mayor popularidad en los últimos años, tanto en su nativa Suecia como internacionalmente. La banda ha vendido más de tres millones de discos en todo el mundo.​</v>
       </c>
       <c r="L129" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M129" t="b">
         <v>1</v>
@@ -5942,10 +5943,10 @@
         <v>https://www.facebook.com/official.darkmoor?sid=6286</v>
       </c>
       <c r="K130" t="str">
-        <v>DARK MOOR es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>​ La agrupación fue de las primeras bandas españolas de power metal, y son influenciados por grupos como Stratovarius, Blind Guardian y Helloween. El grupo ha ido evolucionando su sonido, teniendo una fuerte inspiración de música clásica durante sus primeros álbumes, pasando a un sonido de metal sinfónico e incluso folk metal en sus últimos trabajos. Las temáticas de sus canciones suelen hablar de novelas clásicas, personajes históricos, antiguas leyendas y mitos.</v>
       </c>
       <c r="L130" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M130" t="b">
         <v>1</v>
@@ -5983,10 +5984,10 @@
         <v>https://www.facebook.com/ChezKaneVocalist</v>
       </c>
       <c r="K131" t="str">
-        <v>CHEZ KANE es una banda de hard rock originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Chez Kane es una vocalista y compositora británica de hard rock y AOR. Conocida también como la vocalista de la banda familiar Kane'd, ha destacado con sus álbumes en solitario que reviven el espíritu festivo y los coros del rock de los ochenta.</v>
       </c>
       <c r="L131" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M131" t="b">
         <v>1</v>
@@ -6024,10 +6025,10 @@
         <v>https://www.facebook.com/thebaboonshow</v>
       </c>
       <c r="K132" t="str">
-        <v>THE BABOON SHOW es una banda de punk rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>The Baboon Show es una banda sueca de punk rock formada en Estocolmo en 2003. Famosos por sus giras incansables y la increíble presencia escénica de su líder Cecilia Boström, su sonido mezcla punk, rock clásico y letras con un gran contenido político.</v>
       </c>
       <c r="L132" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M132" t="b">
         <v>1</v>
@@ -6065,10 +6066,10 @@
         <v>https://www.facebook.com/stratovarius</v>
       </c>
       <c r="K133" t="str">
-        <v>STRATOVARIUS es una banda de power metal originaria de Finlandia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Stratovarius es una banda finlandesa de power metal melódico con elementos de música clásica, formada en 1984 en la ciudad de Helsinki por Tuomo Lassila, John Vihervä y Staffan Stråhlman bajo el nombre Black Water. Ha publicado dieciséis álbumes de estudio, seis DVD y seis álbumes en vivo. ​ La influencia de Stratovarius en la década de 1990 tuvo un enorme impacto en la escena europea, con su estilo veloz, melódico y virtuoso, inspiró a bandas como Sonata Arctica, DragonForce,​ Galneryus, Heavenly, Children of Bodom,​ Wintersun,​ Twilight Force,​ Majestica,​ Nightwish, entre otras.</v>
       </c>
       <c r="L133" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M133" t="b">
         <v>1</v>
@@ -6106,10 +6107,10 @@
         <v/>
       </c>
       <c r="K134" t="str">
-        <v>XERIA es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L134" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M134" t="b">
         <v>1</v>
@@ -6147,10 +6148,10 @@
         <v>https://www.facebook.com/OfficialWingsofSteel</v>
       </c>
       <c r="K135" t="str">
-        <v>WINGS OF STEEL es una banda de hard rock originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Wings of Steel es una banda estadounidense de hard rock y heavy metal clásico formada en Los Ángeles, California, en 2019. Liderados por el vocalista Leo Valeri, su música destaca por sus agudos falsetes y riffs reminiscentes de la NWOBHM.</v>
       </c>
       <c r="L135" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M135" t="b">
         <v>1</v>
@@ -6188,10 +6189,10 @@
         <v>https://www.facebook.com/pages/AGAINST-MYSELF/203937595534</v>
       </c>
       <c r="K136" t="str">
-        <v>AGAINST MYSELF es una banda de metal sinfónico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Against Myself es una banda española de metal sinfónico formada en Ciudad Real en 2009. Su estilo destaca por la instrumentación orquestal de teclado, guitarras pesadas y la virtuosa voz femenina de su cantante, con atmósferas de metal progresivo.</v>
       </c>
       <c r="L136" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M136" t="b">
         <v>1</v>
@@ -6229,10 +6230,10 @@
         <v>https://www.facebook.com/employedtoserve</v>
       </c>
       <c r="K137" t="str">
-        <v>EMPLOYED TO SERVE es una banda de metalcore originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Employed to Serve es una banda británica de metalcore y mathcore formada en Woking, Inglaterra, en 2013. Su música combina la pesadez de los acordes de afinación baja con estructuras rítmicas complejas y las potentes voces de Justine Jones.</v>
       </c>
       <c r="L137" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M137" t="b">
         <v>1</v>
@@ -6270,10 +6271,10 @@
         <v>https://www.facebook.com/DAERIAOFICIAL</v>
       </c>
       <c r="K138" t="str">
-        <v>DAERIA es una banda de metal alternativo originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Art Gates Records es un sello discográfico independiente español fundado en mayo de 2012 en la provincia de Valencia.​ La discográfica está especializada principalmente en la producción, promoción y distribución internacional de música metal y sus diferentes subgéneros.​</v>
       </c>
       <c r="L138" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M138" t="b">
         <v>1</v>
@@ -6311,10 +6312,10 @@
         <v>https://www.facebook.com/MindDriller</v>
       </c>
       <c r="K139" t="str">
-        <v>MIND DRILLER es una banda de metal industrial originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Mind Driller es una banda española de metal industrial originaria de Alicante, fundada en el año 2011 por el guitarrista Javier Oriente (integrante de los grupos Blood, Hasswut y Stoneheads). Q. a las voces, Javix a la guitarra, Pharaoh al bajo y Reimon a la batería. El estilo musical de "Mind Driller" es definido como base de metal industrial variado y potente que a diferencia de otras bandas del mismo género cuenta con tres vocalistas.</v>
       </c>
       <c r="L139" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M139" t="b">
         <v>1</v>
@@ -6352,10 +6353,10 @@
         <v/>
       </c>
       <c r="K140" t="str">
-        <v>JORDI WILD DJ SET es una banda de dj set originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Jordi Wild DJ Set es el proyecto de música de baile y rock presentado por el conocido creador de contenido digital, podcaster y youtuber español Jordi Wild. Sus sesiones combinan el rock, metal y punk clásicos con mezclas de música electrónica de alta energía.</v>
       </c>
       <c r="L140" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M140" t="b">
         <v>1</v>
@@ -6393,10 +6394,10 @@
         <v/>
       </c>
       <c r="K141" t="str">
-        <v>GUILT TRIP es una banda de hardcore originaria de Reino Unido. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Nero es un trío británico de música electrónica procedente de Londres, Inglaterra. Está integrado por los productores Daniel Stephens y Joseph Ray junto a su vocalista, Alana Watson, como miembro estable de la banda. ​ También se los suele nombrar Nero UK para evitar confusiones con bandas del mismo nombre. El 6 de diciembre de 2010, Nero fue anunciado como uno de los nominados de la encuesta Sound of 2011 realizada por la BBC.</v>
       </c>
       <c r="L141" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M141" t="b">
         <v>1</v>
@@ -6434,10 +6435,10 @@
         <v>https://www.facebook.com/OfficialDeicide</v>
       </c>
       <c r="K142" t="str">
-        <v>DEICIDE es una banda de death metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Deicide (en español Deicidio del latín deicīda, «dícese de los que dieron muerte a un dios»), es una banda estadounidense de death metal originaria de Tampa, Florida, formada en 1987 por el vocalista y bajista Glen Benton, los hermanos y guitarristas Eric y Brian Hoffman, y el baterista Steve Asheim. ​ La polémica ha acompañado a la banda desde sus inicios, dado lo explícito de sus letras anticristianas y satánicas, que hacen una fuerte crítica hacia el mundo moderno y la idea de Dios, como por varias declaraciones y hechos diversos llevados a cabo por su líder Benton.</v>
       </c>
       <c r="L142" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M142" t="b">
         <v>1</v>
@@ -6475,10 +6476,10 @@
         <v>https://www.facebook.com/helloweenofficial</v>
       </c>
       <c r="K143" t="str">
-        <v>HELLOWEEN es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Helloween es una influyente banda alemana de power metal fundada en Hamburgo en 1984. Considerados como los padres fundadores del género power metal, destacan por sus guitarras gemelas a alta velocidad, coros épicos y melodías alegres.</v>
       </c>
       <c r="L143" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M143" t="b">
         <v>1</v>
@@ -6516,10 +6517,10 @@
         <v>https://www.facebook.com/profile.php?id=100063786306898</v>
       </c>
       <c r="K144" t="str">
-        <v>ANKHARA es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Ankhara es un grupo español de heavy metal con influencias de power metal y metal progresivo. Fundado en 1995, se disolvió en 2004 y en 2013 se reúne nuevamente.</v>
       </c>
       <c r="L144" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M144" t="b">
         <v>1</v>
@@ -6557,10 +6558,10 @@
         <v>https://www.facebook.com/eihwar.music</v>
       </c>
       <c r="K145" t="str">
-        <v>EIHWAR es una banda de pagan folk originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>a Festival) is a music and art festival, held in Sibiu, a town in Romania. The festival, one of the most important projects developed by ARTmania, was first organized in the summer of 2006 and has been held every summer since. The main attraction of the festival is the music: bands perform in the Large Square (Piaţa Mare) during the first two days weekend of the festival. Major bands have performed at the festival including Nightwish, HIM, Opeth, Amorphis, Anathema, Lacrimosa, Tiamat, My Dying Bride and Within Temptation and the festival grows each year.</v>
       </c>
       <c r="L145" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M145" t="b">
         <v>1</v>
@@ -6598,10 +6599,10 @@
         <v>https://www.facebook.com/officialheavenshallburn</v>
       </c>
       <c r="K146" t="str">
-        <v>HEAVEN SHALL BURN es una banda de melodic death metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Heaven Shall Burn es una banda alemana de metal extremo proveniente de Saalfeld, Alemania. Combinan la agresividad del metal con letras antirracistas y contra la injusticia social. Cuatro miembros de la banda son veganos y Straight Edge, siendo Alexander Dietz (guitarra) el único integrante de la banda que no ha adoptado estas ideas. Sin embargo, esto no parece ser motivo de discordia dentro de la misma. Su estilo musical es descrito como una mezcla de death metal melódico y metalcore.</v>
       </c>
       <c r="L146" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M146" t="b">
         <v>1</v>
@@ -6639,10 +6640,10 @@
         <v>https://www.facebook.com/WarCryOficial</v>
       </c>
       <c r="K147" t="str">
-        <v>WARCRY es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>WarCry es una banda de power metal fundada en 2002 en Oviedo (Asturias, España), cuando el vocalista Víctor García y el baterista Alberto Ardines fueron expulsados de Avalanch. Pablo García y Fernando Mon aparecieron como guitarristas invitados en el álbum debut homónimo, pero se hicieron miembros oficiales en 2002 junto con el bajista Álvaro Jardón y el pianista Manuel Ramil. Jardón abandonó la banda a finales de 2003, siendo reemplazado por Roberto García tres meses después.</v>
       </c>
       <c r="L147" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M147" t="b">
         <v>1</v>
@@ -6680,10 +6681,10 @@
         <v>https://www.facebook.com/deathandlegacy</v>
       </c>
       <c r="K148" t="str">
-        <v>DEATH AND LEGACY es una banda de death metal melódico originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Testament (estilizado TestAmenT) es una banda estadounidense de thrash metal de Berkeley, California. Hasta la fecha han publicado trece álbumes de estudio, cuatro álbumes en vivo y seis álbumes recopilatorios, tiene tres discos que entraron en el top-50 en las listas inglesas y en 1999 con el disco The Gathering entró en el top-50 alemán.</v>
       </c>
       <c r="L148" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M148" t="b">
         <v>1</v>
@@ -6721,10 +6722,10 @@
         <v/>
       </c>
       <c r="K149" t="str">
-        <v>LATZEN es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Su Ta Gar es un grupo de heavy metal formado en 1987 en la ciudad de Éibar. En castellano, "Su ta Gar" podría traducirse literalmente como "fuego y llama", pero en realidad es una locución vasca con más de un significado. El significado más importante es similar a otras locuciones como "Jo ta Ke" (una de sus canciones más conocidas) o "buru-belarri", que vienen a usarse en euskera como equivalentes a "Dale duro", "Con ahínco" o "Sin descanso". Sugieren una gran intensidad en la acción y una prolongación en el tiempo, a pesar de toda resistencia o dificultad.</v>
       </c>
       <c r="L149" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M149" t="b">
         <v>1</v>
@@ -6768,7 +6769,7 @@
         <v>2026-07-11</v>
       </c>
       <c r="M150" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -6803,10 +6804,10 @@
         <v>https://www.facebook.com/ten56hq</v>
       </c>
       <c r="K151" t="str">
-        <v>TEN56. es una banda de deathcore originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>ten56. es una banda francesa de deathcore formada en 2020 por el vocalista Aaron Matts tras su salida de Betraying The Martyrs. Junto a Matts, el grupo está compuesto por los guitarristas Quentin Godet y Luka Garotin, el bajo Steeves Hostin y el batería Arnaud Verrier.</v>
       </c>
       <c r="L151" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M151" t="b">
         <v>1</v>
@@ -6844,10 +6845,10 @@
         <v>https://www.facebook.com/halfmeband</v>
       </c>
       <c r="K152" t="str">
-        <v>HALF ME es una banda de metalcore originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Half Me es una banda alemana de metalcore formada en Hamburgo en 2018. Conocidos por un sonido extremadamente denso y agresivo, incorporan elementos de nu metal y deathcore en sus producciones, con letras oscuras y ritmos con gran dinámica.</v>
       </c>
       <c r="L152" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M152" t="b">
         <v>1</v>
@@ -6885,10 +6886,10 @@
         <v>https://www.facebook.com/cabalcph</v>
       </c>
       <c r="K153" t="str">
-        <v>CABAL es una banda de deathcore originaria de Dinamarca. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Cabal es una banda de deathcore y metal extremo originaria de Copenhague, Dinamarca. Formada en 2015, destacan por un sonido brutal que mezcla el peso del deathcore con atmósferas opresivas procedentes del black metal y el sludge.</v>
       </c>
       <c r="L153" t="str">
-        <v>2026-07-11</v>
+        <v>2026-07-12</v>
       </c>
       <c r="M153" t="b">
         <v>1</v>
@@ -6920,19 +6921,19 @@
         <v/>
       </c>
       <c r="I154" t="str">
-        <v/>
+        <v>https://www.instagram.com/rockerizos_</v>
       </c>
       <c r="J154" t="str">
-        <v/>
+        <v>https://www.facebook.com/Rockerazos</v>
       </c>
       <c r="K154" t="str">
-        <v>Rockerizos es una banda de hard rock originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda local burgalesa de hard rock y heavy metal clásico, conocidos por su energía y pasión sobre el escenario.</v>
       </c>
       <c r="L154" t="str">
         <v>2026-07-11</v>
       </c>
       <c r="M154" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -6952,7 +6953,7 @@
         <v>Leyenda alemana de la guitarra, exmiembro de Scorpions y pionero del metal neoclásico.</v>
       </c>
       <c r="F155" t="str">
-        <v>https://www.youtube.com/watch?v=y4velOF3ff8</v>
+        <v>https://www.youtube.com/watch?v=5UgaW0MVqVw</v>
       </c>
       <c r="G155" t="str">
         <v>https://i.scdn.co/image/2526875cb953ea6d353eb5e8787647f9a3cdf0c5</v>
@@ -6961,13 +6962,13 @@
         <v>https://open.spotify.com/artist/2VoP4JXyxNPIoYAFdB5ssQ</v>
       </c>
       <c r="I155" t="str">
-        <v/>
+        <v>https://www.instagram.com/ulijonroth/</v>
       </c>
       <c r="J155" t="str">
         <v>https://www.facebook.com/Uli-Jon-Roth-403059233077097</v>
       </c>
       <c r="K155" t="str">
-        <v>Uli Jon Roth es una banda de heavy metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Leyenda alemana de la guitarra, exmiembro de Scorpions y pionero del metal neoclásico.</v>
       </c>
       <c r="L155" t="str">
         <v>2026-07-11</v>
@@ -6993,16 +6994,16 @@
         <v>Secret Sphere es un grupo de power metal italiano, procedentes de la región de Alessandria. Comenzaron su actividad en el verano de 1997 gracias al talentoso guitarrista Aldo Lonobile. Después de algunos cambios de formación durante los primeros días, la formación actual del grupo grabaron su álbum debut "Mistress Of The Shadowlight" en 1999. En el año 2000 Secret Sphere apareció en prestigioso homenaje a Helloween "Keepers Of Jericho" junto a grandes nombres como Sonata Arctica, Rhapsody, Trick or Treat entre otras.</v>
       </c>
       <c r="F156" t="str">
-        <v>https://www.youtube.com/watch?v=RPy2hKop0y4</v>
+        <v>https://www.youtube.com/watch?v=NOK3sZ5epkU</v>
       </c>
       <c r="G156" t="str">
         <v/>
       </c>
       <c r="H156" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/6RW3PIbCsvSVIB5dzx9MV8</v>
       </c>
       <c r="I156" t="str">
-        <v/>
+        <v>https://www.instagram.com/secretsphere/</v>
       </c>
       <c r="J156" t="str">
         <v>https://www.facebook.com/secretsphere</v>
@@ -7034,22 +7035,22 @@
         <v>Histórica banda granadina de heavy metal y power metal en castellano con más de tres décadas de trayectoria.</v>
       </c>
       <c r="F157" t="str">
-        <v>https://www.youtube.com/watch?v=zSHoeFg-uhQ</v>
+        <v>https://www.youtube.com/watch?v=9BZoM49iEKU</v>
       </c>
       <c r="G157" t="str">
         <v/>
       </c>
       <c r="H157" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/3MbI60af17wgl3P9EXQJQb</v>
       </c>
       <c r="I157" t="str">
-        <v/>
+        <v>https://www.instagram.com/azraelmetaloficial/</v>
       </c>
       <c r="J157" t="str">
-        <v/>
+        <v>https://www.facebook.com/azraelmetalband</v>
       </c>
       <c r="K157" t="str">
-        <v>Azrael es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Histórica banda granadina de heavy metal y power metal en castellano con más de tres décadas de trayectoria.</v>
       </c>
       <c r="L157" t="str">
         <v>2026-07-11</v>
@@ -7075,7 +7076,7 @@
         <v>Potente banda británica de heavy metal clásico con riffs dinámicos y gran puesta en escena.</v>
       </c>
       <c r="F158" t="str">
-        <v>https://www.youtube.com/watch?v=6Bd5LDEJqH4</v>
+        <v>https://www.youtube.com/watch?v=acCkBUtYK68</v>
       </c>
       <c r="G158" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517405e5c32722b5ae52c4f8376b</v>
@@ -7090,7 +7091,7 @@
         <v>https://www.facebook.com/furyofficial</v>
       </c>
       <c r="K158" t="str">
-        <v>Fury es una banda de heavy metal originaria de UK. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Potente banda británica de heavy metal clásico con riffs dinámicos y gran puesta en escena.</v>
       </c>
       <c r="L158" t="str">
         <v>2026-07-11</v>
@@ -7116,22 +7117,22 @@
         <v>Proyecto de power metal comandado por el prestigioso productor Sascha Paeth y el vocalista Tommy Heart.</v>
       </c>
       <c r="F159" t="str">
-        <v>https://www.youtube.com/watch?v=QtpOm5yFxw0</v>
+        <v>https://www.youtube.com/watch?v=cCMc7vZWuAk</v>
       </c>
       <c r="G159" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab67616d00001e02aa45ec1a8328e81af490b4a4</v>
       </c>
       <c r="H159" t="str">
-        <v>https://open.spotify.com/artist/0nKiNlJFtcGhZXZlNkOstJ</v>
+        <v>https://open.spotify.com/intl-es/artist/3z2BhxE5Fn5OaLLPMnXzK8</v>
       </c>
       <c r="I159" t="str">
-        <v/>
+        <v>https://www.instagram.com/mastersofceremony.official/</v>
       </c>
       <c r="J159" t="str">
-        <v/>
+        <v>https://www.facebook.com/saschapaethsmastersofceremony</v>
       </c>
       <c r="K159" t="str">
-        <v>Masters of Ceremony es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Proyecto de power metal comandado por el prestigioso productor Sascha Paeth y el vocalista Tommy Heart.</v>
       </c>
       <c r="L159" t="str">
         <v>2026-07-11</v>
@@ -7163,16 +7164,16 @@
         <v>https://image-cdn-fa.spotifycdn.com/image/ab6761610000517461f85b0265f8496c97063a38</v>
       </c>
       <c r="H160" t="str">
-        <v>https://open.spotify.com/artist/1t20wYnTiAT0Bs7H1hv9Wt</v>
+        <v>https://open.spotify.com/intl-es/artist/4ZCwQot86SbeHASevLgQmr</v>
       </c>
       <c r="I160" t="str">
-        <v>https://www.instagram.com/iameden/</v>
+        <v>https://www.instagram.com/edenmetalband/</v>
       </c>
       <c r="J160" t="str">
-        <v>https://www.facebook.com/iameden</v>
+        <v>https://www.facebook.com/EDENMETALBAND</v>
       </c>
       <c r="K160" t="str">
-        <v>Eden es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Veterana banda asturiana de heavy metal melódico con canciones llenas de épica y fuerza.</v>
       </c>
       <c r="L160" t="str">
         <v>2026-07-11</v>
@@ -7207,13 +7208,13 @@
         <v>https://open.spotify.com/artist/57b3sKD9pGilMb2QlMqArq</v>
       </c>
       <c r="I161" t="str">
-        <v/>
+        <v>https://www.instagram.com/hardcoresuperstarofficial/</v>
       </c>
       <c r="J161" t="str">
         <v>https://www.facebook.com/OfficialHardcoreSuperstar</v>
       </c>
       <c r="K161" t="str">
-        <v>Hardcore Superstar es una banda de sleaze rock originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Referentes indiscutibles del sleaze rock y el hard rock sueco con un directo demoledor.</v>
       </c>
       <c r="L161" t="str">
         <v>2026-07-11</v>
@@ -7254,7 +7255,7 @@
         <v>https://www.facebook.com/savagedheavy</v>
       </c>
       <c r="K162" t="str">
-        <v>Savaged es una banda de speed metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Joven y salvaje promesa barcelonesa de speed y heavy metal tradicional de corte ochentero.</v>
       </c>
       <c r="L162" t="str">
         <v>2026-07-11</v>
@@ -7280,7 +7281,7 @@
         <v>Pioneros indiscutibles del thrash metal estadounidense procedentes de Nueva Jersey.</v>
       </c>
       <c r="F163" t="str">
-        <v>https://www.youtube.com/watch?v=VoMCka5bBdU</v>
+        <v>https://www.youtube.com/watch?v=NZ8XxTkXc2c</v>
       </c>
       <c r="G163" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab6761610000517403cb77f96e45ca6fdb18debe</v>
@@ -7295,7 +7296,7 @@
         <v>https://www.facebook.com/OverkillWreckingCrew</v>
       </c>
       <c r="K163" t="str">
-        <v>Overkill es una banda de thrash metal originaria de EEUU. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Pioneros indiscutibles del thrash metal estadounidense procedentes de Nueva Jersey.</v>
       </c>
       <c r="L163" t="str">
         <v>2026-07-11</v>
@@ -7330,13 +7331,13 @@
         <v>https://open.spotify.com/artist/78LVpk0xhPtf6ptfZjaw5h</v>
       </c>
       <c r="I164" t="str">
-        <v/>
+        <v>https://www.instagram.com/hittenofficial/</v>
       </c>
       <c r="J164" t="str">
-        <v/>
+        <v>https://www.facebook.com/hittenofficial</v>
       </c>
       <c r="K164" t="str">
-        <v>Hitten es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda murciana de heavy metal tradicional, aclamada internacionalmente por su sonido NWOTHM.</v>
       </c>
       <c r="L164" t="str">
         <v>2026-07-11</v>
@@ -7362,7 +7363,7 @@
         <v>Formación de power metal progresivo fundada por Tim Hansen, heredera del sonido clásico del género.</v>
       </c>
       <c r="F165" t="str">
-        <v>https://www.youtube.com/watch?v=Rs1lI8XRFNs</v>
+        <v>https://www.youtube.com/watch?v=3RUweV_Tl3w</v>
       </c>
       <c r="G165" t="str">
         <v>https://image-cdn-ak.spotifycdn.com/image/ab676161000051741bf64d84a5f034bee6855e8e</v>
@@ -7377,7 +7378,7 @@
         <v>https://www.facebook.com/inductionofficial</v>
       </c>
       <c r="K165" t="str">
-        <v>Induction es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Formación de power metal progresivo fundada por Tim Hansen, heredera del sonido clásico del género.</v>
       </c>
       <c r="L165" t="str">
         <v>2026-07-11</v>
@@ -7409,16 +7410,16 @@
         <v/>
       </c>
       <c r="H166" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/77KiwIxgTb2kX0wDMKqnmj</v>
       </c>
       <c r="I166" t="str">
-        <v/>
+        <v>https://www.instagram.com/arsamandirock/</v>
       </c>
       <c r="J166" t="str">
         <v>https://www.facebook.com/ArsAmandiRock</v>
       </c>
       <c r="K166" t="str">
-        <v>Ars Amandi es una banda de folk metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda madrileña pionera del folk metal castellano que fusiona rock pesado con dulzaina y pito castellano.</v>
       </c>
       <c r="L166" t="str">
         <v>2026-07-11</v>
@@ -7459,7 +7460,7 @@
         <v>https://www.facebook.com/profile.php?id=61555780541728</v>
       </c>
       <c r="K167" t="str">
-        <v>Bloodstain es una banda de thrash metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda burgalesa de thrash y death metal con un directo arrollador y riffs contundentes.</v>
       </c>
       <c r="L167" t="str">
         <v>2026-07-11</v>
@@ -7485,22 +7486,22 @@
         <v>Exitoso grupo sueco de glam metal y hard rock melódico con estribillos pegadizos y gran producción.</v>
       </c>
       <c r="F168" t="str">
-        <v>https://www.youtube.com/watch?v=pvqarSnBQN8</v>
+        <v>https://www.youtube.com/watch?v=8XQorbAqzVg</v>
       </c>
       <c r="G168" t="str">
         <v/>
       </c>
       <c r="H168" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/56qqwnRK5BjH8okTscHtY9</v>
       </c>
       <c r="I168" t="str">
-        <v/>
+        <v>https://www.instagram.com/the_poodles_sweden/</v>
       </c>
       <c r="J168" t="str">
         <v>https://www.facebook.com/thepoodles</v>
       </c>
       <c r="K168" t="str">
-        <v>The Poodles es una banda de glam metal originaria de Suecia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Exitoso grupo sueco de glam metal y hard rock melódico con estribillos pegadizos y gran producción.</v>
       </c>
       <c r="L168" t="str">
         <v>2026-07-11</v>
@@ -7526,22 +7527,22 @@
         <v>Banda de metal alternativo y metalcore procedente de Burgos con letras reflexivas y bases pesadas.</v>
       </c>
       <c r="F169" t="str">
-        <v>https://www.youtube.com/watch?v=Y__C9IKkEz4</v>
+        <v>https://www.youtube.com/watch?v=JgIuDD4_s80</v>
       </c>
       <c r="G169" t="str">
         <v/>
       </c>
       <c r="H169" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/4zDokiOegUyKQI68NsajnP</v>
       </c>
       <c r="I169" t="str">
-        <v/>
+        <v>https://www.instagram.com/khoreaband/</v>
       </c>
       <c r="J169" t="str">
-        <v/>
+        <v>https://www.facebook.com/profile.php?id=61571130271291&amp;locale=es_ES</v>
       </c>
       <c r="K169" t="str">
-        <v>Khorea es una banda de metalcore originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda de metal alternativo y metalcore procedente de Burgos con letras reflexivas y bases pesadas.</v>
       </c>
       <c r="L169" t="str">
         <v>2026-07-11</v>
@@ -7567,22 +7568,22 @@
         <v>Legendaria formación alemana de power metal de finales de los 80, muy influyente en el género.</v>
       </c>
       <c r="F170" t="str">
-        <v>https://www.youtube.com/watch?v=kYJvM9e2V34</v>
+        <v>https://www.youtube.com/watch?v=GFOCqLAKiTc</v>
       </c>
       <c r="G170" t="str">
         <v/>
       </c>
       <c r="H170" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/4bJlNp8kcrWMSIM4NObk2D</v>
       </c>
       <c r="I170" t="str">
         <v/>
       </c>
       <c r="J170" t="str">
-        <v/>
+        <v>https://www.facebook.com/heavensgatemetal</v>
       </c>
       <c r="K170" t="str">
-        <v>Heavens Gate es una banda de power metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Legendaria formación alemana de power metal de finales de los 80, muy influyente en el género.</v>
       </c>
       <c r="L170" t="str">
         <v>2026-07-11</v>
@@ -7608,7 +7609,7 @@
         <v>Moderno cuarteto parisino que combina metal alternativo, rock melódico y matices electrónicos.</v>
       </c>
       <c r="F171" t="str">
-        <v>https://www.youtube.com/watch?v=A2WpC9Uo3S8</v>
+        <v>https://www.youtube.com/watch?v=DRqJdqpjXnM</v>
       </c>
       <c r="G171" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab67616100005174510624ce3ecb6e7d0bdb7d09</v>
@@ -7623,7 +7624,7 @@
         <v>https://www.facebook.com/ODCOfficiel</v>
       </c>
       <c r="K171" t="str">
-        <v>ODC es una banda de metal alternativo originaria de Francia. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Moderno cuarteto parisino que combina metal alternativo, rock melódico y matices electrónicos.</v>
       </c>
       <c r="L171" t="str">
         <v>2026-07-11</v>
@@ -7649,7 +7650,7 @@
         <v>Dorothee Pesch, más conocida por su nombre artístico Doro Pesch (Düsseldorf; 3 de junio de 1964), es una cantante de heavy metal alemana.​ Formó parte de las agrupaciones Warlock y Snakebite y se desempeña como solista. Fue una de las primeras cantantes de metal en los años 1980, cuando los hombres dominaban este tipo de música. Se la considera la indiscutible Reina del Metal a nivel mundial, habiendo inspirado a múltiples generaciones.</v>
       </c>
       <c r="F172" t="str">
-        <v>https://www.youtube.com/watch?v=kH3Ml0jiPFA</v>
+        <v>https://www.youtube.com/watch?v=A857YBw8u30</v>
       </c>
       <c r="G172" t="str">
         <v>https://image-cdn-fa.spotifycdn.com/image/ab676161000051740f0c71fd8ca7477c0a7de478</v>
@@ -7664,7 +7665,7 @@
         <v>https://www.facebook.com/DoroPeschOfficialGerman</v>
       </c>
       <c r="K172" t="str">
-        <v>Doro es una banda de heavy metal originaria de Alemania. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Dorothee Pesch, más conocida por su nombre artístico Doro Pesch (Düsseldorf; 3 de junio de 1964), es una cantante de heavy metal alemana.​ Formó parte de las agrupaciones Warlock y Snakebite y se desempeña como solista. Fue una de las primeras cantantes de metal en los años 1980, cuando los hombres dominaban este tipo de música. Se la considera la indiscutible Reina del Metal a nivel mundial, habiendo inspirado a múltiples generaciones.</v>
       </c>
       <c r="L172" t="str">
         <v>2026-07-11</v>
@@ -7731,22 +7732,22 @@
         <v>Banda española de heavy metal tradicional con letras combativas y sonido de la vieja escuela.</v>
       </c>
       <c r="F174" t="str">
-        <v>https://www.youtube.com/watch?v=D0w_NZodwX4</v>
+        <v>https://www.youtube.com/watch?v=82fuY5yiXRA</v>
       </c>
       <c r="G174" t="str">
         <v/>
       </c>
       <c r="H174" t="str">
-        <v/>
+        <v>https://open.spotify.com/intl-es/artist/2ts6YtBKLFEySkArj0lyR5</v>
       </c>
       <c r="I174" t="str">
-        <v/>
+        <v>https://www.instagram.com/officialvindicta</v>
       </c>
       <c r="J174" t="str">
-        <v/>
+        <v>https://www.facebook.com/officialvindictaband</v>
       </c>
       <c r="K174" t="str">
-        <v>Vindicta es una banda de heavy metal originaria de España. Cuenta con una destacada trayectoria en la escena musical alternativa, habiendo editado diversos trabajos discográficos y girado extensamente compartiendo su música con sus seguidores a nivel internacional.</v>
+        <v>Banda española de heavy metal tradicional con letras combativas y sonido de la vieja escuela.</v>
       </c>
       <c r="L174" t="str">
         <v>2026-07-11</v>
@@ -11726,6 +11727,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G175"/>
   </ignoredErrors>
@@ -12136,6 +12138,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>

</xml_diff>